<commit_message>
58013 - updating the code to match the newest version of ASC prompt, 57387 - implementing the changes for inexistent VRCC even though it is marked present on the ICW and IAQ (the changes are tested, but commented out until DU for IAQ is in Prod)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606F359C-1347-44CC-AE74-0BE416A3A6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB68463C-445B-4128-A2BE-6C3B9B8E2D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28200" windowHeight="13530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28200" windowHeight="13530" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="745">
   <si>
     <t>Name</t>
   </si>
@@ -2269,6 +2269,12 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>VRCCDoesNotExist</t>
+  </si>
+  <si>
+    <t>The Recurring Cash Contributions check is marked as “Yes” on the IAQ and listed on the ICW, but no VRCC is present in the application.</t>
   </si>
 </sst>
 </file>
@@ -6917,7 +6923,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C298"/>
+  <dimension ref="A1:C299"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -9253,60 +9259,71 @@
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>432</v>
+        <v>743</v>
       </c>
       <c r="B292" t="s">
-        <v>623</v>
+        <v>744</v>
+      </c>
+      <c r="C292" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B293" t="s">
-        <v>624</v>
-      </c>
-      <c r="C293" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>511</v>
+        <v>433</v>
       </c>
       <c r="B294" t="s">
-        <v>625</v>
+        <v>624</v>
+      </c>
+      <c r="C294" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>434</v>
+        <v>511</v>
       </c>
       <c r="B295" t="s">
-        <v>651</v>
+        <v>625</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B296" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B297" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
+        <v>436</v>
+      </c>
+      <c r="B298" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3">
+      <c r="A299" t="s">
         <v>528</v>
       </c>
-      <c r="B298" t="s">
+      <c r="B299" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating the code for 57387 - changes for income types listed on the IAQ that do not appear in the application, 57814 - Tax Refund check for ASC and ASCWorksheet, 57800 - adding a finding in case sum of cash values is not hte same on both ASC and ASCWorksheet.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB68463C-445B-4128-A2BE-6C3B9B8E2D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C4B63F-A7CD-41EC-AA26-53FD0844B7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28200" windowHeight="13530" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22440" windowHeight="11715" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="756">
   <si>
     <t>Name</t>
   </si>
@@ -2274,7 +2274,40 @@
     <t>VRCCDoesNotExist</t>
   </si>
   <si>
-    <t>The Recurring Cash Contributions check is marked as “Yes” on the IAQ and listed on the ICW, but no VRCC is present in the application.</t>
+    <t>Supporting documents have not been provided for Verification of Recurring Cash Contributions documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>SSBLDoesNotExist</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for Social Security Benefits Letter documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>SECDoesNotExist</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for Self Employment Certification documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>CSCDoesNotExist</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for EmployeeWages/Salary income type documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>IAQ_EWSDocsCheck</t>
+  </si>
+  <si>
+    <t>ASC_FederalTaxCheck</t>
+  </si>
+  <si>
+    <t>Tax Refund listed on Asset Self-Certification and Asset Self-Certification Worksheet do not match.</t>
+  </si>
+  <si>
+    <t>Sum of assets listed on Asset Self-Certification do not match Asset Self-Certification Worksheet.</t>
+  </si>
+  <si>
+    <t>ASC_SumOfAssetsCheck</t>
   </si>
 </sst>
 </file>
@@ -6923,7 +6956,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C299"/>
+  <dimension ref="A1:C306"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -7427,130 +7460,130 @@
         <v>670</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
-      <c r="A64" t="s">
-        <v>158</v>
-      </c>
-      <c r="B64" t="s">
-        <v>121</v>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>751</v>
+      </c>
+      <c r="B63" t="s">
+        <v>750</v>
+      </c>
+      <c r="C63" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>122</v>
+        <v>158</v>
       </c>
       <c r="B65" t="s">
-        <v>594</v>
+        <v>121</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B66" t="s">
-        <v>123</v>
+        <v>594</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>635</v>
+        <v>124</v>
       </c>
       <c r="B67" t="s">
-        <v>636</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>635</v>
+      </c>
+      <c r="B68" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
         <v>543</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B69" t="s">
         <v>671</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" t="s">
-        <v>186</v>
-      </c>
-      <c r="B70" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>125</v>
+        <v>186</v>
       </c>
       <c r="B71" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B73" t="s">
-        <v>595</v>
+        <v>128</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B74" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B75" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B76" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>495</v>
-      </c>
-      <c r="C77" t="s">
-        <v>686</v>
+        <v>598</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B78" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C78" t="s">
-        <v>556</v>
+        <v>686</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C79" t="s">
         <v>556</v>
@@ -7558,395 +7591,401 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>637</v>
+        <v>144</v>
       </c>
       <c r="B80" t="s">
-        <v>638</v>
+        <v>498</v>
+      </c>
+      <c r="C80" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>542</v>
+        <v>637</v>
       </c>
       <c r="B81" t="s">
-        <v>672</v>
+        <v>638</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
+        <v>542</v>
+      </c>
+      <c r="B82" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" t="s">
         <v>719</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" t="s">
         <v>720</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C83" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>147</v>
+        <v>752</v>
       </c>
       <c r="B84" t="s">
-        <v>150</v>
+        <v>753</v>
+      </c>
+      <c r="C84" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>148</v>
+        <v>755</v>
       </c>
       <c r="B85" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3">
-      <c r="A86" t="s">
-        <v>149</v>
-      </c>
-      <c r="B86" t="s">
-        <v>152</v>
+        <v>754</v>
+      </c>
+      <c r="C85" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B87" t="s">
-        <v>580</v>
-      </c>
-      <c r="C87" t="s">
-        <v>691</v>
+        <v>150</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>690</v>
+        <v>148</v>
       </c>
       <c r="B88" t="s">
-        <v>580</v>
+        <v>151</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B89" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B90" t="s">
-        <v>599</v>
+        <v>580</v>
+      </c>
+      <c r="C90" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>132</v>
+        <v>690</v>
       </c>
       <c r="B91" t="s">
-        <v>130</v>
+        <v>580</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>639</v>
+        <v>146</v>
       </c>
       <c r="B92" t="s">
-        <v>640</v>
+        <v>129</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>541</v>
+        <v>131</v>
       </c>
       <c r="B93" t="s">
-        <v>673</v>
+        <v>599</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>132</v>
+      </c>
+      <c r="B94" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>188</v>
+        <v>639</v>
       </c>
       <c r="B95" t="s">
-        <v>189</v>
+        <v>640</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>133</v>
+        <v>541</v>
       </c>
       <c r="B96" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3">
-      <c r="A97" t="s">
-        <v>135</v>
-      </c>
-      <c r="B97" t="s">
-        <v>154</v>
+        <v>673</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>134</v>
+        <v>188</v>
       </c>
       <c r="B98" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B99" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B100" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>629</v>
+        <v>134</v>
       </c>
       <c r="B101" t="s">
-        <v>695</v>
-      </c>
-      <c r="C101" t="s">
-        <v>699</v>
+        <v>155</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>641</v>
+        <v>136</v>
       </c>
       <c r="B102" t="s">
-        <v>642</v>
+        <v>156</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>540</v>
+        <v>137</v>
       </c>
       <c r="B103" t="s">
-        <v>674</v>
+        <v>157</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>721</v>
+        <v>629</v>
       </c>
       <c r="B104" t="s">
-        <v>722</v>
+        <v>695</v>
       </c>
       <c r="C104" t="s">
-        <v>692</v>
+        <v>699</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" t="s">
+        <v>641</v>
+      </c>
+      <c r="B105" t="s">
+        <v>642</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>710</v>
+        <v>540</v>
       </c>
       <c r="B106" t="s">
-        <v>711</v>
-      </c>
-      <c r="C106" t="s">
-        <v>712</v>
+        <v>674</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="B107" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="C107" t="s">
-        <v>712</v>
+        <v>692</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>710</v>
       </c>
       <c r="B109" t="s">
-        <v>163</v>
+        <v>711</v>
+      </c>
+      <c r="C109" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>713</v>
       </c>
       <c r="B110" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3">
-      <c r="A111" t="s">
-        <v>161</v>
-      </c>
-      <c r="B111" t="s">
-        <v>165</v>
+        <v>714</v>
+      </c>
+      <c r="C110" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B112" t="s">
-        <v>600</v>
+        <v>163</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>557</v>
+        <v>160</v>
       </c>
       <c r="B113" t="s">
-        <v>739</v>
-      </c>
-      <c r="C113" t="s">
-        <v>740</v>
+        <v>164</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>647</v>
+        <v>161</v>
       </c>
       <c r="B114" t="s">
-        <v>648</v>
+        <v>165</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>539</v>
+        <v>162</v>
       </c>
       <c r="B115" t="s">
-        <v>675</v>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" t="s">
+        <v>557</v>
+      </c>
+      <c r="B116" t="s">
+        <v>739</v>
+      </c>
+      <c r="C116" t="s">
+        <v>740</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>192</v>
+        <v>647</v>
       </c>
       <c r="B117" t="s">
-        <v>193</v>
+        <v>648</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>166</v>
+        <v>539</v>
       </c>
       <c r="B118" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3">
-      <c r="A119" t="s">
-        <v>167</v>
-      </c>
-      <c r="B119" t="s">
-        <v>169</v>
+        <v>675</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>643</v>
+        <v>192</v>
       </c>
       <c r="B120" t="s">
-        <v>644</v>
+        <v>193</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>538</v>
+        <v>166</v>
       </c>
       <c r="B121" t="s">
-        <v>676</v>
+        <v>168</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>723</v>
+        <v>167</v>
       </c>
       <c r="B122" t="s">
-        <v>724</v>
-      </c>
-      <c r="C122" t="s">
-        <v>692</v>
+        <v>169</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" t="s">
+        <v>643</v>
+      </c>
+      <c r="B123" t="s">
+        <v>644</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>190</v>
+        <v>538</v>
       </c>
       <c r="B124" t="s">
-        <v>191</v>
+        <v>676</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>723</v>
       </c>
       <c r="B125" t="s">
-        <v>172</v>
+        <v>724</v>
       </c>
       <c r="C125" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3">
-      <c r="A126" t="s">
-        <v>170</v>
-      </c>
-      <c r="B126" t="s">
-        <v>173</v>
-      </c>
-      <c r="C126" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="B127" t="s">
-        <v>174</v>
-      </c>
-      <c r="C127" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>203</v>
+        <v>175</v>
       </c>
       <c r="B128" t="s">
-        <v>202</v>
+        <v>172</v>
+      </c>
+      <c r="C128" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B129" t="s">
-        <v>201</v>
+        <v>173</v>
+      </c>
+      <c r="C129" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B130" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C130" t="s">
         <v>588</v>
@@ -7954,1038 +7993,1044 @@
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>645</v>
+        <v>203</v>
       </c>
       <c r="B131" t="s">
-        <v>646</v>
+        <v>202</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>527</v>
+        <v>200</v>
       </c>
       <c r="B132" t="s">
-        <v>677</v>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3">
+      <c r="A133" t="s">
+        <v>176</v>
+      </c>
+      <c r="B133" t="s">
+        <v>177</v>
+      </c>
+      <c r="C133" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="B134" t="s">
-        <v>653</v>
-      </c>
-      <c r="C134" t="s">
-        <v>654</v>
+        <v>646</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>727</v>
+        <v>527</v>
       </c>
       <c r="B135" t="s">
-        <v>728</v>
-      </c>
-      <c r="C135" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" t="s">
-        <v>733</v>
-      </c>
-      <c r="B136" t="s">
-        <v>734</v>
-      </c>
-      <c r="C136" t="s">
-        <v>692</v>
+        <v>677</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>741</v>
+        <v>652</v>
       </c>
       <c r="B137" t="s">
-        <v>730</v>
+        <v>653</v>
       </c>
       <c r="C137" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" t="s">
+        <v>727</v>
+      </c>
+      <c r="B138" t="s">
+        <v>728</v>
+      </c>
+      <c r="C138" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>513</v>
+        <v>733</v>
       </c>
       <c r="B139" t="s">
-        <v>514</v>
+        <v>734</v>
+      </c>
+      <c r="C139" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>661</v>
+        <v>741</v>
       </c>
       <c r="B140" t="s">
-        <v>665</v>
+        <v>730</v>
       </c>
       <c r="C140" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3">
-      <c r="A141" t="s">
-        <v>662</v>
-      </c>
-      <c r="B141" t="s">
-        <v>664</v>
-      </c>
-      <c r="C141" t="s">
-        <v>663</v>
+        <v>692</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>242</v>
+        <v>513</v>
       </c>
       <c r="B142" t="s">
-        <v>243</v>
-      </c>
-      <c r="C142" t="s">
-        <v>588</v>
+        <v>514</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>244</v>
+        <v>661</v>
       </c>
       <c r="B143" t="s">
-        <v>245</v>
+        <v>665</v>
+      </c>
+      <c r="C143" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>258</v>
+        <v>662</v>
       </c>
       <c r="B144" t="s">
-        <v>560</v>
+        <v>664</v>
       </c>
       <c r="C144" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B145" t="s">
-        <v>246</v>
+        <v>243</v>
+      </c>
+      <c r="C145" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>503</v>
+        <v>244</v>
       </c>
       <c r="B146" t="s">
-        <v>512</v>
+        <v>245</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B147" t="s">
-        <v>248</v>
+        <v>560</v>
+      </c>
+      <c r="C147" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B148" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>251</v>
+        <v>503</v>
       </c>
       <c r="B149" t="s">
-        <v>253</v>
+        <v>512</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B150" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B151" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>302</v>
+        <v>251</v>
       </c>
       <c r="B152" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>349</v>
+        <v>255</v>
       </c>
       <c r="B153" t="s">
-        <v>350</v>
+        <v>254</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>657</v>
+        <v>257</v>
       </c>
       <c r="B154" t="s">
-        <v>658</v>
+        <v>256</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>702</v>
+        <v>302</v>
       </c>
       <c r="B155" t="s">
-        <v>703</v>
+        <v>248</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>526</v>
+        <v>349</v>
       </c>
       <c r="B156" t="s">
-        <v>678</v>
+        <v>350</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" t="s">
+        <v>657</v>
+      </c>
+      <c r="B157" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>515</v>
+        <v>702</v>
       </c>
       <c r="B158" t="s">
-        <v>516</v>
+        <v>703</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>259</v>
+        <v>526</v>
       </c>
       <c r="B159" t="s">
-        <v>262</v>
-      </c>
-      <c r="C159" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A160" t="s">
-        <v>261</v>
-      </c>
-      <c r="B160" t="s">
-        <v>561</v>
-      </c>
-      <c r="C160" t="s">
-        <v>696</v>
+        <v>678</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>260</v>
+        <v>515</v>
       </c>
       <c r="B161" t="s">
-        <v>263</v>
+        <v>516</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B162" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C162" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" ht="13.5" customHeight="1">
       <c r="A163" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B163" t="s">
-        <v>267</v>
+        <v>561</v>
+      </c>
+      <c r="C163" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B164" t="s">
-        <v>268</v>
-      </c>
-      <c r="C164" t="s">
-        <v>660</v>
+        <v>263</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>504</v>
+        <v>265</v>
       </c>
       <c r="B165" t="s">
-        <v>570</v>
+        <v>264</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B166" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B167" t="s">
-        <v>273</v>
+        <v>268</v>
+      </c>
+      <c r="C167" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>277</v>
+        <v>504</v>
       </c>
       <c r="B168" t="s">
-        <v>287</v>
+        <v>570</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="B169" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B170" t="s">
-        <v>285</v>
-      </c>
-      <c r="C170" t="s">
-        <v>660</v>
+        <v>273</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B171" t="s">
-        <v>605</v>
+        <v>287</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B172" t="s">
-        <v>284</v>
-      </c>
-      <c r="C172" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B173" t="s">
-        <v>283</v>
+        <v>285</v>
+      </c>
+      <c r="C173" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="B174" t="s">
-        <v>300</v>
+        <v>605</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="B175" t="s">
-        <v>248</v>
+        <v>284</v>
+      </c>
+      <c r="C175" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="B176" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>704</v>
+        <v>299</v>
       </c>
       <c r="B177" t="s">
-        <v>703</v>
+        <v>300</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>537</v>
+        <v>301</v>
       </c>
       <c r="B178" t="s">
-        <v>679</v>
+        <v>248</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>697</v>
+        <v>304</v>
       </c>
       <c r="B179" t="s">
-        <v>698</v>
-      </c>
-      <c r="C179" t="s">
-        <v>692</v>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3">
+      <c r="A180" t="s">
+        <v>704</v>
+      </c>
+      <c r="B180" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>517</v>
+        <v>537</v>
       </c>
       <c r="B181" t="s">
-        <v>518</v>
+        <v>679</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>292</v>
+        <v>697</v>
       </c>
       <c r="B182" t="s">
-        <v>296</v>
+        <v>698</v>
       </c>
       <c r="C182" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3">
-      <c r="A183" t="s">
-        <v>505</v>
-      </c>
-      <c r="B183" t="s">
-        <v>571</v>
+        <v>692</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>293</v>
+        <v>517</v>
       </c>
       <c r="B184" t="s">
-        <v>297</v>
-      </c>
-      <c r="C184" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B185" t="s">
-        <v>298</v>
+        <v>296</v>
+      </c>
+      <c r="C185" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>295</v>
+        <v>505</v>
       </c>
       <c r="B186" t="s">
-        <v>562</v>
+        <v>571</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B187" t="s">
-        <v>248</v>
+        <v>297</v>
+      </c>
+      <c r="C187" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="B188" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="B189" t="s">
-        <v>308</v>
+        <v>562</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B190" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B191" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>705</v>
+        <v>306</v>
       </c>
       <c r="B192" t="s">
-        <v>703</v>
+        <v>308</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>536</v>
+        <v>307</v>
       </c>
       <c r="B193" t="s">
-        <v>680</v>
+        <v>308</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3">
+      <c r="A194" t="s">
+        <v>311</v>
+      </c>
+      <c r="B194" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>519</v>
+        <v>705</v>
       </c>
       <c r="B195" t="s">
-        <v>520</v>
+        <v>703</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>499</v>
+        <v>536</v>
       </c>
       <c r="B196" t="s">
-        <v>320</v>
-      </c>
-      <c r="C196" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3">
-      <c r="A197" t="s">
-        <v>506</v>
-      </c>
-      <c r="B197" t="s">
-        <v>572</v>
+        <v>680</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>315</v>
+        <v>519</v>
       </c>
       <c r="B198" t="s">
-        <v>321</v>
-      </c>
-      <c r="C198" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>316</v>
+        <v>499</v>
       </c>
       <c r="B199" t="s">
-        <v>322</v>
+        <v>320</v>
+      </c>
+      <c r="C199" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>317</v>
+        <v>506</v>
       </c>
       <c r="B200" t="s">
-        <v>323</v>
+        <v>572</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B201" t="s">
-        <v>563</v>
+        <v>321</v>
+      </c>
+      <c r="C201" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B202" t="s">
-        <v>248</v>
+        <v>322</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="B203" t="s">
-        <v>325</v>
-      </c>
-      <c r="C203" t="s">
-        <v>588</v>
+        <v>323</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="B204" t="s">
-        <v>327</v>
+        <v>563</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="B205" t="s">
-        <v>328</v>
+        <v>248</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="B206" t="s">
-        <v>331</v>
+        <v>325</v>
+      </c>
+      <c r="C206" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="B207" t="s">
-        <v>256</v>
+        <v>327</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>706</v>
+        <v>329</v>
       </c>
       <c r="B208" t="s">
-        <v>703</v>
+        <v>328</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>535</v>
+        <v>330</v>
       </c>
       <c r="B209" t="s">
-        <v>681</v>
+        <v>331</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3">
+      <c r="A210" t="s">
+        <v>332</v>
+      </c>
+      <c r="B210" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>521</v>
+        <v>706</v>
       </c>
       <c r="B211" t="s">
-        <v>522</v>
+        <v>703</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>501</v>
+        <v>535</v>
       </c>
       <c r="B212" t="s">
-        <v>338</v>
-      </c>
-      <c r="C212" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3">
-      <c r="A213" t="s">
-        <v>507</v>
-      </c>
-      <c r="B213" t="s">
-        <v>573</v>
+        <v>681</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>336</v>
+        <v>521</v>
       </c>
       <c r="B214" t="s">
-        <v>339</v>
-      </c>
-      <c r="C214" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>337</v>
+        <v>501</v>
       </c>
       <c r="B215" t="s">
-        <v>340</v>
+        <v>338</v>
+      </c>
+      <c r="C215" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="B216" t="s">
-        <v>564</v>
+        <v>573</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="B217" t="s">
-        <v>248</v>
+        <v>339</v>
+      </c>
+      <c r="C217" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="B218" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>346</v>
+        <v>500</v>
       </c>
       <c r="B219" t="s">
-        <v>342</v>
+        <v>564</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B220" t="s">
-        <v>343</v>
+        <v>248</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B221" t="s">
-        <v>256</v>
+        <v>341</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>707</v>
+        <v>346</v>
       </c>
       <c r="B222" t="s">
-        <v>703</v>
+        <v>342</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>534</v>
+        <v>347</v>
       </c>
       <c r="B223" t="s">
-        <v>682</v>
+        <v>343</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3">
+      <c r="A224" t="s">
+        <v>348</v>
+      </c>
+      <c r="B224" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>551</v>
+        <v>707</v>
       </c>
       <c r="B225" t="s">
-        <v>554</v>
-      </c>
-      <c r="C225" t="s">
-        <v>586</v>
+        <v>703</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>552</v>
+        <v>534</v>
       </c>
       <c r="B226" t="s">
-        <v>553</v>
-      </c>
-      <c r="C226" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="227" spans="1:3">
-      <c r="A227" t="s">
-        <v>585</v>
-      </c>
-      <c r="B227" t="s">
-        <v>601</v>
+        <v>682</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>365</v>
+        <v>747</v>
       </c>
       <c r="B228" t="s">
-        <v>351</v>
+        <v>748</v>
+      </c>
+      <c r="C228" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>366</v>
+        <v>551</v>
       </c>
       <c r="B229" t="s">
-        <v>352</v>
+        <v>554</v>
       </c>
       <c r="C229" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>508</v>
+        <v>552</v>
       </c>
       <c r="B230" t="s">
-        <v>574</v>
+        <v>553</v>
+      </c>
+      <c r="C230" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>367</v>
+        <v>585</v>
       </c>
       <c r="B231" t="s">
-        <v>353</v>
+        <v>601</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B232" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B233" t="s">
-        <v>355</v>
+        <v>352</v>
+      </c>
+      <c r="C233" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>370</v>
+        <v>508</v>
       </c>
       <c r="B234" t="s">
-        <v>356</v>
-      </c>
-      <c r="C234" t="s">
-        <v>588</v>
+        <v>574</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B235" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B236" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B237" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B238" t="s">
-        <v>360</v>
+        <v>356</v>
+      </c>
+      <c r="C238" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B239" t="s">
-        <v>361</v>
-      </c>
-      <c r="C239" t="s">
-        <v>588</v>
+        <v>357</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B240" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B241" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B242" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>533</v>
+        <v>375</v>
       </c>
       <c r="B243" t="s">
-        <v>666</v>
+        <v>361</v>
+      </c>
+      <c r="C243" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3">
+      <c r="A244" t="s">
+        <v>376</v>
+      </c>
+      <c r="B244" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>606</v>
+        <v>377</v>
       </c>
       <c r="B245" t="s">
-        <v>607</v>
+        <v>363</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B246" t="s">
-        <v>403</v>
+        <v>364</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>386</v>
+        <v>533</v>
       </c>
       <c r="B247" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="248" spans="1:3">
-      <c r="A248" t="s">
-        <v>387</v>
-      </c>
-      <c r="B248" t="s">
-        <v>401</v>
-      </c>
-      <c r="C248" t="s">
-        <v>588</v>
+        <v>666</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>509</v>
+        <v>606</v>
       </c>
       <c r="B249" t="s">
-        <v>575</v>
+        <v>607</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>404</v>
+        <v>385</v>
       </c>
       <c r="B250" t="s">
-        <v>402</v>
-      </c>
-      <c r="C250" t="s">
-        <v>588</v>
+        <v>403</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B251" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>405</v>
+        <v>387</v>
       </c>
       <c r="B252" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C252" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>389</v>
+        <v>509</v>
       </c>
       <c r="B253" t="s">
-        <v>396</v>
+        <v>575</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="B254" t="s">
-        <v>397</v>
+        <v>402</v>
+      </c>
+      <c r="C254" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B255" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="B256" t="s">
-        <v>399</v>
+        <v>395</v>
+      </c>
+      <c r="C256" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="B257" t="s">
         <v>396</v>
@@ -8993,337 +9038,391 @@
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>532</v>
+        <v>391</v>
       </c>
       <c r="B258" t="s">
-        <v>683</v>
+        <v>397</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3">
+      <c r="A259" t="s">
+        <v>390</v>
+      </c>
+      <c r="B259" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>523</v>
+        <v>392</v>
       </c>
       <c r="B260" t="s">
-        <v>524</v>
+        <v>399</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>411</v>
+        <v>393</v>
       </c>
       <c r="B261" t="s">
-        <v>422</v>
+        <v>396</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>412</v>
+        <v>532</v>
       </c>
       <c r="B262" t="s">
-        <v>423</v>
-      </c>
-      <c r="C262" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3">
-      <c r="A263" t="s">
-        <v>576</v>
-      </c>
-      <c r="B263" t="s">
-        <v>577</v>
+        <v>683</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>413</v>
+        <v>749</v>
       </c>
       <c r="B264" t="s">
-        <v>424</v>
+        <v>746</v>
       </c>
       <c r="C264" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="265" spans="1:3">
-      <c r="A265" t="s">
-        <v>414</v>
-      </c>
-      <c r="B265" t="s">
-        <v>425</v>
-      </c>
-      <c r="C265" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>415</v>
+        <v>745</v>
       </c>
       <c r="B266" t="s">
-        <v>589</v>
+        <v>746</v>
+      </c>
+      <c r="C266" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>416</v>
+        <v>523</v>
       </c>
       <c r="B267" t="s">
-        <v>426</v>
+        <v>524</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="B268" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="B269" t="s">
-        <v>428</v>
+        <v>423</v>
+      </c>
+      <c r="C269" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>419</v>
+        <v>576</v>
       </c>
       <c r="B270" t="s">
-        <v>429</v>
+        <v>577</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="B271" t="s">
-        <v>430</v>
+        <v>424</v>
+      </c>
+      <c r="C271" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="B272" t="s">
-        <v>431</v>
+        <v>425</v>
+      </c>
+      <c r="C272" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>530</v>
+        <v>415</v>
       </c>
       <c r="B273" t="s">
-        <v>684</v>
+        <v>589</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>615</v>
+        <v>416</v>
       </c>
       <c r="B274" t="s">
-        <v>616</v>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3">
+      <c r="A275" t="s">
+        <v>417</v>
+      </c>
+      <c r="B275" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>525</v>
+        <v>418</v>
       </c>
       <c r="B276" t="s">
-        <v>524</v>
+        <v>428</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>438</v>
+        <v>419</v>
       </c>
       <c r="B277" t="s">
-        <v>449</v>
+        <v>429</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>439</v>
+        <v>420</v>
       </c>
       <c r="B278" t="s">
-        <v>450</v>
-      </c>
-      <c r="C278" t="s">
-        <v>588</v>
+        <v>430</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>510</v>
+        <v>421</v>
       </c>
       <c r="B279" t="s">
-        <v>578</v>
+        <v>431</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>440</v>
+        <v>530</v>
       </c>
       <c r="B280" t="s">
-        <v>451</v>
-      </c>
-      <c r="C280" t="s">
-        <v>588</v>
+        <v>684</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>441</v>
+        <v>615</v>
       </c>
       <c r="B281" t="s">
-        <v>452</v>
-      </c>
-      <c r="C281" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="282" spans="1:3">
-      <c r="A282" t="s">
-        <v>442</v>
-      </c>
-      <c r="B282" t="s">
-        <v>590</v>
+        <v>616</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>443</v>
+        <v>525</v>
       </c>
       <c r="B283" t="s">
-        <v>426</v>
+        <v>524</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="B284" t="s">
-        <v>427</v>
+        <v>449</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="B285" t="s">
-        <v>453</v>
+        <v>450</v>
+      </c>
+      <c r="C285" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>446</v>
+        <v>510</v>
       </c>
       <c r="B286" t="s">
-        <v>454</v>
+        <v>578</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="B287" t="s">
-        <v>430</v>
+        <v>451</v>
+      </c>
+      <c r="C287" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="B288" t="s">
-        <v>431</v>
+        <v>452</v>
+      </c>
+      <c r="C288" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>529</v>
+        <v>442</v>
       </c>
       <c r="B289" t="s">
-        <v>684</v>
+        <v>590</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>622</v>
+        <v>443</v>
       </c>
       <c r="B290" t="s">
-        <v>616</v>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3">
+      <c r="A291" t="s">
+        <v>444</v>
+      </c>
+      <c r="B291" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>743</v>
+        <v>445</v>
       </c>
       <c r="B292" t="s">
-        <v>744</v>
-      </c>
-      <c r="C292" t="s">
-        <v>692</v>
+        <v>453</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>432</v>
+        <v>446</v>
       </c>
       <c r="B293" t="s">
-        <v>623</v>
+        <v>454</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
       <c r="B294" t="s">
-        <v>624</v>
-      </c>
-      <c r="C294" t="s">
-        <v>588</v>
+        <v>430</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>511</v>
+        <v>448</v>
       </c>
       <c r="B295" t="s">
-        <v>625</v>
+        <v>431</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>434</v>
+        <v>529</v>
       </c>
       <c r="B296" t="s">
-        <v>651</v>
+        <v>684</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>435</v>
+        <v>622</v>
       </c>
       <c r="B297" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3">
-      <c r="A298" t="s">
-        <v>436</v>
-      </c>
-      <c r="B298" t="s">
-        <v>627</v>
+        <v>616</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
+        <v>743</v>
+      </c>
+      <c r="B299" t="s">
+        <v>744</v>
+      </c>
+      <c r="C299" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3">
+      <c r="A300" t="s">
+        <v>432</v>
+      </c>
+      <c r="B300" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3">
+      <c r="A301" t="s">
+        <v>433</v>
+      </c>
+      <c r="B301" t="s">
+        <v>624</v>
+      </c>
+      <c r="C301" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
+        <v>511</v>
+      </c>
+      <c r="B302" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3">
+      <c r="A303" t="s">
+        <v>434</v>
+      </c>
+      <c r="B303" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3">
+      <c r="A304" t="s">
+        <v>435</v>
+      </c>
+      <c r="B304" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" t="s">
+        <v>436</v>
+      </c>
+      <c r="B305" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" t="s">
         <v>528</v>
       </c>
-      <c r="B299" t="s">
+      <c r="B306" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Resolved merge conflicts with DU
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C4B63F-A7CD-41EC-AA26-53FD0844B7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B626E7BF-8271-444F-B7BE-8604427EA395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="22440" windowHeight="11715" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="760">
   <si>
     <t>Name</t>
   </si>
@@ -2308,6 +2308,18 @@
   </si>
   <si>
     <t>ASC_SumOfAssetsCheck</t>
+  </si>
+  <si>
+    <t>Assets disposed for less than Fair Market Value (FMV) on the Asset Self-Certification but not on the Asset Self-Certification Worksheet.</t>
+  </si>
+  <si>
+    <t>ASC_AssetsOnWorksheet</t>
+  </si>
+  <si>
+    <t>ASC_WorksheetNotFound</t>
+  </si>
+  <si>
+    <t>Asset Self Certification Worksheet is empty or missing from the application.</t>
   </si>
 </sst>
 </file>
@@ -6956,7 +6968,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C306"/>
+  <dimension ref="A1:C308"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -7610,18 +7622,21 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>542</v>
+        <v>719</v>
       </c>
       <c r="B82" t="s">
-        <v>672</v>
+        <v>720</v>
+      </c>
+      <c r="C82" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="B83" t="s">
-        <v>720</v>
+        <v>753</v>
       </c>
       <c r="C83" t="s">
         <v>692</v>
@@ -7629,10 +7644,10 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="B84" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C84" t="s">
         <v>692</v>
@@ -7640,352 +7655,349 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B85" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C85" t="s">
         <v>692</v>
       </c>
     </row>
+    <row r="86" spans="1:3">
+      <c r="A86" t="s">
+        <v>758</v>
+      </c>
+      <c r="B86" t="s">
+        <v>759</v>
+      </c>
+      <c r="C86" t="s">
+        <v>692</v>
+      </c>
+    </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>147</v>
+        <v>542</v>
       </c>
       <c r="B87" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3">
-      <c r="A88" t="s">
-        <v>148</v>
-      </c>
-      <c r="B88" t="s">
-        <v>151</v>
+        <v>672</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B89" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B90" t="s">
-        <v>580</v>
-      </c>
-      <c r="C90" t="s">
-        <v>691</v>
+        <v>151</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>690</v>
+        <v>149</v>
       </c>
       <c r="B91" t="s">
-        <v>580</v>
+        <v>152</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B92" t="s">
-        <v>129</v>
+        <v>580</v>
+      </c>
+      <c r="C92" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>131</v>
+        <v>690</v>
       </c>
       <c r="B93" t="s">
-        <v>599</v>
+        <v>580</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B94" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>639</v>
+        <v>131</v>
       </c>
       <c r="B95" t="s">
-        <v>640</v>
+        <v>599</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>541</v>
+        <v>132</v>
       </c>
       <c r="B96" t="s">
-        <v>673</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" t="s">
+        <v>639</v>
+      </c>
+      <c r="B97" t="s">
+        <v>640</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>188</v>
+        <v>541</v>
       </c>
       <c r="B98" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99" t="s">
-        <v>133</v>
-      </c>
-      <c r="B99" t="s">
-        <v>153</v>
+        <v>673</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="B100" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B101" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B102" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B103" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>629</v>
+        <v>136</v>
       </c>
       <c r="B104" t="s">
-        <v>695</v>
-      </c>
-      <c r="C104" t="s">
-        <v>699</v>
+        <v>156</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>641</v>
+        <v>137</v>
       </c>
       <c r="B105" t="s">
-        <v>642</v>
+        <v>157</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>540</v>
+        <v>629</v>
       </c>
       <c r="B106" t="s">
-        <v>674</v>
+        <v>695</v>
+      </c>
+      <c r="C106" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>721</v>
+        <v>641</v>
       </c>
       <c r="B107" t="s">
-        <v>722</v>
-      </c>
-      <c r="C107" t="s">
-        <v>692</v>
+        <v>642</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" t="s">
+        <v>540</v>
+      </c>
+      <c r="B108" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
+        <v>721</v>
+      </c>
+      <c r="B109" t="s">
+        <v>722</v>
+      </c>
+      <c r="C109" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" t="s">
         <v>710</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B111" t="s">
         <v>711</v>
       </c>
-      <c r="C109" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3">
-      <c r="A110" t="s">
-        <v>713</v>
-      </c>
-      <c r="B110" t="s">
-        <v>714</v>
-      </c>
-      <c r="C110" t="s">
+      <c r="C111" t="s">
         <v>712</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>159</v>
+        <v>713</v>
       </c>
       <c r="B112" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3">
-      <c r="A113" t="s">
-        <v>160</v>
-      </c>
-      <c r="B113" t="s">
-        <v>164</v>
+        <v>714</v>
+      </c>
+      <c r="C112" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B114" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B115" t="s">
-        <v>600</v>
+        <v>164</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>557</v>
+        <v>161</v>
       </c>
       <c r="B116" t="s">
-        <v>739</v>
-      </c>
-      <c r="C116" t="s">
-        <v>740</v>
+        <v>165</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>647</v>
+        <v>162</v>
       </c>
       <c r="B117" t="s">
-        <v>648</v>
+        <v>600</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>539</v>
+        <v>557</v>
       </c>
       <c r="B118" t="s">
-        <v>675</v>
+        <v>739</v>
+      </c>
+      <c r="C118" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" t="s">
+        <v>647</v>
+      </c>
+      <c r="B119" t="s">
+        <v>648</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>192</v>
+        <v>539</v>
       </c>
       <c r="B120" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3">
-      <c r="A121" t="s">
-        <v>166</v>
-      </c>
-      <c r="B121" t="s">
-        <v>168</v>
+        <v>675</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="B122" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>643</v>
+        <v>166</v>
       </c>
       <c r="B123" t="s">
-        <v>644</v>
+        <v>168</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>538</v>
+        <v>167</v>
       </c>
       <c r="B124" t="s">
-        <v>676</v>
+        <v>169</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>723</v>
+        <v>643</v>
       </c>
       <c r="B125" t="s">
-        <v>724</v>
-      </c>
-      <c r="C125" t="s">
-        <v>692</v>
+        <v>644</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" t="s">
+        <v>538</v>
+      </c>
+      <c r="B126" t="s">
+        <v>676</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>190</v>
+        <v>723</v>
       </c>
       <c r="B127" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3">
-      <c r="A128" t="s">
-        <v>175</v>
-      </c>
-      <c r="B128" t="s">
-        <v>172</v>
-      </c>
-      <c r="C128" t="s">
-        <v>588</v>
+        <v>724</v>
+      </c>
+      <c r="C127" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="B129" t="s">
-        <v>173</v>
-      </c>
-      <c r="C129" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B130" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C130" t="s">
         <v>588</v>
@@ -7993,377 +8005,380 @@
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="B131" t="s">
-        <v>202</v>
+        <v>173</v>
+      </c>
+      <c r="C131" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="B132" t="s">
-        <v>201</v>
+        <v>174</v>
+      </c>
+      <c r="C132" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="B133" t="s">
-        <v>177</v>
-      </c>
-      <c r="C133" t="s">
-        <v>588</v>
+        <v>202</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>645</v>
+        <v>200</v>
       </c>
       <c r="B134" t="s">
-        <v>646</v>
+        <v>201</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>527</v>
+        <v>176</v>
       </c>
       <c r="B135" t="s">
-        <v>677</v>
+        <v>177</v>
+      </c>
+      <c r="C135" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3">
+      <c r="A136" t="s">
+        <v>645</v>
+      </c>
+      <c r="B136" t="s">
+        <v>646</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>652</v>
+        <v>527</v>
       </c>
       <c r="B137" t="s">
-        <v>653</v>
-      </c>
-      <c r="C137" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3">
-      <c r="A138" t="s">
-        <v>727</v>
-      </c>
-      <c r="B138" t="s">
-        <v>728</v>
-      </c>
-      <c r="C138" t="s">
-        <v>692</v>
+        <v>677</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>733</v>
+        <v>652</v>
       </c>
       <c r="B139" t="s">
-        <v>734</v>
+        <v>653</v>
       </c>
       <c r="C139" t="s">
-        <v>692</v>
+        <v>654</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>741</v>
+        <v>727</v>
       </c>
       <c r="B140" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="C140" t="s">
         <v>692</v>
       </c>
     </row>
+    <row r="141" spans="1:3">
+      <c r="A141" t="s">
+        <v>733</v>
+      </c>
+      <c r="B141" t="s">
+        <v>734</v>
+      </c>
+      <c r="C141" t="s">
+        <v>692</v>
+      </c>
+    </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>513</v>
+        <v>741</v>
       </c>
       <c r="B142" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" t="s">
-        <v>661</v>
-      </c>
-      <c r="B143" t="s">
-        <v>665</v>
-      </c>
-      <c r="C143" t="s">
-        <v>663</v>
+        <v>730</v>
+      </c>
+      <c r="C142" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>662</v>
+        <v>513</v>
       </c>
       <c r="B144" t="s">
-        <v>664</v>
-      </c>
-      <c r="C144" t="s">
-        <v>663</v>
+        <v>514</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>242</v>
+        <v>661</v>
       </c>
       <c r="B145" t="s">
-        <v>243</v>
+        <v>665</v>
       </c>
       <c r="C145" t="s">
-        <v>588</v>
+        <v>663</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>244</v>
+        <v>662</v>
       </c>
       <c r="B146" t="s">
-        <v>245</v>
+        <v>664</v>
+      </c>
+      <c r="C146" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="B147" t="s">
-        <v>560</v>
+        <v>243</v>
       </c>
       <c r="C147" t="s">
-        <v>650</v>
+        <v>588</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B148" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>503</v>
+        <v>258</v>
       </c>
       <c r="B149" t="s">
-        <v>512</v>
+        <v>560</v>
+      </c>
+      <c r="C149" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B150" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>250</v>
+        <v>503</v>
       </c>
       <c r="B151" t="s">
-        <v>252</v>
+        <v>512</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B152" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B153" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B154" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="B155" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>349</v>
+        <v>257</v>
       </c>
       <c r="B156" t="s">
-        <v>350</v>
+        <v>256</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>657</v>
+        <v>302</v>
       </c>
       <c r="B157" t="s">
-        <v>658</v>
+        <v>248</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>702</v>
+        <v>349</v>
       </c>
       <c r="B158" t="s">
-        <v>703</v>
+        <v>350</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>526</v>
+        <v>657</v>
       </c>
       <c r="B159" t="s">
-        <v>678</v>
+        <v>658</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3">
+      <c r="A160" t="s">
+        <v>702</v>
+      </c>
+      <c r="B160" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
+        <v>526</v>
+      </c>
+      <c r="B161" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3">
+      <c r="A163" t="s">
         <v>515</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B163" t="s">
         <v>516</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3">
-      <c r="A162" t="s">
-        <v>259</v>
-      </c>
-      <c r="B162" t="s">
-        <v>262</v>
-      </c>
-      <c r="C162" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A163" t="s">
-        <v>261</v>
-      </c>
-      <c r="B163" t="s">
-        <v>561</v>
-      </c>
-      <c r="C163" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B164" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C164" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" ht="13.5" customHeight="1">
       <c r="A165" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B165" t="s">
-        <v>264</v>
+        <v>561</v>
+      </c>
+      <c r="C165" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B166" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B167" t="s">
-        <v>268</v>
-      </c>
-      <c r="C167" t="s">
-        <v>660</v>
+        <v>264</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>504</v>
+        <v>266</v>
       </c>
       <c r="B168" t="s">
-        <v>570</v>
+        <v>267</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B169" t="s">
-        <v>271</v>
+        <v>268</v>
+      </c>
+      <c r="C169" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>272</v>
+        <v>504</v>
       </c>
       <c r="B170" t="s">
-        <v>273</v>
+        <v>570</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B171" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="B172" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B173" t="s">
-        <v>285</v>
-      </c>
-      <c r="C173" t="s">
-        <v>660</v>
+        <v>287</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B174" t="s">
-        <v>605</v>
+        <v>286</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B175" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C175" t="s">
         <v>660</v>
@@ -8371,96 +8386,96 @@
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B176" t="s">
-        <v>283</v>
+        <v>605</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="B177" t="s">
-        <v>300</v>
+        <v>284</v>
+      </c>
+      <c r="C177" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="B178" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B179" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>704</v>
+        <v>301</v>
       </c>
       <c r="B180" t="s">
-        <v>703</v>
+        <v>248</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>537</v>
+        <v>304</v>
       </c>
       <c r="B181" t="s">
-        <v>679</v>
+        <v>305</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="B182" t="s">
-        <v>698</v>
-      </c>
-      <c r="C182" t="s">
-        <v>692</v>
+        <v>703</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3">
+      <c r="A183" t="s">
+        <v>537</v>
+      </c>
+      <c r="B183" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>517</v>
+        <v>697</v>
       </c>
       <c r="B184" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3">
-      <c r="A185" t="s">
-        <v>292</v>
-      </c>
-      <c r="B185" t="s">
-        <v>296</v>
-      </c>
-      <c r="C185" t="s">
-        <v>588</v>
+        <v>698</v>
+      </c>
+      <c r="C184" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="B186" t="s">
-        <v>571</v>
+        <v>518</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B187" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C187" t="s">
         <v>588</v>
@@ -8468,109 +8483,109 @@
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>294</v>
+        <v>505</v>
       </c>
       <c r="B188" t="s">
-        <v>298</v>
+        <v>571</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B189" t="s">
-        <v>562</v>
+        <v>297</v>
+      </c>
+      <c r="C189" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B190" t="s">
-        <v>248</v>
+        <v>298</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="B191" t="s">
-        <v>310</v>
+        <v>562</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B192" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B193" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B194" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>705</v>
+        <v>307</v>
       </c>
       <c r="B195" t="s">
-        <v>703</v>
+        <v>308</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>536</v>
+        <v>311</v>
       </c>
       <c r="B196" t="s">
-        <v>680</v>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
+        <v>705</v>
+      </c>
+      <c r="B197" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="B198" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="199" spans="1:3">
-      <c r="A199" t="s">
-        <v>499</v>
-      </c>
-      <c r="B199" t="s">
-        <v>320</v>
-      </c>
-      <c r="C199" t="s">
-        <v>588</v>
+        <v>680</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="B200" t="s">
-        <v>572</v>
+        <v>520</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>315</v>
+        <v>499</v>
       </c>
       <c r="B201" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C201" t="s">
         <v>588</v>
@@ -8578,128 +8593,128 @@
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>316</v>
+        <v>506</v>
       </c>
       <c r="B202" t="s">
-        <v>322</v>
+        <v>572</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B203" t="s">
-        <v>323</v>
+        <v>321</v>
+      </c>
+      <c r="C203" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B204" t="s">
-        <v>563</v>
+        <v>322</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B205" t="s">
-        <v>248</v>
+        <v>323</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B206" t="s">
-        <v>325</v>
-      </c>
-      <c r="C206" t="s">
-        <v>588</v>
+        <v>563</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="B207" t="s">
-        <v>327</v>
+        <v>248</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B208" t="s">
-        <v>328</v>
+        <v>325</v>
+      </c>
+      <c r="C208" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B209" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B210" t="s">
-        <v>256</v>
+        <v>328</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>706</v>
+        <v>330</v>
       </c>
       <c r="B211" t="s">
-        <v>703</v>
+        <v>331</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>535</v>
+        <v>332</v>
       </c>
       <c r="B212" t="s">
-        <v>681</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3">
+      <c r="A213" t="s">
+        <v>706</v>
+      </c>
+      <c r="B213" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="B214" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3">
-      <c r="A215" t="s">
-        <v>501</v>
-      </c>
-      <c r="B215" t="s">
-        <v>338</v>
-      </c>
-      <c r="C215" t="s">
-        <v>588</v>
+        <v>681</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
       <c r="B216" t="s">
-        <v>573</v>
+        <v>522</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>336</v>
+        <v>501</v>
       </c>
       <c r="B217" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C217" t="s">
         <v>588</v>
@@ -8707,303 +8722,303 @@
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>337</v>
+        <v>507</v>
       </c>
       <c r="B218" t="s">
-        <v>340</v>
+        <v>573</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>500</v>
+        <v>336</v>
       </c>
       <c r="B219" t="s">
-        <v>564</v>
+        <v>339</v>
+      </c>
+      <c r="C219" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="B220" t="s">
-        <v>248</v>
+        <v>340</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>345</v>
+        <v>500</v>
       </c>
       <c r="B221" t="s">
-        <v>341</v>
+        <v>564</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B222" t="s">
-        <v>342</v>
+        <v>248</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B223" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B224" t="s">
-        <v>256</v>
+        <v>342</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>707</v>
+        <v>347</v>
       </c>
       <c r="B225" t="s">
-        <v>703</v>
+        <v>343</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>534</v>
+        <v>348</v>
       </c>
       <c r="B226" t="s">
-        <v>682</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3">
+      <c r="A227" t="s">
+        <v>707</v>
+      </c>
+      <c r="B227" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>747</v>
+        <v>534</v>
       </c>
       <c r="B228" t="s">
-        <v>748</v>
-      </c>
-      <c r="C228" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="229" spans="1:3">
-      <c r="A229" t="s">
-        <v>551</v>
-      </c>
-      <c r="B229" t="s">
-        <v>554</v>
-      </c>
-      <c r="C229" t="s">
-        <v>586</v>
+        <v>682</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>552</v>
+        <v>747</v>
       </c>
       <c r="B230" t="s">
-        <v>553</v>
+        <v>748</v>
       </c>
       <c r="C230" t="s">
-        <v>587</v>
+        <v>692</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>585</v>
+        <v>551</v>
       </c>
       <c r="B231" t="s">
-        <v>601</v>
+        <v>554</v>
+      </c>
+      <c r="C231" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>365</v>
+        <v>552</v>
       </c>
       <c r="B232" t="s">
-        <v>351</v>
+        <v>553</v>
+      </c>
+      <c r="C232" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>366</v>
+        <v>585</v>
       </c>
       <c r="B233" t="s">
-        <v>352</v>
-      </c>
-      <c r="C233" t="s">
-        <v>588</v>
+        <v>601</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>508</v>
+        <v>365</v>
       </c>
       <c r="B234" t="s">
-        <v>574</v>
+        <v>351</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B235" t="s">
-        <v>353</v>
+        <v>352</v>
+      </c>
+      <c r="C235" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>368</v>
+        <v>508</v>
       </c>
       <c r="B236" t="s">
-        <v>354</v>
+        <v>574</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B237" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B238" t="s">
-        <v>356</v>
-      </c>
-      <c r="C238" t="s">
-        <v>588</v>
+        <v>354</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B239" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B240" t="s">
-        <v>358</v>
+        <v>356</v>
+      </c>
+      <c r="C240" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B241" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B242" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B243" t="s">
-        <v>361</v>
-      </c>
-      <c r="C243" t="s">
-        <v>588</v>
+        <v>359</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B244" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B245" t="s">
-        <v>363</v>
+        <v>361</v>
+      </c>
+      <c r="C245" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B246" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>533</v>
+        <v>377</v>
       </c>
       <c r="B247" t="s">
-        <v>666</v>
+        <v>363</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3">
+      <c r="A248" t="s">
+        <v>378</v>
+      </c>
+      <c r="B248" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>606</v>
+        <v>533</v>
       </c>
       <c r="B249" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="250" spans="1:3">
-      <c r="A250" t="s">
-        <v>385</v>
-      </c>
-      <c r="B250" t="s">
-        <v>403</v>
+        <v>666</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>386</v>
+        <v>606</v>
       </c>
       <c r="B251" t="s">
-        <v>400</v>
+        <v>607</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B252" t="s">
-        <v>401</v>
-      </c>
-      <c r="C252" t="s">
-        <v>588</v>
+        <v>403</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>509</v>
+        <v>386</v>
       </c>
       <c r="B253" t="s">
-        <v>575</v>
+        <v>400</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>404</v>
+        <v>387</v>
       </c>
       <c r="B254" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C254" t="s">
         <v>588</v>
@@ -9011,85 +9026,93 @@
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>388</v>
+        <v>509</v>
       </c>
       <c r="B255" t="s">
-        <v>394</v>
+        <v>575</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B256" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C256" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B257" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="B258" t="s">
-        <v>397</v>
+        <v>395</v>
+      </c>
+      <c r="C258" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B259" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B260" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B261" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>532</v>
+        <v>392</v>
       </c>
       <c r="B262" t="s">
-        <v>683</v>
+        <v>399</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3">
+      <c r="A263" t="s">
+        <v>393</v>
+      </c>
+      <c r="B263" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>749</v>
+        <v>532</v>
       </c>
       <c r="B264" t="s">
-        <v>746</v>
-      </c>
-      <c r="C264" t="s">
-        <v>692</v>
+        <v>683</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="B266" t="s">
         <v>746</v>
@@ -9098,47 +9121,39 @@
         <v>692</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
-      <c r="A267" t="s">
-        <v>523</v>
-      </c>
-      <c r="B267" t="s">
-        <v>524</v>
-      </c>
-    </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>411</v>
+        <v>745</v>
       </c>
       <c r="B268" t="s">
-        <v>422</v>
+        <v>746</v>
+      </c>
+      <c r="C268" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>412</v>
+        <v>523</v>
       </c>
       <c r="B269" t="s">
-        <v>423</v>
-      </c>
-      <c r="C269" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>576</v>
+        <v>411</v>
       </c>
       <c r="B270" t="s">
-        <v>577</v>
+        <v>422</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B271" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C271" t="s">
         <v>588</v>
@@ -9146,128 +9161,128 @@
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>414</v>
+        <v>576</v>
       </c>
       <c r="B272" t="s">
-        <v>425</v>
-      </c>
-      <c r="C272" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B273" t="s">
-        <v>589</v>
+        <v>424</v>
+      </c>
+      <c r="C273" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B274" t="s">
-        <v>426</v>
+        <v>425</v>
+      </c>
+      <c r="C274" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B275" t="s">
-        <v>427</v>
+        <v>589</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B276" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B277" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B278" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B279" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>530</v>
+        <v>420</v>
       </c>
       <c r="B280" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>615</v>
+        <v>421</v>
       </c>
       <c r="B281" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3">
+      <c r="A282" t="s">
+        <v>530</v>
+      </c>
+      <c r="B282" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>525</v>
+        <v>615</v>
       </c>
       <c r="B283" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="284" spans="1:3">
-      <c r="A284" t="s">
-        <v>438</v>
-      </c>
-      <c r="B284" t="s">
-        <v>449</v>
+        <v>616</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>439</v>
+        <v>525</v>
       </c>
       <c r="B285" t="s">
-        <v>450</v>
-      </c>
-      <c r="C285" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>510</v>
+        <v>438</v>
       </c>
       <c r="B286" t="s">
-        <v>578</v>
+        <v>449</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B287" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C287" t="s">
         <v>588</v>
@@ -9275,154 +9290,173 @@
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>441</v>
+        <v>510</v>
       </c>
       <c r="B288" t="s">
-        <v>452</v>
-      </c>
-      <c r="C288" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B289" t="s">
-        <v>590</v>
+        <v>451</v>
+      </c>
+      <c r="C289" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B290" t="s">
-        <v>426</v>
+        <v>452</v>
+      </c>
+      <c r="C290" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B291" t="s">
-        <v>427</v>
+        <v>590</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B292" t="s">
-        <v>453</v>
+        <v>426</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B293" t="s">
-        <v>454</v>
+        <v>427</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B294" t="s">
-        <v>430</v>
+        <v>453</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B295" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>529</v>
+        <v>447</v>
       </c>
       <c r="B296" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>622</v>
+        <v>448</v>
       </c>
       <c r="B297" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3">
+      <c r="A298" t="s">
+        <v>529</v>
+      </c>
+      <c r="B298" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>743</v>
+        <v>622</v>
       </c>
       <c r="B299" t="s">
-        <v>744</v>
-      </c>
-      <c r="C299" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="300" spans="1:3">
-      <c r="A300" t="s">
-        <v>432</v>
-      </c>
-      <c r="B300" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>433</v>
+        <v>743</v>
       </c>
       <c r="B301" t="s">
-        <v>624</v>
+        <v>744</v>
       </c>
       <c r="C301" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>511</v>
+        <v>432</v>
       </c>
       <c r="B302" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B303" t="s">
-        <v>651</v>
+        <v>624</v>
+      </c>
+      <c r="C303" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>435</v>
+        <v>511</v>
       </c>
       <c r="B304" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="305" spans="1:2">
       <c r="A305" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B305" t="s">
-        <v>627</v>
+        <v>651</v>
       </c>
     </row>
     <row r="306" spans="1:2">
       <c r="A306" t="s">
+        <v>435</v>
+      </c>
+      <c r="B306" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" t="s">
+        <v>436</v>
+      </c>
+      <c r="B307" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" t="s">
         <v>528</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B308" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DU updates for Application summary, integration in Auditfindings and testing
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B626E7BF-8271-444F-B7BE-8604427EA395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B344CECA-6A60-4BF5-BFCA-06F6953E4C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22440" windowHeight="11715" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2268,9 +2268,6 @@
     <t>EDC_DominiumEmployee</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>VRCCDoesNotExist</t>
   </si>
   <si>
@@ -2320,6 +2317,9 @@
   </si>
   <si>
     <t>Asset Self Certification Worksheet is empty or missing from the application.</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2777,7 +2777,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>742</v>
+        <v>759</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7474,10 +7474,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B63" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="C63" t="s">
         <v>692</v>
@@ -7633,10 +7633,10 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
+        <v>751</v>
+      </c>
+      <c r="B83" t="s">
         <v>752</v>
-      </c>
-      <c r="B83" t="s">
-        <v>753</v>
       </c>
       <c r="C83" t="s">
         <v>692</v>
@@ -7644,10 +7644,10 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B84" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C84" t="s">
         <v>692</v>
@@ -7655,10 +7655,10 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B85" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C85" t="s">
         <v>692</v>
@@ -7666,10 +7666,10 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
+        <v>757</v>
+      </c>
+      <c r="B86" t="s">
         <v>758</v>
-      </c>
-      <c r="B86" t="s">
-        <v>759</v>
       </c>
       <c r="C86" t="s">
         <v>692</v>
@@ -8813,10 +8813,10 @@
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
+        <v>746</v>
+      </c>
+      <c r="B230" t="s">
         <v>747</v>
-      </c>
-      <c r="B230" t="s">
-        <v>748</v>
       </c>
       <c r="C230" t="s">
         <v>692</v>
@@ -9112,10 +9112,10 @@
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B266" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C266" t="s">
         <v>692</v>
@@ -9123,10 +9123,10 @@
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
+        <v>744</v>
+      </c>
+      <c r="B268" t="s">
         <v>745</v>
-      </c>
-      <c r="B268" t="s">
-        <v>746</v>
       </c>
       <c r="C268" t="s">
         <v>692</v>
@@ -9392,10 +9392,10 @@
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
+        <v>742</v>
+      </c>
+      <c r="B301" t="s">
         <v>743</v>
-      </c>
-      <c r="B301" t="s">
-        <v>744</v>
       </c>
       <c r="C301" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
57448 - implemented a condition to detect when the ASC is empty or missing from the application, 58031 - added a finding for SCNE if the employment checkbox is checked 'yes' but not documented on the ICW
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B344CECA-6A60-4BF5-BFCA-06F6953E4C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD6162E-D11E-4E80-BDAF-736920B3B7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2190" yWindow="3960" windowWidth="28170" windowHeight="13710" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="760">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="764">
   <si>
     <t>Name</t>
   </si>
@@ -2319,7 +2319,19 @@
     <t>Asset Self Certification Worksheet is empty or missing from the application.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>ASC_IsFound</t>
+  </si>
+  <si>
+    <t>Asset Self Certification is missing from the application.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>SCNE_EmploymentDocumented</t>
+  </si>
+  <si>
+    <t>Currently employment has been documented on the Self-Certification of Non-Employment but no current employment was documented on the ICW for that member.</t>
   </si>
 </sst>
 </file>
@@ -2777,7 +2789,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -6968,7 +6980,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C308"/>
+  <dimension ref="A1:C310"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -7517,148 +7529,148 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>762</v>
+      </c>
+      <c r="B69" t="s">
+        <v>763</v>
+      </c>
+      <c r="C69" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>543</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B70" t="s">
         <v>671</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" t="s">
-        <v>186</v>
-      </c>
-      <c r="B71" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>125</v>
+        <v>186</v>
       </c>
       <c r="B72" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>126</v>
+        <v>759</v>
       </c>
       <c r="B73" t="s">
-        <v>128</v>
+        <v>760</v>
+      </c>
+      <c r="C73" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>138</v>
+        <v>757</v>
       </c>
       <c r="B74" t="s">
-        <v>595</v>
+        <v>758</v>
+      </c>
+      <c r="C74" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B75" t="s">
-        <v>596</v>
+        <v>127</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="B76" t="s">
-        <v>597</v>
+        <v>128</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B77" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B78" t="s">
-        <v>495</v>
-      </c>
-      <c r="C78" t="s">
-        <v>686</v>
+        <v>596</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B79" t="s">
-        <v>497</v>
-      </c>
-      <c r="C79" t="s">
-        <v>556</v>
+        <v>597</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B80" t="s">
-        <v>498</v>
-      </c>
-      <c r="C80" t="s">
-        <v>556</v>
+        <v>598</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>637</v>
+        <v>142</v>
       </c>
       <c r="B81" t="s">
-        <v>638</v>
+        <v>495</v>
+      </c>
+      <c r="C81" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>719</v>
+        <v>143</v>
       </c>
       <c r="B82" t="s">
-        <v>720</v>
+        <v>497</v>
       </c>
       <c r="C82" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>751</v>
+        <v>144</v>
       </c>
       <c r="B83" t="s">
-        <v>752</v>
+        <v>498</v>
       </c>
       <c r="C83" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>754</v>
+        <v>637</v>
       </c>
       <c r="B84" t="s">
-        <v>753</v>
-      </c>
-      <c r="C84" t="s">
-        <v>692</v>
+        <v>638</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>756</v>
+        <v>719</v>
       </c>
       <c r="B85" t="s">
-        <v>755</v>
+        <v>720</v>
       </c>
       <c r="C85" t="s">
         <v>692</v>
@@ -7666,10 +7678,10 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
       <c r="B86" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="C86" t="s">
         <v>692</v>
@@ -7677,349 +7689,349 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>542</v>
+        <v>754</v>
       </c>
       <c r="B87" t="s">
-        <v>672</v>
+        <v>753</v>
+      </c>
+      <c r="C87" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>756</v>
+      </c>
+      <c r="B88" t="s">
+        <v>755</v>
+      </c>
+      <c r="C88" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>147</v>
+        <v>542</v>
       </c>
       <c r="B89" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3">
-      <c r="A90" t="s">
-        <v>148</v>
-      </c>
-      <c r="B90" t="s">
-        <v>151</v>
+        <v>672</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B91" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B92" t="s">
-        <v>580</v>
-      </c>
-      <c r="C92" t="s">
-        <v>691</v>
+        <v>151</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>690</v>
+        <v>149</v>
       </c>
       <c r="B93" t="s">
-        <v>580</v>
+        <v>152</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B94" t="s">
-        <v>129</v>
+        <v>580</v>
+      </c>
+      <c r="C94" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>131</v>
+        <v>690</v>
       </c>
       <c r="B95" t="s">
-        <v>599</v>
+        <v>580</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B96" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>639</v>
+        <v>131</v>
       </c>
       <c r="B97" t="s">
-        <v>640</v>
+        <v>599</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>541</v>
+        <v>132</v>
       </c>
       <c r="B98" t="s">
-        <v>673</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" t="s">
+        <v>639</v>
+      </c>
+      <c r="B99" t="s">
+        <v>640</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>188</v>
+        <v>541</v>
       </c>
       <c r="B100" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3">
-      <c r="A101" t="s">
-        <v>133</v>
-      </c>
-      <c r="B101" t="s">
-        <v>153</v>
+        <v>673</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="B102" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B103" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B104" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B105" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>629</v>
+        <v>136</v>
       </c>
       <c r="B106" t="s">
-        <v>695</v>
-      </c>
-      <c r="C106" t="s">
-        <v>699</v>
+        <v>156</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>641</v>
+        <v>137</v>
       </c>
       <c r="B107" t="s">
-        <v>642</v>
+        <v>157</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>540</v>
+        <v>629</v>
       </c>
       <c r="B108" t="s">
-        <v>674</v>
+        <v>695</v>
+      </c>
+      <c r="C108" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>721</v>
+        <v>641</v>
       </c>
       <c r="B109" t="s">
-        <v>722</v>
-      </c>
-      <c r="C109" t="s">
-        <v>692</v>
+        <v>642</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" t="s">
+        <v>540</v>
+      </c>
+      <c r="B110" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
+        <v>721</v>
+      </c>
+      <c r="B111" t="s">
+        <v>722</v>
+      </c>
+      <c r="C111" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" t="s">
         <v>710</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B113" t="s">
         <v>711</v>
       </c>
-      <c r="C111" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3">
-      <c r="A112" t="s">
-        <v>713</v>
-      </c>
-      <c r="B112" t="s">
-        <v>714</v>
-      </c>
-      <c r="C112" t="s">
+      <c r="C113" t="s">
         <v>712</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>159</v>
+        <v>713</v>
       </c>
       <c r="B114" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3">
-      <c r="A115" t="s">
-        <v>160</v>
-      </c>
-      <c r="B115" t="s">
-        <v>164</v>
+        <v>714</v>
+      </c>
+      <c r="C114" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B116" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B117" t="s">
-        <v>600</v>
+        <v>164</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>557</v>
+        <v>161</v>
       </c>
       <c r="B118" t="s">
-        <v>739</v>
-      </c>
-      <c r="C118" t="s">
-        <v>740</v>
+        <v>165</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>647</v>
+        <v>162</v>
       </c>
       <c r="B119" t="s">
-        <v>648</v>
+        <v>600</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>539</v>
+        <v>557</v>
       </c>
       <c r="B120" t="s">
-        <v>675</v>
+        <v>739</v>
+      </c>
+      <c r="C120" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" t="s">
+        <v>647</v>
+      </c>
+      <c r="B121" t="s">
+        <v>648</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>192</v>
+        <v>539</v>
       </c>
       <c r="B122" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" t="s">
-        <v>166</v>
-      </c>
-      <c r="B123" t="s">
-        <v>168</v>
+        <v>675</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="B124" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>643</v>
+        <v>166</v>
       </c>
       <c r="B125" t="s">
-        <v>644</v>
+        <v>168</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>538</v>
+        <v>167</v>
       </c>
       <c r="B126" t="s">
-        <v>676</v>
+        <v>169</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>723</v>
+        <v>643</v>
       </c>
       <c r="B127" t="s">
-        <v>724</v>
-      </c>
-      <c r="C127" t="s">
-        <v>692</v>
+        <v>644</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" t="s">
+        <v>538</v>
+      </c>
+      <c r="B128" t="s">
+        <v>676</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>190</v>
+        <v>723</v>
       </c>
       <c r="B129" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3">
-      <c r="A130" t="s">
-        <v>175</v>
-      </c>
-      <c r="B130" t="s">
-        <v>172</v>
-      </c>
-      <c r="C130" t="s">
-        <v>588</v>
+        <v>724</v>
+      </c>
+      <c r="C129" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="B131" t="s">
-        <v>173</v>
-      </c>
-      <c r="C131" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B132" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C132" t="s">
         <v>588</v>
@@ -8027,377 +8039,380 @@
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="B133" t="s">
-        <v>202</v>
+        <v>173</v>
+      </c>
+      <c r="C133" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="B134" t="s">
-        <v>201</v>
+        <v>174</v>
+      </c>
+      <c r="C134" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="B135" t="s">
-        <v>177</v>
-      </c>
-      <c r="C135" t="s">
-        <v>588</v>
+        <v>202</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>645</v>
+        <v>200</v>
       </c>
       <c r="B136" t="s">
-        <v>646</v>
+        <v>201</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>527</v>
+        <v>176</v>
       </c>
       <c r="B137" t="s">
-        <v>677</v>
+        <v>177</v>
+      </c>
+      <c r="C137" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" t="s">
+        <v>645</v>
+      </c>
+      <c r="B138" t="s">
+        <v>646</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>652</v>
+        <v>527</v>
       </c>
       <c r="B139" t="s">
-        <v>653</v>
-      </c>
-      <c r="C139" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3">
-      <c r="A140" t="s">
-        <v>727</v>
-      </c>
-      <c r="B140" t="s">
-        <v>728</v>
-      </c>
-      <c r="C140" t="s">
-        <v>692</v>
+        <v>677</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>733</v>
+        <v>652</v>
       </c>
       <c r="B141" t="s">
-        <v>734</v>
+        <v>653</v>
       </c>
       <c r="C141" t="s">
-        <v>692</v>
+        <v>654</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>741</v>
+        <v>727</v>
       </c>
       <c r="B142" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="C142" t="s">
         <v>692</v>
       </c>
     </row>
+    <row r="143" spans="1:3">
+      <c r="A143" t="s">
+        <v>733</v>
+      </c>
+      <c r="B143" t="s">
+        <v>734</v>
+      </c>
+      <c r="C143" t="s">
+        <v>692</v>
+      </c>
+    </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>513</v>
+        <v>741</v>
       </c>
       <c r="B144" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3">
-      <c r="A145" t="s">
-        <v>661</v>
-      </c>
-      <c r="B145" t="s">
-        <v>665</v>
-      </c>
-      <c r="C145" t="s">
-        <v>663</v>
+        <v>730</v>
+      </c>
+      <c r="C144" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>662</v>
+        <v>513</v>
       </c>
       <c r="B146" t="s">
-        <v>664</v>
-      </c>
-      <c r="C146" t="s">
-        <v>663</v>
+        <v>514</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>242</v>
+        <v>661</v>
       </c>
       <c r="B147" t="s">
-        <v>243</v>
+        <v>665</v>
       </c>
       <c r="C147" t="s">
-        <v>588</v>
+        <v>663</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>244</v>
+        <v>662</v>
       </c>
       <c r="B148" t="s">
-        <v>245</v>
+        <v>664</v>
+      </c>
+      <c r="C148" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="B149" t="s">
-        <v>560</v>
+        <v>243</v>
       </c>
       <c r="C149" t="s">
-        <v>650</v>
+        <v>588</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B150" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>503</v>
+        <v>258</v>
       </c>
       <c r="B151" t="s">
-        <v>512</v>
+        <v>560</v>
+      </c>
+      <c r="C151" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B152" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>250</v>
+        <v>503</v>
       </c>
       <c r="B153" t="s">
-        <v>252</v>
+        <v>512</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B154" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B155" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B156" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="B157" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>349</v>
+        <v>257</v>
       </c>
       <c r="B158" t="s">
-        <v>350</v>
+        <v>256</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>657</v>
+        <v>302</v>
       </c>
       <c r="B159" t="s">
-        <v>658</v>
+        <v>248</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>702</v>
+        <v>349</v>
       </c>
       <c r="B160" t="s">
-        <v>703</v>
+        <v>350</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>526</v>
+        <v>657</v>
       </c>
       <c r="B161" t="s">
-        <v>678</v>
+        <v>658</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3">
+      <c r="A162" t="s">
+        <v>702</v>
+      </c>
+      <c r="B162" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
+        <v>526</v>
+      </c>
+      <c r="B163" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3">
+      <c r="A165" t="s">
         <v>515</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B165" t="s">
         <v>516</v>
-      </c>
-    </row>
-    <row r="164" spans="1:3">
-      <c r="A164" t="s">
-        <v>259</v>
-      </c>
-      <c r="B164" t="s">
-        <v>262</v>
-      </c>
-      <c r="C164" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A165" t="s">
-        <v>261</v>
-      </c>
-      <c r="B165" t="s">
-        <v>561</v>
-      </c>
-      <c r="C165" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B166" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C166" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="13.5" customHeight="1">
       <c r="A167" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B167" t="s">
-        <v>264</v>
+        <v>561</v>
+      </c>
+      <c r="C167" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B168" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B169" t="s">
-        <v>268</v>
-      </c>
-      <c r="C169" t="s">
-        <v>660</v>
+        <v>264</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>504</v>
+        <v>266</v>
       </c>
       <c r="B170" t="s">
-        <v>570</v>
+        <v>267</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B171" t="s">
-        <v>271</v>
+        <v>268</v>
+      </c>
+      <c r="C171" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>272</v>
+        <v>504</v>
       </c>
       <c r="B172" t="s">
-        <v>273</v>
+        <v>570</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B173" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="B174" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B175" t="s">
-        <v>285</v>
-      </c>
-      <c r="C175" t="s">
-        <v>660</v>
+        <v>287</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B176" t="s">
-        <v>605</v>
+        <v>286</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B177" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C177" t="s">
         <v>660</v>
@@ -8405,96 +8420,96 @@
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B178" t="s">
-        <v>283</v>
+        <v>605</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="B179" t="s">
-        <v>300</v>
+        <v>284</v>
+      </c>
+      <c r="C179" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="B180" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B181" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>704</v>
+        <v>301</v>
       </c>
       <c r="B182" t="s">
-        <v>703</v>
+        <v>248</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>537</v>
+        <v>304</v>
       </c>
       <c r="B183" t="s">
-        <v>679</v>
+        <v>305</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="B184" t="s">
-        <v>698</v>
-      </c>
-      <c r="C184" t="s">
-        <v>692</v>
+        <v>703</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3">
+      <c r="A185" t="s">
+        <v>537</v>
+      </c>
+      <c r="B185" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>517</v>
+        <v>697</v>
       </c>
       <c r="B186" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3">
-      <c r="A187" t="s">
-        <v>292</v>
-      </c>
-      <c r="B187" t="s">
-        <v>296</v>
-      </c>
-      <c r="C187" t="s">
-        <v>588</v>
+        <v>698</v>
+      </c>
+      <c r="C186" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="B188" t="s">
-        <v>571</v>
+        <v>518</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B189" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C189" t="s">
         <v>588</v>
@@ -8502,109 +8517,109 @@
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>294</v>
+        <v>505</v>
       </c>
       <c r="B190" t="s">
-        <v>298</v>
+        <v>571</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B191" t="s">
-        <v>562</v>
+        <v>297</v>
+      </c>
+      <c r="C191" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B192" t="s">
-        <v>248</v>
+        <v>298</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="B193" t="s">
-        <v>310</v>
+        <v>562</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B194" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B195" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B196" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>705</v>
+        <v>307</v>
       </c>
       <c r="B197" t="s">
-        <v>703</v>
+        <v>308</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>536</v>
+        <v>311</v>
       </c>
       <c r="B198" t="s">
-        <v>680</v>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3">
+      <c r="A199" t="s">
+        <v>705</v>
+      </c>
+      <c r="B199" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="B200" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="201" spans="1:3">
-      <c r="A201" t="s">
-        <v>499</v>
-      </c>
-      <c r="B201" t="s">
-        <v>320</v>
-      </c>
-      <c r="C201" t="s">
-        <v>588</v>
+        <v>680</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="B202" t="s">
-        <v>572</v>
+        <v>520</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>315</v>
+        <v>499</v>
       </c>
       <c r="B203" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C203" t="s">
         <v>588</v>
@@ -8612,128 +8627,128 @@
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>316</v>
+        <v>506</v>
       </c>
       <c r="B204" t="s">
-        <v>322</v>
+        <v>572</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B205" t="s">
-        <v>323</v>
+        <v>321</v>
+      </c>
+      <c r="C205" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B206" t="s">
-        <v>563</v>
+        <v>322</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B207" t="s">
-        <v>248</v>
+        <v>323</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B208" t="s">
-        <v>325</v>
-      </c>
-      <c r="C208" t="s">
-        <v>588</v>
+        <v>563</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="B209" t="s">
-        <v>327</v>
+        <v>248</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B210" t="s">
-        <v>328</v>
+        <v>325</v>
+      </c>
+      <c r="C210" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B211" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B212" t="s">
-        <v>256</v>
+        <v>328</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>706</v>
+        <v>330</v>
       </c>
       <c r="B213" t="s">
-        <v>703</v>
+        <v>331</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>535</v>
+        <v>332</v>
       </c>
       <c r="B214" t="s">
-        <v>681</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3">
+      <c r="A215" t="s">
+        <v>706</v>
+      </c>
+      <c r="B215" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="B216" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3">
-      <c r="A217" t="s">
-        <v>501</v>
-      </c>
-      <c r="B217" t="s">
-        <v>338</v>
-      </c>
-      <c r="C217" t="s">
-        <v>588</v>
+        <v>681</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
       <c r="B218" t="s">
-        <v>573</v>
+        <v>522</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>336</v>
+        <v>501</v>
       </c>
       <c r="B219" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C219" t="s">
         <v>588</v>
@@ -8741,303 +8756,303 @@
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>337</v>
+        <v>507</v>
       </c>
       <c r="B220" t="s">
-        <v>340</v>
+        <v>573</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>500</v>
+        <v>336</v>
       </c>
       <c r="B221" t="s">
-        <v>564</v>
+        <v>339</v>
+      </c>
+      <c r="C221" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="B222" t="s">
-        <v>248</v>
+        <v>340</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>345</v>
+        <v>500</v>
       </c>
       <c r="B223" t="s">
-        <v>341</v>
+        <v>564</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B224" t="s">
-        <v>342</v>
+        <v>248</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B225" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B226" t="s">
-        <v>256</v>
+        <v>342</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>707</v>
+        <v>347</v>
       </c>
       <c r="B227" t="s">
-        <v>703</v>
+        <v>343</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>534</v>
+        <v>348</v>
       </c>
       <c r="B228" t="s">
-        <v>682</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3">
+      <c r="A229" t="s">
+        <v>707</v>
+      </c>
+      <c r="B229" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>746</v>
+        <v>534</v>
       </c>
       <c r="B230" t="s">
-        <v>747</v>
-      </c>
-      <c r="C230" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3">
-      <c r="A231" t="s">
-        <v>551</v>
-      </c>
-      <c r="B231" t="s">
-        <v>554</v>
-      </c>
-      <c r="C231" t="s">
-        <v>586</v>
+        <v>682</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>552</v>
+        <v>746</v>
       </c>
       <c r="B232" t="s">
-        <v>553</v>
+        <v>747</v>
       </c>
       <c r="C232" t="s">
-        <v>587</v>
+        <v>692</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>585</v>
+        <v>551</v>
       </c>
       <c r="B233" t="s">
-        <v>601</v>
+        <v>554</v>
+      </c>
+      <c r="C233" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>365</v>
+        <v>552</v>
       </c>
       <c r="B234" t="s">
-        <v>351</v>
+        <v>553</v>
+      </c>
+      <c r="C234" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>366</v>
+        <v>585</v>
       </c>
       <c r="B235" t="s">
-        <v>352</v>
-      </c>
-      <c r="C235" t="s">
-        <v>588</v>
+        <v>601</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>508</v>
+        <v>365</v>
       </c>
       <c r="B236" t="s">
-        <v>574</v>
+        <v>351</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B237" t="s">
-        <v>353</v>
+        <v>352</v>
+      </c>
+      <c r="C237" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>368</v>
+        <v>508</v>
       </c>
       <c r="B238" t="s">
-        <v>354</v>
+        <v>574</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B239" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B240" t="s">
-        <v>356</v>
-      </c>
-      <c r="C240" t="s">
-        <v>588</v>
+        <v>354</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B241" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B242" t="s">
-        <v>358</v>
+        <v>356</v>
+      </c>
+      <c r="C242" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B243" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B244" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B245" t="s">
-        <v>361</v>
-      </c>
-      <c r="C245" t="s">
-        <v>588</v>
+        <v>359</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B246" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B247" t="s">
-        <v>363</v>
+        <v>361</v>
+      </c>
+      <c r="C247" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B248" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>533</v>
+        <v>377</v>
       </c>
       <c r="B249" t="s">
-        <v>666</v>
+        <v>363</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3">
+      <c r="A250" t="s">
+        <v>378</v>
+      </c>
+      <c r="B250" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>606</v>
+        <v>533</v>
       </c>
       <c r="B251" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="252" spans="1:3">
-      <c r="A252" t="s">
-        <v>385</v>
-      </c>
-      <c r="B252" t="s">
-        <v>403</v>
+        <v>666</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>386</v>
+        <v>606</v>
       </c>
       <c r="B253" t="s">
-        <v>400</v>
+        <v>607</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B254" t="s">
-        <v>401</v>
-      </c>
-      <c r="C254" t="s">
-        <v>588</v>
+        <v>403</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>509</v>
+        <v>386</v>
       </c>
       <c r="B255" t="s">
-        <v>575</v>
+        <v>400</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>404</v>
+        <v>387</v>
       </c>
       <c r="B256" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C256" t="s">
         <v>588</v>
@@ -9045,85 +9060,93 @@
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>388</v>
+        <v>509</v>
       </c>
       <c r="B257" t="s">
-        <v>394</v>
+        <v>575</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B258" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C258" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B259" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="B260" t="s">
-        <v>397</v>
+        <v>395</v>
+      </c>
+      <c r="C260" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B261" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B262" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B263" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>532</v>
+        <v>392</v>
       </c>
       <c r="B264" t="s">
-        <v>683</v>
+        <v>399</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3">
+      <c r="A265" t="s">
+        <v>393</v>
+      </c>
+      <c r="B265" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>748</v>
+        <v>532</v>
       </c>
       <c r="B266" t="s">
-        <v>745</v>
-      </c>
-      <c r="C266" t="s">
-        <v>692</v>
+        <v>683</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="B268" t="s">
         <v>745</v>
@@ -9132,47 +9155,39 @@
         <v>692</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
-      <c r="A269" t="s">
-        <v>523</v>
-      </c>
-      <c r="B269" t="s">
-        <v>524</v>
-      </c>
-    </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>411</v>
+        <v>744</v>
       </c>
       <c r="B270" t="s">
-        <v>422</v>
+        <v>745</v>
+      </c>
+      <c r="C270" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>412</v>
+        <v>523</v>
       </c>
       <c r="B271" t="s">
-        <v>423</v>
-      </c>
-      <c r="C271" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>576</v>
+        <v>411</v>
       </c>
       <c r="B272" t="s">
-        <v>577</v>
+        <v>422</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B273" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C273" t="s">
         <v>588</v>
@@ -9180,128 +9195,128 @@
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>414</v>
+        <v>576</v>
       </c>
       <c r="B274" t="s">
-        <v>425</v>
-      </c>
-      <c r="C274" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B275" t="s">
-        <v>589</v>
+        <v>424</v>
+      </c>
+      <c r="C275" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B276" t="s">
-        <v>426</v>
+        <v>425</v>
+      </c>
+      <c r="C276" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B277" t="s">
-        <v>427</v>
+        <v>589</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B278" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B279" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B280" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B281" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>530</v>
+        <v>420</v>
       </c>
       <c r="B282" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>615</v>
+        <v>421</v>
       </c>
       <c r="B283" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3">
+      <c r="A284" t="s">
+        <v>530</v>
+      </c>
+      <c r="B284" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>525</v>
+        <v>615</v>
       </c>
       <c r="B285" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="286" spans="1:3">
-      <c r="A286" t="s">
-        <v>438</v>
-      </c>
-      <c r="B286" t="s">
-        <v>449</v>
+        <v>616</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>439</v>
+        <v>525</v>
       </c>
       <c r="B287" t="s">
-        <v>450</v>
-      </c>
-      <c r="C287" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>510</v>
+        <v>438</v>
       </c>
       <c r="B288" t="s">
-        <v>578</v>
+        <v>449</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B289" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C289" t="s">
         <v>588</v>
@@ -9309,154 +9324,173 @@
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>441</v>
+        <v>510</v>
       </c>
       <c r="B290" t="s">
-        <v>452</v>
-      </c>
-      <c r="C290" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B291" t="s">
-        <v>590</v>
+        <v>451</v>
+      </c>
+      <c r="C291" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B292" t="s">
-        <v>426</v>
+        <v>452</v>
+      </c>
+      <c r="C292" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B293" t="s">
-        <v>427</v>
+        <v>590</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B294" t="s">
-        <v>453</v>
+        <v>426</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B295" t="s">
-        <v>454</v>
+        <v>427</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B296" t="s">
-        <v>430</v>
+        <v>453</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B297" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>529</v>
+        <v>447</v>
       </c>
       <c r="B298" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>622</v>
+        <v>448</v>
       </c>
       <c r="B299" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3">
+      <c r="A300" t="s">
+        <v>529</v>
+      </c>
+      <c r="B300" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>742</v>
+        <v>622</v>
       </c>
       <c r="B301" t="s">
-        <v>743</v>
-      </c>
-      <c r="C301" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="302" spans="1:3">
-      <c r="A302" t="s">
-        <v>432</v>
-      </c>
-      <c r="B302" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>433</v>
+        <v>742</v>
       </c>
       <c r="B303" t="s">
-        <v>624</v>
+        <v>743</v>
       </c>
       <c r="C303" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
+        <v>432</v>
+      </c>
+      <c r="B304" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3">
+      <c r="A305" t="s">
+        <v>433</v>
+      </c>
+      <c r="B305" t="s">
+        <v>624</v>
+      </c>
+      <c r="C305" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3">
+      <c r="A306" t="s">
         <v>511</v>
       </c>
-      <c r="B304" t="s">
+      <c r="B306" t="s">
         <v>625</v>
       </c>
     </row>
-    <row r="305" spans="1:2">
-      <c r="A305" t="s">
+    <row r="307" spans="1:3">
+      <c r="A307" t="s">
         <v>434</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B307" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="306" spans="1:2">
-      <c r="A306" t="s">
+    <row r="308" spans="1:3">
+      <c r="A308" t="s">
         <v>435</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B308" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="307" spans="1:2">
-      <c r="A307" t="s">
+    <row r="309" spans="1:3">
+      <c r="A309" t="s">
         <v>436</v>
       </c>
-      <c r="B307" t="s">
+      <c r="B309" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="308" spans="1:2">
-      <c r="A308" t="s">
+    <row r="310" spans="1:3">
+      <c r="A310" t="s">
         <v>528</v>
       </c>
-      <c r="B308" t="s">
+      <c r="B310" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DU for AS and IAQ is disabled
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD6162E-D11E-4E80-BDAF-736920B3B7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95B4A76B-7CF5-4A6E-A573-2AAE1BD1A386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2190" yWindow="3960" windowWidth="28170" windowHeight="13710" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2325,13 +2325,13 @@
     <t>Asset Self Certification is missing from the application.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>SCNE_EmploymentDocumented</t>
   </si>
   <si>
     <t>Currently employment has been documented on the Self-Certification of Non-Employment but no current employment was documented on the ICW for that member.</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2789,7 +2789,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7529,10 +7529,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>761</v>
+      </c>
+      <c r="B69" t="s">
         <v>762</v>
-      </c>
-      <c r="B69" t="s">
-        <v>763</v>
       </c>
       <c r="C69" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Changes for 58031 - SCNE employed checkbox marked yes, 58073 - updated the validation logic to ensure blank ASCWs are excluded from comparison with the ASC, 57074 - if the letter version is 'yearly' no Move In Date finding is created for the SSBL, 58054 - new MID prompt validation
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95B4A76B-7CF5-4A6E-A573-2AAE1BD1A386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CCA124-D571-4C79-B2DF-958740E9F480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="20970" windowHeight="9660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="772">
   <si>
     <t>Name</t>
   </si>
@@ -2325,13 +2325,37 @@
     <t>Asset Self Certification is missing from the application.</t>
   </si>
   <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
     <t>SCNE_EmploymentDocumented</t>
   </si>
   <si>
-    <t>Currently employment has been documented on the Self-Certification of Non-Employment but no current employment was documented on the ICW for that member.</t>
-  </si>
-  <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>Currently employment has been documented on the Self-Certification of Non-Employment. Manual review required.</t>
+  </si>
+  <si>
+    <t>HHD_IsSigned</t>
+  </si>
+  <si>
+    <t>HHD_IsDated</t>
+  </si>
+  <si>
+    <t>The member signature is missing from the Housing History Disclosure.</t>
+  </si>
+  <si>
+    <t>The date signed is missing from the Housing History Disclosure.</t>
+  </si>
+  <si>
+    <t>HHD_OwningCurrentAddress</t>
+  </si>
+  <si>
+    <t>The applicant reported owning their current residence, but Real Estate was marked as "No" on the ICW.</t>
+  </si>
+  <si>
+    <t>HHD_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Housing History Disclosure. Needs manual review.</t>
   </si>
 </sst>
 </file>
@@ -2789,7 +2813,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -6980,7 +7004,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C310"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -7015,400 +7039,400 @@
         <v>692</v>
       </c>
     </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B6" t="s">
+        <v>766</v>
+      </c>
+      <c r="C6" t="s">
+        <v>692</v>
+      </c>
+    </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>765</v>
       </c>
       <c r="B7" t="s">
-        <v>496</v>
+        <v>767</v>
+      </c>
+      <c r="C7" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>768</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>769</v>
+      </c>
+      <c r="C8" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>179</v>
+        <v>770</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" t="s">
-        <v>74</v>
+        <v>771</v>
+      </c>
+      <c r="C9" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>180</v>
       </c>
       <c r="B11" t="s">
-        <v>207</v>
-      </c>
-      <c r="C11" t="s">
-        <v>659</v>
+        <v>496</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>549</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>550</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>687</v>
+        <v>179</v>
       </c>
       <c r="B13" t="s">
-        <v>688</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>531</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
-        <v>667</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>700</v>
+        <v>206</v>
       </c>
       <c r="B15" t="s">
-        <v>701</v>
+        <v>207</v>
       </c>
       <c r="C15" t="s">
-        <v>692</v>
+        <v>659</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>715</v>
+        <v>549</v>
       </c>
       <c r="B16" t="s">
-        <v>716</v>
-      </c>
-      <c r="C16" t="s">
-        <v>692</v>
+        <v>550</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>729</v>
+        <v>687</v>
       </c>
       <c r="B17" t="s">
-        <v>730</v>
-      </c>
-      <c r="C17" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>732</v>
+        <v>531</v>
       </c>
       <c r="B18" t="s">
-        <v>737</v>
-      </c>
-      <c r="C18" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>700</v>
+      </c>
+      <c r="B19" t="s">
+        <v>701</v>
+      </c>
+      <c r="C19" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>715</v>
       </c>
       <c r="B20" t="s">
-        <v>182</v>
+        <v>716</v>
+      </c>
+      <c r="C20" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>79</v>
+        <v>729</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>730</v>
+      </c>
+      <c r="C21" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>558</v>
+        <v>732</v>
       </c>
       <c r="B22" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" t="s">
-        <v>76</v>
+        <v>737</v>
+      </c>
+      <c r="C22" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>82</v>
+        <v>181</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>79</v>
       </c>
       <c r="B25" t="s">
-        <v>197</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>558</v>
       </c>
       <c r="B26" t="s">
-        <v>199</v>
+        <v>559</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>81</v>
+        <v>196</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>198</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>631</v>
+        <v>84</v>
       </c>
       <c r="B31" t="s">
-        <v>632</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>655</v>
+        <v>86</v>
       </c>
       <c r="B32" t="s">
-        <v>656</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>546</v>
+        <v>81</v>
       </c>
       <c r="B33" t="s">
-        <v>668</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>717</v>
+        <v>89</v>
       </c>
       <c r="B34" t="s">
-        <v>718</v>
-      </c>
-      <c r="C34" t="s">
-        <v>692</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>631</v>
+      </c>
+      <c r="B35" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>183</v>
+        <v>655</v>
       </c>
       <c r="B36" t="s">
-        <v>185</v>
+        <v>656</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>91</v>
+        <v>546</v>
       </c>
       <c r="B37" t="s">
-        <v>92</v>
+        <v>668</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>93</v>
+        <v>717</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>101</v>
-      </c>
-      <c r="B39" t="s">
-        <v>95</v>
+        <v>718</v>
+      </c>
+      <c r="C38" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>102</v>
+        <v>183</v>
       </c>
       <c r="B40" t="s">
-        <v>96</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B43" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" t="s">
-        <v>588</v>
+        <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>633</v>
+        <v>103</v>
       </c>
       <c r="B45" t="s">
-        <v>634</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>545</v>
+        <v>104</v>
       </c>
       <c r="B46" t="s">
-        <v>669</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>693</v>
+        <v>105</v>
       </c>
       <c r="B47" t="s">
-        <v>694</v>
+        <v>99</v>
       </c>
       <c r="C47" t="s">
-        <v>692</v>
+        <v>588</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>106</v>
+      </c>
+      <c r="B48" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>184</v>
+        <v>633</v>
       </c>
       <c r="B49" t="s">
-        <v>591</v>
+        <v>634</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>107</v>
+        <v>545</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
-      </c>
-      <c r="C50" t="s">
-        <v>588</v>
+        <v>669</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>117</v>
+        <v>693</v>
       </c>
       <c r="B51" t="s">
-        <v>118</v>
+        <v>694</v>
       </c>
       <c r="C51" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>119</v>
-      </c>
-      <c r="B52" t="s">
-        <v>120</v>
-      </c>
-      <c r="C52" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>113</v>
+        <v>184</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
-      </c>
-      <c r="C53" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C54" t="s">
         <v>588</v>
@@ -7416,10 +7440,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B55" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C55" t="s">
         <v>588</v>
@@ -7427,26 +7451,32 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>120</v>
+      </c>
+      <c r="C56" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>204</v>
+        <v>113</v>
       </c>
       <c r="B57" t="s">
-        <v>494</v>
+        <v>109</v>
+      </c>
+      <c r="C57" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>205</v>
+        <v>114</v>
       </c>
       <c r="B58" t="s">
-        <v>592</v>
+        <v>110</v>
       </c>
       <c r="C58" t="s">
         <v>588</v>
@@ -7454,112 +7484,123 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>579</v>
+        <v>115</v>
       </c>
       <c r="B59" t="s">
-        <v>593</v>
+        <v>111</v>
+      </c>
+      <c r="C59" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>547</v>
+        <v>116</v>
       </c>
       <c r="B60" t="s">
-        <v>548</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>555</v>
+        <v>204</v>
       </c>
       <c r="B61" t="s">
-        <v>630</v>
+        <v>494</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>544</v>
+        <v>205</v>
       </c>
       <c r="B62" t="s">
-        <v>670</v>
+        <v>592</v>
+      </c>
+      <c r="C62" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>750</v>
+        <v>579</v>
       </c>
       <c r="B63" t="s">
-        <v>749</v>
-      </c>
-      <c r="C63" t="s">
-        <v>692</v>
+        <v>593</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>547</v>
+      </c>
+      <c r="B64" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>158</v>
+        <v>555</v>
       </c>
       <c r="B65" t="s">
-        <v>121</v>
+        <v>630</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>122</v>
+        <v>544</v>
       </c>
       <c r="B66" t="s">
-        <v>594</v>
+        <v>670</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>124</v>
+        <v>750</v>
       </c>
       <c r="B67" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" t="s">
-        <v>635</v>
-      </c>
-      <c r="B68" t="s">
-        <v>636</v>
+        <v>749</v>
+      </c>
+      <c r="C67" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>761</v>
+        <v>158</v>
       </c>
       <c r="B69" t="s">
-        <v>762</v>
-      </c>
-      <c r="C69" t="s">
-        <v>692</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>543</v>
+        <v>122</v>
       </c>
       <c r="B70" t="s">
-        <v>671</v>
+        <v>594</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>124</v>
+      </c>
+      <c r="B71" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>186</v>
+        <v>635</v>
       </c>
       <c r="B72" t="s">
-        <v>187</v>
+        <v>636</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B73" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="C73" t="s">
         <v>692</v>
@@ -7567,520 +7608,509 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>757</v>
+        <v>543</v>
       </c>
       <c r="B74" t="s">
-        <v>758</v>
-      </c>
-      <c r="C74" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>125</v>
-      </c>
-      <c r="B75" t="s">
-        <v>127</v>
+        <v>671</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
       <c r="B76" t="s">
-        <v>128</v>
+        <v>187</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>138</v>
+        <v>759</v>
       </c>
       <c r="B77" t="s">
-        <v>595</v>
+        <v>760</v>
+      </c>
+      <c r="C77" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>139</v>
+        <v>757</v>
       </c>
       <c r="B78" t="s">
-        <v>596</v>
+        <v>758</v>
+      </c>
+      <c r="C78" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B79" t="s">
-        <v>597</v>
+        <v>127</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="B80" t="s">
-        <v>598</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B81" t="s">
-        <v>495</v>
-      </c>
-      <c r="C81" t="s">
-        <v>686</v>
+        <v>595</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B82" t="s">
-        <v>497</v>
-      </c>
-      <c r="C82" t="s">
-        <v>556</v>
+        <v>596</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B83" t="s">
-        <v>498</v>
-      </c>
-      <c r="C83" t="s">
-        <v>556</v>
+        <v>597</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>637</v>
+        <v>141</v>
       </c>
       <c r="B84" t="s">
-        <v>638</v>
+        <v>598</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>719</v>
+        <v>142</v>
       </c>
       <c r="B85" t="s">
-        <v>720</v>
+        <v>495</v>
       </c>
       <c r="C85" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>751</v>
+        <v>143</v>
       </c>
       <c r="B86" t="s">
-        <v>752</v>
+        <v>497</v>
       </c>
       <c r="C86" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>754</v>
+        <v>144</v>
       </c>
       <c r="B87" t="s">
-        <v>753</v>
+        <v>498</v>
       </c>
       <c r="C87" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>756</v>
+        <v>637</v>
       </c>
       <c r="B88" t="s">
-        <v>755</v>
-      </c>
-      <c r="C88" t="s">
-        <v>692</v>
+        <v>638</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>542</v>
+        <v>719</v>
       </c>
       <c r="B89" t="s">
-        <v>672</v>
+        <v>720</v>
+      </c>
+      <c r="C89" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" t="s">
+        <v>751</v>
+      </c>
+      <c r="B90" t="s">
+        <v>752</v>
+      </c>
+      <c r="C90" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>147</v>
+        <v>754</v>
       </c>
       <c r="B91" t="s">
-        <v>150</v>
+        <v>753</v>
+      </c>
+      <c r="C91" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>148</v>
+        <v>756</v>
       </c>
       <c r="B92" t="s">
-        <v>151</v>
+        <v>755</v>
+      </c>
+      <c r="C92" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>149</v>
+        <v>542</v>
       </c>
       <c r="B93" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" t="s">
-        <v>145</v>
-      </c>
-      <c r="B94" t="s">
-        <v>580</v>
-      </c>
-      <c r="C94" t="s">
-        <v>691</v>
+        <v>672</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>690</v>
+        <v>147</v>
       </c>
       <c r="B95" t="s">
-        <v>580</v>
+        <v>150</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="B97" t="s">
-        <v>599</v>
+        <v>152</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="B98" t="s">
-        <v>130</v>
+        <v>580</v>
+      </c>
+      <c r="C98" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>639</v>
+        <v>690</v>
       </c>
       <c r="B99" t="s">
-        <v>640</v>
+        <v>580</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>541</v>
+        <v>146</v>
       </c>
       <c r="B100" t="s">
-        <v>673</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" t="s">
+        <v>131</v>
+      </c>
+      <c r="B101" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>188</v>
+        <v>132</v>
       </c>
       <c r="B102" t="s">
-        <v>189</v>
+        <v>130</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>133</v>
+        <v>639</v>
       </c>
       <c r="B103" t="s">
-        <v>153</v>
+        <v>640</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>135</v>
+        <v>541</v>
       </c>
       <c r="B104" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3">
-      <c r="A105" t="s">
-        <v>134</v>
-      </c>
-      <c r="B105" t="s">
-        <v>155</v>
+        <v>673</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>136</v>
+        <v>188</v>
       </c>
       <c r="B106" t="s">
-        <v>156</v>
+        <v>189</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B107" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>629</v>
+        <v>135</v>
       </c>
       <c r="B108" t="s">
-        <v>695</v>
-      </c>
-      <c r="C108" t="s">
-        <v>699</v>
+        <v>154</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>641</v>
+        <v>134</v>
       </c>
       <c r="B109" t="s">
-        <v>642</v>
+        <v>155</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>540</v>
+        <v>136</v>
       </c>
       <c r="B110" t="s">
-        <v>674</v>
+        <v>156</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>721</v>
+        <v>137</v>
       </c>
       <c r="B111" t="s">
-        <v>722</v>
-      </c>
-      <c r="C111" t="s">
-        <v>692</v>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" t="s">
+        <v>629</v>
+      </c>
+      <c r="B112" t="s">
+        <v>695</v>
+      </c>
+      <c r="C112" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>710</v>
+        <v>641</v>
       </c>
       <c r="B113" t="s">
-        <v>711</v>
-      </c>
-      <c r="C113" t="s">
-        <v>712</v>
+        <v>642</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>713</v>
+        <v>540</v>
       </c>
       <c r="B114" t="s">
-        <v>714</v>
-      </c>
-      <c r="C114" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3">
-      <c r="A116" t="s">
-        <v>159</v>
-      </c>
-      <c r="B116" t="s">
-        <v>163</v>
+        <v>674</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" t="s">
+        <v>721</v>
+      </c>
+      <c r="B115" t="s">
+        <v>722</v>
+      </c>
+      <c r="C115" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>160</v>
+        <v>710</v>
       </c>
       <c r="B117" t="s">
-        <v>164</v>
+        <v>711</v>
+      </c>
+      <c r="C117" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>161</v>
+        <v>713</v>
       </c>
       <c r="B118" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3">
-      <c r="A119" t="s">
-        <v>162</v>
-      </c>
-      <c r="B119" t="s">
-        <v>600</v>
+        <v>714</v>
+      </c>
+      <c r="C118" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>557</v>
+        <v>159</v>
       </c>
       <c r="B120" t="s">
-        <v>739</v>
-      </c>
-      <c r="C120" t="s">
-        <v>740</v>
+        <v>163</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>647</v>
+        <v>160</v>
       </c>
       <c r="B121" t="s">
-        <v>648</v>
+        <v>164</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>539</v>
+        <v>161</v>
       </c>
       <c r="B122" t="s">
-        <v>675</v>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" t="s">
+        <v>162</v>
+      </c>
+      <c r="B123" t="s">
+        <v>600</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>192</v>
+        <v>557</v>
       </c>
       <c r="B124" t="s">
-        <v>193</v>
+        <v>739</v>
+      </c>
+      <c r="C124" t="s">
+        <v>740</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>166</v>
+        <v>647</v>
       </c>
       <c r="B125" t="s">
-        <v>168</v>
+        <v>648</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>167</v>
+        <v>539</v>
       </c>
       <c r="B126" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3">
-      <c r="A127" t="s">
-        <v>643</v>
-      </c>
-      <c r="B127" t="s">
-        <v>644</v>
+        <v>675</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>538</v>
+        <v>192</v>
       </c>
       <c r="B128" t="s">
-        <v>676</v>
+        <v>193</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>723</v>
+        <v>166</v>
       </c>
       <c r="B129" t="s">
-        <v>724</v>
-      </c>
-      <c r="C129" t="s">
-        <v>692</v>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3">
+      <c r="A130" t="s">
+        <v>167</v>
+      </c>
+      <c r="B130" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>190</v>
+        <v>643</v>
       </c>
       <c r="B131" t="s">
-        <v>191</v>
+        <v>644</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>175</v>
+        <v>538</v>
       </c>
       <c r="B132" t="s">
-        <v>172</v>
-      </c>
-      <c r="C132" t="s">
-        <v>588</v>
+        <v>676</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>170</v>
+        <v>723</v>
       </c>
       <c r="B133" t="s">
-        <v>173</v>
+        <v>724</v>
       </c>
       <c r="C133" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" t="s">
-        <v>171</v>
-      </c>
-      <c r="B134" t="s">
-        <v>174</v>
-      </c>
-      <c r="C134" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>203</v>
+        <v>190</v>
       </c>
       <c r="B135" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="B136" t="s">
-        <v>201</v>
+        <v>172</v>
+      </c>
+      <c r="C136" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B137" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C137" t="s">
         <v>588</v>
@@ -8088,1049 +8118,1055 @@
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>645</v>
+        <v>171</v>
       </c>
       <c r="B138" t="s">
-        <v>646</v>
+        <v>174</v>
+      </c>
+      <c r="C138" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>527</v>
+        <v>203</v>
       </c>
       <c r="B139" t="s">
-        <v>677</v>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
+        <v>200</v>
+      </c>
+      <c r="B140" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>652</v>
+        <v>176</v>
       </c>
       <c r="B141" t="s">
-        <v>653</v>
+        <v>177</v>
       </c>
       <c r="C141" t="s">
-        <v>654</v>
+        <v>588</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>727</v>
+        <v>645</v>
       </c>
       <c r="B142" t="s">
-        <v>728</v>
-      </c>
-      <c r="C142" t="s">
-        <v>692</v>
+        <v>646</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>733</v>
+        <v>527</v>
       </c>
       <c r="B143" t="s">
-        <v>734</v>
-      </c>
-      <c r="C143" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3">
-      <c r="A144" t="s">
-        <v>741</v>
-      </c>
-      <c r="B144" t="s">
-        <v>730</v>
-      </c>
-      <c r="C144" t="s">
-        <v>692</v>
+        <v>677</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" t="s">
+        <v>652</v>
+      </c>
+      <c r="B145" t="s">
+        <v>653</v>
+      </c>
+      <c r="C145" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>513</v>
+        <v>727</v>
       </c>
       <c r="B146" t="s">
-        <v>514</v>
+        <v>728</v>
+      </c>
+      <c r="C146" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>661</v>
+        <v>733</v>
       </c>
       <c r="B147" t="s">
-        <v>665</v>
+        <v>734</v>
       </c>
       <c r="C147" t="s">
-        <v>663</v>
+        <v>692</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>662</v>
+        <v>741</v>
       </c>
       <c r="B148" t="s">
-        <v>664</v>
+        <v>730</v>
       </c>
       <c r="C148" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3">
-      <c r="A149" t="s">
-        <v>242</v>
-      </c>
-      <c r="B149" t="s">
-        <v>243</v>
-      </c>
-      <c r="C149" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>244</v>
+        <v>513</v>
       </c>
       <c r="B150" t="s">
-        <v>245</v>
+        <v>514</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>258</v>
+        <v>661</v>
       </c>
       <c r="B151" t="s">
-        <v>560</v>
+        <v>665</v>
       </c>
       <c r="C151" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>247</v>
+        <v>662</v>
       </c>
       <c r="B152" t="s">
-        <v>246</v>
+        <v>664</v>
+      </c>
+      <c r="C152" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>503</v>
+        <v>242</v>
       </c>
       <c r="B153" t="s">
-        <v>512</v>
+        <v>243</v>
+      </c>
+      <c r="C153" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B154" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="B155" t="s">
-        <v>252</v>
+        <v>560</v>
+      </c>
+      <c r="C155" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B156" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>255</v>
+        <v>503</v>
       </c>
       <c r="B157" t="s">
-        <v>254</v>
+        <v>512</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B158" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>302</v>
+        <v>250</v>
       </c>
       <c r="B159" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>349</v>
+        <v>251</v>
       </c>
       <c r="B160" t="s">
-        <v>350</v>
+        <v>253</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>657</v>
+        <v>255</v>
       </c>
       <c r="B161" t="s">
-        <v>658</v>
+        <v>254</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>702</v>
+        <v>257</v>
       </c>
       <c r="B162" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>526</v>
+        <v>302</v>
       </c>
       <c r="B163" t="s">
-        <v>678</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3">
+      <c r="A164" t="s">
+        <v>349</v>
+      </c>
+      <c r="B164" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>515</v>
+        <v>657</v>
       </c>
       <c r="B165" t="s">
-        <v>516</v>
+        <v>658</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>259</v>
+        <v>702</v>
       </c>
       <c r="B166" t="s">
-        <v>262</v>
-      </c>
-      <c r="C166" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" ht="13.5" customHeight="1">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>261</v>
+        <v>526</v>
       </c>
       <c r="B167" t="s">
-        <v>561</v>
-      </c>
-      <c r="C167" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3">
-      <c r="A168" t="s">
-        <v>260</v>
-      </c>
-      <c r="B168" t="s">
-        <v>263</v>
+        <v>678</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>265</v>
+        <v>515</v>
       </c>
       <c r="B169" t="s">
-        <v>264</v>
+        <v>516</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="B170" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C170" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" ht="13.5" customHeight="1">
       <c r="A171" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="B171" t="s">
-        <v>268</v>
+        <v>561</v>
       </c>
       <c r="C171" t="s">
-        <v>660</v>
+        <v>696</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>504</v>
+        <v>260</v>
       </c>
       <c r="B172" t="s">
-        <v>570</v>
+        <v>263</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B173" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="B174" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="B175" t="s">
-        <v>287</v>
+        <v>268</v>
+      </c>
+      <c r="C175" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>278</v>
+        <v>504</v>
       </c>
       <c r="B176" t="s">
-        <v>286</v>
+        <v>570</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="B177" t="s">
-        <v>285</v>
-      </c>
-      <c r="C177" t="s">
-        <v>660</v>
+        <v>271</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="B178" t="s">
-        <v>605</v>
+        <v>273</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B179" t="s">
-        <v>284</v>
-      </c>
-      <c r="C179" t="s">
-        <v>660</v>
+        <v>287</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B180" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="B181" t="s">
-        <v>300</v>
+        <v>285</v>
+      </c>
+      <c r="C181" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>301</v>
+        <v>280</v>
       </c>
       <c r="B182" t="s">
-        <v>248</v>
+        <v>605</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>304</v>
+        <v>281</v>
       </c>
       <c r="B183" t="s">
-        <v>305</v>
+        <v>284</v>
+      </c>
+      <c r="C183" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>704</v>
+        <v>282</v>
       </c>
       <c r="B184" t="s">
-        <v>703</v>
+        <v>283</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>537</v>
+        <v>299</v>
       </c>
       <c r="B185" t="s">
-        <v>679</v>
+        <v>300</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>697</v>
+        <v>301</v>
       </c>
       <c r="B186" t="s">
-        <v>698</v>
-      </c>
-      <c r="C186" t="s">
-        <v>692</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3">
+      <c r="A187" t="s">
+        <v>304</v>
+      </c>
+      <c r="B187" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>517</v>
+        <v>704</v>
       </c>
       <c r="B188" t="s">
-        <v>518</v>
+        <v>703</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>292</v>
+        <v>537</v>
       </c>
       <c r="B189" t="s">
-        <v>296</v>
-      </c>
-      <c r="C189" t="s">
-        <v>588</v>
+        <v>679</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>505</v>
+        <v>697</v>
       </c>
       <c r="B190" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3">
-      <c r="A191" t="s">
-        <v>293</v>
-      </c>
-      <c r="B191" t="s">
-        <v>297</v>
-      </c>
-      <c r="C191" t="s">
-        <v>588</v>
+        <v>698</v>
+      </c>
+      <c r="C190" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>294</v>
+        <v>517</v>
       </c>
       <c r="B192" t="s">
-        <v>298</v>
+        <v>518</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B193" t="s">
-        <v>562</v>
+        <v>296</v>
+      </c>
+      <c r="C193" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>303</v>
+        <v>505</v>
       </c>
       <c r="B194" t="s">
-        <v>248</v>
+        <v>571</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="B195" t="s">
-        <v>310</v>
+        <v>297</v>
+      </c>
+      <c r="C195" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="B196" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="B197" t="s">
-        <v>308</v>
+        <v>562</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="B198" t="s">
-        <v>312</v>
+        <v>248</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>705</v>
+        <v>309</v>
       </c>
       <c r="B199" t="s">
-        <v>703</v>
+        <v>310</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>536</v>
+        <v>306</v>
       </c>
       <c r="B200" t="s">
-        <v>680</v>
+        <v>308</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3">
+      <c r="A201" t="s">
+        <v>307</v>
+      </c>
+      <c r="B201" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>519</v>
+        <v>311</v>
       </c>
       <c r="B202" t="s">
-        <v>520</v>
+        <v>312</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>499</v>
+        <v>705</v>
       </c>
       <c r="B203" t="s">
-        <v>320</v>
-      </c>
-      <c r="C203" t="s">
-        <v>588</v>
+        <v>703</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>506</v>
+        <v>536</v>
       </c>
       <c r="B204" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="205" spans="1:3">
-      <c r="A205" t="s">
-        <v>315</v>
-      </c>
-      <c r="B205" t="s">
-        <v>321</v>
-      </c>
-      <c r="C205" t="s">
-        <v>588</v>
+        <v>680</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>316</v>
+        <v>519</v>
       </c>
       <c r="B206" t="s">
-        <v>322</v>
+        <v>520</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>317</v>
+        <v>499</v>
       </c>
       <c r="B207" t="s">
-        <v>323</v>
+        <v>320</v>
+      </c>
+      <c r="C207" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>318</v>
+        <v>506</v>
       </c>
       <c r="B208" t="s">
-        <v>563</v>
+        <v>572</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B209" t="s">
-        <v>248</v>
+        <v>321</v>
+      </c>
+      <c r="C209" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="B210" t="s">
-        <v>325</v>
-      </c>
-      <c r="C210" t="s">
-        <v>588</v>
+        <v>322</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="B211" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="B212" t="s">
-        <v>328</v>
+        <v>563</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="B213" t="s">
-        <v>331</v>
+        <v>248</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="B214" t="s">
-        <v>256</v>
+        <v>325</v>
+      </c>
+      <c r="C214" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>706</v>
+        <v>326</v>
       </c>
       <c r="B215" t="s">
-        <v>703</v>
+        <v>327</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>535</v>
+        <v>329</v>
       </c>
       <c r="B216" t="s">
-        <v>681</v>
+        <v>328</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3">
+      <c r="A217" t="s">
+        <v>330</v>
+      </c>
+      <c r="B217" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>521</v>
+        <v>332</v>
       </c>
       <c r="B218" t="s">
-        <v>522</v>
+        <v>256</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>501</v>
+        <v>706</v>
       </c>
       <c r="B219" t="s">
-        <v>338</v>
-      </c>
-      <c r="C219" t="s">
-        <v>588</v>
+        <v>703</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>507</v>
+        <v>535</v>
       </c>
       <c r="B220" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="221" spans="1:3">
-      <c r="A221" t="s">
-        <v>336</v>
-      </c>
-      <c r="B221" t="s">
-        <v>339</v>
-      </c>
-      <c r="C221" t="s">
-        <v>588</v>
+        <v>681</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>337</v>
+        <v>521</v>
       </c>
       <c r="B222" t="s">
-        <v>340</v>
+        <v>522</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B223" t="s">
-        <v>564</v>
+        <v>338</v>
+      </c>
+      <c r="C223" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>344</v>
+        <v>507</v>
       </c>
       <c r="B224" t="s">
-        <v>248</v>
+        <v>573</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="B225" t="s">
-        <v>341</v>
+        <v>339</v>
+      </c>
+      <c r="C225" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="B226" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>347</v>
+        <v>500</v>
       </c>
       <c r="B227" t="s">
-        <v>343</v>
+        <v>564</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="B228" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>707</v>
+        <v>345</v>
       </c>
       <c r="B229" t="s">
-        <v>703</v>
+        <v>341</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>534</v>
+        <v>346</v>
       </c>
       <c r="B230" t="s">
-        <v>682</v>
+        <v>342</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3">
+      <c r="A231" t="s">
+        <v>347</v>
+      </c>
+      <c r="B231" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>746</v>
+        <v>348</v>
       </c>
       <c r="B232" t="s">
-        <v>747</v>
-      </c>
-      <c r="C232" t="s">
-        <v>692</v>
+        <v>256</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>551</v>
+        <v>707</v>
       </c>
       <c r="B233" t="s">
-        <v>554</v>
-      </c>
-      <c r="C233" t="s">
-        <v>586</v>
+        <v>703</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>552</v>
+        <v>534</v>
       </c>
       <c r="B234" t="s">
-        <v>553</v>
-      </c>
-      <c r="C234" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
-        <v>585</v>
-      </c>
-      <c r="B235" t="s">
-        <v>601</v>
+        <v>682</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>365</v>
+        <v>746</v>
       </c>
       <c r="B236" t="s">
-        <v>351</v>
+        <v>747</v>
+      </c>
+      <c r="C236" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>366</v>
+        <v>551</v>
       </c>
       <c r="B237" t="s">
-        <v>352</v>
+        <v>554</v>
       </c>
       <c r="C237" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>508</v>
+        <v>552</v>
       </c>
       <c r="B238" t="s">
-        <v>574</v>
+        <v>553</v>
+      </c>
+      <c r="C238" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>367</v>
+        <v>585</v>
       </c>
       <c r="B239" t="s">
-        <v>353</v>
+        <v>601</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B240" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B241" t="s">
-        <v>355</v>
+        <v>352</v>
+      </c>
+      <c r="C241" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>370</v>
+        <v>508</v>
       </c>
       <c r="B242" t="s">
-        <v>356</v>
-      </c>
-      <c r="C242" t="s">
-        <v>588</v>
+        <v>574</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B243" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B244" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B245" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B246" t="s">
-        <v>360</v>
+        <v>356</v>
+      </c>
+      <c r="C246" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B247" t="s">
-        <v>361</v>
-      </c>
-      <c r="C247" t="s">
-        <v>588</v>
+        <v>357</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B248" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B249" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B250" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>533</v>
+        <v>375</v>
       </c>
       <c r="B251" t="s">
-        <v>666</v>
+        <v>361</v>
+      </c>
+      <c r="C251" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3">
+      <c r="A252" t="s">
+        <v>376</v>
+      </c>
+      <c r="B252" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>606</v>
+        <v>377</v>
       </c>
       <c r="B253" t="s">
-        <v>607</v>
+        <v>363</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B254" t="s">
-        <v>403</v>
+        <v>364</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>386</v>
+        <v>533</v>
       </c>
       <c r="B255" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="256" spans="1:3">
-      <c r="A256" t="s">
-        <v>387</v>
-      </c>
-      <c r="B256" t="s">
-        <v>401</v>
-      </c>
-      <c r="C256" t="s">
-        <v>588</v>
+        <v>666</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>509</v>
+        <v>606</v>
       </c>
       <c r="B257" t="s">
-        <v>575</v>
+        <v>607</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>404</v>
+        <v>385</v>
       </c>
       <c r="B258" t="s">
-        <v>402</v>
-      </c>
-      <c r="C258" t="s">
-        <v>588</v>
+        <v>403</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B259" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>405</v>
+        <v>387</v>
       </c>
       <c r="B260" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C260" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>389</v>
+        <v>509</v>
       </c>
       <c r="B261" t="s">
-        <v>396</v>
+        <v>575</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="B262" t="s">
-        <v>397</v>
+        <v>402</v>
+      </c>
+      <c r="C262" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B263" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="B264" t="s">
-        <v>399</v>
+        <v>395</v>
+      </c>
+      <c r="C264" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="B265" t="s">
         <v>396</v>
@@ -9138,359 +9174,391 @@
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>532</v>
+        <v>391</v>
       </c>
       <c r="B266" t="s">
-        <v>683</v>
+        <v>397</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3">
+      <c r="A267" t="s">
+        <v>390</v>
+      </c>
+      <c r="B267" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>748</v>
+        <v>392</v>
       </c>
       <c r="B268" t="s">
-        <v>745</v>
-      </c>
-      <c r="C268" t="s">
-        <v>692</v>
+        <v>399</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3">
+      <c r="A269" t="s">
+        <v>393</v>
+      </c>
+      <c r="B269" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>744</v>
+        <v>532</v>
       </c>
       <c r="B270" t="s">
-        <v>745</v>
-      </c>
-      <c r="C270" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="271" spans="1:3">
-      <c r="A271" t="s">
-        <v>523</v>
-      </c>
-      <c r="B271" t="s">
-        <v>524</v>
+        <v>683</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>411</v>
+        <v>748</v>
       </c>
       <c r="B272" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="273" spans="1:3">
-      <c r="A273" t="s">
-        <v>412</v>
-      </c>
-      <c r="B273" t="s">
-        <v>423</v>
-      </c>
-      <c r="C273" t="s">
-        <v>588</v>
+        <v>745</v>
+      </c>
+      <c r="C272" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>576</v>
+        <v>744</v>
       </c>
       <c r="B274" t="s">
-        <v>577</v>
+        <v>745</v>
+      </c>
+      <c r="C274" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>413</v>
+        <v>523</v>
       </c>
       <c r="B275" t="s">
-        <v>424</v>
-      </c>
-      <c r="C275" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B276" t="s">
-        <v>425</v>
-      </c>
-      <c r="C276" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B277" t="s">
-        <v>589</v>
+        <v>423</v>
+      </c>
+      <c r="C277" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>416</v>
+        <v>576</v>
       </c>
       <c r="B278" t="s">
-        <v>426</v>
+        <v>577</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="B279" t="s">
-        <v>427</v>
+        <v>424</v>
+      </c>
+      <c r="C279" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B280" t="s">
-        <v>428</v>
+        <v>425</v>
+      </c>
+      <c r="C280" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="B281" t="s">
-        <v>429</v>
+        <v>589</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B282" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="B283" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>530</v>
+        <v>418</v>
       </c>
       <c r="B284" t="s">
-        <v>684</v>
+        <v>428</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>615</v>
+        <v>419</v>
       </c>
       <c r="B285" t="s">
-        <v>616</v>
+        <v>429</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3">
+      <c r="A286" t="s">
+        <v>420</v>
+      </c>
+      <c r="B286" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>525</v>
+        <v>421</v>
       </c>
       <c r="B287" t="s">
-        <v>524</v>
+        <v>431</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>438</v>
+        <v>530</v>
       </c>
       <c r="B288" t="s">
-        <v>449</v>
+        <v>684</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>439</v>
+        <v>615</v>
       </c>
       <c r="B289" t="s">
-        <v>450</v>
-      </c>
-      <c r="C289" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="290" spans="1:3">
-      <c r="A290" t="s">
-        <v>510</v>
-      </c>
-      <c r="B290" t="s">
-        <v>578</v>
+        <v>616</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>440</v>
+        <v>525</v>
       </c>
       <c r="B291" t="s">
-        <v>451</v>
-      </c>
-      <c r="C291" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="B292" t="s">
-        <v>452</v>
-      </c>
-      <c r="C292" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B293" t="s">
-        <v>590</v>
+        <v>450</v>
+      </c>
+      <c r="C293" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>443</v>
+        <v>510</v>
       </c>
       <c r="B294" t="s">
-        <v>426</v>
+        <v>578</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="B295" t="s">
-        <v>427</v>
+        <v>451</v>
+      </c>
+      <c r="C295" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="B296" t="s">
-        <v>453</v>
+        <v>452</v>
+      </c>
+      <c r="C296" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="B297" t="s">
-        <v>454</v>
+        <v>590</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="B298" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="B299" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>529</v>
+        <v>445</v>
       </c>
       <c r="B300" t="s">
-        <v>684</v>
+        <v>453</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>622</v>
+        <v>446</v>
       </c>
       <c r="B301" t="s">
-        <v>616</v>
+        <v>454</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
+        <v>447</v>
+      </c>
+      <c r="B302" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>742</v>
+        <v>448</v>
       </c>
       <c r="B303" t="s">
-        <v>743</v>
-      </c>
-      <c r="C303" t="s">
-        <v>692</v>
+        <v>431</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>432</v>
+        <v>529</v>
       </c>
       <c r="B304" t="s">
-        <v>623</v>
+        <v>684</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>433</v>
+        <v>622</v>
       </c>
       <c r="B305" t="s">
-        <v>624</v>
-      </c>
-      <c r="C305" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="306" spans="1:3">
-      <c r="A306" t="s">
-        <v>511</v>
-      </c>
-      <c r="B306" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>434</v>
+        <v>742</v>
       </c>
       <c r="B307" t="s">
-        <v>651</v>
+        <v>743</v>
+      </c>
+      <c r="C307" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="B308" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="B309" t="s">
-        <v>627</v>
+        <v>624</v>
+      </c>
+      <c r="C309" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
+        <v>511</v>
+      </c>
+      <c r="B310" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3">
+      <c r="A311" t="s">
+        <v>434</v>
+      </c>
+      <c r="B311" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3">
+      <c r="A312" t="s">
+        <v>435</v>
+      </c>
+      <c r="B312" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3">
+      <c r="A313" t="s">
+        <v>436</v>
+      </c>
+      <c r="B313" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3">
+      <c r="A314" t="s">
         <v>528</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B314" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Commnetd out HHD, added ASC for DU
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CCA124-D571-4C79-B2DF-958740E9F480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE21DE6-8270-4C54-ACD0-6F084B1E2989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="20970" windowHeight="9660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2325,9 +2325,6 @@
     <t>Asset Self Certification is missing from the application.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>SCNE_EmploymentDocumented</t>
   </si>
   <si>
@@ -2356,6 +2353,9 @@
   </si>
   <si>
     <t>Unable to validate findings for Housing History Disclosure. Needs manual review.</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2813,7 +2813,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>761</v>
+        <v>771</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7041,10 +7041,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C6" t="s">
         <v>692</v>
@@ -7052,10 +7052,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B7" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C7" t="s">
         <v>692</v>
@@ -7063,10 +7063,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
+        <v>767</v>
+      </c>
+      <c r="B8" t="s">
         <v>768</v>
-      </c>
-      <c r="B8" t="s">
-        <v>769</v>
       </c>
       <c r="C8" t="s">
         <v>692</v>
@@ -7074,10 +7074,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
+        <v>769</v>
+      </c>
+      <c r="B9" t="s">
         <v>770</v>
-      </c>
-      <c r="B9" t="s">
-        <v>771</v>
       </c>
       <c r="C9" t="s">
         <v>692</v>
@@ -7597,10 +7597,10 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
+        <v>761</v>
+      </c>
+      <c r="B73" t="s">
         <v>762</v>
-      </c>
-      <c r="B73" t="s">
-        <v>763</v>
       </c>
       <c r="C73" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Changes for 57813 for checking if the applicant owns the current address and it is also documented on the IAQ; if not documented on the IAQ, it is adding a finding
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE21DE6-8270-4C54-ACD0-6F084B1E2989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC06EB4-9A42-4549-8476-C2408D58E816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4395" yWindow="4740" windowWidth="28170" windowHeight="13710" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="772">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="775">
   <si>
     <t>Name</t>
   </si>
@@ -2217,9 +2217,6 @@
     <t>Not all adults in the household have signed the VAWA.</t>
   </si>
   <si>
-    <t>The Housing History Disclosure form is a required document but missing from the application.</t>
-  </si>
-  <si>
     <t>HousingDisclosureExists</t>
   </si>
   <si>
@@ -2337,25 +2334,37 @@
     <t>HHD_IsDated</t>
   </si>
   <si>
-    <t>The member signature is missing from the Housing History Disclosure.</t>
-  </si>
-  <si>
-    <t>The date signed is missing from the Housing History Disclosure.</t>
-  </si>
-  <si>
     <t>HHD_OwningCurrentAddress</t>
   </si>
   <si>
-    <t>The applicant reported owning their current residence, but Real Estate was marked as "No" on the ICW.</t>
-  </si>
-  <si>
     <t>HHD_FindingError</t>
   </si>
   <si>
     <t>Unable to validate findings for Housing History Disclosure. Needs manual review.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for Child Support Calcs documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>Housing History Disclosure is a required document but it is missing from the application.</t>
+  </si>
+  <si>
+    <t>Housing History Disclosure has not been signed.</t>
+  </si>
+  <si>
+    <t>Housing History Disclosure has not been dated.</t>
+  </si>
+  <si>
+    <t>Housing History Disclosure date is not within 120 days of the Move-In date.</t>
+  </si>
+  <si>
+    <t>Housing History Disclosure form states the applicant owns their current address but they documented no Real Estate on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>HHD_MoveInDateCheck</t>
   </si>
 </sst>
 </file>
@@ -2813,7 +2822,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4617,10 +4626,10 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B21" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
@@ -6011,18 +6020,18 @@
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B39" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B40" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7004,7 +7013,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C314"/>
+  <dimension ref="A1:C315"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -7030,10 +7039,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B5" t="s">
-        <v>725</v>
+        <v>769</v>
       </c>
       <c r="C5" t="s">
         <v>692</v>
@@ -7041,10 +7050,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B6" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="C6" t="s">
         <v>692</v>
@@ -7052,10 +7061,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B7" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="C7" t="s">
         <v>692</v>
@@ -7063,10 +7072,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="B8" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="C8" t="s">
         <v>692</v>
@@ -7074,99 +7083,99 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="B9" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C9" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B11" t="s">
-        <v>496</v>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>765</v>
+      </c>
+      <c r="B10" t="s">
+        <v>766</v>
+      </c>
+      <c r="C10" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>180</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>496</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
-        <v>178</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>179</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>206</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>207</v>
-      </c>
-      <c r="C15" t="s">
-        <v>659</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>549</v>
+        <v>206</v>
       </c>
       <c r="B16" t="s">
-        <v>550</v>
+        <v>207</v>
+      </c>
+      <c r="C16" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>687</v>
+        <v>549</v>
       </c>
       <c r="B17" t="s">
-        <v>688</v>
+        <v>550</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>531</v>
+        <v>687</v>
       </c>
       <c r="B18" t="s">
-        <v>667</v>
+        <v>688</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>700</v>
+        <v>531</v>
       </c>
       <c r="B19" t="s">
-        <v>701</v>
-      </c>
-      <c r="C19" t="s">
-        <v>692</v>
+        <v>667</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>715</v>
+        <v>700</v>
       </c>
       <c r="B20" t="s">
-        <v>716</v>
+        <v>701</v>
       </c>
       <c r="C20" t="s">
         <v>692</v>
@@ -7174,10 +7183,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>729</v>
+        <v>715</v>
       </c>
       <c r="B21" t="s">
-        <v>730</v>
+        <v>716</v>
       </c>
       <c r="C21" t="s">
         <v>692</v>
@@ -7185,265 +7194,265 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="B22" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="C22" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" t="s">
-        <v>182</v>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>731</v>
+      </c>
+      <c r="B23" t="s">
+        <v>736</v>
+      </c>
+      <c r="C23" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>181</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>558</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>559</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>558</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>559</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>197</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B30" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>198</v>
       </c>
       <c r="B31" t="s">
-        <v>85</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>631</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>632</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>655</v>
+        <v>631</v>
       </c>
       <c r="B36" t="s">
-        <v>656</v>
+        <v>632</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>546</v>
+        <v>655</v>
       </c>
       <c r="B37" t="s">
-        <v>668</v>
+        <v>656</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>546</v>
+      </c>
+      <c r="B38" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
         <v>717</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>718</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>183</v>
-      </c>
-      <c r="B40" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>183</v>
       </c>
       <c r="B41" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B42" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
-      </c>
-      <c r="C47" t="s">
-        <v>588</v>
+        <v>98</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>99</v>
+      </c>
+      <c r="C48" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>633</v>
+        <v>106</v>
       </c>
       <c r="B49" t="s">
-        <v>634</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>545</v>
+        <v>633</v>
       </c>
       <c r="B50" t="s">
-        <v>669</v>
+        <v>634</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>545</v>
+      </c>
+      <c r="B51" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>693</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B52" t="s">
         <v>694</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C52" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>184</v>
-      </c>
-      <c r="B53" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>107</v>
+        <v>184</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
-      </c>
-      <c r="C54" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B55" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C55" t="s">
         <v>588</v>
@@ -7451,10 +7460,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B56" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C56" t="s">
         <v>588</v>
@@ -7462,10 +7471,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B57" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C57" t="s">
         <v>588</v>
@@ -7473,10 +7482,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B58" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C58" t="s">
         <v>588</v>
@@ -7484,10 +7493,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B59" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C59" t="s">
         <v>588</v>
@@ -7495,150 +7504,150 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="C60" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="B61" t="s">
-        <v>494</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B62" t="s">
-        <v>592</v>
-      </c>
-      <c r="C62" t="s">
-        <v>588</v>
+        <v>494</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>579</v>
+        <v>205</v>
       </c>
       <c r="B63" t="s">
-        <v>593</v>
+        <v>592</v>
+      </c>
+      <c r="C63" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>547</v>
+        <v>579</v>
       </c>
       <c r="B64" t="s">
-        <v>548</v>
+        <v>593</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="B65" t="s">
-        <v>630</v>
+        <v>548</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="B66" t="s">
-        <v>670</v>
+        <v>630</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>750</v>
+        <v>544</v>
       </c>
       <c r="B67" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
         <v>749</v>
       </c>
-      <c r="C67" t="s">
+      <c r="B68" t="s">
+        <v>748</v>
+      </c>
+      <c r="C68" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" t="s">
-        <v>158</v>
-      </c>
-      <c r="B69" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>122</v>
+        <v>158</v>
       </c>
       <c r="B70" t="s">
-        <v>594</v>
+        <v>121</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B71" t="s">
-        <v>123</v>
+        <v>594</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>635</v>
+        <v>124</v>
       </c>
       <c r="B72" t="s">
-        <v>636</v>
+        <v>123</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>761</v>
+        <v>635</v>
       </c>
       <c r="B73" t="s">
-        <v>762</v>
-      </c>
-      <c r="C73" t="s">
-        <v>692</v>
+        <v>636</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
+        <v>760</v>
+      </c>
+      <c r="B74" t="s">
+        <v>761</v>
+      </c>
+      <c r="C74" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
         <v>543</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
         <v>671</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76" t="s">
-        <v>186</v>
-      </c>
-      <c r="B76" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>759</v>
+        <v>186</v>
       </c>
       <c r="B77" t="s">
-        <v>760</v>
-      </c>
-      <c r="C77" t="s">
-        <v>692</v>
+        <v>187</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B78" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="C78" t="s">
         <v>692</v>
@@ -7646,80 +7655,80 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>125</v>
+        <v>756</v>
       </c>
       <c r="B79" t="s">
-        <v>127</v>
+        <v>757</v>
+      </c>
+      <c r="C79" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B80" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B81" t="s">
-        <v>595</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B82" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B83" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B84" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B85" t="s">
-        <v>495</v>
-      </c>
-      <c r="C85" t="s">
-        <v>686</v>
+        <v>598</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B86" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C86" t="s">
-        <v>556</v>
+        <v>686</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B87" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C87" t="s">
         <v>556</v>
@@ -7727,29 +7736,29 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>637</v>
+        <v>144</v>
       </c>
       <c r="B88" t="s">
-        <v>638</v>
+        <v>498</v>
+      </c>
+      <c r="C88" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>719</v>
+        <v>637</v>
       </c>
       <c r="B89" t="s">
-        <v>720</v>
-      </c>
-      <c r="C89" t="s">
-        <v>692</v>
+        <v>638</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>751</v>
+        <v>719</v>
       </c>
       <c r="B90" t="s">
-        <v>752</v>
+        <v>720</v>
       </c>
       <c r="C90" t="s">
         <v>692</v>
@@ -7757,10 +7766,10 @@
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="B91" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="C91" t="s">
         <v>692</v>
@@ -7768,10 +7777,10 @@
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="B92" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="C92" t="s">
         <v>692</v>
@@ -7779,338 +7788,338 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
+        <v>755</v>
+      </c>
+      <c r="B93" t="s">
+        <v>754</v>
+      </c>
+      <c r="C93" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
         <v>542</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B94" t="s">
         <v>672</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3">
-      <c r="A95" t="s">
-        <v>147</v>
-      </c>
-      <c r="B95" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B96" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B97" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B98" t="s">
-        <v>580</v>
-      </c>
-      <c r="C98" t="s">
-        <v>691</v>
+        <v>152</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>690</v>
+        <v>145</v>
       </c>
       <c r="B99" t="s">
         <v>580</v>
       </c>
+      <c r="C99" t="s">
+        <v>691</v>
+      </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>146</v>
+        <v>690</v>
       </c>
       <c r="B100" t="s">
-        <v>129</v>
+        <v>580</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="B101" t="s">
-        <v>599</v>
+        <v>129</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B102" t="s">
-        <v>130</v>
+        <v>599</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>639</v>
+        <v>132</v>
       </c>
       <c r="B103" t="s">
-        <v>640</v>
+        <v>130</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
+        <v>639</v>
+      </c>
+      <c r="B104" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" t="s">
         <v>541</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B105" t="s">
         <v>673</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3">
-      <c r="A106" t="s">
-        <v>188</v>
-      </c>
-      <c r="B106" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="B107" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B108" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B109" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B110" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B111" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>629</v>
+        <v>137</v>
       </c>
       <c r="B112" t="s">
-        <v>695</v>
-      </c>
-      <c r="C112" t="s">
-        <v>699</v>
+        <v>157</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>641</v>
+        <v>629</v>
       </c>
       <c r="B113" t="s">
-        <v>642</v>
+        <v>695</v>
+      </c>
+      <c r="C113" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>540</v>
+        <v>641</v>
       </c>
       <c r="B114" t="s">
-        <v>674</v>
+        <v>642</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
+        <v>540</v>
+      </c>
+      <c r="B115" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" t="s">
         <v>721</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B116" t="s">
         <v>722</v>
       </c>
-      <c r="C115" t="s">
+      <c r="C116" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3">
-      <c r="A117" t="s">
-        <v>710</v>
-      </c>
-      <c r="B117" t="s">
-        <v>711</v>
-      </c>
-      <c r="C117" t="s">
-        <v>712</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="B118" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C118" t="s">
         <v>712</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
-      <c r="A120" t="s">
-        <v>159</v>
-      </c>
-      <c r="B120" t="s">
-        <v>163</v>
+    <row r="119" spans="1:3">
+      <c r="A119" t="s">
+        <v>713</v>
+      </c>
+      <c r="B119" t="s">
+        <v>714</v>
+      </c>
+      <c r="C119" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B121" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B122" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B123" t="s">
-        <v>600</v>
+        <v>165</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>557</v>
+        <v>162</v>
       </c>
       <c r="B124" t="s">
-        <v>739</v>
-      </c>
-      <c r="C124" t="s">
-        <v>740</v>
+        <v>600</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>647</v>
+        <v>557</v>
       </c>
       <c r="B125" t="s">
-        <v>648</v>
+        <v>738</v>
+      </c>
+      <c r="C125" t="s">
+        <v>739</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
+        <v>647</v>
+      </c>
+      <c r="B126" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3">
+      <c r="A127" t="s">
         <v>539</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B127" t="s">
         <v>675</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3">
-      <c r="A128" t="s">
-        <v>192</v>
-      </c>
-      <c r="B128" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="B129" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B130" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>643</v>
+        <v>167</v>
       </c>
       <c r="B131" t="s">
-        <v>644</v>
+        <v>169</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>538</v>
+        <v>643</v>
       </c>
       <c r="B132" t="s">
-        <v>676</v>
+        <v>644</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
+        <v>538</v>
+      </c>
+      <c r="B133" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
         <v>723</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B134" t="s">
         <v>724</v>
       </c>
-      <c r="C133" t="s">
+      <c r="C134" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" t="s">
-        <v>190</v>
-      </c>
-      <c r="B135" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B136" t="s">
-        <v>172</v>
-      </c>
-      <c r="C136" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B137" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C137" t="s">
         <v>588</v>
@@ -8118,10 +8127,10 @@
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B138" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C138" t="s">
         <v>588</v>
@@ -8129,75 +8138,75 @@
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="B139" t="s">
-        <v>202</v>
+        <v>174</v>
+      </c>
+      <c r="C139" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B140" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="B141" t="s">
-        <v>177</v>
-      </c>
-      <c r="C141" t="s">
-        <v>588</v>
+        <v>201</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>645</v>
+        <v>176</v>
       </c>
       <c r="B142" t="s">
-        <v>646</v>
+        <v>177</v>
+      </c>
+      <c r="C142" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
+        <v>645</v>
+      </c>
+      <c r="B143" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3">
+      <c r="A144" t="s">
         <v>527</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B144" t="s">
         <v>677</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3">
-      <c r="A145" t="s">
-        <v>652</v>
-      </c>
-      <c r="B145" t="s">
-        <v>653</v>
-      </c>
-      <c r="C145" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>727</v>
+        <v>652</v>
       </c>
       <c r="B146" t="s">
-        <v>728</v>
+        <v>653</v>
       </c>
       <c r="C146" t="s">
-        <v>692</v>
+        <v>654</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="B147" t="s">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="C147" t="s">
         <v>692</v>
@@ -8205,40 +8214,40 @@
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>741</v>
+        <v>732</v>
       </c>
       <c r="B148" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="C148" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
-      <c r="A150" t="s">
-        <v>513</v>
-      </c>
-      <c r="B150" t="s">
-        <v>514</v>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
+        <v>740</v>
+      </c>
+      <c r="B149" t="s">
+        <v>729</v>
+      </c>
+      <c r="C149" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>661</v>
+        <v>513</v>
       </c>
       <c r="B151" t="s">
-        <v>665</v>
-      </c>
-      <c r="C151" t="s">
-        <v>663</v>
+        <v>514</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B152" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C152" t="s">
         <v>663</v>
@@ -8246,405 +8255,408 @@
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>242</v>
+        <v>662</v>
       </c>
       <c r="B153" t="s">
-        <v>243</v>
+        <v>664</v>
       </c>
       <c r="C153" t="s">
-        <v>588</v>
+        <v>663</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B154" t="s">
-        <v>245</v>
+        <v>243</v>
+      </c>
+      <c r="C154" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B155" t="s">
-        <v>560</v>
-      </c>
-      <c r="C155" t="s">
-        <v>650</v>
+        <v>245</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="B156" t="s">
-        <v>246</v>
+        <v>560</v>
+      </c>
+      <c r="C156" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>503</v>
+        <v>247</v>
       </c>
       <c r="B157" t="s">
-        <v>512</v>
+        <v>246</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>249</v>
+        <v>503</v>
       </c>
       <c r="B158" t="s">
-        <v>248</v>
+        <v>512</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B159" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B160" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B161" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B162" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>302</v>
+        <v>257</v>
       </c>
       <c r="B163" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>349</v>
+        <v>302</v>
       </c>
       <c r="B164" t="s">
-        <v>350</v>
+        <v>248</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>657</v>
+        <v>349</v>
       </c>
       <c r="B165" t="s">
-        <v>658</v>
+        <v>350</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>702</v>
+        <v>657</v>
       </c>
       <c r="B166" t="s">
-        <v>703</v>
+        <v>658</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
+        <v>702</v>
+      </c>
+      <c r="B167" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3">
+      <c r="A168" t="s">
         <v>526</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B168" t="s">
         <v>678</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3">
-      <c r="A169" t="s">
-        <v>515</v>
-      </c>
-      <c r="B169" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
+        <v>515</v>
+      </c>
+      <c r="B170" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3">
+      <c r="A171" t="s">
         <v>259</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B171" t="s">
         <v>262</v>
       </c>
-      <c r="C170" t="s">
+      <c r="C171" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A171" t="s">
+    <row r="172" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A172" t="s">
         <v>261</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B172" t="s">
         <v>561</v>
       </c>
-      <c r="C171" t="s">
+      <c r="C172" t="s">
         <v>696</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3">
-      <c r="A172" t="s">
-        <v>260</v>
-      </c>
-      <c r="B172" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B173" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B174" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B175" t="s">
-        <v>268</v>
-      </c>
-      <c r="C175" t="s">
-        <v>660</v>
+        <v>267</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>504</v>
+        <v>269</v>
       </c>
       <c r="B176" t="s">
-        <v>570</v>
+        <v>268</v>
+      </c>
+      <c r="C176" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>270</v>
+        <v>504</v>
       </c>
       <c r="B177" t="s">
-        <v>271</v>
+        <v>570</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B178" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B179" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B180" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B181" t="s">
-        <v>285</v>
-      </c>
-      <c r="C181" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B182" t="s">
-        <v>605</v>
+        <v>285</v>
+      </c>
+      <c r="C182" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B183" t="s">
-        <v>284</v>
-      </c>
-      <c r="C183" t="s">
-        <v>660</v>
+        <v>605</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B184" t="s">
-        <v>283</v>
+        <v>284</v>
+      </c>
+      <c r="C184" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="B185" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B186" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B187" t="s">
-        <v>305</v>
+        <v>248</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>704</v>
+        <v>304</v>
       </c>
       <c r="B188" t="s">
-        <v>703</v>
+        <v>305</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>537</v>
+        <v>704</v>
       </c>
       <c r="B189" t="s">
-        <v>679</v>
+        <v>703</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
+        <v>537</v>
+      </c>
+      <c r="B190" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3">
+      <c r="A191" t="s">
         <v>697</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B191" t="s">
         <v>698</v>
       </c>
-      <c r="C190" t="s">
+      <c r="C191" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3">
-      <c r="A192" t="s">
-        <v>517</v>
-      </c>
-      <c r="B192" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>292</v>
+        <v>517</v>
       </c>
       <c r="B193" t="s">
-        <v>296</v>
-      </c>
-      <c r="C193" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>505</v>
+        <v>292</v>
       </c>
       <c r="B194" t="s">
-        <v>571</v>
+        <v>296</v>
+      </c>
+      <c r="C194" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>293</v>
+        <v>505</v>
       </c>
       <c r="B195" t="s">
-        <v>297</v>
-      </c>
-      <c r="C195" t="s">
-        <v>588</v>
+        <v>571</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B196" t="s">
-        <v>298</v>
+        <v>297</v>
+      </c>
+      <c r="C196" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B197" t="s">
-        <v>562</v>
+        <v>298</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="B198" t="s">
-        <v>248</v>
+        <v>562</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B199" t="s">
-        <v>310</v>
+        <v>248</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B200" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B201" t="s">
         <v>308</v>
@@ -8652,640 +8664,637 @@
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B202" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>705</v>
+        <v>311</v>
       </c>
       <c r="B203" t="s">
-        <v>703</v>
+        <v>312</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
+        <v>705</v>
+      </c>
+      <c r="B204" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3">
+      <c r="A205" t="s">
         <v>536</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B205" t="s">
         <v>680</v>
-      </c>
-    </row>
-    <row r="206" spans="1:3">
-      <c r="A206" t="s">
-        <v>519</v>
-      </c>
-      <c r="B206" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>499</v>
+        <v>519</v>
       </c>
       <c r="B207" t="s">
-        <v>320</v>
-      </c>
-      <c r="C207" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="B208" t="s">
-        <v>572</v>
+        <v>320</v>
+      </c>
+      <c r="C208" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>315</v>
+        <v>506</v>
       </c>
       <c r="B209" t="s">
-        <v>321</v>
-      </c>
-      <c r="C209" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B210" t="s">
-        <v>322</v>
+        <v>321</v>
+      </c>
+      <c r="C210" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B211" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B212" t="s">
-        <v>563</v>
+        <v>323</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B213" t="s">
-        <v>248</v>
+        <v>563</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B214" t="s">
-        <v>325</v>
-      </c>
-      <c r="C214" t="s">
-        <v>588</v>
+        <v>248</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B215" t="s">
-        <v>327</v>
+        <v>325</v>
+      </c>
+      <c r="C215" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B216" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B217" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B218" t="s">
-        <v>256</v>
+        <v>331</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>706</v>
+        <v>332</v>
       </c>
       <c r="B219" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
+        <v>706</v>
+      </c>
+      <c r="B220" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3">
+      <c r="A221" t="s">
         <v>535</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B221" t="s">
         <v>681</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3">
-      <c r="A222" t="s">
-        <v>521</v>
-      </c>
-      <c r="B222" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="B223" t="s">
-        <v>338</v>
-      </c>
-      <c r="C223" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B224" t="s">
-        <v>573</v>
+        <v>338</v>
+      </c>
+      <c r="C224" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>336</v>
+        <v>507</v>
       </c>
       <c r="B225" t="s">
-        <v>339</v>
-      </c>
-      <c r="C225" t="s">
-        <v>588</v>
+        <v>573</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B226" t="s">
-        <v>340</v>
+        <v>339</v>
+      </c>
+      <c r="C226" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>500</v>
+        <v>337</v>
       </c>
       <c r="B227" t="s">
-        <v>564</v>
+        <v>340</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>344</v>
+        <v>500</v>
       </c>
       <c r="B228" t="s">
-        <v>248</v>
+        <v>564</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B229" t="s">
-        <v>341</v>
+        <v>248</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B230" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B231" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B232" t="s">
-        <v>256</v>
+        <v>343</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>707</v>
+        <v>348</v>
       </c>
       <c r="B233" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
+        <v>707</v>
+      </c>
+      <c r="B234" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3">
+      <c r="A235" t="s">
         <v>534</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B235" t="s">
         <v>682</v>
-      </c>
-    </row>
-    <row r="236" spans="1:3">
-      <c r="A236" t="s">
-        <v>746</v>
-      </c>
-      <c r="B236" t="s">
-        <v>747</v>
-      </c>
-      <c r="C236" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>551</v>
+        <v>745</v>
       </c>
       <c r="B237" t="s">
-        <v>554</v>
+        <v>746</v>
       </c>
       <c r="C237" t="s">
-        <v>586</v>
+        <v>692</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B238" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C238" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>585</v>
+        <v>552</v>
       </c>
       <c r="B239" t="s">
-        <v>601</v>
+        <v>553</v>
+      </c>
+      <c r="C239" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>365</v>
+        <v>585</v>
       </c>
       <c r="B240" t="s">
-        <v>351</v>
+        <v>601</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B241" t="s">
-        <v>352</v>
-      </c>
-      <c r="C241" t="s">
-        <v>588</v>
+        <v>351</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>508</v>
+        <v>366</v>
       </c>
       <c r="B242" t="s">
-        <v>574</v>
+        <v>352</v>
+      </c>
+      <c r="C242" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>367</v>
+        <v>508</v>
       </c>
       <c r="B243" t="s">
-        <v>353</v>
+        <v>574</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B244" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B245" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B246" t="s">
-        <v>356</v>
-      </c>
-      <c r="C246" t="s">
-        <v>588</v>
+        <v>355</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B247" t="s">
-        <v>357</v>
+        <v>356</v>
+      </c>
+      <c r="C247" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B248" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B249" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B250" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B251" t="s">
-        <v>361</v>
-      </c>
-      <c r="C251" t="s">
-        <v>588</v>
+        <v>360</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B252" t="s">
-        <v>362</v>
+        <v>361</v>
+      </c>
+      <c r="C252" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B253" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B254" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
+        <v>378</v>
+      </c>
+      <c r="B255" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3">
+      <c r="A256" t="s">
         <v>533</v>
       </c>
-      <c r="B255" t="s">
+      <c r="B256" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="257" spans="1:3">
-      <c r="A257" t="s">
-        <v>606</v>
-      </c>
-      <c r="B257" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>385</v>
+        <v>606</v>
       </c>
       <c r="B258" t="s">
-        <v>403</v>
+        <v>607</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B259" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B260" t="s">
-        <v>401</v>
-      </c>
-      <c r="C260" t="s">
-        <v>588</v>
+        <v>400</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>509</v>
+        <v>387</v>
       </c>
       <c r="B261" t="s">
-        <v>575</v>
+        <v>401</v>
+      </c>
+      <c r="C261" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>404</v>
+        <v>509</v>
       </c>
       <c r="B262" t="s">
-        <v>402</v>
-      </c>
-      <c r="C262" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="B263" t="s">
-        <v>394</v>
+        <v>402</v>
+      </c>
+      <c r="C263" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
       <c r="B264" t="s">
-        <v>395</v>
-      </c>
-      <c r="C264" t="s">
-        <v>565</v>
+        <v>394</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="B265" t="s">
-        <v>396</v>
+        <v>395</v>
+      </c>
+      <c r="C265" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B266" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B267" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B268" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B269" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
+        <v>393</v>
+      </c>
+      <c r="B270" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3">
+      <c r="A271" t="s">
         <v>532</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B271" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
-      <c r="A272" t="s">
-        <v>748</v>
-      </c>
-      <c r="B272" t="s">
-        <v>745</v>
-      </c>
-      <c r="C272" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="274" spans="1:3">
-      <c r="A274" t="s">
-        <v>744</v>
-      </c>
-      <c r="B274" t="s">
-        <v>745</v>
-      </c>
-      <c r="C274" t="s">
+    <row r="273" spans="1:3">
+      <c r="A273" t="s">
+        <v>747</v>
+      </c>
+      <c r="B273" t="s">
+        <v>768</v>
+      </c>
+      <c r="C273" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>523</v>
+        <v>743</v>
       </c>
       <c r="B275" t="s">
-        <v>524</v>
+        <v>744</v>
+      </c>
+      <c r="C275" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>411</v>
+        <v>523</v>
       </c>
       <c r="B276" t="s">
-        <v>422</v>
+        <v>524</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B277" t="s">
-        <v>423</v>
-      </c>
-      <c r="C277" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>576</v>
+        <v>412</v>
       </c>
       <c r="B278" t="s">
-        <v>577</v>
+        <v>423</v>
+      </c>
+      <c r="C278" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>413</v>
+        <v>576</v>
       </c>
       <c r="B279" t="s">
-        <v>424</v>
-      </c>
-      <c r="C279" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B280" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C280" t="s">
         <v>588</v>
@@ -9293,128 +9302,128 @@
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B281" t="s">
-        <v>589</v>
+        <v>425</v>
+      </c>
+      <c r="C281" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B282" t="s">
-        <v>426</v>
+        <v>589</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B283" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B284" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B285" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B286" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B287" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>530</v>
+        <v>421</v>
       </c>
       <c r="B288" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
+        <v>530</v>
+      </c>
+      <c r="B289" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3">
+      <c r="A290" t="s">
         <v>615</v>
       </c>
-      <c r="B289" t="s">
+      <c r="B290" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="291" spans="1:3">
-      <c r="A291" t="s">
-        <v>525</v>
-      </c>
-      <c r="B291" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>438</v>
+        <v>525</v>
       </c>
       <c r="B292" t="s">
-        <v>449</v>
+        <v>524</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B293" t="s">
-        <v>450</v>
-      </c>
-      <c r="C293" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>510</v>
+        <v>439</v>
       </c>
       <c r="B294" t="s">
-        <v>578</v>
+        <v>450</v>
+      </c>
+      <c r="C294" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>440</v>
+        <v>510</v>
       </c>
       <c r="B295" t="s">
-        <v>451</v>
-      </c>
-      <c r="C295" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B296" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C296" t="s">
         <v>588</v>
@@ -9422,143 +9431,154 @@
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B297" t="s">
-        <v>590</v>
+        <v>452</v>
+      </c>
+      <c r="C297" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B298" t="s">
-        <v>426</v>
+        <v>590</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B299" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B300" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B301" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B302" t="s">
-        <v>430</v>
+        <v>454</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B303" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>529</v>
+        <v>448</v>
       </c>
       <c r="B304" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
+        <v>529</v>
+      </c>
+      <c r="B305" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3">
+      <c r="A306" t="s">
         <v>622</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B306" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="307" spans="1:3">
-      <c r="A307" t="s">
-        <v>742</v>
-      </c>
-      <c r="B307" t="s">
-        <v>743</v>
-      </c>
-      <c r="C307" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>432</v>
+        <v>741</v>
       </c>
       <c r="B308" t="s">
-        <v>623</v>
+        <v>742</v>
+      </c>
+      <c r="C308" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B309" t="s">
-        <v>624</v>
-      </c>
-      <c r="C309" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>511</v>
+        <v>433</v>
       </c>
       <c r="B310" t="s">
-        <v>625</v>
+        <v>624</v>
+      </c>
+      <c r="C310" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>434</v>
+        <v>511</v>
       </c>
       <c r="B311" t="s">
-        <v>651</v>
+        <v>625</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B312" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B313" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
+        <v>436</v>
+      </c>
+      <c r="B314" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3">
+      <c r="A315" t="s">
         <v>528</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B315" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates done to DU code for resolving Emgu in unattended runs
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC06EB4-9A42-4549-8476-C2408D58E816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA776A3-303B-45E8-AF71-E9EE17DD402E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4395" yWindow="4740" windowWidth="28170" windowHeight="13710" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2343,9 +2343,6 @@
     <t>Unable to validate findings for Housing History Disclosure. Needs manual review.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Supporting documents have not been provided for Child Support Calcs documented on the Income &amp; Asset Questionnaire.</t>
   </si>
   <si>
@@ -2365,6 +2362,9 @@
   </si>
   <si>
     <t>HHD_MoveInDateCheck</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2822,7 +2822,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7042,7 +7042,7 @@
         <v>725</v>
       </c>
       <c r="B5" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C5" t="s">
         <v>692</v>
@@ -7053,7 +7053,7 @@
         <v>762</v>
       </c>
       <c r="B6" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C6" t="s">
         <v>692</v>
@@ -7064,7 +7064,7 @@
         <v>763</v>
       </c>
       <c r="B7" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C7" t="s">
         <v>692</v>
@@ -7075,7 +7075,7 @@
         <v>764</v>
       </c>
       <c r="B8" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C8" t="s">
         <v>692</v>
@@ -7083,10 +7083,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B9" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C9" t="s">
         <v>692</v>
@@ -9237,7 +9237,7 @@
         <v>747</v>
       </c>
       <c r="B273" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C273" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
DU changes for MID and HHD. Tested the new prompt changes for SSBL - 58078.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA776A3-303B-45E8-AF71-E9EE17DD402E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAE5491-6AF6-469C-AF31-5F503270C954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28200" windowHeight="13665" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Adding DU for VOE
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAE5491-6AF6-469C-AF31-5F503270C954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1841A8E9-F3C3-4AAC-B5CD-0F6E2BE7CDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28200" windowHeight="13665" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Changes for HHD DU (57856), SC Signature Section (58136) and ASC Signature Section (58137)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1841A8E9-F3C3-4AAC-B5CD-0F6E2BE7CDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF1BBB7-0FB6-4B1B-BA91-6BA63C849F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21060" windowHeight="9615" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Changes to VOE, SC DU
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF1BBB7-0FB6-4B1B-BA91-6BA63C849F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0F0D0B5-399D-4F36-8E88-35521A3FDFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21060" windowHeight="9615" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
uncommented code for 57387, 57813, as IAQ DU is deployed, and minor changes for 57850 - DU for MID (also a minor change for HHD DU)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0F0D0B5-399D-4F36-8E88-35521A3FDFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF9B40B-20F3-4186-A637-370E7A37503F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="28260" windowHeight="13665" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updates to SC, VOE and Reassign in BE
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF9B40B-20F3-4186-A637-370E7A37503F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2018818D-CD00-4E5B-8108-77ACFC35F8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="28260" windowHeight="13665" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
58056, 58164 - updated the ASC present but empty finding, updated the code for the latest version of the SEC prompt
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2018818D-CD00-4E5B-8108-77ACFC35F8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B9E2DE-6B95-406B-B0DF-DD29C700AEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="4245" windowWidth="28260" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2319,9 +2319,6 @@
     <t>ASC_IsFound</t>
   </si>
   <si>
-    <t>Asset Self Certification is missing from the application.</t>
-  </si>
-  <si>
     <t>SCNE_EmploymentDocumented</t>
   </si>
   <si>
@@ -2364,7 +2361,10 @@
     <t>HHD_MoveInDateCheck</t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>Asset Self Certification is empty.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -7042,7 +7042,7 @@
         <v>725</v>
       </c>
       <c r="B5" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C5" t="s">
         <v>692</v>
@@ -7050,10 +7050,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B6" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C6" t="s">
         <v>692</v>
@@ -7061,10 +7061,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B7" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C7" t="s">
         <v>692</v>
@@ -7072,10 +7072,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B8" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C8" t="s">
         <v>692</v>
@@ -7083,10 +7083,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B9" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C9" t="s">
         <v>692</v>
@@ -7094,10 +7094,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>764</v>
+      </c>
+      <c r="B10" t="s">
         <v>765</v>
-      </c>
-      <c r="B10" t="s">
-        <v>766</v>
       </c>
       <c r="C10" t="s">
         <v>692</v>
@@ -7617,10 +7617,10 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
+        <v>759</v>
+      </c>
+      <c r="B74" t="s">
         <v>760</v>
-      </c>
-      <c r="B74" t="s">
-        <v>761</v>
       </c>
       <c r="C74" t="s">
         <v>692</v>
@@ -7647,7 +7647,7 @@
         <v>758</v>
       </c>
       <c r="B78" t="s">
-        <v>759</v>
+        <v>773</v>
       </c>
       <c r="C78" t="s">
         <v>692</v>
@@ -9237,7 +9237,7 @@
         <v>747</v>
       </c>
       <c r="B273" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C273" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Added ASFA DU code
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B9E2DE-6B95-406B-B0DF-DD29C700AEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBD1648-DE06-40CA-8298-0AE9AC2F044A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="4245" windowWidth="28260" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2364,7 +2364,7 @@
     <t>Asset Self Certification is empty.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Tests for 58173, 58175, and added a finding in PS for 57449
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBD1648-DE06-40CA-8298-0AE9AC2F044A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68658DF6-A6A8-4117-9896-83A177AE4E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="777">
   <si>
     <t>Name</t>
   </si>
@@ -2364,7 +2364,13 @@
     <t>Asset Self Certification is empty.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>PS_NegativePaystubs</t>
+  </si>
+  <si>
+    <t>Negative value identified on paystub. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -7013,7 +7019,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C315"/>
+  <dimension ref="A1:C316"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -8384,287 +8390,290 @@
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
+        <v>775</v>
+      </c>
+      <c r="B168" t="s">
+        <v>776</v>
+      </c>
+      <c r="C168" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3">
+      <c r="A169" t="s">
         <v>526</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B169" t="s">
         <v>678</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3">
-      <c r="A170" t="s">
-        <v>515</v>
-      </c>
-      <c r="B170" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
+        <v>515</v>
+      </c>
+      <c r="B171" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3">
+      <c r="A172" t="s">
         <v>259</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B172" t="s">
         <v>262</v>
       </c>
-      <c r="C171" t="s">
+      <c r="C172" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A172" t="s">
+    <row r="173" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A173" t="s">
         <v>261</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B173" t="s">
         <v>561</v>
       </c>
-      <c r="C172" t="s">
+      <c r="C173" t="s">
         <v>696</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3">
-      <c r="A173" t="s">
-        <v>260</v>
-      </c>
-      <c r="B173" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B174" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B175" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B176" t="s">
-        <v>268</v>
-      </c>
-      <c r="C176" t="s">
-        <v>660</v>
+        <v>267</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>504</v>
+        <v>269</v>
       </c>
       <c r="B177" t="s">
-        <v>570</v>
+        <v>268</v>
+      </c>
+      <c r="C177" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>270</v>
+        <v>504</v>
       </c>
       <c r="B178" t="s">
-        <v>271</v>
+        <v>570</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B179" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B180" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B181" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B182" t="s">
-        <v>285</v>
-      </c>
-      <c r="C182" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B183" t="s">
-        <v>605</v>
+        <v>285</v>
+      </c>
+      <c r="C183" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B184" t="s">
-        <v>284</v>
-      </c>
-      <c r="C184" t="s">
-        <v>660</v>
+        <v>605</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B185" t="s">
-        <v>283</v>
+        <v>284</v>
+      </c>
+      <c r="C185" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="B186" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B187" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B188" t="s">
-        <v>305</v>
+        <v>248</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>704</v>
+        <v>304</v>
       </c>
       <c r="B189" t="s">
-        <v>703</v>
+        <v>305</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>537</v>
+        <v>704</v>
       </c>
       <c r="B190" t="s">
-        <v>679</v>
+        <v>703</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
+        <v>537</v>
+      </c>
+      <c r="B191" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
         <v>697</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>698</v>
       </c>
-      <c r="C191" t="s">
+      <c r="C192" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3">
-      <c r="A193" t="s">
-        <v>517</v>
-      </c>
-      <c r="B193" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>292</v>
+        <v>517</v>
       </c>
       <c r="B194" t="s">
-        <v>296</v>
-      </c>
-      <c r="C194" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>505</v>
+        <v>292</v>
       </c>
       <c r="B195" t="s">
-        <v>571</v>
+        <v>296</v>
+      </c>
+      <c r="C195" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>293</v>
+        <v>505</v>
       </c>
       <c r="B196" t="s">
-        <v>297</v>
-      </c>
-      <c r="C196" t="s">
-        <v>588</v>
+        <v>571</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B197" t="s">
-        <v>298</v>
+        <v>297</v>
+      </c>
+      <c r="C197" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B198" t="s">
-        <v>562</v>
+        <v>298</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="B199" t="s">
-        <v>248</v>
+        <v>562</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B200" t="s">
-        <v>310</v>
+        <v>248</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B201" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B202" t="s">
         <v>308</v>
@@ -8672,640 +8681,637 @@
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B203" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>705</v>
+        <v>311</v>
       </c>
       <c r="B204" t="s">
-        <v>703</v>
+        <v>312</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
+        <v>705</v>
+      </c>
+      <c r="B205" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3">
+      <c r="A206" t="s">
         <v>536</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B206" t="s">
         <v>680</v>
-      </c>
-    </row>
-    <row r="207" spans="1:3">
-      <c r="A207" t="s">
-        <v>519</v>
-      </c>
-      <c r="B207" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>499</v>
+        <v>519</v>
       </c>
       <c r="B208" t="s">
-        <v>320</v>
-      </c>
-      <c r="C208" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="B209" t="s">
-        <v>572</v>
+        <v>320</v>
+      </c>
+      <c r="C209" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>315</v>
+        <v>506</v>
       </c>
       <c r="B210" t="s">
-        <v>321</v>
-      </c>
-      <c r="C210" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B211" t="s">
-        <v>322</v>
+        <v>321</v>
+      </c>
+      <c r="C211" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B212" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B213" t="s">
-        <v>563</v>
+        <v>323</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B214" t="s">
-        <v>248</v>
+        <v>563</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B215" t="s">
-        <v>325</v>
-      </c>
-      <c r="C215" t="s">
-        <v>588</v>
+        <v>248</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B216" t="s">
-        <v>327</v>
+        <v>325</v>
+      </c>
+      <c r="C216" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B217" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B218" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B219" t="s">
-        <v>256</v>
+        <v>331</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>706</v>
+        <v>332</v>
       </c>
       <c r="B220" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
+        <v>706</v>
+      </c>
+      <c r="B221" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3">
+      <c r="A222" t="s">
         <v>535</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B222" t="s">
         <v>681</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
-        <v>521</v>
-      </c>
-      <c r="B223" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="B224" t="s">
-        <v>338</v>
-      </c>
-      <c r="C224" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B225" t="s">
-        <v>573</v>
+        <v>338</v>
+      </c>
+      <c r="C225" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>336</v>
+        <v>507</v>
       </c>
       <c r="B226" t="s">
-        <v>339</v>
-      </c>
-      <c r="C226" t="s">
-        <v>588</v>
+        <v>573</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B227" t="s">
-        <v>340</v>
+        <v>339</v>
+      </c>
+      <c r="C227" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>500</v>
+        <v>337</v>
       </c>
       <c r="B228" t="s">
-        <v>564</v>
+        <v>340</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>344</v>
+        <v>500</v>
       </c>
       <c r="B229" t="s">
-        <v>248</v>
+        <v>564</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B230" t="s">
-        <v>341</v>
+        <v>248</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B231" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B232" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B233" t="s">
-        <v>256</v>
+        <v>343</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>707</v>
+        <v>348</v>
       </c>
       <c r="B234" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
+        <v>707</v>
+      </c>
+      <c r="B235" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3">
+      <c r="A236" t="s">
         <v>534</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B236" t="s">
         <v>682</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3">
-      <c r="A237" t="s">
-        <v>745</v>
-      </c>
-      <c r="B237" t="s">
-        <v>746</v>
-      </c>
-      <c r="C237" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>551</v>
+        <v>745</v>
       </c>
       <c r="B238" t="s">
-        <v>554</v>
+        <v>746</v>
       </c>
       <c r="C238" t="s">
-        <v>586</v>
+        <v>692</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B239" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C239" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>585</v>
+        <v>552</v>
       </c>
       <c r="B240" t="s">
-        <v>601</v>
+        <v>553</v>
+      </c>
+      <c r="C240" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>365</v>
+        <v>585</v>
       </c>
       <c r="B241" t="s">
-        <v>351</v>
+        <v>601</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B242" t="s">
-        <v>352</v>
-      </c>
-      <c r="C242" t="s">
-        <v>588</v>
+        <v>351</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>508</v>
+        <v>366</v>
       </c>
       <c r="B243" t="s">
-        <v>574</v>
+        <v>352</v>
+      </c>
+      <c r="C243" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>367</v>
+        <v>508</v>
       </c>
       <c r="B244" t="s">
-        <v>353</v>
+        <v>574</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B245" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B246" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B247" t="s">
-        <v>356</v>
-      </c>
-      <c r="C247" t="s">
-        <v>588</v>
+        <v>355</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B248" t="s">
-        <v>357</v>
+        <v>356</v>
+      </c>
+      <c r="C248" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B249" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B250" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B251" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B252" t="s">
-        <v>361</v>
-      </c>
-      <c r="C252" t="s">
-        <v>588</v>
+        <v>360</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B253" t="s">
-        <v>362</v>
+        <v>361</v>
+      </c>
+      <c r="C253" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B254" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B255" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
+        <v>378</v>
+      </c>
+      <c r="B256" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3">
+      <c r="A257" t="s">
         <v>533</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B257" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="258" spans="1:3">
-      <c r="A258" t="s">
-        <v>606</v>
-      </c>
-      <c r="B258" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>385</v>
+        <v>606</v>
       </c>
       <c r="B259" t="s">
-        <v>403</v>
+        <v>607</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B260" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B261" t="s">
-        <v>401</v>
-      </c>
-      <c r="C261" t="s">
-        <v>588</v>
+        <v>400</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>509</v>
+        <v>387</v>
       </c>
       <c r="B262" t="s">
-        <v>575</v>
+        <v>401</v>
+      </c>
+      <c r="C262" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>404</v>
+        <v>509</v>
       </c>
       <c r="B263" t="s">
-        <v>402</v>
-      </c>
-      <c r="C263" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="B264" t="s">
-        <v>394</v>
+        <v>402</v>
+      </c>
+      <c r="C264" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
       <c r="B265" t="s">
-        <v>395</v>
-      </c>
-      <c r="C265" t="s">
-        <v>565</v>
+        <v>394</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="B266" t="s">
-        <v>396</v>
+        <v>395</v>
+      </c>
+      <c r="C266" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B267" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B268" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B269" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B270" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
+        <v>393</v>
+      </c>
+      <c r="B271" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3">
+      <c r="A272" t="s">
         <v>532</v>
       </c>
-      <c r="B271" t="s">
+      <c r="B272" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="273" spans="1:3">
-      <c r="A273" t="s">
+    <row r="274" spans="1:3">
+      <c r="A274" t="s">
         <v>747</v>
       </c>
-      <c r="B273" t="s">
+      <c r="B274" t="s">
         <v>766</v>
       </c>
-      <c r="C273" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="275" spans="1:3">
-      <c r="A275" t="s">
-        <v>743</v>
-      </c>
-      <c r="B275" t="s">
-        <v>744</v>
-      </c>
-      <c r="C275" t="s">
+      <c r="C274" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>523</v>
+        <v>743</v>
       </c>
       <c r="B276" t="s">
-        <v>524</v>
+        <v>744</v>
+      </c>
+      <c r="C276" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>411</v>
+        <v>523</v>
       </c>
       <c r="B277" t="s">
-        <v>422</v>
+        <v>524</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B278" t="s">
-        <v>423</v>
-      </c>
-      <c r="C278" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>576</v>
+        <v>412</v>
       </c>
       <c r="B279" t="s">
-        <v>577</v>
+        <v>423</v>
+      </c>
+      <c r="C279" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>413</v>
+        <v>576</v>
       </c>
       <c r="B280" t="s">
-        <v>424</v>
-      </c>
-      <c r="C280" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B281" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C281" t="s">
         <v>588</v>
@@ -9313,128 +9319,128 @@
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B282" t="s">
-        <v>589</v>
+        <v>425</v>
+      </c>
+      <c r="C282" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B283" t="s">
-        <v>426</v>
+        <v>589</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B284" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B285" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B286" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B287" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B288" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>530</v>
+        <v>421</v>
       </c>
       <c r="B289" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
+        <v>530</v>
+      </c>
+      <c r="B290" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3">
+      <c r="A291" t="s">
         <v>615</v>
       </c>
-      <c r="B290" t="s">
+      <c r="B291" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="292" spans="1:3">
-      <c r="A292" t="s">
-        <v>525</v>
-      </c>
-      <c r="B292" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>438</v>
+        <v>525</v>
       </c>
       <c r="B293" t="s">
-        <v>449</v>
+        <v>524</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B294" t="s">
-        <v>450</v>
-      </c>
-      <c r="C294" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>510</v>
+        <v>439</v>
       </c>
       <c r="B295" t="s">
-        <v>578</v>
+        <v>450</v>
+      </c>
+      <c r="C295" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>440</v>
+        <v>510</v>
       </c>
       <c r="B296" t="s">
-        <v>451</v>
-      </c>
-      <c r="C296" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B297" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C297" t="s">
         <v>588</v>
@@ -9442,143 +9448,154 @@
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B298" t="s">
-        <v>590</v>
+        <v>452</v>
+      </c>
+      <c r="C298" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B299" t="s">
-        <v>426</v>
+        <v>590</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B300" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B301" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B302" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B303" t="s">
-        <v>430</v>
+        <v>454</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B304" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>529</v>
+        <v>448</v>
       </c>
       <c r="B305" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
+        <v>529</v>
+      </c>
+      <c r="B306" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3">
+      <c r="A307" t="s">
         <v>622</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B307" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="308" spans="1:3">
-      <c r="A308" t="s">
-        <v>741</v>
-      </c>
-      <c r="B308" t="s">
-        <v>742</v>
-      </c>
-      <c r="C308" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>432</v>
+        <v>741</v>
       </c>
       <c r="B309" t="s">
-        <v>623</v>
+        <v>742</v>
+      </c>
+      <c r="C309" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B310" t="s">
-        <v>624</v>
-      </c>
-      <c r="C310" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>511</v>
+        <v>433</v>
       </c>
       <c r="B311" t="s">
-        <v>625</v>
+        <v>624</v>
+      </c>
+      <c r="C311" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>434</v>
+        <v>511</v>
       </c>
       <c r="B312" t="s">
-        <v>651</v>
+        <v>625</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B313" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B314" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
+        <v>436</v>
+      </c>
+      <c r="B315" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3">
+      <c r="A316" t="s">
         <v>528</v>
       </c>
-      <c r="B315" t="s">
+      <c r="B316" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated ASFA to handle all scenarios with DU
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68658DF6-A6A8-4117-9896-83A177AE4E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D8F043-B753-4843-97C2-BC54A2F525A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="778">
   <si>
     <t>Name</t>
   </si>
@@ -2364,13 +2364,16 @@
     <t>Asset Self Certification is empty.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>PS_NegativePaystubs</t>
   </si>
   <si>
     <t>Negative value identified on paystub. Manual review required.</t>
+  </si>
+  <si>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>FindAllASFAAssistance_Threshold</t>
   </si>
 </sst>
 </file>
@@ -2828,7 +2831,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -5683,7 +5686,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1011"/>
+  <dimension ref="A1:Z1012"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -6018,29 +6021,36 @@
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>689</v>
+        <v>777</v>
       </c>
       <c r="B38" t="s">
-        <v>689</v>
+        <v>777</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>730</v>
+        <v>689</v>
       </c>
       <c r="B39" t="s">
-        <v>730</v>
+        <v>689</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
+        <v>730</v>
+      </c>
+      <c r="B40" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A41" t="s">
         <v>737</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="42" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7011,6 +7021,7 @@
     <row r="1009" ht="14.25" customHeight="1"/>
     <row r="1010" ht="14.25" customHeight="1"/>
     <row r="1011" ht="14.25" customHeight="1"/>
+    <row r="1012" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8390,10 +8401,10 @@
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
+        <v>774</v>
+      </c>
+      <c r="B168" t="s">
         <v>775</v>
-      </c>
-      <c r="B168" t="s">
-        <v>776</v>
       </c>
       <c r="C168" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Changes for 58080 - adding the 'hourly' frequency pay period calculation for VOE, 58180 - changed the signature check for HHD to be based not only on the IsSigned field, but also on the Signature Date, and 58165 - changed the way we validate the all requested fields
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D8F043-B753-4843-97C2-BC54A2F525A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB70091C-BD59-4B9B-AFE4-1D0CF9C4F84C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2370,10 +2370,10 @@
     <t>Negative value identified on paystub. Manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>FindAllASFAAssistance_Threshold</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2831,7 +2831,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -6021,10 +6021,10 @@
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B38" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Changes for SCNE new prompt 58055, testing SCNE DU, an additional change for ASC at verification of null fields, also changed the check for 58183
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB70091C-BD59-4B9B-AFE4-1D0CF9C4F84C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E1E4BB-F59D-42DA-B6BD-0B2997875A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28170" windowHeight="14670" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="778">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="784">
   <si>
     <t>Name</t>
   </si>
@@ -2374,6 +2374,24 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>SCNE_EmploymentNo</t>
+  </si>
+  <si>
+    <t>SCNE_NotExpectingEmployment12Months</t>
+  </si>
+  <si>
+    <t>SCNE_ExpectingEmployment12Months</t>
+  </si>
+  <si>
+    <t>Employment expected in 12 months field is Yes, but the following documentation for Yes is not documented appropriated.</t>
+  </si>
+  <si>
+    <t>Employment expected in 12 months field is No, but the following documentation for No is not documented appropriated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employment field is No, but the following documentation for unemployment is not documented appropriately. </t>
   </si>
 </sst>
 </file>
@@ -7030,10 +7048,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C316"/>
+  <dimension ref="A1:C319"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.5703125" customWidth="1"/>
     <col min="2" max="2" width="153.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -7645,170 +7663,170 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>543</v>
+        <v>780</v>
       </c>
       <c r="B75" t="s">
-        <v>671</v>
+        <v>781</v>
+      </c>
+      <c r="C75" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>779</v>
+      </c>
+      <c r="B76" t="s">
+        <v>782</v>
+      </c>
+      <c r="C76" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>186</v>
+        <v>778</v>
       </c>
       <c r="B77" t="s">
-        <v>187</v>
+        <v>783</v>
+      </c>
+      <c r="C77" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>758</v>
+        <v>543</v>
       </c>
       <c r="B78" t="s">
-        <v>773</v>
-      </c>
-      <c r="C78" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3">
-      <c r="A79" t="s">
-        <v>756</v>
-      </c>
-      <c r="B79" t="s">
-        <v>757</v>
-      </c>
-      <c r="C79" t="s">
-        <v>692</v>
+        <v>671</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>125</v>
+        <v>186</v>
       </c>
       <c r="B80" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>126</v>
+        <v>758</v>
       </c>
       <c r="B81" t="s">
-        <v>128</v>
+        <v>773</v>
+      </c>
+      <c r="C81" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>138</v>
+        <v>756</v>
       </c>
       <c r="B82" t="s">
-        <v>595</v>
+        <v>757</v>
+      </c>
+      <c r="C82" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B83" t="s">
-        <v>596</v>
+        <v>127</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="B84" t="s">
-        <v>597</v>
+        <v>128</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B85" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B86" t="s">
-        <v>495</v>
-      </c>
-      <c r="C86" t="s">
-        <v>686</v>
+        <v>596</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B87" t="s">
-        <v>497</v>
-      </c>
-      <c r="C87" t="s">
-        <v>556</v>
+        <v>597</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B88" t="s">
-        <v>498</v>
-      </c>
-      <c r="C88" t="s">
-        <v>556</v>
+        <v>598</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>637</v>
+        <v>142</v>
       </c>
       <c r="B89" t="s">
-        <v>638</v>
+        <v>495</v>
+      </c>
+      <c r="C89" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>719</v>
+        <v>143</v>
       </c>
       <c r="B90" t="s">
-        <v>720</v>
+        <v>497</v>
       </c>
       <c r="C90" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>750</v>
+        <v>144</v>
       </c>
       <c r="B91" t="s">
-        <v>751</v>
+        <v>498</v>
       </c>
       <c r="C91" t="s">
-        <v>692</v>
+        <v>556</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>753</v>
+        <v>637</v>
       </c>
       <c r="B92" t="s">
-        <v>752</v>
-      </c>
-      <c r="C92" t="s">
-        <v>692</v>
+        <v>638</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>755</v>
+        <v>719</v>
       </c>
       <c r="B93" t="s">
-        <v>754</v>
+        <v>720</v>
       </c>
       <c r="C93" t="s">
         <v>692</v>
@@ -7816,376 +7834,382 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>542</v>
+        <v>750</v>
       </c>
       <c r="B94" t="s">
-        <v>672</v>
+        <v>751</v>
+      </c>
+      <c r="C94" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" t="s">
+        <v>753</v>
+      </c>
+      <c r="B95" t="s">
+        <v>752</v>
+      </c>
+      <c r="C95" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>147</v>
+        <v>755</v>
       </c>
       <c r="B96" t="s">
-        <v>150</v>
+        <v>754</v>
+      </c>
+      <c r="C96" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>148</v>
+        <v>542</v>
       </c>
       <c r="B97" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3">
-      <c r="A98" t="s">
-        <v>149</v>
-      </c>
-      <c r="B98" t="s">
-        <v>152</v>
+        <v>672</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B99" t="s">
-        <v>580</v>
-      </c>
-      <c r="C99" t="s">
-        <v>691</v>
+        <v>150</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>690</v>
+        <v>148</v>
       </c>
       <c r="B100" t="s">
-        <v>580</v>
+        <v>151</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B101" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B102" t="s">
-        <v>599</v>
+        <v>580</v>
+      </c>
+      <c r="C102" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>132</v>
+        <v>690</v>
       </c>
       <c r="B103" t="s">
-        <v>130</v>
+        <v>580</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>639</v>
+        <v>146</v>
       </c>
       <c r="B104" t="s">
-        <v>640</v>
+        <v>129</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>541</v>
+        <v>131</v>
       </c>
       <c r="B105" t="s">
-        <v>673</v>
+        <v>599</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="A106" t="s">
+        <v>132</v>
+      </c>
+      <c r="B106" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>188</v>
+        <v>639</v>
       </c>
       <c r="B107" t="s">
-        <v>189</v>
+        <v>640</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>133</v>
+        <v>541</v>
       </c>
       <c r="B108" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3">
-      <c r="A109" t="s">
-        <v>135</v>
-      </c>
-      <c r="B109" t="s">
-        <v>154</v>
+        <v>673</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>134</v>
+        <v>188</v>
       </c>
       <c r="B110" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B111" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B112" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>629</v>
+        <v>134</v>
       </c>
       <c r="B113" t="s">
-        <v>695</v>
-      </c>
-      <c r="C113" t="s">
-        <v>699</v>
+        <v>155</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>641</v>
+        <v>136</v>
       </c>
       <c r="B114" t="s">
-        <v>642</v>
+        <v>156</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>540</v>
+        <v>137</v>
       </c>
       <c r="B115" t="s">
-        <v>674</v>
+        <v>157</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>721</v>
+        <v>629</v>
       </c>
       <c r="B116" t="s">
-        <v>722</v>
+        <v>695</v>
       </c>
       <c r="C116" t="s">
-        <v>692</v>
+        <v>699</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" t="s">
+        <v>641</v>
+      </c>
+      <c r="B117" t="s">
+        <v>642</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>710</v>
+        <v>540</v>
       </c>
       <c r="B118" t="s">
-        <v>711</v>
-      </c>
-      <c r="C118" t="s">
-        <v>712</v>
+        <v>674</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="B119" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="C119" t="s">
-        <v>712</v>
+        <v>692</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>159</v>
+        <v>710</v>
       </c>
       <c r="B121" t="s">
-        <v>163</v>
+        <v>711</v>
+      </c>
+      <c r="C121" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>160</v>
+        <v>713</v>
       </c>
       <c r="B122" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" t="s">
-        <v>161</v>
-      </c>
-      <c r="B123" t="s">
-        <v>165</v>
+        <v>714</v>
+      </c>
+      <c r="C122" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B124" t="s">
-        <v>600</v>
+        <v>163</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>557</v>
+        <v>160</v>
       </c>
       <c r="B125" t="s">
-        <v>738</v>
-      </c>
-      <c r="C125" t="s">
-        <v>739</v>
+        <v>164</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>647</v>
+        <v>161</v>
       </c>
       <c r="B126" t="s">
-        <v>648</v>
+        <v>165</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>539</v>
+        <v>162</v>
       </c>
       <c r="B127" t="s">
-        <v>675</v>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" t="s">
+        <v>557</v>
+      </c>
+      <c r="B128" t="s">
+        <v>738</v>
+      </c>
+      <c r="C128" t="s">
+        <v>739</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>192</v>
+        <v>647</v>
       </c>
       <c r="B129" t="s">
-        <v>193</v>
+        <v>648</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>166</v>
+        <v>539</v>
       </c>
       <c r="B130" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" t="s">
-        <v>167</v>
-      </c>
-      <c r="B131" t="s">
-        <v>169</v>
+        <v>675</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>643</v>
+        <v>192</v>
       </c>
       <c r="B132" t="s">
-        <v>644</v>
+        <v>193</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>538</v>
+        <v>166</v>
       </c>
       <c r="B133" t="s">
-        <v>676</v>
+        <v>168</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>723</v>
+        <v>167</v>
       </c>
       <c r="B134" t="s">
-        <v>724</v>
-      </c>
-      <c r="C134" t="s">
-        <v>692</v>
+        <v>169</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3">
+      <c r="A135" t="s">
+        <v>643</v>
+      </c>
+      <c r="B135" t="s">
+        <v>644</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>190</v>
+        <v>538</v>
       </c>
       <c r="B136" t="s">
-        <v>191</v>
+        <v>676</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>175</v>
+        <v>723</v>
       </c>
       <c r="B137" t="s">
-        <v>172</v>
+        <v>724</v>
       </c>
       <c r="C137" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3">
-      <c r="A138" t="s">
-        <v>170</v>
-      </c>
-      <c r="B138" t="s">
-        <v>173</v>
-      </c>
-      <c r="C138" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="B139" t="s">
-        <v>174</v>
-      </c>
-      <c r="C139" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>203</v>
+        <v>175</v>
       </c>
       <c r="B140" t="s">
-        <v>202</v>
+        <v>172</v>
+      </c>
+      <c r="C140" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B141" t="s">
-        <v>201</v>
+        <v>173</v>
+      </c>
+      <c r="C141" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B142" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C142" t="s">
         <v>588</v>
@@ -8193,1147 +8217,1144 @@
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>645</v>
+        <v>203</v>
       </c>
       <c r="B143" t="s">
-        <v>646</v>
+        <v>202</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>527</v>
+        <v>200</v>
       </c>
       <c r="B144" t="s">
-        <v>677</v>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" t="s">
+        <v>176</v>
+      </c>
+      <c r="B145" t="s">
+        <v>177</v>
+      </c>
+      <c r="C145" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="B146" t="s">
-        <v>653</v>
-      </c>
-      <c r="C146" t="s">
-        <v>654</v>
+        <v>646</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>726</v>
+        <v>527</v>
       </c>
       <c r="B147" t="s">
-        <v>727</v>
-      </c>
-      <c r="C147" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3">
-      <c r="A148" t="s">
-        <v>732</v>
-      </c>
-      <c r="B148" t="s">
-        <v>733</v>
-      </c>
-      <c r="C148" t="s">
-        <v>692</v>
+        <v>677</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>740</v>
+        <v>652</v>
       </c>
       <c r="B149" t="s">
-        <v>729</v>
+        <v>653</v>
       </c>
       <c r="C149" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" t="s">
+        <v>726</v>
+      </c>
+      <c r="B150" t="s">
+        <v>727</v>
+      </c>
+      <c r="C150" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>513</v>
+        <v>732</v>
       </c>
       <c r="B151" t="s">
-        <v>514</v>
+        <v>733</v>
+      </c>
+      <c r="C151" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>661</v>
+        <v>740</v>
       </c>
       <c r="B152" t="s">
-        <v>665</v>
+        <v>729</v>
       </c>
       <c r="C152" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3">
-      <c r="A153" t="s">
-        <v>662</v>
-      </c>
-      <c r="B153" t="s">
-        <v>664</v>
-      </c>
-      <c r="C153" t="s">
-        <v>663</v>
+        <v>692</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>242</v>
+        <v>513</v>
       </c>
       <c r="B154" t="s">
-        <v>243</v>
-      </c>
-      <c r="C154" t="s">
-        <v>588</v>
+        <v>514</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>244</v>
+        <v>661</v>
       </c>
       <c r="B155" t="s">
-        <v>245</v>
+        <v>665</v>
+      </c>
+      <c r="C155" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>258</v>
+        <v>662</v>
       </c>
       <c r="B156" t="s">
-        <v>560</v>
+        <v>664</v>
       </c>
       <c r="C156" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B157" t="s">
-        <v>246</v>
+        <v>243</v>
+      </c>
+      <c r="C157" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>503</v>
+        <v>244</v>
       </c>
       <c r="B158" t="s">
-        <v>512</v>
+        <v>245</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B159" t="s">
-        <v>248</v>
+        <v>560</v>
+      </c>
+      <c r="C159" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B160" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>251</v>
+        <v>503</v>
       </c>
       <c r="B161" t="s">
-        <v>253</v>
+        <v>512</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B162" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B163" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>302</v>
+        <v>251</v>
       </c>
       <c r="B164" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>349</v>
+        <v>255</v>
       </c>
       <c r="B165" t="s">
-        <v>350</v>
+        <v>254</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>657</v>
+        <v>257</v>
       </c>
       <c r="B166" t="s">
-        <v>658</v>
+        <v>256</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>702</v>
+        <v>302</v>
       </c>
       <c r="B167" t="s">
-        <v>703</v>
+        <v>248</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>774</v>
+        <v>349</v>
       </c>
       <c r="B168" t="s">
-        <v>775</v>
-      </c>
-      <c r="C168" t="s">
-        <v>692</v>
+        <v>350</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>526</v>
+        <v>657</v>
       </c>
       <c r="B169" t="s">
-        <v>678</v>
+        <v>658</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3">
+      <c r="A170" t="s">
+        <v>702</v>
+      </c>
+      <c r="B170" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>515</v>
+        <v>774</v>
       </c>
       <c r="B171" t="s">
-        <v>516</v>
+        <v>775</v>
+      </c>
+      <c r="C171" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>259</v>
+        <v>526</v>
       </c>
       <c r="B172" t="s">
-        <v>262</v>
-      </c>
-      <c r="C172" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A173" t="s">
-        <v>261</v>
-      </c>
-      <c r="B173" t="s">
-        <v>561</v>
-      </c>
-      <c r="C173" t="s">
-        <v>696</v>
+        <v>678</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>260</v>
+        <v>515</v>
       </c>
       <c r="B174" t="s">
-        <v>263</v>
+        <v>516</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B175" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C175" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" ht="13.5" customHeight="1">
       <c r="A176" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B176" t="s">
-        <v>267</v>
+        <v>561</v>
+      </c>
+      <c r="C176" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B177" t="s">
-        <v>268</v>
-      </c>
-      <c r="C177" t="s">
-        <v>660</v>
+        <v>263</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>504</v>
+        <v>265</v>
       </c>
       <c r="B178" t="s">
-        <v>570</v>
+        <v>264</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B179" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B180" t="s">
-        <v>273</v>
+        <v>268</v>
+      </c>
+      <c r="C180" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>277</v>
+        <v>504</v>
       </c>
       <c r="B181" t="s">
-        <v>287</v>
+        <v>570</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="B182" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B183" t="s">
-        <v>285</v>
-      </c>
-      <c r="C183" t="s">
-        <v>660</v>
+        <v>273</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B184" t="s">
-        <v>605</v>
+        <v>287</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B185" t="s">
-        <v>284</v>
-      </c>
-      <c r="C185" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B186" t="s">
-        <v>283</v>
+        <v>285</v>
+      </c>
+      <c r="C186" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="B187" t="s">
-        <v>300</v>
+        <v>605</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="B188" t="s">
-        <v>248</v>
+        <v>284</v>
+      </c>
+      <c r="C188" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="B189" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>704</v>
+        <v>299</v>
       </c>
       <c r="B190" t="s">
-        <v>703</v>
+        <v>300</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>537</v>
+        <v>301</v>
       </c>
       <c r="B191" t="s">
-        <v>679</v>
+        <v>248</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>697</v>
+        <v>304</v>
       </c>
       <c r="B192" t="s">
-        <v>698</v>
-      </c>
-      <c r="C192" t="s">
-        <v>692</v>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3">
+      <c r="A193" t="s">
+        <v>704</v>
+      </c>
+      <c r="B193" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>517</v>
+        <v>537</v>
       </c>
       <c r="B194" t="s">
-        <v>518</v>
+        <v>679</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>292</v>
+        <v>697</v>
       </c>
       <c r="B195" t="s">
-        <v>296</v>
+        <v>698</v>
       </c>
       <c r="C195" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="196" spans="1:3">
-      <c r="A196" t="s">
-        <v>505</v>
-      </c>
-      <c r="B196" t="s">
-        <v>571</v>
+        <v>692</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>293</v>
+        <v>517</v>
       </c>
       <c r="B197" t="s">
-        <v>297</v>
-      </c>
-      <c r="C197" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B198" t="s">
-        <v>298</v>
+        <v>296</v>
+      </c>
+      <c r="C198" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>295</v>
+        <v>505</v>
       </c>
       <c r="B199" t="s">
-        <v>562</v>
+        <v>571</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B200" t="s">
-        <v>248</v>
+        <v>297</v>
+      </c>
+      <c r="C200" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="B201" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="B202" t="s">
-        <v>308</v>
+        <v>562</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B203" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B204" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>705</v>
+        <v>306</v>
       </c>
       <c r="B205" t="s">
-        <v>703</v>
+        <v>308</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>536</v>
+        <v>307</v>
       </c>
       <c r="B206" t="s">
-        <v>680</v>
+        <v>308</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3">
+      <c r="A207" t="s">
+        <v>311</v>
+      </c>
+      <c r="B207" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>519</v>
+        <v>705</v>
       </c>
       <c r="B208" t="s">
-        <v>520</v>
+        <v>703</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>499</v>
+        <v>536</v>
       </c>
       <c r="B209" t="s">
-        <v>320</v>
-      </c>
-      <c r="C209" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="210" spans="1:3">
-      <c r="A210" t="s">
-        <v>506</v>
-      </c>
-      <c r="B210" t="s">
-        <v>572</v>
+        <v>680</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>315</v>
+        <v>519</v>
       </c>
       <c r="B211" t="s">
-        <v>321</v>
-      </c>
-      <c r="C211" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>316</v>
+        <v>499</v>
       </c>
       <c r="B212" t="s">
-        <v>322</v>
+        <v>320</v>
+      </c>
+      <c r="C212" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>317</v>
+        <v>506</v>
       </c>
       <c r="B213" t="s">
-        <v>323</v>
+        <v>572</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B214" t="s">
-        <v>563</v>
+        <v>321</v>
+      </c>
+      <c r="C214" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B215" t="s">
-        <v>248</v>
+        <v>322</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="B216" t="s">
-        <v>325</v>
-      </c>
-      <c r="C216" t="s">
-        <v>588</v>
+        <v>323</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="B217" t="s">
-        <v>327</v>
+        <v>563</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="B218" t="s">
-        <v>328</v>
+        <v>248</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="B219" t="s">
-        <v>331</v>
+        <v>325</v>
+      </c>
+      <c r="C219" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="B220" t="s">
-        <v>256</v>
+        <v>327</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>706</v>
+        <v>329</v>
       </c>
       <c r="B221" t="s">
-        <v>703</v>
+        <v>328</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>535</v>
+        <v>330</v>
       </c>
       <c r="B222" t="s">
-        <v>681</v>
+        <v>331</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3">
+      <c r="A223" t="s">
+        <v>332</v>
+      </c>
+      <c r="B223" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>521</v>
+        <v>706</v>
       </c>
       <c r="B224" t="s">
-        <v>522</v>
+        <v>703</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>501</v>
+        <v>535</v>
       </c>
       <c r="B225" t="s">
-        <v>338</v>
-      </c>
-      <c r="C225" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="226" spans="1:3">
-      <c r="A226" t="s">
-        <v>507</v>
-      </c>
-      <c r="B226" t="s">
-        <v>573</v>
+        <v>681</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>336</v>
+        <v>521</v>
       </c>
       <c r="B227" t="s">
-        <v>339</v>
-      </c>
-      <c r="C227" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>337</v>
+        <v>501</v>
       </c>
       <c r="B228" t="s">
-        <v>340</v>
+        <v>338</v>
+      </c>
+      <c r="C228" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="B229" t="s">
-        <v>564</v>
+        <v>573</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="B230" t="s">
-        <v>248</v>
+        <v>339</v>
+      </c>
+      <c r="C230" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="B231" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>346</v>
+        <v>500</v>
       </c>
       <c r="B232" t="s">
-        <v>342</v>
+        <v>564</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B233" t="s">
-        <v>343</v>
+        <v>248</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B234" t="s">
-        <v>256</v>
+        <v>341</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>707</v>
+        <v>346</v>
       </c>
       <c r="B235" t="s">
-        <v>703</v>
+        <v>342</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>534</v>
+        <v>347</v>
       </c>
       <c r="B236" t="s">
-        <v>682</v>
+        <v>343</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3">
+      <c r="A237" t="s">
+        <v>348</v>
+      </c>
+      <c r="B237" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>745</v>
+        <v>707</v>
       </c>
       <c r="B238" t="s">
-        <v>746</v>
-      </c>
-      <c r="C238" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>551</v>
+        <v>534</v>
       </c>
       <c r="B239" t="s">
-        <v>554</v>
-      </c>
-      <c r="C239" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="240" spans="1:3">
-      <c r="A240" t="s">
-        <v>552</v>
-      </c>
-      <c r="B240" t="s">
-        <v>553</v>
-      </c>
-      <c r="C240" t="s">
-        <v>587</v>
+        <v>682</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>585</v>
+        <v>745</v>
       </c>
       <c r="B241" t="s">
-        <v>601</v>
+        <v>746</v>
+      </c>
+      <c r="C241" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>365</v>
+        <v>551</v>
       </c>
       <c r="B242" t="s">
-        <v>351</v>
+        <v>554</v>
+      </c>
+      <c r="C242" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>366</v>
+        <v>552</v>
       </c>
       <c r="B243" t="s">
-        <v>352</v>
+        <v>553</v>
       </c>
       <c r="C243" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>508</v>
+        <v>585</v>
       </c>
       <c r="B244" t="s">
-        <v>574</v>
+        <v>601</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B245" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B246" t="s">
-        <v>354</v>
+        <v>352</v>
+      </c>
+      <c r="C246" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>369</v>
+        <v>508</v>
       </c>
       <c r="B247" t="s">
-        <v>355</v>
+        <v>574</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B248" t="s">
-        <v>356</v>
-      </c>
-      <c r="C248" t="s">
-        <v>588</v>
+        <v>353</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B249" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B250" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B251" t="s">
-        <v>359</v>
+        <v>356</v>
+      </c>
+      <c r="C251" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B252" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B253" t="s">
-        <v>361</v>
-      </c>
-      <c r="C253" t="s">
-        <v>588</v>
+        <v>358</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B254" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B255" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B256" t="s">
-        <v>364</v>
+        <v>361</v>
+      </c>
+      <c r="C256" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>533</v>
+        <v>376</v>
       </c>
       <c r="B257" t="s">
-        <v>666</v>
+        <v>362</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3">
+      <c r="A258" t="s">
+        <v>377</v>
+      </c>
+      <c r="B258" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>606</v>
+        <v>378</v>
       </c>
       <c r="B259" t="s">
-        <v>607</v>
+        <v>364</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>385</v>
+        <v>533</v>
       </c>
       <c r="B260" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="261" spans="1:3">
-      <c r="A261" t="s">
-        <v>386</v>
-      </c>
-      <c r="B261" t="s">
-        <v>400</v>
+        <v>666</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>387</v>
+        <v>606</v>
       </c>
       <c r="B262" t="s">
-        <v>401</v>
-      </c>
-      <c r="C262" t="s">
-        <v>588</v>
+        <v>607</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>509</v>
+        <v>385</v>
       </c>
       <c r="B263" t="s">
-        <v>575</v>
+        <v>403</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
       <c r="B264" t="s">
-        <v>402</v>
-      </c>
-      <c r="C264" t="s">
-        <v>588</v>
+        <v>400</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B265" t="s">
-        <v>394</v>
+        <v>401</v>
+      </c>
+      <c r="C265" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>405</v>
+        <v>509</v>
       </c>
       <c r="B266" t="s">
-        <v>395</v>
-      </c>
-      <c r="C266" t="s">
-        <v>565</v>
+        <v>575</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="B267" t="s">
-        <v>396</v>
+        <v>402</v>
+      </c>
+      <c r="C267" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B268" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="B269" t="s">
-        <v>398</v>
+        <v>395</v>
+      </c>
+      <c r="C269" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B270" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B271" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>532</v>
+        <v>390</v>
       </c>
       <c r="B272" t="s">
-        <v>683</v>
+        <v>398</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3">
+      <c r="A273" t="s">
+        <v>392</v>
+      </c>
+      <c r="B273" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>747</v>
+        <v>393</v>
       </c>
       <c r="B274" t="s">
-        <v>766</v>
-      </c>
-      <c r="C274" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="276" spans="1:3">
-      <c r="A276" t="s">
-        <v>743</v>
-      </c>
-      <c r="B276" t="s">
-        <v>744</v>
-      </c>
-      <c r="C276" t="s">
-        <v>692</v>
+        <v>396</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3">
+      <c r="A275" t="s">
+        <v>532</v>
+      </c>
+      <c r="B275" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>523</v>
+        <v>747</v>
       </c>
       <c r="B277" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="278" spans="1:3">
-      <c r="A278" t="s">
-        <v>411</v>
-      </c>
-      <c r="B278" t="s">
-        <v>422</v>
+        <v>766</v>
+      </c>
+      <c r="C277" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>412</v>
+        <v>743</v>
       </c>
       <c r="B279" t="s">
-        <v>423</v>
+        <v>744</v>
       </c>
       <c r="C279" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>576</v>
+        <v>523</v>
       </c>
       <c r="B280" t="s">
-        <v>577</v>
+        <v>524</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B281" t="s">
-        <v>424</v>
-      </c>
-      <c r="C281" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B282" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C282" t="s">
         <v>588</v>
@@ -9341,128 +9362,128 @@
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>415</v>
+        <v>576</v>
       </c>
       <c r="B283" t="s">
-        <v>589</v>
+        <v>577</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B284" t="s">
-        <v>426</v>
+        <v>424</v>
+      </c>
+      <c r="C284" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B285" t="s">
-        <v>427</v>
+        <v>425</v>
+      </c>
+      <c r="C285" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B286" t="s">
-        <v>428</v>
+        <v>589</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B287" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B288" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="B289" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>530</v>
+        <v>419</v>
       </c>
       <c r="B290" t="s">
-        <v>684</v>
+        <v>429</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>615</v>
+        <v>420</v>
       </c>
       <c r="B291" t="s">
-        <v>616</v>
+        <v>430</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3">
+      <c r="A292" t="s">
+        <v>421</v>
+      </c>
+      <c r="B292" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="B293" t="s">
-        <v>524</v>
+        <v>684</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>438</v>
+        <v>615</v>
       </c>
       <c r="B294" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="295" spans="1:3">
-      <c r="A295" t="s">
-        <v>439</v>
-      </c>
-      <c r="B295" t="s">
-        <v>450</v>
-      </c>
-      <c r="C295" t="s">
-        <v>588</v>
+        <v>616</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>510</v>
+        <v>525</v>
       </c>
       <c r="B296" t="s">
-        <v>578</v>
+        <v>524</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B297" t="s">
-        <v>451</v>
-      </c>
-      <c r="C297" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B298" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C298" t="s">
         <v>588</v>
@@ -9470,143 +9491,173 @@
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>442</v>
+        <v>510</v>
       </c>
       <c r="B299" t="s">
-        <v>590</v>
+        <v>578</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B300" t="s">
-        <v>426</v>
+        <v>451</v>
+      </c>
+      <c r="C300" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B301" t="s">
-        <v>427</v>
+        <v>452</v>
+      </c>
+      <c r="C301" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B302" t="s">
-        <v>453</v>
+        <v>590</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B303" t="s">
-        <v>454</v>
+        <v>426</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="B304" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B305" t="s">
-        <v>431</v>
+        <v>453</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>529</v>
+        <v>446</v>
       </c>
       <c r="B306" t="s">
-        <v>684</v>
+        <v>454</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>622</v>
+        <v>447</v>
       </c>
       <c r="B307" t="s">
-        <v>616</v>
+        <v>430</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3">
+      <c r="A308" t="s">
+        <v>448</v>
+      </c>
+      <c r="B308" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>741</v>
+        <v>529</v>
       </c>
       <c r="B309" t="s">
-        <v>742</v>
-      </c>
-      <c r="C309" t="s">
-        <v>692</v>
+        <v>684</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>432</v>
+        <v>622</v>
       </c>
       <c r="B310" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3">
-      <c r="A311" t="s">
-        <v>433</v>
-      </c>
-      <c r="B311" t="s">
-        <v>624</v>
-      </c>
-      <c r="C311" t="s">
-        <v>588</v>
+        <v>616</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>511</v>
+        <v>741</v>
       </c>
       <c r="B312" t="s">
-        <v>625</v>
+        <v>742</v>
+      </c>
+      <c r="C312" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B313" t="s">
-        <v>651</v>
+        <v>623</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B314" t="s">
-        <v>626</v>
+        <v>624</v>
+      </c>
+      <c r="C314" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>436</v>
+        <v>511</v>
       </c>
       <c r="B315" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
+        <v>434</v>
+      </c>
+      <c r="B316" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3">
+      <c r="A317" t="s">
+        <v>435</v>
+      </c>
+      <c r="B317" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3">
+      <c r="A318" t="s">
+        <v>436</v>
+      </c>
+      <c r="B318" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3">
+      <c r="A319" t="s">
         <v>528</v>
       </c>
-      <c r="B316" t="s">
+      <c r="B319" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added DU for CZI
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E1E4BB-F59D-42DA-B6BD-0B2997875A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334A87BA-021E-4576-B114-A24A08158F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28170" windowHeight="14670" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="786">
   <si>
     <t>Name</t>
   </si>
@@ -2373,9 +2373,6 @@
     <t>FindAllASFAAssistance_Threshold</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>SCNE_EmploymentNo</t>
   </si>
   <si>
@@ -2392,6 +2389,15 @@
   </si>
   <si>
     <t xml:space="preserve">Employment field is No, but the following documentation for unemployment is not documented appropriately. </t>
+  </si>
+  <si>
+    <t>DU_TenantURL</t>
+  </si>
+  <si>
+    <t>DU_AppCredentials</t>
+  </si>
+  <si>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2849,7 +2855,7 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4455,7 +4461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z995"/>
+  <dimension ref="A1:Z996"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -4645,110 +4651,117 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>784</v>
       </c>
       <c r="B20" t="s">
-        <v>502</v>
+        <v>784</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>735</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>734</v>
+        <v>502</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
+        <v>735</v>
+      </c>
+      <c r="B22" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A23" t="s">
         <v>604</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" t="s">
-        <v>49</v>
-      </c>
-    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
         <v>69</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
+    <row r="34" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="35" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="36" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="37" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="38" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="39" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="40" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="41" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="42" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
     <row r="51" ht="14.25" customHeight="1"/>
@@ -5696,6 +5709,7 @@
     <row r="993" ht="14.25" customHeight="1"/>
     <row r="994" ht="14.25" customHeight="1"/>
     <row r="995" ht="14.25" customHeight="1"/>
+    <row r="996" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6069,7 +6083,14 @@
         <v>737</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="42" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A42" t="s">
+        <v>783</v>
+      </c>
+      <c r="B42" t="s">
+        <v>783</v>
+      </c>
+    </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7663,10 +7684,10 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
+        <v>779</v>
+      </c>
+      <c r="B75" t="s">
         <v>780</v>
-      </c>
-      <c r="B75" t="s">
-        <v>781</v>
       </c>
       <c r="C75" t="s">
         <v>692</v>
@@ -7674,10 +7695,10 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B76" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C76" t="s">
         <v>692</v>
@@ -7685,10 +7706,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B77" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C77" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Changes for 58192 - do not perform checks for VS when the employer is Social Security, 58193 - add finding for present VOE, and 58188 - retry scope for MID, ASFA, CZI, and HHD
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334A87BA-021E-4576-B114-A24A08158F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FBA7AE-2595-448B-A870-ED4E9A43D739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="788">
   <si>
     <t>Name</t>
   </si>
@@ -2397,7 +2397,13 @@
     <t>DU_AppCredentials</t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>VOE_Exists</t>
+  </si>
+  <si>
+    <t>Verification of Employment email receipt and clarification verification require manual review.</t>
   </si>
 </sst>
 </file>
@@ -7069,7 +7075,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C319"/>
+  <dimension ref="A1:C320"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8492,279 +8498,282 @@
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>515</v>
+        <v>786</v>
       </c>
       <c r="B174" t="s">
-        <v>516</v>
+        <v>787</v>
+      </c>
+      <c r="C174" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
+        <v>515</v>
+      </c>
+      <c r="B175" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3">
+      <c r="A176" t="s">
         <v>259</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B176" t="s">
         <v>262</v>
       </c>
-      <c r="C175" t="s">
+      <c r="C176" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A176" t="s">
+    <row r="177" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A177" t="s">
         <v>261</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>561</v>
       </c>
-      <c r="C176" t="s">
+      <c r="C177" t="s">
         <v>696</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3">
-      <c r="A177" t="s">
-        <v>260</v>
-      </c>
-      <c r="B177" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B178" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B179" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B180" t="s">
-        <v>268</v>
-      </c>
-      <c r="C180" t="s">
-        <v>660</v>
+        <v>267</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>504</v>
+        <v>269</v>
       </c>
       <c r="B181" t="s">
-        <v>570</v>
+        <v>268</v>
+      </c>
+      <c r="C181" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>270</v>
+        <v>504</v>
       </c>
       <c r="B182" t="s">
-        <v>271</v>
+        <v>570</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B183" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B184" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B185" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B186" t="s">
-        <v>285</v>
-      </c>
-      <c r="C186" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B187" t="s">
-        <v>605</v>
+        <v>285</v>
+      </c>
+      <c r="C187" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B188" t="s">
-        <v>284</v>
-      </c>
-      <c r="C188" t="s">
-        <v>660</v>
+        <v>605</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B189" t="s">
-        <v>283</v>
+        <v>284</v>
+      </c>
+      <c r="C189" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="B190" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B191" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B192" t="s">
-        <v>305</v>
+        <v>248</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>704</v>
+        <v>304</v>
       </c>
       <c r="B193" t="s">
-        <v>703</v>
+        <v>305</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>537</v>
+        <v>704</v>
       </c>
       <c r="B194" t="s">
-        <v>679</v>
+        <v>703</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
+        <v>537</v>
+      </c>
+      <c r="B195" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3">
+      <c r="A196" t="s">
         <v>697</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B196" t="s">
         <v>698</v>
       </c>
-      <c r="C195" t="s">
+      <c r="C196" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3">
-      <c r="A197" t="s">
-        <v>517</v>
-      </c>
-      <c r="B197" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>292</v>
+        <v>517</v>
       </c>
       <c r="B198" t="s">
-        <v>296</v>
-      </c>
-      <c r="C198" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>505</v>
+        <v>292</v>
       </c>
       <c r="B199" t="s">
-        <v>571</v>
+        <v>296</v>
+      </c>
+      <c r="C199" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>293</v>
+        <v>505</v>
       </c>
       <c r="B200" t="s">
-        <v>297</v>
-      </c>
-      <c r="C200" t="s">
-        <v>588</v>
+        <v>571</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B201" t="s">
-        <v>298</v>
+        <v>297</v>
+      </c>
+      <c r="C201" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B202" t="s">
-        <v>562</v>
+        <v>298</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="B203" t="s">
-        <v>248</v>
+        <v>562</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B204" t="s">
-        <v>310</v>
+        <v>248</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B205" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B206" t="s">
         <v>308</v>
@@ -8772,640 +8781,637 @@
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B207" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>705</v>
+        <v>311</v>
       </c>
       <c r="B208" t="s">
-        <v>703</v>
+        <v>312</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
+        <v>705</v>
+      </c>
+      <c r="B209" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3">
+      <c r="A210" t="s">
         <v>536</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B210" t="s">
         <v>680</v>
-      </c>
-    </row>
-    <row r="211" spans="1:3">
-      <c r="A211" t="s">
-        <v>519</v>
-      </c>
-      <c r="B211" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>499</v>
+        <v>519</v>
       </c>
       <c r="B212" t="s">
-        <v>320</v>
-      </c>
-      <c r="C212" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="B213" t="s">
-        <v>572</v>
+        <v>320</v>
+      </c>
+      <c r="C213" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>315</v>
+        <v>506</v>
       </c>
       <c r="B214" t="s">
-        <v>321</v>
-      </c>
-      <c r="C214" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B215" t="s">
-        <v>322</v>
+        <v>321</v>
+      </c>
+      <c r="C215" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B216" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B217" t="s">
-        <v>563</v>
+        <v>323</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B218" t="s">
-        <v>248</v>
+        <v>563</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B219" t="s">
-        <v>325</v>
-      </c>
-      <c r="C219" t="s">
-        <v>588</v>
+        <v>248</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B220" t="s">
-        <v>327</v>
+        <v>325</v>
+      </c>
+      <c r="C220" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B221" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B222" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B223" t="s">
-        <v>256</v>
+        <v>331</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>706</v>
+        <v>332</v>
       </c>
       <c r="B224" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
+        <v>706</v>
+      </c>
+      <c r="B225" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3">
+      <c r="A226" t="s">
         <v>535</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B226" t="s">
         <v>681</v>
-      </c>
-    </row>
-    <row r="227" spans="1:3">
-      <c r="A227" t="s">
-        <v>521</v>
-      </c>
-      <c r="B227" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="B228" t="s">
-        <v>338</v>
-      </c>
-      <c r="C228" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B229" t="s">
-        <v>573</v>
+        <v>338</v>
+      </c>
+      <c r="C229" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>336</v>
+        <v>507</v>
       </c>
       <c r="B230" t="s">
-        <v>339</v>
-      </c>
-      <c r="C230" t="s">
-        <v>588</v>
+        <v>573</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B231" t="s">
-        <v>340</v>
+        <v>339</v>
+      </c>
+      <c r="C231" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>500</v>
+        <v>337</v>
       </c>
       <c r="B232" t="s">
-        <v>564</v>
+        <v>340</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>344</v>
+        <v>500</v>
       </c>
       <c r="B233" t="s">
-        <v>248</v>
+        <v>564</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B234" t="s">
-        <v>341</v>
+        <v>248</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B235" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B236" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B237" t="s">
-        <v>256</v>
+        <v>343</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>707</v>
+        <v>348</v>
       </c>
       <c r="B238" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
+        <v>707</v>
+      </c>
+      <c r="B239" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3">
+      <c r="A240" t="s">
         <v>534</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B240" t="s">
         <v>682</v>
-      </c>
-    </row>
-    <row r="241" spans="1:3">
-      <c r="A241" t="s">
-        <v>745</v>
-      </c>
-      <c r="B241" t="s">
-        <v>746</v>
-      </c>
-      <c r="C241" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>551</v>
+        <v>745</v>
       </c>
       <c r="B242" t="s">
-        <v>554</v>
+        <v>746</v>
       </c>
       <c r="C242" t="s">
-        <v>586</v>
+        <v>692</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B243" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C243" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>585</v>
+        <v>552</v>
       </c>
       <c r="B244" t="s">
-        <v>601</v>
+        <v>553</v>
+      </c>
+      <c r="C244" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>365</v>
+        <v>585</v>
       </c>
       <c r="B245" t="s">
-        <v>351</v>
+        <v>601</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B246" t="s">
-        <v>352</v>
-      </c>
-      <c r="C246" t="s">
-        <v>588</v>
+        <v>351</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>508</v>
+        <v>366</v>
       </c>
       <c r="B247" t="s">
-        <v>574</v>
+        <v>352</v>
+      </c>
+      <c r="C247" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>367</v>
+        <v>508</v>
       </c>
       <c r="B248" t="s">
-        <v>353</v>
+        <v>574</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B249" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B250" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B251" t="s">
-        <v>356</v>
-      </c>
-      <c r="C251" t="s">
-        <v>588</v>
+        <v>355</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B252" t="s">
-        <v>357</v>
+        <v>356</v>
+      </c>
+      <c r="C252" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B253" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B254" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B255" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B256" t="s">
-        <v>361</v>
-      </c>
-      <c r="C256" t="s">
-        <v>588</v>
+        <v>360</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B257" t="s">
-        <v>362</v>
+        <v>361</v>
+      </c>
+      <c r="C257" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B258" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B259" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
+        <v>378</v>
+      </c>
+      <c r="B260" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3">
+      <c r="A261" t="s">
         <v>533</v>
       </c>
-      <c r="B260" t="s">
+      <c r="B261" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="262" spans="1:3">
-      <c r="A262" t="s">
-        <v>606</v>
-      </c>
-      <c r="B262" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>385</v>
+        <v>606</v>
       </c>
       <c r="B263" t="s">
-        <v>403</v>
+        <v>607</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B264" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B265" t="s">
-        <v>401</v>
-      </c>
-      <c r="C265" t="s">
-        <v>588</v>
+        <v>400</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>509</v>
+        <v>387</v>
       </c>
       <c r="B266" t="s">
-        <v>575</v>
+        <v>401</v>
+      </c>
+      <c r="C266" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>404</v>
+        <v>509</v>
       </c>
       <c r="B267" t="s">
-        <v>402</v>
-      </c>
-      <c r="C267" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="B268" t="s">
-        <v>394</v>
+        <v>402</v>
+      </c>
+      <c r="C268" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
       <c r="B269" t="s">
-        <v>395</v>
-      </c>
-      <c r="C269" t="s">
-        <v>565</v>
+        <v>394</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="B270" t="s">
-        <v>396</v>
+        <v>395</v>
+      </c>
+      <c r="C270" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B271" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B272" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B273" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B274" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
+        <v>393</v>
+      </c>
+      <c r="B275" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3">
+      <c r="A276" t="s">
         <v>532</v>
       </c>
-      <c r="B275" t="s">
+      <c r="B276" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
-      <c r="A277" t="s">
+    <row r="278" spans="1:3">
+      <c r="A278" t="s">
         <v>747</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B278" t="s">
         <v>766</v>
       </c>
-      <c r="C277" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="279" spans="1:3">
-      <c r="A279" t="s">
-        <v>743</v>
-      </c>
-      <c r="B279" t="s">
-        <v>744</v>
-      </c>
-      <c r="C279" t="s">
+      <c r="C278" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>523</v>
+        <v>743</v>
       </c>
       <c r="B280" t="s">
-        <v>524</v>
+        <v>744</v>
+      </c>
+      <c r="C280" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>411</v>
+        <v>523</v>
       </c>
       <c r="B281" t="s">
-        <v>422</v>
+        <v>524</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B282" t="s">
-        <v>423</v>
-      </c>
-      <c r="C282" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>576</v>
+        <v>412</v>
       </c>
       <c r="B283" t="s">
-        <v>577</v>
+        <v>423</v>
+      </c>
+      <c r="C283" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>413</v>
+        <v>576</v>
       </c>
       <c r="B284" t="s">
-        <v>424</v>
-      </c>
-      <c r="C284" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B285" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C285" t="s">
         <v>588</v>
@@ -9413,128 +9419,128 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B286" t="s">
-        <v>589</v>
+        <v>425</v>
+      </c>
+      <c r="C286" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B287" t="s">
-        <v>426</v>
+        <v>589</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B288" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B289" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B290" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B291" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B292" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>530</v>
+        <v>421</v>
       </c>
       <c r="B293" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
+        <v>530</v>
+      </c>
+      <c r="B294" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3">
+      <c r="A295" t="s">
         <v>615</v>
       </c>
-      <c r="B294" t="s">
+      <c r="B295" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="296" spans="1:3">
-      <c r="A296" t="s">
-        <v>525</v>
-      </c>
-      <c r="B296" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>438</v>
+        <v>525</v>
       </c>
       <c r="B297" t="s">
-        <v>449</v>
+        <v>524</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B298" t="s">
-        <v>450</v>
-      </c>
-      <c r="C298" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>510</v>
+        <v>439</v>
       </c>
       <c r="B299" t="s">
-        <v>578</v>
+        <v>450</v>
+      </c>
+      <c r="C299" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>440</v>
+        <v>510</v>
       </c>
       <c r="B300" t="s">
-        <v>451</v>
-      </c>
-      <c r="C300" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B301" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C301" t="s">
         <v>588</v>
@@ -9542,143 +9548,154 @@
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B302" t="s">
-        <v>590</v>
+        <v>452</v>
+      </c>
+      <c r="C302" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B303" t="s">
-        <v>426</v>
+        <v>590</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B304" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B305" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B306" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B307" t="s">
-        <v>430</v>
+        <v>454</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B308" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>529</v>
+        <v>448</v>
       </c>
       <c r="B309" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
+        <v>529</v>
+      </c>
+      <c r="B310" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3">
+      <c r="A311" t="s">
         <v>622</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B311" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="312" spans="1:3">
-      <c r="A312" t="s">
-        <v>741</v>
-      </c>
-      <c r="B312" t="s">
-        <v>742</v>
-      </c>
-      <c r="C312" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>432</v>
+        <v>741</v>
       </c>
       <c r="B313" t="s">
-        <v>623</v>
+        <v>742</v>
+      </c>
+      <c r="C313" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B314" t="s">
-        <v>624</v>
-      </c>
-      <c r="C314" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>511</v>
+        <v>433</v>
       </c>
       <c r="B315" t="s">
-        <v>625</v>
+        <v>624</v>
+      </c>
+      <c r="C315" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>434</v>
+        <v>511</v>
       </c>
       <c r="B316" t="s">
-        <v>651</v>
+        <v>625</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B317" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B318" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
+        <v>436</v>
+      </c>
+      <c r="B319" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3">
+      <c r="A320" t="s">
         <v>528</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B320" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changes for 58201 - removing page numbers in Yardi findings, 58188 - added retry scopes for all document types fro DU extraction, and 57831 - added a new check for pay increase in paystubs
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FBA7AE-2595-448B-A870-ED4E9A43D739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A22F4ED-41A4-46C5-B1F6-4907B867EB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="790">
   <si>
     <t>Name</t>
   </si>
@@ -2404,6 +2404,12 @@
   </si>
   <si>
     <t>Verification of Employment email receipt and clarification verification require manual review.</t>
+  </si>
+  <si>
+    <t>PS_PayIncreaseAcrossPS</t>
+  </si>
+  <si>
+    <t>Regular pay rate has increase across paystubs. Manual review is required.</t>
   </si>
 </sst>
 </file>
@@ -7075,7 +7081,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C320"/>
+  <dimension ref="A1:C321"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8490,298 +8496,301 @@
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
+        <v>788</v>
+      </c>
+      <c r="B172" t="s">
+        <v>789</v>
+      </c>
+      <c r="C172" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3">
+      <c r="A173" t="s">
         <v>526</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B173" t="s">
         <v>678</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3">
-      <c r="A174" t="s">
-        <v>786</v>
-      </c>
-      <c r="B174" t="s">
-        <v>787</v>
-      </c>
-      <c r="C174" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>515</v>
+        <v>786</v>
       </c>
       <c r="B175" t="s">
-        <v>516</v>
+        <v>787</v>
+      </c>
+      <c r="C175" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
+        <v>515</v>
+      </c>
+      <c r="B176" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3">
+      <c r="A177" t="s">
         <v>259</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>262</v>
       </c>
-      <c r="C176" t="s">
+      <c r="C177" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A177" t="s">
+    <row r="178" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A178" t="s">
         <v>261</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>561</v>
       </c>
-      <c r="C177" t="s">
+      <c r="C178" t="s">
         <v>696</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3">
-      <c r="A178" t="s">
-        <v>260</v>
-      </c>
-      <c r="B178" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B179" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B180" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B181" t="s">
-        <v>268</v>
-      </c>
-      <c r="C181" t="s">
-        <v>660</v>
+        <v>267</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>504</v>
+        <v>269</v>
       </c>
       <c r="B182" t="s">
-        <v>570</v>
+        <v>268</v>
+      </c>
+      <c r="C182" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>270</v>
+        <v>504</v>
       </c>
       <c r="B183" t="s">
-        <v>271</v>
+        <v>570</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B184" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B185" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B186" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B187" t="s">
-        <v>285</v>
-      </c>
-      <c r="C187" t="s">
-        <v>660</v>
+        <v>286</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B188" t="s">
-        <v>605</v>
+        <v>285</v>
+      </c>
+      <c r="C188" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B189" t="s">
-        <v>284</v>
-      </c>
-      <c r="C189" t="s">
-        <v>660</v>
+        <v>605</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B190" t="s">
-        <v>283</v>
+        <v>284</v>
+      </c>
+      <c r="C190" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="B191" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B192" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B193" t="s">
-        <v>305</v>
+        <v>248</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>704</v>
+        <v>304</v>
       </c>
       <c r="B194" t="s">
-        <v>703</v>
+        <v>305</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>537</v>
+        <v>704</v>
       </c>
       <c r="B195" t="s">
-        <v>679</v>
+        <v>703</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
+        <v>537</v>
+      </c>
+      <c r="B196" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
         <v>697</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B197" t="s">
         <v>698</v>
       </c>
-      <c r="C196" t="s">
+      <c r="C197" t="s">
         <v>692</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3">
-      <c r="A198" t="s">
-        <v>517</v>
-      </c>
-      <c r="B198" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>292</v>
+        <v>517</v>
       </c>
       <c r="B199" t="s">
-        <v>296</v>
-      </c>
-      <c r="C199" t="s">
-        <v>588</v>
+        <v>518</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>505</v>
+        <v>292</v>
       </c>
       <c r="B200" t="s">
-        <v>571</v>
+        <v>296</v>
+      </c>
+      <c r="C200" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>293</v>
+        <v>505</v>
       </c>
       <c r="B201" t="s">
-        <v>297</v>
-      </c>
-      <c r="C201" t="s">
-        <v>588</v>
+        <v>571</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B202" t="s">
-        <v>298</v>
+        <v>297</v>
+      </c>
+      <c r="C202" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B203" t="s">
-        <v>562</v>
+        <v>298</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="B204" t="s">
-        <v>248</v>
+        <v>562</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B205" t="s">
-        <v>310</v>
+        <v>248</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B206" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B207" t="s">
         <v>308</v>
@@ -8789,640 +8798,637 @@
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B208" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>705</v>
+        <v>311</v>
       </c>
       <c r="B209" t="s">
-        <v>703</v>
+        <v>312</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
+        <v>705</v>
+      </c>
+      <c r="B210" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3">
+      <c r="A211" t="s">
         <v>536</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B211" t="s">
         <v>680</v>
-      </c>
-    </row>
-    <row r="212" spans="1:3">
-      <c r="A212" t="s">
-        <v>519</v>
-      </c>
-      <c r="B212" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>499</v>
+        <v>519</v>
       </c>
       <c r="B213" t="s">
-        <v>320</v>
-      </c>
-      <c r="C213" t="s">
-        <v>588</v>
+        <v>520</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="B214" t="s">
-        <v>572</v>
+        <v>320</v>
+      </c>
+      <c r="C214" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>315</v>
+        <v>506</v>
       </c>
       <c r="B215" t="s">
-        <v>321</v>
-      </c>
-      <c r="C215" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B216" t="s">
-        <v>322</v>
+        <v>321</v>
+      </c>
+      <c r="C216" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B217" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B218" t="s">
-        <v>563</v>
+        <v>323</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B219" t="s">
-        <v>248</v>
+        <v>563</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B220" t="s">
-        <v>325</v>
-      </c>
-      <c r="C220" t="s">
-        <v>588</v>
+        <v>248</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B221" t="s">
-        <v>327</v>
+        <v>325</v>
+      </c>
+      <c r="C221" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B222" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B223" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B224" t="s">
-        <v>256</v>
+        <v>331</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>706</v>
+        <v>332</v>
       </c>
       <c r="B225" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
+        <v>706</v>
+      </c>
+      <c r="B226" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3">
+      <c r="A227" t="s">
         <v>535</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B227" t="s">
         <v>681</v>
-      </c>
-    </row>
-    <row r="228" spans="1:3">
-      <c r="A228" t="s">
-        <v>521</v>
-      </c>
-      <c r="B228" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="B229" t="s">
-        <v>338</v>
-      </c>
-      <c r="C229" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B230" t="s">
-        <v>573</v>
+        <v>338</v>
+      </c>
+      <c r="C230" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>336</v>
+        <v>507</v>
       </c>
       <c r="B231" t="s">
-        <v>339</v>
-      </c>
-      <c r="C231" t="s">
-        <v>588</v>
+        <v>573</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B232" t="s">
-        <v>340</v>
+        <v>339</v>
+      </c>
+      <c r="C232" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>500</v>
+        <v>337</v>
       </c>
       <c r="B233" t="s">
-        <v>564</v>
+        <v>340</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>344</v>
+        <v>500</v>
       </c>
       <c r="B234" t="s">
-        <v>248</v>
+        <v>564</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B235" t="s">
-        <v>341</v>
+        <v>248</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B236" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B237" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B238" t="s">
-        <v>256</v>
+        <v>343</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>707</v>
+        <v>348</v>
       </c>
       <c r="B239" t="s">
-        <v>703</v>
+        <v>256</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
+        <v>707</v>
+      </c>
+      <c r="B240" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3">
+      <c r="A241" t="s">
         <v>534</v>
       </c>
-      <c r="B240" t="s">
+      <c r="B241" t="s">
         <v>682</v>
-      </c>
-    </row>
-    <row r="242" spans="1:3">
-      <c r="A242" t="s">
-        <v>745</v>
-      </c>
-      <c r="B242" t="s">
-        <v>746</v>
-      </c>
-      <c r="C242" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>551</v>
+        <v>745</v>
       </c>
       <c r="B243" t="s">
-        <v>554</v>
+        <v>746</v>
       </c>
       <c r="C243" t="s">
-        <v>586</v>
+        <v>692</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B244" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C244" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>585</v>
+        <v>552</v>
       </c>
       <c r="B245" t="s">
-        <v>601</v>
+        <v>553</v>
+      </c>
+      <c r="C245" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>365</v>
+        <v>585</v>
       </c>
       <c r="B246" t="s">
-        <v>351</v>
+        <v>601</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B247" t="s">
-        <v>352</v>
-      </c>
-      <c r="C247" t="s">
-        <v>588</v>
+        <v>351</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>508</v>
+        <v>366</v>
       </c>
       <c r="B248" t="s">
-        <v>574</v>
+        <v>352</v>
+      </c>
+      <c r="C248" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>367</v>
+        <v>508</v>
       </c>
       <c r="B249" t="s">
-        <v>353</v>
+        <v>574</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B250" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B251" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B252" t="s">
-        <v>356</v>
-      </c>
-      <c r="C252" t="s">
-        <v>588</v>
+        <v>355</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B253" t="s">
-        <v>357</v>
+        <v>356</v>
+      </c>
+      <c r="C253" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B254" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B255" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B256" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B257" t="s">
-        <v>361</v>
-      </c>
-      <c r="C257" t="s">
-        <v>588</v>
+        <v>360</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B258" t="s">
-        <v>362</v>
+        <v>361</v>
+      </c>
+      <c r="C258" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B259" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B260" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
+        <v>378</v>
+      </c>
+      <c r="B261" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3">
+      <c r="A262" t="s">
         <v>533</v>
       </c>
-      <c r="B261" t="s">
+      <c r="B262" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3">
-      <c r="A263" t="s">
-        <v>606</v>
-      </c>
-      <c r="B263" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>385</v>
+        <v>606</v>
       </c>
       <c r="B264" t="s">
-        <v>403</v>
+        <v>607</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B265" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B266" t="s">
-        <v>401</v>
-      </c>
-      <c r="C266" t="s">
-        <v>588</v>
+        <v>400</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>509</v>
+        <v>387</v>
       </c>
       <c r="B267" t="s">
-        <v>575</v>
+        <v>401</v>
+      </c>
+      <c r="C267" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>404</v>
+        <v>509</v>
       </c>
       <c r="B268" t="s">
-        <v>402</v>
-      </c>
-      <c r="C268" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="B269" t="s">
-        <v>394</v>
+        <v>402</v>
+      </c>
+      <c r="C269" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>405</v>
+        <v>388</v>
       </c>
       <c r="B270" t="s">
-        <v>395</v>
-      </c>
-      <c r="C270" t="s">
-        <v>565</v>
+        <v>394</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="B271" t="s">
-        <v>396</v>
+        <v>395</v>
+      </c>
+      <c r="C271" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B272" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B273" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B274" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B275" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
+        <v>393</v>
+      </c>
+      <c r="B276" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3">
+      <c r="A277" t="s">
         <v>532</v>
       </c>
-      <c r="B276" t="s">
+      <c r="B277" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
-      <c r="A278" t="s">
+    <row r="279" spans="1:3">
+      <c r="A279" t="s">
         <v>747</v>
       </c>
-      <c r="B278" t="s">
+      <c r="B279" t="s">
         <v>766</v>
       </c>
-      <c r="C278" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="280" spans="1:3">
-      <c r="A280" t="s">
-        <v>743</v>
-      </c>
-      <c r="B280" t="s">
-        <v>744</v>
-      </c>
-      <c r="C280" t="s">
+      <c r="C279" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>523</v>
+        <v>743</v>
       </c>
       <c r="B281" t="s">
-        <v>524</v>
+        <v>744</v>
+      </c>
+      <c r="C281" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>411</v>
+        <v>523</v>
       </c>
       <c r="B282" t="s">
-        <v>422</v>
+        <v>524</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B283" t="s">
-        <v>423</v>
-      </c>
-      <c r="C283" t="s">
-        <v>588</v>
+        <v>422</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>576</v>
+        <v>412</v>
       </c>
       <c r="B284" t="s">
-        <v>577</v>
+        <v>423</v>
+      </c>
+      <c r="C284" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>413</v>
+        <v>576</v>
       </c>
       <c r="B285" t="s">
-        <v>424</v>
-      </c>
-      <c r="C285" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B286" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C286" t="s">
         <v>588</v>
@@ -9430,128 +9436,128 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B287" t="s">
-        <v>589</v>
+        <v>425</v>
+      </c>
+      <c r="C287" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B288" t="s">
-        <v>426</v>
+        <v>589</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B289" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B290" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B291" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B292" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B293" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>530</v>
+        <v>421</v>
       </c>
       <c r="B294" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
+        <v>530</v>
+      </c>
+      <c r="B295" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3">
+      <c r="A296" t="s">
         <v>615</v>
       </c>
-      <c r="B295" t="s">
+      <c r="B296" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="297" spans="1:3">
-      <c r="A297" t="s">
-        <v>525</v>
-      </c>
-      <c r="B297" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>438</v>
+        <v>525</v>
       </c>
       <c r="B298" t="s">
-        <v>449</v>
+        <v>524</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B299" t="s">
-        <v>450</v>
-      </c>
-      <c r="C299" t="s">
-        <v>588</v>
+        <v>449</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>510</v>
+        <v>439</v>
       </c>
       <c r="B300" t="s">
-        <v>578</v>
+        <v>450</v>
+      </c>
+      <c r="C300" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>440</v>
+        <v>510</v>
       </c>
       <c r="B301" t="s">
-        <v>451</v>
-      </c>
-      <c r="C301" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B302" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C302" t="s">
         <v>588</v>
@@ -9559,143 +9565,154 @@
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B303" t="s">
-        <v>590</v>
+        <v>452</v>
+      </c>
+      <c r="C303" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B304" t="s">
-        <v>426</v>
+        <v>590</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B305" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B306" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B307" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B308" t="s">
-        <v>430</v>
+        <v>454</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B309" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>529</v>
+        <v>448</v>
       </c>
       <c r="B310" t="s">
-        <v>684</v>
+        <v>431</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
+        <v>529</v>
+      </c>
+      <c r="B311" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3">
+      <c r="A312" t="s">
         <v>622</v>
       </c>
-      <c r="B311" t="s">
+      <c r="B312" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3">
-      <c r="A313" t="s">
-        <v>741</v>
-      </c>
-      <c r="B313" t="s">
-        <v>742</v>
-      </c>
-      <c r="C313" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>432</v>
+        <v>741</v>
       </c>
       <c r="B314" t="s">
-        <v>623</v>
+        <v>742</v>
+      </c>
+      <c r="C314" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B315" t="s">
-        <v>624</v>
-      </c>
-      <c r="C315" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>511</v>
+        <v>433</v>
       </c>
       <c r="B316" t="s">
-        <v>625</v>
+        <v>624</v>
+      </c>
+      <c r="C316" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>434</v>
+        <v>511</v>
       </c>
       <c r="B317" t="s">
-        <v>651</v>
+        <v>625</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B318" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B319" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
+        <v>436</v>
+      </c>
+      <c r="B320" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" t="s">
         <v>528</v>
       </c>
-      <c r="B320" t="s">
+      <c r="B321" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changes for 58187 - updated str_Frequency in PS to be replaced withfrequency stated, otherwise to adda  finding if both are null
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A22F4ED-41A4-46C5-B1F6-4907B867EB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4330DBD4-1A88-4E08-8596-702C7B8E256A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="794">
   <si>
     <t>Name</t>
   </si>
@@ -2410,6 +2410,18 @@
   </si>
   <si>
     <t>Regular pay rate has increase across paystubs. Manual review is required.</t>
+  </si>
+  <si>
+    <t>PS_FrequencyError</t>
+  </si>
+  <si>
+    <t>Pay frequency could not be determined from the paystubs to compare to the Exact Day Calculator.</t>
+  </si>
+  <si>
+    <t>EDC_Missing</t>
+  </si>
+  <si>
+    <t>The ICW includes multiple employments; however, Exact Day Calculator is available for only one of them.</t>
   </si>
 </sst>
 </file>
@@ -7081,7 +7093,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C321"/>
+  <dimension ref="A1:C323"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8326,40 +8338,40 @@
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>740</v>
+        <v>792</v>
       </c>
       <c r="B152" t="s">
-        <v>729</v>
+        <v>793</v>
       </c>
       <c r="C152" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
-      <c r="A154" t="s">
-        <v>513</v>
-      </c>
-      <c r="B154" t="s">
-        <v>514</v>
+    <row r="153" spans="1:3">
+      <c r="A153" t="s">
+        <v>740</v>
+      </c>
+      <c r="B153" t="s">
+        <v>729</v>
+      </c>
+      <c r="C153" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>661</v>
+        <v>513</v>
       </c>
       <c r="B155" t="s">
-        <v>665</v>
-      </c>
-      <c r="C155" t="s">
-        <v>663</v>
+        <v>514</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B156" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C156" t="s">
         <v>663</v>
@@ -8367,293 +8379,296 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>242</v>
+        <v>662</v>
       </c>
       <c r="B157" t="s">
-        <v>243</v>
+        <v>664</v>
       </c>
       <c r="C157" t="s">
-        <v>588</v>
+        <v>663</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B158" t="s">
-        <v>245</v>
+        <v>243</v>
+      </c>
+      <c r="C158" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B159" t="s">
-        <v>560</v>
-      </c>
-      <c r="C159" t="s">
-        <v>650</v>
+        <v>245</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="B160" t="s">
-        <v>246</v>
+        <v>560</v>
+      </c>
+      <c r="C160" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>503</v>
+        <v>790</v>
       </c>
       <c r="B161" t="s">
-        <v>512</v>
+        <v>791</v>
+      </c>
+      <c r="C161" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B162" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>250</v>
+        <v>503</v>
       </c>
       <c r="B163" t="s">
-        <v>252</v>
+        <v>512</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B164" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B165" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B166" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="B167" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>349</v>
+        <v>257</v>
       </c>
       <c r="B168" t="s">
-        <v>350</v>
+        <v>256</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>657</v>
+        <v>302</v>
       </c>
       <c r="B169" t="s">
-        <v>658</v>
+        <v>248</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>702</v>
+        <v>349</v>
       </c>
       <c r="B170" t="s">
-        <v>703</v>
+        <v>350</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>774</v>
+        <v>657</v>
       </c>
       <c r="B171" t="s">
-        <v>775</v>
-      </c>
-      <c r="C171" t="s">
-        <v>692</v>
+        <v>658</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>788</v>
+        <v>702</v>
       </c>
       <c r="B172" t="s">
-        <v>789</v>
-      </c>
-      <c r="C172" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>526</v>
+        <v>774</v>
       </c>
       <c r="B173" t="s">
-        <v>678</v>
+        <v>775</v>
+      </c>
+      <c r="C173" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3">
+      <c r="A174" t="s">
+        <v>788</v>
+      </c>
+      <c r="B174" t="s">
+        <v>789</v>
+      </c>
+      <c r="C174" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>786</v>
+        <v>526</v>
       </c>
       <c r="B175" t="s">
-        <v>787</v>
-      </c>
-      <c r="C175" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3">
-      <c r="A176" t="s">
-        <v>515</v>
-      </c>
-      <c r="B176" t="s">
-        <v>516</v>
+        <v>678</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>259</v>
+        <v>786</v>
       </c>
       <c r="B177" t="s">
-        <v>262</v>
+        <v>787</v>
       </c>
       <c r="C177" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" ht="13.5" customHeight="1">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>261</v>
+        <v>515</v>
       </c>
       <c r="B178" t="s">
-        <v>561</v>
-      </c>
-      <c r="C178" t="s">
-        <v>696</v>
+        <v>516</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B179" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3">
+        <v>262</v>
+      </c>
+      <c r="C179" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="13.5" customHeight="1">
       <c r="A180" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B180" t="s">
-        <v>264</v>
+        <v>561</v>
+      </c>
+      <c r="C180" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B181" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B182" t="s">
-        <v>268</v>
-      </c>
-      <c r="C182" t="s">
-        <v>660</v>
+        <v>264</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>504</v>
+        <v>266</v>
       </c>
       <c r="B183" t="s">
-        <v>570</v>
+        <v>267</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B184" t="s">
-        <v>271</v>
+        <v>268</v>
+      </c>
+      <c r="C184" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>272</v>
+        <v>504</v>
       </c>
       <c r="B185" t="s">
-        <v>273</v>
+        <v>570</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B186" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="B187" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B188" t="s">
-        <v>285</v>
-      </c>
-      <c r="C188" t="s">
-        <v>660</v>
+        <v>287</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B189" t="s">
-        <v>605</v>
+        <v>286</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B190" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C190" t="s">
         <v>660</v>
@@ -8661,96 +8676,96 @@
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B191" t="s">
-        <v>283</v>
+        <v>605</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="B192" t="s">
-        <v>300</v>
+        <v>284</v>
+      </c>
+      <c r="C192" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="B193" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B194" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>704</v>
+        <v>301</v>
       </c>
       <c r="B195" t="s">
-        <v>703</v>
+        <v>248</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>537</v>
+        <v>304</v>
       </c>
       <c r="B196" t="s">
-        <v>679</v>
+        <v>305</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="B197" t="s">
-        <v>698</v>
-      </c>
-      <c r="C197" t="s">
-        <v>692</v>
+        <v>703</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3">
+      <c r="A198" t="s">
+        <v>537</v>
+      </c>
+      <c r="B198" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>517</v>
+        <v>697</v>
       </c>
       <c r="B199" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="200" spans="1:3">
-      <c r="A200" t="s">
-        <v>292</v>
-      </c>
-      <c r="B200" t="s">
-        <v>296</v>
-      </c>
-      <c r="C200" t="s">
-        <v>588</v>
+        <v>698</v>
+      </c>
+      <c r="C199" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="B201" t="s">
-        <v>571</v>
+        <v>518</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B202" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C202" t="s">
         <v>588</v>
@@ -8758,109 +8773,109 @@
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>294</v>
+        <v>505</v>
       </c>
       <c r="B203" t="s">
-        <v>298</v>
+        <v>571</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B204" t="s">
-        <v>562</v>
+        <v>297</v>
+      </c>
+      <c r="C204" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B205" t="s">
-        <v>248</v>
+        <v>298</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="B206" t="s">
-        <v>310</v>
+        <v>562</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B207" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B208" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B209" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>705</v>
+        <v>307</v>
       </c>
       <c r="B210" t="s">
-        <v>703</v>
+        <v>308</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>536</v>
+        <v>311</v>
       </c>
       <c r="B211" t="s">
-        <v>680</v>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3">
+      <c r="A212" t="s">
+        <v>705</v>
+      </c>
+      <c r="B212" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="B213" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="214" spans="1:3">
-      <c r="A214" t="s">
-        <v>499</v>
-      </c>
-      <c r="B214" t="s">
-        <v>320</v>
-      </c>
-      <c r="C214" t="s">
-        <v>588</v>
+        <v>680</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="B215" t="s">
-        <v>572</v>
+        <v>520</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>315</v>
+        <v>499</v>
       </c>
       <c r="B216" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C216" t="s">
         <v>588</v>
@@ -8868,128 +8883,128 @@
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>316</v>
+        <v>506</v>
       </c>
       <c r="B217" t="s">
-        <v>322</v>
+        <v>572</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B218" t="s">
-        <v>323</v>
+        <v>321</v>
+      </c>
+      <c r="C218" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B219" t="s">
-        <v>563</v>
+        <v>322</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B220" t="s">
-        <v>248</v>
+        <v>323</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B221" t="s">
-        <v>325</v>
-      </c>
-      <c r="C221" t="s">
-        <v>588</v>
+        <v>563</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="B222" t="s">
-        <v>327</v>
+        <v>248</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B223" t="s">
-        <v>328</v>
+        <v>325</v>
+      </c>
+      <c r="C223" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B224" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B225" t="s">
-        <v>256</v>
+        <v>328</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>706</v>
+        <v>330</v>
       </c>
       <c r="B226" t="s">
-        <v>703</v>
+        <v>331</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>535</v>
+        <v>332</v>
       </c>
       <c r="B227" t="s">
-        <v>681</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3">
+      <c r="A228" t="s">
+        <v>706</v>
+      </c>
+      <c r="B228" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="B229" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3">
-      <c r="A230" t="s">
-        <v>501</v>
-      </c>
-      <c r="B230" t="s">
-        <v>338</v>
-      </c>
-      <c r="C230" t="s">
-        <v>588</v>
+        <v>681</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
       <c r="B231" t="s">
-        <v>573</v>
+        <v>522</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>336</v>
+        <v>501</v>
       </c>
       <c r="B232" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C232" t="s">
         <v>588</v>
@@ -8997,303 +9012,303 @@
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>337</v>
+        <v>507</v>
       </c>
       <c r="B233" t="s">
-        <v>340</v>
+        <v>573</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>500</v>
+        <v>336</v>
       </c>
       <c r="B234" t="s">
-        <v>564</v>
+        <v>339</v>
+      </c>
+      <c r="C234" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="B235" t="s">
-        <v>248</v>
+        <v>340</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>345</v>
+        <v>500</v>
       </c>
       <c r="B236" t="s">
-        <v>341</v>
+        <v>564</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B237" t="s">
-        <v>342</v>
+        <v>248</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B238" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B239" t="s">
-        <v>256</v>
+        <v>342</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>707</v>
+        <v>347</v>
       </c>
       <c r="B240" t="s">
-        <v>703</v>
+        <v>343</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>534</v>
+        <v>348</v>
       </c>
       <c r="B241" t="s">
-        <v>682</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3">
+      <c r="A242" t="s">
+        <v>707</v>
+      </c>
+      <c r="B242" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>745</v>
+        <v>534</v>
       </c>
       <c r="B243" t="s">
-        <v>746</v>
-      </c>
-      <c r="C243" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="244" spans="1:3">
-      <c r="A244" t="s">
-        <v>551</v>
-      </c>
-      <c r="B244" t="s">
-        <v>554</v>
-      </c>
-      <c r="C244" t="s">
-        <v>586</v>
+        <v>682</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>552</v>
+        <v>745</v>
       </c>
       <c r="B245" t="s">
-        <v>553</v>
+        <v>746</v>
       </c>
       <c r="C245" t="s">
-        <v>587</v>
+        <v>692</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>585</v>
+        <v>551</v>
       </c>
       <c r="B246" t="s">
-        <v>601</v>
+        <v>554</v>
+      </c>
+      <c r="C246" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>365</v>
+        <v>552</v>
       </c>
       <c r="B247" t="s">
-        <v>351</v>
+        <v>553</v>
+      </c>
+      <c r="C247" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>366</v>
+        <v>585</v>
       </c>
       <c r="B248" t="s">
-        <v>352</v>
-      </c>
-      <c r="C248" t="s">
-        <v>588</v>
+        <v>601</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>508</v>
+        <v>365</v>
       </c>
       <c r="B249" t="s">
-        <v>574</v>
+        <v>351</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B250" t="s">
-        <v>353</v>
+        <v>352</v>
+      </c>
+      <c r="C250" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>368</v>
+        <v>508</v>
       </c>
       <c r="B251" t="s">
-        <v>354</v>
+        <v>574</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B252" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B253" t="s">
-        <v>356</v>
-      </c>
-      <c r="C253" t="s">
-        <v>588</v>
+        <v>354</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B254" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B255" t="s">
-        <v>358</v>
+        <v>356</v>
+      </c>
+      <c r="C255" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B256" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B257" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B258" t="s">
-        <v>361</v>
-      </c>
-      <c r="C258" t="s">
-        <v>588</v>
+        <v>359</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B259" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B260" t="s">
-        <v>363</v>
+        <v>361</v>
+      </c>
+      <c r="C260" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B261" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>533</v>
+        <v>377</v>
       </c>
       <c r="B262" t="s">
-        <v>666</v>
+        <v>363</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3">
+      <c r="A263" t="s">
+        <v>378</v>
+      </c>
+      <c r="B263" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>606</v>
+        <v>533</v>
       </c>
       <c r="B264" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="265" spans="1:3">
-      <c r="A265" t="s">
-        <v>385</v>
-      </c>
-      <c r="B265" t="s">
-        <v>403</v>
+        <v>666</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>386</v>
+        <v>606</v>
       </c>
       <c r="B266" t="s">
-        <v>400</v>
+        <v>607</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B267" t="s">
-        <v>401</v>
-      </c>
-      <c r="C267" t="s">
-        <v>588</v>
+        <v>403</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>509</v>
+        <v>386</v>
       </c>
       <c r="B268" t="s">
-        <v>575</v>
+        <v>400</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>404</v>
+        <v>387</v>
       </c>
       <c r="B269" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C269" t="s">
         <v>588</v>
@@ -9301,134 +9316,134 @@
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>388</v>
+        <v>509</v>
       </c>
       <c r="B270" t="s">
-        <v>394</v>
+        <v>575</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B271" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C271" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B272" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="B273" t="s">
-        <v>397</v>
+        <v>395</v>
+      </c>
+      <c r="C273" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B274" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B275" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B276" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>532</v>
+        <v>392</v>
       </c>
       <c r="B277" t="s">
-        <v>683</v>
+        <v>399</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3">
+      <c r="A278" t="s">
+        <v>393</v>
+      </c>
+      <c r="B278" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>747</v>
+        <v>532</v>
       </c>
       <c r="B279" t="s">
-        <v>766</v>
-      </c>
-      <c r="C279" t="s">
-        <v>692</v>
+        <v>683</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B281" t="s">
-        <v>744</v>
+        <v>766</v>
       </c>
       <c r="C281" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
-      <c r="A282" t="s">
-        <v>523</v>
-      </c>
-      <c r="B282" t="s">
-        <v>524</v>
-      </c>
-    </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>411</v>
+        <v>743</v>
       </c>
       <c r="B283" t="s">
-        <v>422</v>
+        <v>744</v>
+      </c>
+      <c r="C283" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>412</v>
+        <v>523</v>
       </c>
       <c r="B284" t="s">
-        <v>423</v>
-      </c>
-      <c r="C284" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>576</v>
+        <v>411</v>
       </c>
       <c r="B285" t="s">
-        <v>577</v>
+        <v>422</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B286" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C286" t="s">
         <v>588</v>
@@ -9436,128 +9451,128 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>414</v>
+        <v>576</v>
       </c>
       <c r="B287" t="s">
-        <v>425</v>
-      </c>
-      <c r="C287" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B288" t="s">
-        <v>589</v>
+        <v>424</v>
+      </c>
+      <c r="C288" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B289" t="s">
-        <v>426</v>
+        <v>425</v>
+      </c>
+      <c r="C289" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B290" t="s">
-        <v>427</v>
+        <v>589</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B291" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B292" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B293" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B294" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>530</v>
+        <v>420</v>
       </c>
       <c r="B295" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>615</v>
+        <v>421</v>
       </c>
       <c r="B296" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3">
+      <c r="A297" t="s">
+        <v>530</v>
+      </c>
+      <c r="B297" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>525</v>
+        <v>615</v>
       </c>
       <c r="B298" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="299" spans="1:3">
-      <c r="A299" t="s">
-        <v>438</v>
-      </c>
-      <c r="B299" t="s">
-        <v>449</v>
+        <v>616</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>439</v>
+        <v>525</v>
       </c>
       <c r="B300" t="s">
-        <v>450</v>
-      </c>
-      <c r="C300" t="s">
-        <v>588</v>
+        <v>524</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>510</v>
+        <v>438</v>
       </c>
       <c r="B301" t="s">
-        <v>578</v>
+        <v>449</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B302" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C302" t="s">
         <v>588</v>
@@ -9565,154 +9580,173 @@
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>441</v>
+        <v>510</v>
       </c>
       <c r="B303" t="s">
-        <v>452</v>
-      </c>
-      <c r="C303" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B304" t="s">
-        <v>590</v>
+        <v>451</v>
+      </c>
+      <c r="C304" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B305" t="s">
-        <v>426</v>
+        <v>452</v>
+      </c>
+      <c r="C305" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B306" t="s">
-        <v>427</v>
+        <v>590</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B307" t="s">
-        <v>453</v>
+        <v>426</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B308" t="s">
-        <v>454</v>
+        <v>427</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B309" t="s">
-        <v>430</v>
+        <v>453</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B310" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>529</v>
+        <v>447</v>
       </c>
       <c r="B311" t="s">
-        <v>684</v>
+        <v>430</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>622</v>
+        <v>448</v>
       </c>
       <c r="B312" t="s">
-        <v>616</v>
+        <v>431</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3">
+      <c r="A313" t="s">
+        <v>529</v>
+      </c>
+      <c r="B313" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>741</v>
+        <v>622</v>
       </c>
       <c r="B314" t="s">
-        <v>742</v>
-      </c>
-      <c r="C314" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="315" spans="1:3">
-      <c r="A315" t="s">
-        <v>432</v>
-      </c>
-      <c r="B315" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>433</v>
+        <v>741</v>
       </c>
       <c r="B316" t="s">
-        <v>624</v>
+        <v>742</v>
       </c>
       <c r="C316" t="s">
-        <v>588</v>
+        <v>692</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>511</v>
+        <v>432</v>
       </c>
       <c r="B317" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B318" t="s">
-        <v>651</v>
+        <v>624</v>
+      </c>
+      <c r="C318" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>435</v>
+        <v>511</v>
       </c>
       <c r="B319" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B320" t="s">
-        <v>627</v>
+        <v>651</v>
       </c>
     </row>
     <row r="321" spans="1:2">
       <c r="A321" t="s">
+        <v>435</v>
+      </c>
+      <c r="B321" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" t="s">
+        <v>436</v>
+      </c>
+      <c r="B322" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" t="s">
         <v>528</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B323" t="s">
         <v>685</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changes for 1904 - Dominium Dev board story (Matching SSNs on Member Information Documents) and 58139 from our board, but commented them out as they were not tested before today's prod release
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4330DBD4-1A88-4E08-8596-702C7B8E256A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27436A5D-783B-4852-B261-6D06762FAB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="796">
   <si>
     <t>Name</t>
   </si>
@@ -633,15 +633,9 @@
     <t>AS_MemNameNotListed</t>
   </si>
   <si>
-    <t>The household members do not match that listed on the ICW.</t>
-  </si>
-  <si>
     <t>AS_TaxRefund</t>
   </si>
   <si>
-    <t>The tax refund listed on the Application Summary and ICW do not match.</t>
-  </si>
-  <si>
     <t>SR_SSNCheck</t>
   </si>
   <si>
@@ -1524,9 +1518,6 @@
     <t>Replace_JObjectInJSON</t>
   </si>
   <si>
-    <t>Asset sources from the asset checklist do not match that listed on the ICW.</t>
-  </si>
-  <si>
     <t>Tax Refund provided does not match that listed on the ICW.</t>
   </si>
   <si>
@@ -1818,12 +1809,6 @@
     <t>Income &amp; Asset Questionnaire is missing from the application.</t>
   </si>
   <si>
-    <t>Income Sources listed on Income &amp; Asset Questionnaire does not match the ICW</t>
-  </si>
-  <si>
-    <t>Income Types listed on Income &amp; Asset Questionnaire does not match the ICW</t>
-  </si>
-  <si>
     <t>Signature is missing from the Self Certification of Non Employment.</t>
   </si>
   <si>
@@ -1932,9 +1917,6 @@
     <t>SC_AllFullTimeStudents</t>
   </si>
   <si>
-    <t>Assets Type and  value does not match that listed on the ICW.</t>
-  </si>
-  <si>
     <t>AS_CheckDateWithMoveIn</t>
   </si>
   <si>
@@ -2422,6 +2404,30 @@
   </si>
   <si>
     <t>The ICW includes multiple employments; however, Exact Day Calculator is available for only one of them.</t>
+  </si>
+  <si>
+    <t>MID_DuplicateSSNs</t>
+  </si>
+  <si>
+    <t>Member Information Documents have matching SSNs (last 4 digits) that are not all 9s.</t>
+  </si>
+  <si>
+    <t>Asset sources from the asset checklist do not match that listed on the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>Income Sources listed on Income &amp; Asset Questionnaire does not match the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>Income Types listed on Income &amp; Asset Questionnaire does not match the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>Assets Type and  value does not match that listed on the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>The household members do not match that listed on the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>The tax refund listed on the Application Summary and Income Calculation Worksheet do not match.</t>
   </si>
 </sst>
 </file>
@@ -2876,210 +2882,210 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B7" t="s">
-        <v>785</v>
+        <v>779</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B9" t="s">
         <v>210</v>
-      </c>
-      <c r="B9" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B10" t="s">
         <v>211</v>
-      </c>
-      <c r="B10" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B12" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B13" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>708</v>
+        <v>702</v>
       </c>
       <c r="B14" t="s">
-        <v>709</v>
+        <v>703</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B15" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B16" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B17" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C17" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C18" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B19" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="C19" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B20" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C20" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B21" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B22" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B23" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B24" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B25" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B26" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
+        <v>286</v>
+      </c>
+      <c r="B27" t="s">
         <v>288</v>
       </c>
-      <c r="B27" t="s">
-        <v>290</v>
-      </c>
       <c r="C27" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
+        <v>287</v>
+      </c>
+      <c r="B28" t="s">
         <v>289</v>
-      </c>
-      <c r="B28" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B29" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B30" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B31" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
@@ -3092,85 +3098,85 @@
     </row>
     <row r="33" spans="1:4" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B33" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B34" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B35" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B36" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B37" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B38" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B39" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B40" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B41" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B42" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D42" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="14.25" customHeight="1"/>
@@ -4152,242 +4158,242 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B1" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="B3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B5" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B6" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B7" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B8" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B9" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B11" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B12" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B13" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B14" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B15" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B16" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B17" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B18" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B19" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B20" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B21" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B22" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B23" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B24" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B25" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B26" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B27" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B28" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B29" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B30" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4395,87 +4401,87 @@
         <v>1040</v>
       </c>
       <c r="B31" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B32" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B33" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B34" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B35" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B36" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B37" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B38" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B39" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B40" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B41" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -4675,10 +4681,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>784</v>
+        <v>778</v>
       </c>
       <c r="B20" t="s">
-        <v>784</v>
+        <v>778</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -4686,23 +4692,23 @@
         <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="B22" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="B23" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5861,90 +5867,90 @@
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="B12" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="B13" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="B14" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="B15" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="B16" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="B17" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="B18" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="B19" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="B20" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="B21" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
@@ -5957,162 +5963,162 @@
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B24" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B27" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B28" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B29" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B30" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B32" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="B33" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="B34" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="B35" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="B36" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
       <c r="B37" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>776</v>
+        <v>770</v>
       </c>
       <c r="B38" t="s">
-        <v>776</v>
+        <v>770</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
       <c r="B39" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>730</v>
+        <v>724</v>
       </c>
       <c r="B40" t="s">
-        <v>730</v>
+        <v>724</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="B41" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>783</v>
+        <v>777</v>
       </c>
       <c r="B42" t="s">
-        <v>783</v>
+        <v>777</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7093,7 +7099,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C323"/>
+  <dimension ref="A1:C324"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7119,68 +7125,68 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="B5" t="s">
-        <v>767</v>
+        <v>761</v>
       </c>
       <c r="C5" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="B6" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="C6" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
       <c r="B7" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
       <c r="C7" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="B8" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="C8" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>772</v>
+        <v>766</v>
       </c>
       <c r="B9" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="C9" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="B10" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="C10" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -7188,7 +7194,7 @@
         <v>180</v>
       </c>
       <c r="B12" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7217,81 +7223,81 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B16" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C16" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="B17" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="B18" t="s">
-        <v>688</v>
+        <v>682</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="B19" t="s">
-        <v>667</v>
+        <v>661</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>700</v>
+        <v>694</v>
       </c>
       <c r="B20" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="C20" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="B21" t="s">
-        <v>716</v>
+        <v>710</v>
       </c>
       <c r="C21" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>728</v>
+        <v>722</v>
       </c>
       <c r="B22" t="s">
-        <v>729</v>
+        <v>723</v>
       </c>
       <c r="C22" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>731</v>
+        <v>725</v>
       </c>
       <c r="B23" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="C23" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -7312,10 +7318,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="B27" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -7339,15 +7345,15 @@
         <v>196</v>
       </c>
       <c r="B30" t="s">
-        <v>197</v>
+        <v>794</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B31" t="s">
-        <v>199</v>
+        <v>795</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -7384,37 +7390,37 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>631</v>
+        <v>625</v>
       </c>
       <c r="B36" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="B37" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="B38" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>717</v>
+        <v>711</v>
       </c>
       <c r="B39" t="s">
-        <v>718</v>
+        <v>712</v>
       </c>
       <c r="C39" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -7481,7 +7487,7 @@
         <v>99</v>
       </c>
       <c r="C48" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -7494,1337 +7500,1337 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="B50" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="B51" t="s">
-        <v>669</v>
+        <v>663</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>693</v>
+        <v>788</v>
       </c>
       <c r="B52" t="s">
-        <v>694</v>
-      </c>
-      <c r="C52" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" t="s">
-        <v>184</v>
-      </c>
-      <c r="B54" t="s">
-        <v>591</v>
+        <v>789</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>687</v>
+      </c>
+      <c r="B53" t="s">
+        <v>688</v>
+      </c>
+      <c r="C53" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>184</v>
       </c>
       <c r="B55" t="s">
-        <v>108</v>
-      </c>
-      <c r="C55" t="s">
         <v>588</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B56" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C56" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B57" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C57" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B58" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C58" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C59" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B60" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C60" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B61" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="C61" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>494</v>
+        <v>112</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B63" t="s">
-        <v>592</v>
-      </c>
-      <c r="C63" t="s">
-        <v>588</v>
+        <v>790</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>579</v>
+        <v>203</v>
       </c>
       <c r="B64" t="s">
-        <v>593</v>
+        <v>791</v>
+      </c>
+      <c r="C64" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>547</v>
+        <v>576</v>
       </c>
       <c r="B65" t="s">
-        <v>548</v>
+        <v>792</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>555</v>
+        <v>544</v>
       </c>
       <c r="B66" t="s">
-        <v>630</v>
+        <v>545</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
       <c r="B67" t="s">
-        <v>670</v>
+        <v>793</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>749</v>
+        <v>541</v>
       </c>
       <c r="B68" t="s">
-        <v>748</v>
-      </c>
-      <c r="C68" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" t="s">
-        <v>158</v>
-      </c>
-      <c r="B70" t="s">
-        <v>121</v>
+        <v>664</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>743</v>
+      </c>
+      <c r="B69" t="s">
+        <v>742</v>
+      </c>
+      <c r="C69" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>122</v>
+        <v>158</v>
       </c>
       <c r="B71" t="s">
-        <v>594</v>
+        <v>121</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B72" t="s">
-        <v>123</v>
+        <v>589</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>635</v>
+        <v>124</v>
       </c>
       <c r="B73" t="s">
-        <v>636</v>
+        <v>123</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>759</v>
+        <v>629</v>
       </c>
       <c r="B74" t="s">
-        <v>760</v>
-      </c>
-      <c r="C74" t="s">
-        <v>692</v>
+        <v>630</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>779</v>
+        <v>753</v>
       </c>
       <c r="B75" t="s">
-        <v>780</v>
+        <v>754</v>
       </c>
       <c r="C75" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="B76" t="s">
-        <v>781</v>
+        <v>774</v>
       </c>
       <c r="C76" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="B77" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="C77" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>543</v>
+        <v>771</v>
       </c>
       <c r="B78" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3">
-      <c r="A80" t="s">
-        <v>186</v>
-      </c>
-      <c r="B80" t="s">
-        <v>187</v>
+        <v>776</v>
+      </c>
+      <c r="C78" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>540</v>
+      </c>
+      <c r="B79" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>758</v>
+        <v>186</v>
       </c>
       <c r="B81" t="s">
-        <v>773</v>
-      </c>
-      <c r="C81" t="s">
-        <v>692</v>
+        <v>187</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="B82" t="s">
-        <v>757</v>
+        <v>767</v>
       </c>
       <c r="C82" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>125</v>
+        <v>750</v>
       </c>
       <c r="B83" t="s">
-        <v>127</v>
+        <v>751</v>
+      </c>
+      <c r="C83" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B84" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B85" t="s">
-        <v>595</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B86" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B87" t="s">
-        <v>597</v>
+        <v>591</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B88" t="s">
-        <v>598</v>
+        <v>592</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B89" t="s">
-        <v>495</v>
-      </c>
-      <c r="C89" t="s">
-        <v>686</v>
+        <v>593</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B90" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="C90" t="s">
-        <v>556</v>
+        <v>680</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B91" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="C91" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>637</v>
+        <v>144</v>
       </c>
       <c r="B92" t="s">
-        <v>638</v>
+        <v>495</v>
+      </c>
+      <c r="C92" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>719</v>
+        <v>631</v>
       </c>
       <c r="B93" t="s">
-        <v>720</v>
-      </c>
-      <c r="C93" t="s">
-        <v>692</v>
+        <v>632</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>750</v>
+        <v>713</v>
       </c>
       <c r="B94" t="s">
-        <v>751</v>
+        <v>714</v>
       </c>
       <c r="C94" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>753</v>
+        <v>744</v>
       </c>
       <c r="B95" t="s">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="C95" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>755</v>
+        <v>747</v>
       </c>
       <c r="B96" t="s">
-        <v>754</v>
+        <v>746</v>
       </c>
       <c r="C96" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>542</v>
+        <v>749</v>
       </c>
       <c r="B97" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99" t="s">
-        <v>147</v>
-      </c>
-      <c r="B99" t="s">
-        <v>150</v>
+        <v>748</v>
+      </c>
+      <c r="C97" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" t="s">
+        <v>539</v>
+      </c>
+      <c r="B98" t="s">
+        <v>666</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B100" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B101" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B102" t="s">
-        <v>580</v>
-      </c>
-      <c r="C102" t="s">
-        <v>691</v>
+        <v>152</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>690</v>
+        <v>145</v>
       </c>
       <c r="B103" t="s">
-        <v>580</v>
+        <v>577</v>
+      </c>
+      <c r="C103" t="s">
+        <v>685</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>146</v>
+        <v>684</v>
       </c>
       <c r="B104" t="s">
-        <v>129</v>
+        <v>577</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="B105" t="s">
-        <v>599</v>
+        <v>129</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B106" t="s">
-        <v>130</v>
+        <v>594</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>639</v>
+        <v>132</v>
       </c>
       <c r="B107" t="s">
-        <v>640</v>
+        <v>130</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>541</v>
+        <v>633</v>
       </c>
       <c r="B108" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3">
-      <c r="A110" t="s">
-        <v>188</v>
-      </c>
-      <c r="B110" t="s">
-        <v>189</v>
+        <v>634</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" t="s">
+        <v>538</v>
+      </c>
+      <c r="B109" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="B111" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B112" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B113" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B114" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B115" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>629</v>
+        <v>137</v>
       </c>
       <c r="B116" t="s">
-        <v>695</v>
-      </c>
-      <c r="C116" t="s">
-        <v>699</v>
+        <v>157</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>641</v>
+        <v>624</v>
       </c>
       <c r="B117" t="s">
-        <v>642</v>
+        <v>689</v>
+      </c>
+      <c r="C117" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>540</v>
+        <v>635</v>
       </c>
       <c r="B118" t="s">
-        <v>674</v>
+        <v>636</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>721</v>
+        <v>537</v>
       </c>
       <c r="B119" t="s">
-        <v>722</v>
-      </c>
-      <c r="C119" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3">
-      <c r="A121" t="s">
-        <v>710</v>
-      </c>
-      <c r="B121" t="s">
-        <v>711</v>
-      </c>
-      <c r="C121" t="s">
-        <v>712</v>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3">
+      <c r="A120" t="s">
+        <v>715</v>
+      </c>
+      <c r="B120" t="s">
+        <v>716</v>
+      </c>
+      <c r="C120" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>713</v>
+        <v>704</v>
       </c>
       <c r="B122" t="s">
-        <v>714</v>
+        <v>705</v>
       </c>
       <c r="C122" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3">
-      <c r="A124" t="s">
-        <v>159</v>
-      </c>
-      <c r="B124" t="s">
-        <v>163</v>
+        <v>706</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" t="s">
+        <v>707</v>
+      </c>
+      <c r="B123" t="s">
+        <v>708</v>
+      </c>
+      <c r="C123" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B125" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B126" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B127" t="s">
-        <v>600</v>
+        <v>165</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>557</v>
+        <v>162</v>
       </c>
       <c r="B128" t="s">
-        <v>738</v>
-      </c>
-      <c r="C128" t="s">
-        <v>739</v>
+        <v>595</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>647</v>
+        <v>554</v>
       </c>
       <c r="B129" t="s">
-        <v>648</v>
+        <v>732</v>
+      </c>
+      <c r="C129" t="s">
+        <v>733</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>539</v>
+        <v>641</v>
       </c>
       <c r="B130" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" t="s">
-        <v>192</v>
-      </c>
-      <c r="B132" t="s">
-        <v>193</v>
+        <v>642</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
+        <v>536</v>
+      </c>
+      <c r="B131" t="s">
+        <v>669</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="B133" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B134" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>643</v>
+        <v>167</v>
       </c>
       <c r="B135" t="s">
-        <v>644</v>
+        <v>169</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>538</v>
+        <v>637</v>
       </c>
       <c r="B136" t="s">
-        <v>676</v>
+        <v>638</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>723</v>
+        <v>535</v>
       </c>
       <c r="B137" t="s">
-        <v>724</v>
-      </c>
-      <c r="C137" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3">
-      <c r="A139" t="s">
-        <v>190</v>
-      </c>
-      <c r="B139" t="s">
-        <v>191</v>
+        <v>670</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" t="s">
+        <v>717</v>
+      </c>
+      <c r="B138" t="s">
+        <v>718</v>
+      </c>
+      <c r="C138" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B140" t="s">
-        <v>172</v>
-      </c>
-      <c r="C140" t="s">
-        <v>588</v>
+        <v>191</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B141" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C141" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B142" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C142" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="B143" t="s">
-        <v>202</v>
+        <v>174</v>
+      </c>
+      <c r="C143" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
+        <v>201</v>
+      </c>
+      <c r="B144" t="s">
         <v>200</v>
-      </c>
-      <c r="B144" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="B145" t="s">
-        <v>177</v>
-      </c>
-      <c r="C145" t="s">
-        <v>588</v>
+        <v>199</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>645</v>
+        <v>176</v>
       </c>
       <c r="B146" t="s">
-        <v>646</v>
+        <v>177</v>
+      </c>
+      <c r="C146" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>527</v>
+        <v>639</v>
       </c>
       <c r="B147" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3">
-      <c r="A149" t="s">
-        <v>652</v>
-      </c>
-      <c r="B149" t="s">
-        <v>653</v>
-      </c>
-      <c r="C149" t="s">
-        <v>654</v>
+        <v>640</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3">
+      <c r="A148" t="s">
+        <v>524</v>
+      </c>
+      <c r="B148" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>726</v>
+        <v>646</v>
       </c>
       <c r="B150" t="s">
-        <v>727</v>
+        <v>647</v>
       </c>
       <c r="C150" t="s">
-        <v>692</v>
+        <v>648</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>732</v>
+        <v>720</v>
       </c>
       <c r="B151" t="s">
-        <v>733</v>
+        <v>721</v>
       </c>
       <c r="C151" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>792</v>
+        <v>726</v>
       </c>
       <c r="B152" t="s">
-        <v>793</v>
+        <v>727</v>
       </c>
       <c r="C152" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>740</v>
+        <v>786</v>
       </c>
       <c r="B153" t="s">
-        <v>729</v>
+        <v>787</v>
       </c>
       <c r="C153" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3">
-      <c r="A155" t="s">
-        <v>513</v>
-      </c>
-      <c r="B155" t="s">
-        <v>514</v>
+        <v>686</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3">
+      <c r="A154" t="s">
+        <v>734</v>
+      </c>
+      <c r="B154" t="s">
+        <v>723</v>
+      </c>
+      <c r="C154" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>661</v>
+        <v>510</v>
       </c>
       <c r="B156" t="s">
-        <v>665</v>
-      </c>
-      <c r="C156" t="s">
-        <v>663</v>
+        <v>511</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
       <c r="B157" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
       <c r="C157" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>242</v>
+        <v>656</v>
       </c>
       <c r="B158" t="s">
-        <v>243</v>
+        <v>658</v>
       </c>
       <c r="C158" t="s">
-        <v>588</v>
+        <v>657</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B159" t="s">
-        <v>245</v>
+        <v>241</v>
+      </c>
+      <c r="C159" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="B160" t="s">
-        <v>560</v>
-      </c>
-      <c r="C160" t="s">
-        <v>650</v>
+        <v>243</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>790</v>
+        <v>256</v>
       </c>
       <c r="B161" t="s">
-        <v>791</v>
+        <v>557</v>
       </c>
       <c r="C161" t="s">
-        <v>692</v>
+        <v>644</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>247</v>
+        <v>784</v>
       </c>
       <c r="B162" t="s">
-        <v>246</v>
+        <v>785</v>
+      </c>
+      <c r="C162" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>503</v>
+        <v>245</v>
       </c>
       <c r="B163" t="s">
-        <v>512</v>
+        <v>244</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>249</v>
+        <v>500</v>
       </c>
       <c r="B164" t="s">
-        <v>248</v>
+        <v>509</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B165" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B166" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B167" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B168" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="B169" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>349</v>
+        <v>300</v>
       </c>
       <c r="B170" t="s">
-        <v>350</v>
+        <v>246</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>657</v>
+        <v>347</v>
       </c>
       <c r="B171" t="s">
-        <v>658</v>
+        <v>348</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>702</v>
+        <v>651</v>
       </c>
       <c r="B172" t="s">
-        <v>703</v>
+        <v>652</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>774</v>
+        <v>696</v>
       </c>
       <c r="B173" t="s">
-        <v>775</v>
-      </c>
-      <c r="C173" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>788</v>
+        <v>768</v>
       </c>
       <c r="B174" t="s">
-        <v>789</v>
+        <v>769</v>
       </c>
       <c r="C174" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>526</v>
+        <v>782</v>
       </c>
       <c r="B175" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3">
-      <c r="A177" t="s">
-        <v>786</v>
-      </c>
-      <c r="B177" t="s">
-        <v>787</v>
-      </c>
-      <c r="C177" t="s">
-        <v>692</v>
+        <v>783</v>
+      </c>
+      <c r="C175" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3">
+      <c r="A176" t="s">
+        <v>523</v>
+      </c>
+      <c r="B176" t="s">
+        <v>672</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>515</v>
+        <v>780</v>
       </c>
       <c r="B178" t="s">
-        <v>516</v>
+        <v>781</v>
+      </c>
+      <c r="C178" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
+        <v>512</v>
+      </c>
+      <c r="B179" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3">
+      <c r="A180" t="s">
+        <v>257</v>
+      </c>
+      <c r="B180" t="s">
+        <v>260</v>
+      </c>
+      <c r="C180" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A181" t="s">
         <v>259</v>
       </c>
-      <c r="B179" t="s">
-        <v>262</v>
-      </c>
-      <c r="C179" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A180" t="s">
-        <v>261</v>
-      </c>
-      <c r="B180" t="s">
-        <v>561</v>
-      </c>
-      <c r="C180" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3">
-      <c r="A181" t="s">
-        <v>260</v>
-      </c>
       <c r="B181" t="s">
-        <v>263</v>
+        <v>558</v>
+      </c>
+      <c r="C181" t="s">
+        <v>690</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="B182" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B183" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B184" t="s">
-        <v>268</v>
-      </c>
-      <c r="C184" t="s">
-        <v>660</v>
+        <v>265</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>504</v>
+        <v>267</v>
       </c>
       <c r="B185" t="s">
-        <v>570</v>
+        <v>266</v>
+      </c>
+      <c r="C185" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>270</v>
+        <v>501</v>
       </c>
       <c r="B186" t="s">
-        <v>271</v>
+        <v>567</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B187" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B188" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B189" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B190" t="s">
-        <v>285</v>
-      </c>
-      <c r="C190" t="s">
-        <v>660</v>
+        <v>284</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B191" t="s">
-        <v>605</v>
+        <v>283</v>
+      </c>
+      <c r="C191" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B192" t="s">
-        <v>284</v>
-      </c>
-      <c r="C192" t="s">
-        <v>660</v>
+        <v>600</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
+        <v>279</v>
+      </c>
+      <c r="B193" t="s">
         <v>282</v>
       </c>
-      <c r="B193" t="s">
-        <v>283</v>
+      <c r="C193" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="B194" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B195" t="s">
-        <v>248</v>
+        <v>298</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B196" t="s">
-        <v>305</v>
+        <v>246</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>704</v>
+        <v>302</v>
       </c>
       <c r="B197" t="s">
-        <v>703</v>
+        <v>303</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>537</v>
+        <v>698</v>
       </c>
       <c r="B198" t="s">
-        <v>679</v>
+        <v>697</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>697</v>
+        <v>534</v>
       </c>
       <c r="B199" t="s">
-        <v>698</v>
-      </c>
-      <c r="C199" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3">
+      <c r="A200" t="s">
+        <v>691</v>
+      </c>
+      <c r="B200" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="201" spans="1:3">
-      <c r="A201" t="s">
-        <v>517</v>
-      </c>
-      <c r="B201" t="s">
-        <v>518</v>
+      <c r="C200" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>292</v>
+        <v>514</v>
       </c>
       <c r="B202" t="s">
-        <v>296</v>
-      </c>
-      <c r="C202" t="s">
-        <v>588</v>
+        <v>515</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>505</v>
+        <v>290</v>
       </c>
       <c r="B203" t="s">
-        <v>571</v>
+        <v>294</v>
+      </c>
+      <c r="C203" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>293</v>
+        <v>502</v>
       </c>
       <c r="B204" t="s">
-        <v>297</v>
-      </c>
-      <c r="C204" t="s">
-        <v>588</v>
+        <v>568</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B205" t="s">
-        <v>298</v>
+        <v>295</v>
+      </c>
+      <c r="C205" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B206" t="s">
-        <v>562</v>
+        <v>296</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B207" t="s">
-        <v>248</v>
+        <v>559</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="B208" t="s">
-        <v>310</v>
+        <v>246</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B209" t="s">
         <v>308</v>
@@ -8832,922 +8838,930 @@
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B210" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="B211" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>705</v>
+        <v>309</v>
       </c>
       <c r="B212" t="s">
-        <v>703</v>
+        <v>310</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>536</v>
+        <v>699</v>
       </c>
       <c r="B213" t="s">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3">
-      <c r="A215" t="s">
-        <v>519</v>
-      </c>
-      <c r="B215" t="s">
-        <v>520</v>
+        <v>697</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3">
+      <c r="A214" t="s">
+        <v>533</v>
+      </c>
+      <c r="B214" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>499</v>
+        <v>516</v>
       </c>
       <c r="B216" t="s">
-        <v>320</v>
-      </c>
-      <c r="C216" t="s">
-        <v>588</v>
+        <v>517</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>506</v>
+        <v>496</v>
       </c>
       <c r="B217" t="s">
-        <v>572</v>
+        <v>318</v>
+      </c>
+      <c r="C217" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>315</v>
+        <v>503</v>
       </c>
       <c r="B218" t="s">
-        <v>321</v>
-      </c>
-      <c r="C218" t="s">
-        <v>588</v>
+        <v>569</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B219" t="s">
-        <v>322</v>
+        <v>319</v>
+      </c>
+      <c r="C219" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B220" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B221" t="s">
-        <v>563</v>
+        <v>321</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B222" t="s">
-        <v>248</v>
+        <v>560</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="B223" t="s">
-        <v>325</v>
-      </c>
-      <c r="C223" t="s">
-        <v>588</v>
+        <v>246</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B224" t="s">
-        <v>327</v>
+        <v>323</v>
+      </c>
+      <c r="C224" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B225" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B226" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B227" t="s">
-        <v>256</v>
+        <v>329</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>706</v>
+        <v>330</v>
       </c>
       <c r="B228" t="s">
-        <v>703</v>
+        <v>254</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>535</v>
+        <v>700</v>
       </c>
       <c r="B229" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3">
-      <c r="A231" t="s">
-        <v>521</v>
-      </c>
-      <c r="B231" t="s">
-        <v>522</v>
+        <v>697</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3">
+      <c r="A230" t="s">
+        <v>532</v>
+      </c>
+      <c r="B230" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="B232" t="s">
-        <v>338</v>
-      </c>
-      <c r="C232" t="s">
-        <v>588</v>
+        <v>519</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="B233" t="s">
-        <v>573</v>
+        <v>336</v>
+      </c>
+      <c r="C233" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>336</v>
+        <v>504</v>
       </c>
       <c r="B234" t="s">
-        <v>339</v>
-      </c>
-      <c r="C234" t="s">
-        <v>588</v>
+        <v>570</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
+        <v>334</v>
+      </c>
+      <c r="B235" t="s">
         <v>337</v>
       </c>
-      <c r="B235" t="s">
-        <v>340</v>
+      <c r="C235" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>500</v>
+        <v>335</v>
       </c>
       <c r="B236" t="s">
-        <v>564</v>
+        <v>338</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>344</v>
+        <v>497</v>
       </c>
       <c r="B237" t="s">
-        <v>248</v>
+        <v>561</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B238" t="s">
-        <v>341</v>
+        <v>246</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B239" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B240" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B241" t="s">
-        <v>256</v>
+        <v>341</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>707</v>
+        <v>346</v>
       </c>
       <c r="B242" t="s">
-        <v>703</v>
+        <v>254</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>534</v>
+        <v>701</v>
       </c>
       <c r="B243" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="245" spans="1:3">
-      <c r="A245" t="s">
-        <v>745</v>
-      </c>
-      <c r="B245" t="s">
-        <v>746</v>
-      </c>
-      <c r="C245" t="s">
-        <v>692</v>
+        <v>697</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3">
+      <c r="A244" t="s">
+        <v>531</v>
+      </c>
+      <c r="B244" t="s">
+        <v>676</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>551</v>
+        <v>739</v>
       </c>
       <c r="B246" t="s">
-        <v>554</v>
+        <v>740</v>
       </c>
       <c r="C246" t="s">
-        <v>586</v>
+        <v>686</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="B247" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C247" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>585</v>
+        <v>549</v>
       </c>
       <c r="B248" t="s">
-        <v>601</v>
+        <v>550</v>
+      </c>
+      <c r="C248" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>365</v>
+        <v>582</v>
       </c>
       <c r="B249" t="s">
-        <v>351</v>
+        <v>596</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B250" t="s">
-        <v>352</v>
-      </c>
-      <c r="C250" t="s">
-        <v>588</v>
+        <v>349</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>508</v>
+        <v>364</v>
       </c>
       <c r="B251" t="s">
-        <v>574</v>
+        <v>350</v>
+      </c>
+      <c r="C251" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>367</v>
+        <v>505</v>
       </c>
       <c r="B252" t="s">
-        <v>353</v>
+        <v>571</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B253" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B254" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B255" t="s">
-        <v>356</v>
-      </c>
-      <c r="C255" t="s">
-        <v>588</v>
+        <v>353</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B256" t="s">
-        <v>357</v>
+        <v>354</v>
+      </c>
+      <c r="C256" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B257" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B258" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B259" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B260" t="s">
-        <v>361</v>
-      </c>
-      <c r="C260" t="s">
-        <v>588</v>
+        <v>358</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B261" t="s">
-        <v>362</v>
+        <v>359</v>
+      </c>
+      <c r="C261" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B262" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B263" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>533</v>
+        <v>376</v>
       </c>
       <c r="B264" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="266" spans="1:3">
-      <c r="A266" t="s">
-        <v>606</v>
-      </c>
-      <c r="B266" t="s">
-        <v>607</v>
+        <v>362</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3">
+      <c r="A265" t="s">
+        <v>530</v>
+      </c>
+      <c r="B265" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>385</v>
+        <v>601</v>
       </c>
       <c r="B267" t="s">
-        <v>403</v>
+        <v>602</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B268" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B269" t="s">
-        <v>401</v>
-      </c>
-      <c r="C269" t="s">
-        <v>588</v>
+        <v>398</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>509</v>
+        <v>385</v>
       </c>
       <c r="B270" t="s">
-        <v>575</v>
+        <v>399</v>
+      </c>
+      <c r="C270" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>404</v>
+        <v>506</v>
       </c>
       <c r="B271" t="s">
-        <v>402</v>
-      </c>
-      <c r="C271" t="s">
-        <v>588</v>
+        <v>572</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>388</v>
+        <v>402</v>
       </c>
       <c r="B272" t="s">
-        <v>394</v>
+        <v>400</v>
+      </c>
+      <c r="C272" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>405</v>
+        <v>386</v>
       </c>
       <c r="B273" t="s">
-        <v>395</v>
-      </c>
-      <c r="C273" t="s">
-        <v>565</v>
+        <v>392</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>389</v>
+        <v>403</v>
       </c>
       <c r="B274" t="s">
-        <v>396</v>
+        <v>393</v>
+      </c>
+      <c r="C274" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B275" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B276" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="B277" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B278" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>532</v>
+        <v>391</v>
       </c>
       <c r="B279" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="281" spans="1:3">
-      <c r="A281" t="s">
-        <v>747</v>
-      </c>
-      <c r="B281" t="s">
-        <v>766</v>
-      </c>
-      <c r="C281" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="283" spans="1:3">
-      <c r="A283" t="s">
-        <v>743</v>
-      </c>
-      <c r="B283" t="s">
-        <v>744</v>
-      </c>
-      <c r="C283" t="s">
-        <v>692</v>
+        <v>394</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3">
+      <c r="A280" t="s">
+        <v>529</v>
+      </c>
+      <c r="B280" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3">
+      <c r="A282" t="s">
+        <v>741</v>
+      </c>
+      <c r="B282" t="s">
+        <v>760</v>
+      </c>
+      <c r="C282" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>523</v>
+        <v>737</v>
       </c>
       <c r="B284" t="s">
-        <v>524</v>
+        <v>738</v>
+      </c>
+      <c r="C284" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>411</v>
+        <v>520</v>
       </c>
       <c r="B285" t="s">
-        <v>422</v>
+        <v>521</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="B286" t="s">
-        <v>423</v>
-      </c>
-      <c r="C286" t="s">
-        <v>588</v>
+        <v>420</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>576</v>
+        <v>410</v>
       </c>
       <c r="B287" t="s">
-        <v>577</v>
+        <v>421</v>
+      </c>
+      <c r="C287" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>413</v>
+        <v>573</v>
       </c>
       <c r="B288" t="s">
-        <v>424</v>
-      </c>
-      <c r="C288" t="s">
-        <v>588</v>
+        <v>574</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B289" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C289" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B290" t="s">
-        <v>589</v>
+        <v>423</v>
+      </c>
+      <c r="C290" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B291" t="s">
-        <v>426</v>
+        <v>586</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B292" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B293" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B294" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B295" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="B296" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>530</v>
+        <v>419</v>
       </c>
       <c r="B297" t="s">
-        <v>684</v>
+        <v>429</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>615</v>
+        <v>527</v>
       </c>
       <c r="B298" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="300" spans="1:3">
-      <c r="A300" t="s">
-        <v>525</v>
-      </c>
-      <c r="B300" t="s">
-        <v>524</v>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3">
+      <c r="A299" t="s">
+        <v>610</v>
+      </c>
+      <c r="B299" t="s">
+        <v>611</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>438</v>
+        <v>522</v>
       </c>
       <c r="B301" t="s">
-        <v>449</v>
+        <v>521</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="B302" t="s">
-        <v>450</v>
-      </c>
-      <c r="C302" t="s">
-        <v>588</v>
+        <v>447</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>510</v>
+        <v>437</v>
       </c>
       <c r="B303" t="s">
-        <v>578</v>
+        <v>448</v>
+      </c>
+      <c r="C303" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>440</v>
+        <v>507</v>
       </c>
       <c r="B304" t="s">
-        <v>451</v>
-      </c>
-      <c r="C304" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="B305" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="C305" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B306" t="s">
-        <v>590</v>
+        <v>450</v>
+      </c>
+      <c r="C306" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B307" t="s">
-        <v>426</v>
+        <v>587</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B308" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B309" t="s">
-        <v>453</v>
+        <v>425</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B310" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="B311" t="s">
-        <v>430</v>
+        <v>452</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B312" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>529</v>
+        <v>446</v>
       </c>
       <c r="B313" t="s">
-        <v>684</v>
+        <v>429</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>622</v>
+        <v>526</v>
       </c>
       <c r="B314" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3">
-      <c r="A316" t="s">
-        <v>741</v>
-      </c>
-      <c r="B316" t="s">
-        <v>742</v>
-      </c>
-      <c r="C316" t="s">
-        <v>692</v>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3">
+      <c r="A315" t="s">
+        <v>617</v>
+      </c>
+      <c r="B315" t="s">
+        <v>611</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>432</v>
+        <v>735</v>
       </c>
       <c r="B317" t="s">
-        <v>623</v>
+        <v>736</v>
+      </c>
+      <c r="C317" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="B318" t="s">
-        <v>624</v>
-      </c>
-      <c r="C318" t="s">
-        <v>588</v>
+        <v>618</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>511</v>
+        <v>431</v>
       </c>
       <c r="B319" t="s">
-        <v>625</v>
+        <v>619</v>
+      </c>
+      <c r="C319" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>434</v>
+        <v>508</v>
       </c>
       <c r="B320" t="s">
-        <v>651</v>
+        <v>620</v>
       </c>
     </row>
     <row r="321" spans="1:2">
       <c r="A321" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="B321" t="s">
-        <v>626</v>
+        <v>645</v>
       </c>
     </row>
     <row r="322" spans="1:2">
       <c r="A322" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="B322" t="s">
-        <v>627</v>
+        <v>621</v>
       </c>
     </row>
     <row r="323" spans="1:2">
       <c r="A323" t="s">
-        <v>528</v>
+        <v>434</v>
       </c>
       <c r="B323" t="s">
-        <v>685</v>
+        <v>622</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" t="s">
+        <v>525</v>
+      </c>
+      <c r="B324" t="s">
+        <v>679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the verbiage finding for 58139
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27436A5D-783B-4852-B261-6D06762FAB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8840FB17-A854-4246-B1F1-00938FA7E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28350" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2403,9 +2403,6 @@
     <t>EDC_Missing</t>
   </si>
   <si>
-    <t>The ICW includes multiple employments; however, Exact Day Calculator is available for only one of them.</t>
-  </si>
-  <si>
     <t>MID_DuplicateSSNs</t>
   </si>
   <si>
@@ -2428,6 +2425,9 @@
   </si>
   <si>
     <t>The tax refund listed on the Application Summary and Income Calculation Worksheet do not match.</t>
+  </si>
+  <si>
+    <t>The ICW includes multiple employments; however, Exact Day Calculator is not available for all of them.</t>
   </si>
 </sst>
 </file>
@@ -7345,7 +7345,7 @@
         <v>196</v>
       </c>
       <c r="B30" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -7353,7 +7353,7 @@
         <v>197</v>
       </c>
       <c r="B31" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -7516,10 +7516,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>787</v>
+      </c>
+      <c r="B52" t="s">
         <v>788</v>
-      </c>
-      <c r="B52" t="s">
-        <v>789</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -7620,7 +7620,7 @@
         <v>202</v>
       </c>
       <c r="B63" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -7628,7 +7628,7 @@
         <v>203</v>
       </c>
       <c r="B64" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C64" t="s">
         <v>585</v>
@@ -7639,7 +7639,7 @@
         <v>576</v>
       </c>
       <c r="B65" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -7655,7 +7655,7 @@
         <v>552</v>
       </c>
       <c r="B67" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -8355,7 +8355,7 @@
         <v>786</v>
       </c>
       <c r="B153" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="C153" t="s">
         <v>686</v>

</xml_diff>

<commit_message>
updated classification prompt to the lastest version
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8840FB17-A854-4246-B1F1-00938FA7E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9059C4-E889-4027-95E7-61B656ADBF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28350" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="797">
   <si>
     <t>Name</t>
   </si>
@@ -2428,6 +2428,9 @@
   </si>
   <si>
     <t>The ICW includes multiple employments; however, Exact Day Calculator is not available for all of them.</t>
+  </si>
+  <si>
+    <t>Completion Details</t>
   </si>
 </sst>
 </file>
@@ -4149,7 +4152,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80DB68E2-2057-45AB-A45E-3EB9CF844C19}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.5703125" bestFit="1" customWidth="1"/>
@@ -4481,6 +4484,14 @@
         <v>483</v>
       </c>
       <c r="B41" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>796</v>
+      </c>
+      <c r="B42" t="s">
         <v>480</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new enhancement for 1911 on Dominium Dev Board - added the HHD check for checkboxes
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90512B6F-241D-4135-A468-D1404153DF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473B82F7-70B9-4496-BC6B-3FF12C42F1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="799">
   <si>
     <t>Name</t>
   </si>
@@ -2431,6 +2431,12 @@
   </si>
   <si>
     <t>Completion Details</t>
+  </si>
+  <si>
+    <t>HHD_PropertyCheckbox</t>
+  </si>
+  <si>
+    <t>None of the "Rent", "Own", or "Other" checkboxes are selected on Housing History Disclosure for this property.</t>
   </si>
 </sst>
 </file>
@@ -7110,7 +7116,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C324"/>
+  <dimension ref="A1:C325"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7191,99 +7197,99 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>758</v>
+        <v>797</v>
       </c>
       <c r="B10" t="s">
-        <v>759</v>
+        <v>798</v>
       </c>
       <c r="C10" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>180</v>
-      </c>
-      <c r="B12" t="s">
-        <v>493</v>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>758</v>
+      </c>
+      <c r="B11" t="s">
+        <v>759</v>
+      </c>
+      <c r="C11" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>180</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>493</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>179</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>178</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>179</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>204</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>205</v>
-      </c>
-      <c r="C16" t="s">
-        <v>653</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>546</v>
+        <v>204</v>
       </c>
       <c r="B17" t="s">
-        <v>547</v>
+        <v>205</v>
+      </c>
+      <c r="C17" t="s">
+        <v>653</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>681</v>
+        <v>546</v>
       </c>
       <c r="B18" t="s">
-        <v>682</v>
+        <v>547</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>528</v>
+        <v>681</v>
       </c>
       <c r="B19" t="s">
-        <v>661</v>
+        <v>682</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>694</v>
+        <v>528</v>
       </c>
       <c r="B20" t="s">
-        <v>695</v>
-      </c>
-      <c r="C20" t="s">
-        <v>686</v>
+        <v>661</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>709</v>
+        <v>694</v>
       </c>
       <c r="B21" t="s">
-        <v>710</v>
+        <v>695</v>
       </c>
       <c r="C21" t="s">
         <v>686</v>
@@ -7291,10 +7297,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>722</v>
+        <v>709</v>
       </c>
       <c r="B22" t="s">
-        <v>723</v>
+        <v>710</v>
       </c>
       <c r="C22" t="s">
         <v>686</v>
@@ -7302,273 +7308,273 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="B23" t="s">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="C23" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>181</v>
-      </c>
-      <c r="B25" t="s">
-        <v>182</v>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>725</v>
+      </c>
+      <c r="B24" t="s">
+        <v>730</v>
+      </c>
+      <c r="C24" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>181</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>555</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
-        <v>556</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>80</v>
+        <v>555</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>556</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>196</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>793</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B31" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>197</v>
       </c>
       <c r="B32" t="s">
-        <v>85</v>
+        <v>794</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>625</v>
+        <v>89</v>
       </c>
       <c r="B36" t="s">
-        <v>626</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>649</v>
+        <v>625</v>
       </c>
       <c r="B37" t="s">
-        <v>650</v>
+        <v>626</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>543</v>
+        <v>649</v>
       </c>
       <c r="B38" t="s">
-        <v>662</v>
+        <v>650</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>543</v>
+      </c>
+      <c r="B39" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
         <v>711</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>712</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C40" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>183</v>
-      </c>
-      <c r="B41" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>183</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B45" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B47" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
-      </c>
-      <c r="C48" t="s">
-        <v>585</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>99</v>
+      </c>
+      <c r="C49" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>627</v>
+        <v>106</v>
       </c>
       <c r="B50" t="s">
-        <v>628</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>542</v>
+        <v>627</v>
       </c>
       <c r="B51" t="s">
-        <v>663</v>
+        <v>628</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>787</v>
+        <v>542</v>
       </c>
       <c r="B52" t="s">
-        <v>788</v>
+        <v>663</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>787</v>
+      </c>
+      <c r="B53" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
         <v>687</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>688</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C54" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>184</v>
-      </c>
-      <c r="B55" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>107</v>
+        <v>184</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
-      </c>
-      <c r="C56" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B57" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C57" t="s">
         <v>585</v>
@@ -7576,10 +7582,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B58" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C58" t="s">
         <v>585</v>
@@ -7587,10 +7593,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B59" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C59" t="s">
         <v>585</v>
@@ -7598,10 +7604,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C60" t="s">
         <v>585</v>
@@ -7609,10 +7615,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B61" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C61" t="s">
         <v>585</v>
@@ -7620,123 +7626,123 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="C62" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="B63" t="s">
-        <v>789</v>
+        <v>112</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B64" t="s">
-        <v>790</v>
-      </c>
-      <c r="C64" t="s">
-        <v>585</v>
+        <v>789</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>576</v>
+        <v>203</v>
       </c>
       <c r="B65" t="s">
-        <v>791</v>
+        <v>790</v>
+      </c>
+      <c r="C65" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>544</v>
+        <v>576</v>
       </c>
       <c r="B66" t="s">
-        <v>545</v>
+        <v>791</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="B67" t="s">
-        <v>792</v>
+        <v>545</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="B68" t="s">
-        <v>664</v>
+        <v>792</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>541</v>
+      </c>
+      <c r="B69" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>743</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B70" t="s">
         <v>742</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C70" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" t="s">
-        <v>158</v>
-      </c>
-      <c r="B71" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>158</v>
       </c>
       <c r="B72" t="s">
-        <v>589</v>
+        <v>121</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
-        <v>123</v>
+        <v>589</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>629</v>
+        <v>124</v>
       </c>
       <c r="B74" t="s">
-        <v>630</v>
+        <v>123</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>753</v>
+        <v>629</v>
       </c>
       <c r="B75" t="s">
-        <v>754</v>
-      </c>
-      <c r="C75" t="s">
-        <v>686</v>
+        <v>630</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>773</v>
+        <v>753</v>
       </c>
       <c r="B76" t="s">
-        <v>774</v>
+        <v>754</v>
       </c>
       <c r="C76" t="s">
         <v>686</v>
@@ -7744,10 +7750,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="B77" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C77" t="s">
         <v>686</v>
@@ -7755,10 +7761,10 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B78" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C78" t="s">
         <v>686</v>
@@ -7766,37 +7772,37 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
+        <v>771</v>
+      </c>
+      <c r="B79" t="s">
+        <v>776</v>
+      </c>
+      <c r="C79" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
         <v>540</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B80" t="s">
         <v>665</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3">
-      <c r="A81" t="s">
-        <v>186</v>
-      </c>
-      <c r="B81" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>752</v>
+        <v>186</v>
       </c>
       <c r="B82" t="s">
-        <v>767</v>
-      </c>
-      <c r="C82" t="s">
-        <v>686</v>
+        <v>187</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B83" t="s">
-        <v>751</v>
+        <v>767</v>
       </c>
       <c r="C83" t="s">
         <v>686</v>
@@ -7804,80 +7810,80 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>125</v>
+        <v>750</v>
       </c>
       <c r="B84" t="s">
-        <v>127</v>
+        <v>751</v>
+      </c>
+      <c r="C84" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B85" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B86" t="s">
-        <v>590</v>
+        <v>128</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B87" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B88" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B89" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B90" t="s">
-        <v>492</v>
-      </c>
-      <c r="C90" t="s">
-        <v>680</v>
+        <v>593</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B91" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C91" t="s">
-        <v>553</v>
+        <v>680</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B92" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C92" t="s">
         <v>553</v>
@@ -7885,29 +7891,29 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>631</v>
+        <v>144</v>
       </c>
       <c r="B93" t="s">
-        <v>632</v>
+        <v>495</v>
+      </c>
+      <c r="C93" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>713</v>
+        <v>631</v>
       </c>
       <c r="B94" t="s">
-        <v>714</v>
-      </c>
-      <c r="C94" t="s">
-        <v>686</v>
+        <v>632</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>744</v>
+        <v>713</v>
       </c>
       <c r="B95" t="s">
-        <v>745</v>
+        <v>714</v>
       </c>
       <c r="C95" t="s">
         <v>686</v>
@@ -7915,10 +7921,10 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="B96" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C96" t="s">
         <v>686</v>
@@ -7926,10 +7932,10 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B97" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C97" t="s">
         <v>686</v>
@@ -7937,338 +7943,338 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
+        <v>749</v>
+      </c>
+      <c r="B98" t="s">
+        <v>748</v>
+      </c>
+      <c r="C98" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" t="s">
         <v>539</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B99" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3">
-      <c r="A100" t="s">
-        <v>147</v>
-      </c>
-      <c r="B100" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B101" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B102" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B103" t="s">
-        <v>577</v>
-      </c>
-      <c r="C103" t="s">
-        <v>685</v>
+        <v>152</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>684</v>
+        <v>145</v>
       </c>
       <c r="B104" t="s">
         <v>577</v>
       </c>
+      <c r="C104" t="s">
+        <v>685</v>
+      </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>146</v>
+        <v>684</v>
       </c>
       <c r="B105" t="s">
-        <v>129</v>
+        <v>577</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="B106" t="s">
-        <v>594</v>
+        <v>129</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B107" t="s">
-        <v>130</v>
+        <v>594</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>633</v>
+        <v>132</v>
       </c>
       <c r="B108" t="s">
-        <v>634</v>
+        <v>130</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
+        <v>633</v>
+      </c>
+      <c r="B109" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" t="s">
         <v>538</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B110" t="s">
         <v>667</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3">
-      <c r="A111" t="s">
-        <v>188</v>
-      </c>
-      <c r="B111" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="B112" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B113" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B114" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B115" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B116" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>624</v>
+        <v>137</v>
       </c>
       <c r="B117" t="s">
-        <v>689</v>
-      </c>
-      <c r="C117" t="s">
-        <v>693</v>
+        <v>157</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>635</v>
+        <v>624</v>
       </c>
       <c r="B118" t="s">
-        <v>636</v>
+        <v>689</v>
+      </c>
+      <c r="C118" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>537</v>
+        <v>635</v>
       </c>
       <c r="B119" t="s">
-        <v>668</v>
+        <v>636</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
+        <v>537</v>
+      </c>
+      <c r="B120" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" t="s">
         <v>715</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B121" t="s">
         <v>716</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C121" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3">
-      <c r="A122" t="s">
-        <v>704</v>
-      </c>
-      <c r="B122" t="s">
-        <v>705</v>
-      </c>
-      <c r="C122" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B123" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C123" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
-      <c r="A125" t="s">
-        <v>159</v>
-      </c>
-      <c r="B125" t="s">
-        <v>163</v>
+    <row r="124" spans="1:3">
+      <c r="A124" t="s">
+        <v>707</v>
+      </c>
+      <c r="B124" t="s">
+        <v>708</v>
+      </c>
+      <c r="C124" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B126" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B127" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B128" t="s">
-        <v>595</v>
+        <v>165</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>554</v>
+        <v>162</v>
       </c>
       <c r="B129" t="s">
-        <v>732</v>
-      </c>
-      <c r="C129" t="s">
-        <v>733</v>
+        <v>595</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>641</v>
+        <v>554</v>
       </c>
       <c r="B130" t="s">
-        <v>642</v>
+        <v>732</v>
+      </c>
+      <c r="C130" t="s">
+        <v>733</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
+        <v>641</v>
+      </c>
+      <c r="B131" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3">
+      <c r="A132" t="s">
         <v>536</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B132" t="s">
         <v>669</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" t="s">
-        <v>192</v>
-      </c>
-      <c r="B133" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="B134" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B135" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>637</v>
+        <v>167</v>
       </c>
       <c r="B136" t="s">
-        <v>638</v>
+        <v>169</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>535</v>
+        <v>637</v>
       </c>
       <c r="B137" t="s">
-        <v>670</v>
+        <v>638</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
+        <v>535</v>
+      </c>
+      <c r="B138" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3">
+      <c r="A139" t="s">
         <v>717</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B139" t="s">
         <v>718</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C139" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3">
-      <c r="A140" t="s">
-        <v>190</v>
-      </c>
-      <c r="B140" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B141" t="s">
-        <v>172</v>
-      </c>
-      <c r="C141" t="s">
-        <v>585</v>
+        <v>191</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B142" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C142" t="s">
         <v>585</v>
@@ -8276,10 +8282,10 @@
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B143" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C143" t="s">
         <v>585</v>
@@ -8287,75 +8293,75 @@
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>201</v>
+        <v>171</v>
       </c>
       <c r="B144" t="s">
-        <v>200</v>
+        <v>174</v>
+      </c>
+      <c r="C144" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B145" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="B146" t="s">
-        <v>177</v>
-      </c>
-      <c r="C146" t="s">
-        <v>585</v>
+        <v>199</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>639</v>
+        <v>176</v>
       </c>
       <c r="B147" t="s">
-        <v>640</v>
+        <v>177</v>
+      </c>
+      <c r="C147" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
+        <v>639</v>
+      </c>
+      <c r="B148" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
         <v>524</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B149" t="s">
         <v>671</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3">
-      <c r="A150" t="s">
-        <v>646</v>
-      </c>
-      <c r="B150" t="s">
-        <v>647</v>
-      </c>
-      <c r="C150" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>720</v>
+        <v>646</v>
       </c>
       <c r="B151" t="s">
-        <v>721</v>
+        <v>647</v>
       </c>
       <c r="C151" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="B152" t="s">
-        <v>727</v>
+        <v>721</v>
       </c>
       <c r="C152" t="s">
         <v>686</v>
@@ -8363,10 +8369,10 @@
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>786</v>
+        <v>726</v>
       </c>
       <c r="B153" t="s">
-        <v>795</v>
+        <v>727</v>
       </c>
       <c r="C153" t="s">
         <v>686</v>
@@ -8374,40 +8380,40 @@
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>734</v>
+        <v>786</v>
       </c>
       <c r="B154" t="s">
-        <v>723</v>
+        <v>795</v>
       </c>
       <c r="C154" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="156" spans="1:3">
-      <c r="A156" t="s">
-        <v>510</v>
-      </c>
-      <c r="B156" t="s">
-        <v>511</v>
+    <row r="155" spans="1:3">
+      <c r="A155" t="s">
+        <v>734</v>
+      </c>
+      <c r="B155" t="s">
+        <v>723</v>
+      </c>
+      <c r="C155" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>655</v>
+        <v>510</v>
       </c>
       <c r="B157" t="s">
-        <v>659</v>
-      </c>
-      <c r="C157" t="s">
-        <v>657</v>
+        <v>511</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B158" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C158" t="s">
         <v>657</v>
@@ -8415,150 +8421,150 @@
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>240</v>
+        <v>656</v>
       </c>
       <c r="B159" t="s">
-        <v>241</v>
+        <v>658</v>
       </c>
       <c r="C159" t="s">
-        <v>585</v>
+        <v>657</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B160" t="s">
-        <v>243</v>
+        <v>241</v>
+      </c>
+      <c r="C160" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="B161" t="s">
-        <v>557</v>
-      </c>
-      <c r="C161" t="s">
-        <v>644</v>
+        <v>243</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>784</v>
+        <v>256</v>
       </c>
       <c r="B162" t="s">
-        <v>785</v>
+        <v>557</v>
       </c>
       <c r="C162" t="s">
-        <v>686</v>
+        <v>644</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>245</v>
+        <v>784</v>
       </c>
       <c r="B163" t="s">
-        <v>244</v>
+        <v>785</v>
+      </c>
+      <c r="C163" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>500</v>
+        <v>245</v>
       </c>
       <c r="B164" t="s">
-        <v>509</v>
+        <v>244</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>247</v>
+        <v>500</v>
       </c>
       <c r="B165" t="s">
-        <v>246</v>
+        <v>509</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B166" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B167" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B168" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B169" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>300</v>
+        <v>255</v>
       </c>
       <c r="B170" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>347</v>
+        <v>300</v>
       </c>
       <c r="B171" t="s">
-        <v>348</v>
+        <v>246</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>651</v>
+        <v>347</v>
       </c>
       <c r="B172" t="s">
-        <v>652</v>
+        <v>348</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>696</v>
+        <v>651</v>
       </c>
       <c r="B173" t="s">
-        <v>697</v>
+        <v>652</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>768</v>
+        <v>696</v>
       </c>
       <c r="B174" t="s">
-        <v>769</v>
-      </c>
-      <c r="C174" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>782</v>
+        <v>768</v>
       </c>
       <c r="B175" t="s">
-        <v>783</v>
+        <v>769</v>
       </c>
       <c r="C175" t="s">
         <v>686</v>
@@ -8566,298 +8572,301 @@
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
+        <v>782</v>
+      </c>
+      <c r="B176" t="s">
+        <v>783</v>
+      </c>
+      <c r="C176" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3">
+      <c r="A177" t="s">
         <v>523</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>672</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3">
-      <c r="A178" t="s">
-        <v>780</v>
-      </c>
-      <c r="B178" t="s">
-        <v>781</v>
-      </c>
-      <c r="C178" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>512</v>
+        <v>780</v>
       </c>
       <c r="B179" t="s">
-        <v>513</v>
+        <v>781</v>
+      </c>
+      <c r="C179" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
+        <v>512</v>
+      </c>
+      <c r="B180" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3">
+      <c r="A181" t="s">
         <v>257</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B181" t="s">
         <v>260</v>
       </c>
-      <c r="C180" t="s">
+      <c r="C181" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A181" t="s">
+    <row r="182" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A182" t="s">
         <v>259</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B182" t="s">
         <v>558</v>
       </c>
-      <c r="C181" t="s">
+      <c r="C182" t="s">
         <v>690</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3">
-      <c r="A182" t="s">
-        <v>258</v>
-      </c>
-      <c r="B182" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B183" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B184" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B185" t="s">
-        <v>266</v>
-      </c>
-      <c r="C185" t="s">
-        <v>654</v>
+        <v>265</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>501</v>
+        <v>267</v>
       </c>
       <c r="B186" t="s">
-        <v>567</v>
+        <v>266</v>
+      </c>
+      <c r="C186" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>268</v>
+        <v>501</v>
       </c>
       <c r="B187" t="s">
-        <v>269</v>
+        <v>567</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B188" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B189" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B190" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B191" t="s">
-        <v>283</v>
-      </c>
-      <c r="C191" t="s">
-        <v>654</v>
+        <v>284</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B192" t="s">
-        <v>600</v>
+        <v>283</v>
+      </c>
+      <c r="C192" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B193" t="s">
-        <v>282</v>
-      </c>
-      <c r="C193" t="s">
-        <v>654</v>
+        <v>600</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B194" t="s">
-        <v>281</v>
+        <v>282</v>
+      </c>
+      <c r="C194" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
       <c r="B195" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B196" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B197" t="s">
-        <v>303</v>
+        <v>246</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>698</v>
+        <v>302</v>
       </c>
       <c r="B198" t="s">
-        <v>697</v>
+        <v>303</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>534</v>
+        <v>698</v>
       </c>
       <c r="B199" t="s">
-        <v>673</v>
+        <v>697</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
+        <v>534</v>
+      </c>
+      <c r="B200" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3">
+      <c r="A201" t="s">
         <v>691</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B201" t="s">
         <v>692</v>
       </c>
-      <c r="C200" t="s">
+      <c r="C201" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="202" spans="1:3">
-      <c r="A202" t="s">
-        <v>514</v>
-      </c>
-      <c r="B202" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>290</v>
+        <v>514</v>
       </c>
       <c r="B203" t="s">
-        <v>294</v>
-      </c>
-      <c r="C203" t="s">
-        <v>585</v>
+        <v>515</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>502</v>
+        <v>290</v>
       </c>
       <c r="B204" t="s">
-        <v>568</v>
+        <v>294</v>
+      </c>
+      <c r="C204" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>291</v>
+        <v>502</v>
       </c>
       <c r="B205" t="s">
-        <v>295</v>
-      </c>
-      <c r="C205" t="s">
-        <v>585</v>
+        <v>568</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B206" t="s">
-        <v>296</v>
+        <v>295</v>
+      </c>
+      <c r="C206" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B207" t="s">
-        <v>559</v>
+        <v>296</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="B208" t="s">
-        <v>246</v>
+        <v>559</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="B209" t="s">
-        <v>308</v>
+        <v>246</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B210" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B211" t="s">
         <v>306</v>
@@ -8865,640 +8874,637 @@
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B212" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>699</v>
+        <v>309</v>
       </c>
       <c r="B213" t="s">
-        <v>697</v>
+        <v>310</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
+        <v>699</v>
+      </c>
+      <c r="B214" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3">
+      <c r="A215" t="s">
         <v>533</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B215" t="s">
         <v>674</v>
-      </c>
-    </row>
-    <row r="216" spans="1:3">
-      <c r="A216" t="s">
-        <v>516</v>
-      </c>
-      <c r="B216" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>496</v>
+        <v>516</v>
       </c>
       <c r="B217" t="s">
-        <v>318</v>
-      </c>
-      <c r="C217" t="s">
-        <v>585</v>
+        <v>517</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="B218" t="s">
-        <v>569</v>
+        <v>318</v>
+      </c>
+      <c r="C218" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>313</v>
+        <v>503</v>
       </c>
       <c r="B219" t="s">
-        <v>319</v>
-      </c>
-      <c r="C219" t="s">
-        <v>585</v>
+        <v>569</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B220" t="s">
-        <v>320</v>
+        <v>319</v>
+      </c>
+      <c r="C220" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B221" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B222" t="s">
-        <v>560</v>
+        <v>321</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B223" t="s">
-        <v>246</v>
+        <v>560</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B224" t="s">
-        <v>323</v>
-      </c>
-      <c r="C224" t="s">
-        <v>585</v>
+        <v>246</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B225" t="s">
-        <v>325</v>
+        <v>323</v>
+      </c>
+      <c r="C225" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B226" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B227" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B228" t="s">
-        <v>254</v>
+        <v>329</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>700</v>
+        <v>330</v>
       </c>
       <c r="B229" t="s">
-        <v>697</v>
+        <v>254</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
+        <v>700</v>
+      </c>
+      <c r="B230" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3">
+      <c r="A231" t="s">
         <v>532</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>675</v>
-      </c>
-    </row>
-    <row r="232" spans="1:3">
-      <c r="A232" t="s">
-        <v>518</v>
-      </c>
-      <c r="B232" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>498</v>
+        <v>518</v>
       </c>
       <c r="B233" t="s">
-        <v>336</v>
-      </c>
-      <c r="C233" t="s">
-        <v>585</v>
+        <v>519</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="B234" t="s">
-        <v>570</v>
+        <v>336</v>
+      </c>
+      <c r="C234" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>334</v>
+        <v>504</v>
       </c>
       <c r="B235" t="s">
-        <v>337</v>
-      </c>
-      <c r="C235" t="s">
-        <v>585</v>
+        <v>570</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B236" t="s">
-        <v>338</v>
+        <v>337</v>
+      </c>
+      <c r="C236" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>497</v>
+        <v>335</v>
       </c>
       <c r="B237" t="s">
-        <v>561</v>
+        <v>338</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>342</v>
+        <v>497</v>
       </c>
       <c r="B238" t="s">
-        <v>246</v>
+        <v>561</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B239" t="s">
-        <v>339</v>
+        <v>246</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B240" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B241" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B242" t="s">
-        <v>254</v>
+        <v>341</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>701</v>
+        <v>346</v>
       </c>
       <c r="B243" t="s">
-        <v>697</v>
+        <v>254</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
+        <v>701</v>
+      </c>
+      <c r="B244" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3">
+      <c r="A245" t="s">
         <v>531</v>
       </c>
-      <c r="B244" t="s">
+      <c r="B245" t="s">
         <v>676</v>
-      </c>
-    </row>
-    <row r="246" spans="1:3">
-      <c r="A246" t="s">
-        <v>739</v>
-      </c>
-      <c r="B246" t="s">
-        <v>740</v>
-      </c>
-      <c r="C246" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>548</v>
+        <v>739</v>
       </c>
       <c r="B247" t="s">
-        <v>551</v>
+        <v>740</v>
       </c>
       <c r="C247" t="s">
-        <v>583</v>
+        <v>686</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B248" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C248" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>582</v>
+        <v>549</v>
       </c>
       <c r="B249" t="s">
-        <v>596</v>
+        <v>550</v>
+      </c>
+      <c r="C249" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>363</v>
+        <v>582</v>
       </c>
       <c r="B250" t="s">
-        <v>349</v>
+        <v>596</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B251" t="s">
-        <v>350</v>
-      </c>
-      <c r="C251" t="s">
-        <v>585</v>
+        <v>349</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>505</v>
+        <v>364</v>
       </c>
       <c r="B252" t="s">
-        <v>571</v>
+        <v>350</v>
+      </c>
+      <c r="C252" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>365</v>
+        <v>505</v>
       </c>
       <c r="B253" t="s">
-        <v>351</v>
+        <v>571</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B254" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B255" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B256" t="s">
-        <v>354</v>
-      </c>
-      <c r="C256" t="s">
-        <v>585</v>
+        <v>353</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B257" t="s">
-        <v>355</v>
+        <v>354</v>
+      </c>
+      <c r="C257" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B258" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B259" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B260" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B261" t="s">
-        <v>359</v>
-      </c>
-      <c r="C261" t="s">
-        <v>585</v>
+        <v>358</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B262" t="s">
-        <v>360</v>
+        <v>359</v>
+      </c>
+      <c r="C262" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B263" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B264" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
+        <v>376</v>
+      </c>
+      <c r="B265" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3">
+      <c r="A266" t="s">
         <v>530</v>
       </c>
-      <c r="B265" t="s">
+      <c r="B266" t="s">
         <v>660</v>
-      </c>
-    </row>
-    <row r="267" spans="1:3">
-      <c r="A267" t="s">
-        <v>601</v>
-      </c>
-      <c r="B267" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>383</v>
+        <v>601</v>
       </c>
       <c r="B268" t="s">
-        <v>401</v>
+        <v>602</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B269" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B270" t="s">
-        <v>399</v>
-      </c>
-      <c r="C270" t="s">
-        <v>585</v>
+        <v>398</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>506</v>
+        <v>385</v>
       </c>
       <c r="B271" t="s">
-        <v>572</v>
+        <v>399</v>
+      </c>
+      <c r="C271" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>402</v>
+        <v>506</v>
       </c>
       <c r="B272" t="s">
-        <v>400</v>
-      </c>
-      <c r="C272" t="s">
-        <v>585</v>
+        <v>572</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
       <c r="B273" t="s">
-        <v>392</v>
+        <v>400</v>
+      </c>
+      <c r="C273" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>403</v>
+        <v>386</v>
       </c>
       <c r="B274" t="s">
-        <v>393</v>
-      </c>
-      <c r="C274" t="s">
-        <v>562</v>
+        <v>392</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="B275" t="s">
-        <v>394</v>
+        <v>393</v>
+      </c>
+      <c r="C275" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B276" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B277" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B278" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B279" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
+        <v>391</v>
+      </c>
+      <c r="B280" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3">
+      <c r="A281" t="s">
         <v>529</v>
       </c>
-      <c r="B280" t="s">
+      <c r="B281" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
-      <c r="A282" t="s">
+    <row r="283" spans="1:3">
+      <c r="A283" t="s">
         <v>741</v>
       </c>
-      <c r="B282" t="s">
+      <c r="B283" t="s">
         <v>760</v>
       </c>
-      <c r="C282" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="284" spans="1:3">
-      <c r="A284" t="s">
-        <v>737</v>
-      </c>
-      <c r="B284" t="s">
-        <v>738</v>
-      </c>
-      <c r="C284" t="s">
+      <c r="C283" t="s">
         <v>686</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>520</v>
+        <v>737</v>
       </c>
       <c r="B285" t="s">
-        <v>521</v>
+        <v>738</v>
+      </c>
+      <c r="C285" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>409</v>
+        <v>520</v>
       </c>
       <c r="B286" t="s">
-        <v>420</v>
+        <v>521</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B287" t="s">
-        <v>421</v>
-      </c>
-      <c r="C287" t="s">
-        <v>585</v>
+        <v>420</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>573</v>
+        <v>410</v>
       </c>
       <c r="B288" t="s">
-        <v>574</v>
+        <v>421</v>
+      </c>
+      <c r="C288" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>411</v>
+        <v>573</v>
       </c>
       <c r="B289" t="s">
-        <v>422</v>
-      </c>
-      <c r="C289" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B290" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C290" t="s">
         <v>585</v>
@@ -9506,128 +9512,128 @@
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B291" t="s">
-        <v>586</v>
+        <v>423</v>
+      </c>
+      <c r="C291" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B292" t="s">
-        <v>424</v>
+        <v>586</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B293" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B294" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B295" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B296" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B297" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>527</v>
+        <v>419</v>
       </c>
       <c r="B298" t="s">
-        <v>678</v>
+        <v>429</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
+        <v>527</v>
+      </c>
+      <c r="B299" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3">
+      <c r="A300" t="s">
         <v>610</v>
       </c>
-      <c r="B299" t="s">
+      <c r="B300" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="301" spans="1:3">
-      <c r="A301" t="s">
-        <v>522</v>
-      </c>
-      <c r="B301" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>436</v>
+        <v>522</v>
       </c>
       <c r="B302" t="s">
-        <v>447</v>
+        <v>521</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B303" t="s">
-        <v>448</v>
-      </c>
-      <c r="C303" t="s">
-        <v>585</v>
+        <v>447</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>507</v>
+        <v>437</v>
       </c>
       <c r="B304" t="s">
-        <v>575</v>
+        <v>448</v>
+      </c>
+      <c r="C304" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>438</v>
+        <v>507</v>
       </c>
       <c r="B305" t="s">
-        <v>449</v>
-      </c>
-      <c r="C305" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B306" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C306" t="s">
         <v>585</v>
@@ -9635,143 +9641,154 @@
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B307" t="s">
-        <v>587</v>
+        <v>450</v>
+      </c>
+      <c r="C307" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B308" t="s">
-        <v>424</v>
+        <v>587</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B309" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B310" t="s">
-        <v>451</v>
+        <v>425</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B311" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B312" t="s">
-        <v>428</v>
+        <v>452</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B313" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>526</v>
+        <v>446</v>
       </c>
       <c r="B314" t="s">
-        <v>678</v>
+        <v>429</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
+        <v>526</v>
+      </c>
+      <c r="B315" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3">
+      <c r="A316" t="s">
         <v>617</v>
       </c>
-      <c r="B315" t="s">
+      <c r="B316" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="317" spans="1:3">
-      <c r="A317" t="s">
-        <v>735</v>
-      </c>
-      <c r="B317" t="s">
-        <v>736</v>
-      </c>
-      <c r="C317" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>430</v>
+        <v>735</v>
       </c>
       <c r="B318" t="s">
-        <v>618</v>
+        <v>736</v>
+      </c>
+      <c r="C318" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B319" t="s">
-        <v>619</v>
-      </c>
-      <c r="C319" t="s">
-        <v>585</v>
+        <v>618</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>508</v>
+        <v>431</v>
       </c>
       <c r="B320" t="s">
-        <v>620</v>
+        <v>619</v>
+      </c>
+      <c r="C320" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="321" spans="1:2">
       <c r="A321" t="s">
-        <v>432</v>
+        <v>508</v>
       </c>
       <c r="B321" t="s">
-        <v>645</v>
+        <v>620</v>
       </c>
     </row>
     <row r="322" spans="1:2">
       <c r="A322" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B322" t="s">
-        <v>621</v>
+        <v>645</v>
       </c>
     </row>
     <row r="323" spans="1:2">
       <c r="A323" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B323" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="324" spans="1:2">
       <c r="A324" t="s">
+        <v>434</v>
+      </c>
+      <c r="B324" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" t="s">
         <v>525</v>
       </c>
-      <c r="B324" t="s">
+      <c r="B325" t="s">
         <v>679</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changes for 1920, 1921 on Dominium Board; added a check for Wait Unit Number and a check for incomplete SSBL - only the first page uploaded
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473B82F7-70B9-4496-BC6B-3FF12C42F1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00960130-42BC-4120-BDBF-74A2E8B5D1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="803">
   <si>
     <t>Name</t>
   </si>
@@ -2437,6 +2437,18 @@
   </si>
   <si>
     <t>None of the "Rent", "Own", or "Other" checkboxes are selected on Housing History Disclosure for this property.</t>
+  </si>
+  <si>
+    <t>AS_WaitUnitNumber</t>
+  </si>
+  <si>
+    <t>The application is currently assigned to a "Wait" unit. The file will need to be assigned to an actual unit number and resubmitted.</t>
+  </si>
+  <si>
+    <t>SSBL_Incomplete</t>
+  </si>
+  <si>
+    <t>Social Security Benefits Letter is incomplete. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -7116,7 +7128,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C325"/>
+  <dimension ref="A1:C327"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7434,158 +7446,158 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>543</v>
+        <v>711</v>
       </c>
       <c r="B39" t="s">
-        <v>662</v>
+        <v>712</v>
+      </c>
+      <c r="C39" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>711</v>
+        <v>799</v>
       </c>
       <c r="B40" t="s">
-        <v>712</v>
+        <v>800</v>
       </c>
       <c r="C40" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>183</v>
-      </c>
-      <c r="B42" t="s">
-        <v>185</v>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>543</v>
+      </c>
+      <c r="B41" t="s">
+        <v>662</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>183</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B46" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B48" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B49" t="s">
-        <v>99</v>
-      </c>
-      <c r="C49" t="s">
-        <v>585</v>
+        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B50" t="s">
-        <v>100</v>
+        <v>99</v>
+      </c>
+      <c r="C50" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>627</v>
+        <v>106</v>
       </c>
       <c r="B51" t="s">
-        <v>628</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>542</v>
+        <v>627</v>
       </c>
       <c r="B52" t="s">
-        <v>663</v>
+        <v>628</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>787</v>
+        <v>542</v>
       </c>
       <c r="B53" t="s">
-        <v>788</v>
+        <v>663</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>787</v>
+      </c>
+      <c r="B54" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
         <v>687</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>688</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C55" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" t="s">
-        <v>184</v>
-      </c>
-      <c r="B56" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>184</v>
       </c>
       <c r="B57" t="s">
-        <v>108</v>
-      </c>
-      <c r="C57" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C58" t="s">
         <v>585</v>
@@ -7593,10 +7605,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C59" t="s">
         <v>585</v>
@@ -7604,10 +7616,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B60" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C60" t="s">
         <v>585</v>
@@ -7615,10 +7627,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B61" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C61" t="s">
         <v>585</v>
@@ -7626,10 +7638,10 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C62" t="s">
         <v>585</v>
@@ -7637,123 +7649,123 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B63" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="C63" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="B64" t="s">
-        <v>789</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B65" t="s">
-        <v>790</v>
-      </c>
-      <c r="C65" t="s">
-        <v>585</v>
+        <v>789</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>576</v>
+        <v>203</v>
       </c>
       <c r="B66" t="s">
-        <v>791</v>
+        <v>790</v>
+      </c>
+      <c r="C66" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>544</v>
+        <v>576</v>
       </c>
       <c r="B67" t="s">
-        <v>545</v>
+        <v>791</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="B68" t="s">
-        <v>792</v>
+        <v>545</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="B69" t="s">
-        <v>664</v>
+        <v>792</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>541</v>
+      </c>
+      <c r="B70" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
         <v>743</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B71" t="s">
         <v>742</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C71" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3">
-      <c r="A72" t="s">
-        <v>158</v>
-      </c>
-      <c r="B72" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>158</v>
       </c>
       <c r="B73" t="s">
-        <v>589</v>
+        <v>121</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B74" t="s">
-        <v>123</v>
+        <v>589</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>629</v>
+        <v>124</v>
       </c>
       <c r="B75" t="s">
-        <v>630</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>753</v>
+        <v>629</v>
       </c>
       <c r="B76" t="s">
-        <v>754</v>
-      </c>
-      <c r="C76" t="s">
-        <v>686</v>
+        <v>630</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>773</v>
+        <v>753</v>
       </c>
       <c r="B77" t="s">
-        <v>774</v>
+        <v>754</v>
       </c>
       <c r="C77" t="s">
         <v>686</v>
@@ -7761,10 +7773,10 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="B78" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C78" t="s">
         <v>686</v>
@@ -7772,10 +7784,10 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B79" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C79" t="s">
         <v>686</v>
@@ -7783,37 +7795,37 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
+        <v>771</v>
+      </c>
+      <c r="B80" t="s">
+        <v>776</v>
+      </c>
+      <c r="C80" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
         <v>540</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B81" t="s">
         <v>665</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82" t="s">
-        <v>186</v>
-      </c>
-      <c r="B82" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>752</v>
+        <v>186</v>
       </c>
       <c r="B83" t="s">
-        <v>767</v>
-      </c>
-      <c r="C83" t="s">
-        <v>686</v>
+        <v>187</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B84" t="s">
-        <v>751</v>
+        <v>767</v>
       </c>
       <c r="C84" t="s">
         <v>686</v>
@@ -7821,80 +7833,80 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>125</v>
+        <v>750</v>
       </c>
       <c r="B85" t="s">
-        <v>127</v>
+        <v>751</v>
+      </c>
+      <c r="C85" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B86" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B87" t="s">
-        <v>590</v>
+        <v>128</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B88" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B89" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B90" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B91" t="s">
-        <v>492</v>
-      </c>
-      <c r="C91" t="s">
-        <v>680</v>
+        <v>593</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B92" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C92" t="s">
-        <v>553</v>
+        <v>680</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B93" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C93" t="s">
         <v>553</v>
@@ -7902,29 +7914,29 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>631</v>
+        <v>144</v>
       </c>
       <c r="B94" t="s">
-        <v>632</v>
+        <v>495</v>
+      </c>
+      <c r="C94" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>713</v>
+        <v>631</v>
       </c>
       <c r="B95" t="s">
-        <v>714</v>
-      </c>
-      <c r="C95" t="s">
-        <v>686</v>
+        <v>632</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>744</v>
+        <v>713</v>
       </c>
       <c r="B96" t="s">
-        <v>745</v>
+        <v>714</v>
       </c>
       <c r="C96" t="s">
         <v>686</v>
@@ -7932,10 +7944,10 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="B97" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C97" t="s">
         <v>686</v>
@@ -7943,10 +7955,10 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B98" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C98" t="s">
         <v>686</v>
@@ -7954,338 +7966,338 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
+        <v>749</v>
+      </c>
+      <c r="B99" t="s">
+        <v>748</v>
+      </c>
+      <c r="C99" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" t="s">
         <v>539</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B100" t="s">
         <v>666</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3">
-      <c r="A101" t="s">
-        <v>147</v>
-      </c>
-      <c r="B101" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B102" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B103" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B104" t="s">
-        <v>577</v>
-      </c>
-      <c r="C104" t="s">
-        <v>685</v>
+        <v>152</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>684</v>
+        <v>145</v>
       </c>
       <c r="B105" t="s">
         <v>577</v>
       </c>
+      <c r="C105" t="s">
+        <v>685</v>
+      </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>146</v>
+        <v>684</v>
       </c>
       <c r="B106" t="s">
-        <v>129</v>
+        <v>577</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="B107" t="s">
-        <v>594</v>
+        <v>129</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B108" t="s">
-        <v>130</v>
+        <v>594</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>633</v>
+        <v>132</v>
       </c>
       <c r="B109" t="s">
-        <v>634</v>
+        <v>130</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
+        <v>633</v>
+      </c>
+      <c r="B110" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" t="s">
         <v>538</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B111" t="s">
         <v>667</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3">
-      <c r="A112" t="s">
-        <v>188</v>
-      </c>
-      <c r="B112" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="B113" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B114" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B115" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B116" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B117" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>624</v>
+        <v>137</v>
       </c>
       <c r="B118" t="s">
-        <v>689</v>
-      </c>
-      <c r="C118" t="s">
-        <v>693</v>
+        <v>157</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>635</v>
+        <v>624</v>
       </c>
       <c r="B119" t="s">
-        <v>636</v>
+        <v>689</v>
+      </c>
+      <c r="C119" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>537</v>
+        <v>635</v>
       </c>
       <c r="B120" t="s">
-        <v>668</v>
+        <v>636</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
+        <v>537</v>
+      </c>
+      <c r="B121" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" t="s">
         <v>715</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B122" t="s">
         <v>716</v>
       </c>
-      <c r="C121" t="s">
+      <c r="C122" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" t="s">
-        <v>704</v>
-      </c>
-      <c r="B123" t="s">
-        <v>705</v>
-      </c>
-      <c r="C123" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B124" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C124" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
-      <c r="A126" t="s">
-        <v>159</v>
-      </c>
-      <c r="B126" t="s">
-        <v>163</v>
+    <row r="125" spans="1:3">
+      <c r="A125" t="s">
+        <v>707</v>
+      </c>
+      <c r="B125" t="s">
+        <v>708</v>
+      </c>
+      <c r="C125" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B127" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B128" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B129" t="s">
-        <v>595</v>
+        <v>165</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>554</v>
+        <v>162</v>
       </c>
       <c r="B130" t="s">
-        <v>732</v>
-      </c>
-      <c r="C130" t="s">
-        <v>733</v>
+        <v>595</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>641</v>
+        <v>554</v>
       </c>
       <c r="B131" t="s">
-        <v>642</v>
+        <v>732</v>
+      </c>
+      <c r="C131" t="s">
+        <v>733</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
+        <v>641</v>
+      </c>
+      <c r="B132" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3">
+      <c r="A133" t="s">
         <v>536</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B133" t="s">
         <v>669</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" t="s">
-        <v>192</v>
-      </c>
-      <c r="B134" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="B135" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B136" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>637</v>
+        <v>167</v>
       </c>
       <c r="B137" t="s">
-        <v>638</v>
+        <v>169</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>535</v>
+        <v>637</v>
       </c>
       <c r="B138" t="s">
-        <v>670</v>
+        <v>638</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
+        <v>535</v>
+      </c>
+      <c r="B139" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
         <v>717</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B140" t="s">
         <v>718</v>
       </c>
-      <c r="C139" t="s">
+      <c r="C140" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3">
-      <c r="A141" t="s">
-        <v>190</v>
-      </c>
-      <c r="B141" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B142" t="s">
-        <v>172</v>
-      </c>
-      <c r="C142" t="s">
-        <v>585</v>
+        <v>191</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B143" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C143" t="s">
         <v>585</v>
@@ -8293,10 +8305,10 @@
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B144" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C144" t="s">
         <v>585</v>
@@ -8304,75 +8316,75 @@
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>201</v>
+        <v>171</v>
       </c>
       <c r="B145" t="s">
-        <v>200</v>
+        <v>174</v>
+      </c>
+      <c r="C145" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B146" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="B147" t="s">
-        <v>177</v>
-      </c>
-      <c r="C147" t="s">
-        <v>585</v>
+        <v>199</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>639</v>
+        <v>176</v>
       </c>
       <c r="B148" t="s">
-        <v>640</v>
+        <v>177</v>
+      </c>
+      <c r="C148" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
+        <v>639</v>
+      </c>
+      <c r="B149" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" t="s">
         <v>524</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B150" t="s">
         <v>671</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3">
-      <c r="A151" t="s">
-        <v>646</v>
-      </c>
-      <c r="B151" t="s">
-        <v>647</v>
-      </c>
-      <c r="C151" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>720</v>
+        <v>646</v>
       </c>
       <c r="B152" t="s">
-        <v>721</v>
+        <v>647</v>
       </c>
       <c r="C152" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="B153" t="s">
-        <v>727</v>
+        <v>721</v>
       </c>
       <c r="C153" t="s">
         <v>686</v>
@@ -8380,10 +8392,10 @@
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>786</v>
+        <v>726</v>
       </c>
       <c r="B154" t="s">
-        <v>795</v>
+        <v>727</v>
       </c>
       <c r="C154" t="s">
         <v>686</v>
@@ -8391,40 +8403,40 @@
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>734</v>
+        <v>786</v>
       </c>
       <c r="B155" t="s">
-        <v>723</v>
+        <v>795</v>
       </c>
       <c r="C155" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
-      <c r="A157" t="s">
-        <v>510</v>
-      </c>
-      <c r="B157" t="s">
-        <v>511</v>
+    <row r="156" spans="1:3">
+      <c r="A156" t="s">
+        <v>734</v>
+      </c>
+      <c r="B156" t="s">
+        <v>723</v>
+      </c>
+      <c r="C156" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>655</v>
+        <v>510</v>
       </c>
       <c r="B158" t="s">
-        <v>659</v>
-      </c>
-      <c r="C158" t="s">
-        <v>657</v>
+        <v>511</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B159" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C159" t="s">
         <v>657</v>
@@ -8432,150 +8444,150 @@
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>240</v>
+        <v>656</v>
       </c>
       <c r="B160" t="s">
-        <v>241</v>
+        <v>658</v>
       </c>
       <c r="C160" t="s">
-        <v>585</v>
+        <v>657</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B161" t="s">
-        <v>243</v>
+        <v>241</v>
+      </c>
+      <c r="C161" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="B162" t="s">
-        <v>557</v>
-      </c>
-      <c r="C162" t="s">
-        <v>644</v>
+        <v>243</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>784</v>
+        <v>256</v>
       </c>
       <c r="B163" t="s">
-        <v>785</v>
+        <v>557</v>
       </c>
       <c r="C163" t="s">
-        <v>686</v>
+        <v>644</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>245</v>
+        <v>784</v>
       </c>
       <c r="B164" t="s">
-        <v>244</v>
+        <v>785</v>
+      </c>
+      <c r="C164" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>500</v>
+        <v>245</v>
       </c>
       <c r="B165" t="s">
-        <v>509</v>
+        <v>244</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>247</v>
+        <v>500</v>
       </c>
       <c r="B166" t="s">
-        <v>246</v>
+        <v>509</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B167" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B168" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B169" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B170" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>300</v>
+        <v>255</v>
       </c>
       <c r="B171" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>347</v>
+        <v>300</v>
       </c>
       <c r="B172" t="s">
-        <v>348</v>
+        <v>246</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>651</v>
+        <v>347</v>
       </c>
       <c r="B173" t="s">
-        <v>652</v>
+        <v>348</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>696</v>
+        <v>651</v>
       </c>
       <c r="B174" t="s">
-        <v>697</v>
+        <v>652</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>768</v>
+        <v>696</v>
       </c>
       <c r="B175" t="s">
-        <v>769</v>
-      </c>
-      <c r="C175" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>782</v>
+        <v>768</v>
       </c>
       <c r="B176" t="s">
-        <v>783</v>
+        <v>769</v>
       </c>
       <c r="C176" t="s">
         <v>686</v>
@@ -8583,298 +8595,301 @@
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
+        <v>782</v>
+      </c>
+      <c r="B177" t="s">
+        <v>783</v>
+      </c>
+      <c r="C177" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3">
+      <c r="A178" t="s">
         <v>523</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>672</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3">
-      <c r="A179" t="s">
-        <v>780</v>
-      </c>
-      <c r="B179" t="s">
-        <v>781</v>
-      </c>
-      <c r="C179" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>512</v>
+        <v>780</v>
       </c>
       <c r="B180" t="s">
-        <v>513</v>
+        <v>781</v>
+      </c>
+      <c r="C180" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
+        <v>512</v>
+      </c>
+      <c r="B181" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3">
+      <c r="A182" t="s">
         <v>257</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B182" t="s">
         <v>260</v>
       </c>
-      <c r="C181" t="s">
+      <c r="C182" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A182" t="s">
+    <row r="183" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A183" t="s">
         <v>259</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B183" t="s">
         <v>558</v>
       </c>
-      <c r="C182" t="s">
+      <c r="C183" t="s">
         <v>690</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3">
-      <c r="A183" t="s">
-        <v>258</v>
-      </c>
-      <c r="B183" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B184" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B185" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B186" t="s">
-        <v>266</v>
-      </c>
-      <c r="C186" t="s">
-        <v>654</v>
+        <v>265</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>501</v>
+        <v>267</v>
       </c>
       <c r="B187" t="s">
-        <v>567</v>
+        <v>266</v>
+      </c>
+      <c r="C187" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>268</v>
+        <v>501</v>
       </c>
       <c r="B188" t="s">
-        <v>269</v>
+        <v>567</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B189" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B190" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B191" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B192" t="s">
-        <v>283</v>
-      </c>
-      <c r="C192" t="s">
-        <v>654</v>
+        <v>284</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B193" t="s">
-        <v>600</v>
+        <v>283</v>
+      </c>
+      <c r="C193" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B194" t="s">
-        <v>282</v>
-      </c>
-      <c r="C194" t="s">
-        <v>654</v>
+        <v>600</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B195" t="s">
-        <v>281</v>
+        <v>282</v>
+      </c>
+      <c r="C195" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
       <c r="B196" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B197" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B198" t="s">
-        <v>303</v>
+        <v>246</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>698</v>
+        <v>302</v>
       </c>
       <c r="B199" t="s">
-        <v>697</v>
+        <v>303</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>534</v>
+        <v>698</v>
       </c>
       <c r="B200" t="s">
-        <v>673</v>
+        <v>697</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
+        <v>534</v>
+      </c>
+      <c r="B201" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3">
+      <c r="A202" t="s">
         <v>691</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B202" t="s">
         <v>692</v>
       </c>
-      <c r="C201" t="s">
+      <c r="C202" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="203" spans="1:3">
-      <c r="A203" t="s">
-        <v>514</v>
-      </c>
-      <c r="B203" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>290</v>
+        <v>514</v>
       </c>
       <c r="B204" t="s">
-        <v>294</v>
-      </c>
-      <c r="C204" t="s">
-        <v>585</v>
+        <v>515</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>502</v>
+        <v>290</v>
       </c>
       <c r="B205" t="s">
-        <v>568</v>
+        <v>294</v>
+      </c>
+      <c r="C205" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>291</v>
+        <v>502</v>
       </c>
       <c r="B206" t="s">
-        <v>295</v>
-      </c>
-      <c r="C206" t="s">
-        <v>585</v>
+        <v>568</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B207" t="s">
-        <v>296</v>
+        <v>295</v>
+      </c>
+      <c r="C207" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B208" t="s">
-        <v>559</v>
+        <v>296</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="B209" t="s">
-        <v>246</v>
+        <v>559</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="B210" t="s">
-        <v>308</v>
+        <v>246</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B211" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B212" t="s">
         <v>306</v>
@@ -8882,640 +8897,637 @@
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B213" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>699</v>
+        <v>309</v>
       </c>
       <c r="B214" t="s">
-        <v>697</v>
+        <v>310</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
+        <v>699</v>
+      </c>
+      <c r="B215" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3">
+      <c r="A216" t="s">
         <v>533</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B216" t="s">
         <v>674</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3">
-      <c r="A217" t="s">
-        <v>516</v>
-      </c>
-      <c r="B217" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>496</v>
+        <v>516</v>
       </c>
       <c r="B218" t="s">
-        <v>318</v>
-      </c>
-      <c r="C218" t="s">
-        <v>585</v>
+        <v>517</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="B219" t="s">
-        <v>569</v>
+        <v>318</v>
+      </c>
+      <c r="C219" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>313</v>
+        <v>503</v>
       </c>
       <c r="B220" t="s">
-        <v>319</v>
-      </c>
-      <c r="C220" t="s">
-        <v>585</v>
+        <v>569</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B221" t="s">
-        <v>320</v>
+        <v>319</v>
+      </c>
+      <c r="C221" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B222" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B223" t="s">
-        <v>560</v>
+        <v>321</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B224" t="s">
-        <v>246</v>
+        <v>560</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B225" t="s">
-        <v>323</v>
-      </c>
-      <c r="C225" t="s">
-        <v>585</v>
+        <v>246</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B226" t="s">
-        <v>325</v>
+        <v>323</v>
+      </c>
+      <c r="C226" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B227" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B228" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B229" t="s">
-        <v>254</v>
+        <v>329</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>700</v>
+        <v>330</v>
       </c>
       <c r="B230" t="s">
-        <v>697</v>
+        <v>254</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
+        <v>700</v>
+      </c>
+      <c r="B231" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3">
+      <c r="A232" t="s">
         <v>532</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B232" t="s">
         <v>675</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3">
-      <c r="A233" t="s">
-        <v>518</v>
-      </c>
-      <c r="B233" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>498</v>
+        <v>518</v>
       </c>
       <c r="B234" t="s">
-        <v>336</v>
-      </c>
-      <c r="C234" t="s">
-        <v>585</v>
+        <v>519</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="B235" t="s">
-        <v>570</v>
+        <v>336</v>
+      </c>
+      <c r="C235" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>334</v>
+        <v>504</v>
       </c>
       <c r="B236" t="s">
-        <v>337</v>
-      </c>
-      <c r="C236" t="s">
-        <v>585</v>
+        <v>570</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B237" t="s">
-        <v>338</v>
+        <v>337</v>
+      </c>
+      <c r="C237" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>497</v>
+        <v>335</v>
       </c>
       <c r="B238" t="s">
-        <v>561</v>
+        <v>338</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>342</v>
+        <v>497</v>
       </c>
       <c r="B239" t="s">
-        <v>246</v>
+        <v>561</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B240" t="s">
-        <v>339</v>
+        <v>246</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B241" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B242" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B243" t="s">
-        <v>254</v>
+        <v>341</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>701</v>
+        <v>346</v>
       </c>
       <c r="B244" t="s">
-        <v>697</v>
+        <v>254</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
+        <v>701</v>
+      </c>
+      <c r="B245" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3">
+      <c r="A246" t="s">
         <v>531</v>
       </c>
-      <c r="B245" t="s">
+      <c r="B246" t="s">
         <v>676</v>
-      </c>
-    </row>
-    <row r="247" spans="1:3">
-      <c r="A247" t="s">
-        <v>739</v>
-      </c>
-      <c r="B247" t="s">
-        <v>740</v>
-      </c>
-      <c r="C247" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>548</v>
+        <v>739</v>
       </c>
       <c r="B248" t="s">
-        <v>551</v>
+        <v>740</v>
       </c>
       <c r="C248" t="s">
-        <v>583</v>
+        <v>686</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B249" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C249" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>582</v>
+        <v>549</v>
       </c>
       <c r="B250" t="s">
-        <v>596</v>
+        <v>550</v>
+      </c>
+      <c r="C250" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>363</v>
+        <v>582</v>
       </c>
       <c r="B251" t="s">
-        <v>349</v>
+        <v>596</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B252" t="s">
-        <v>350</v>
-      </c>
-      <c r="C252" t="s">
-        <v>585</v>
+        <v>349</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>505</v>
+        <v>364</v>
       </c>
       <c r="B253" t="s">
-        <v>571</v>
+        <v>350</v>
+      </c>
+      <c r="C253" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>365</v>
+        <v>505</v>
       </c>
       <c r="B254" t="s">
-        <v>351</v>
+        <v>571</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B255" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B256" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B257" t="s">
-        <v>354</v>
-      </c>
-      <c r="C257" t="s">
-        <v>585</v>
+        <v>353</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B258" t="s">
-        <v>355</v>
+        <v>354</v>
+      </c>
+      <c r="C258" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B259" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B260" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B261" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B262" t="s">
-        <v>359</v>
-      </c>
-      <c r="C262" t="s">
-        <v>585</v>
+        <v>358</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B263" t="s">
-        <v>360</v>
+        <v>359</v>
+      </c>
+      <c r="C263" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B264" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B265" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
+        <v>376</v>
+      </c>
+      <c r="B266" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3">
+      <c r="A267" t="s">
         <v>530</v>
       </c>
-      <c r="B266" t="s">
+      <c r="B267" t="s">
         <v>660</v>
-      </c>
-    </row>
-    <row r="268" spans="1:3">
-      <c r="A268" t="s">
-        <v>601</v>
-      </c>
-      <c r="B268" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>383</v>
+        <v>601</v>
       </c>
       <c r="B269" t="s">
-        <v>401</v>
+        <v>602</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B270" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B271" t="s">
-        <v>399</v>
-      </c>
-      <c r="C271" t="s">
-        <v>585</v>
+        <v>398</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>506</v>
+        <v>385</v>
       </c>
       <c r="B272" t="s">
-        <v>572</v>
+        <v>399</v>
+      </c>
+      <c r="C272" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>402</v>
+        <v>506</v>
       </c>
       <c r="B273" t="s">
-        <v>400</v>
-      </c>
-      <c r="C273" t="s">
-        <v>585</v>
+        <v>572</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
       <c r="B274" t="s">
-        <v>392</v>
+        <v>400</v>
+      </c>
+      <c r="C274" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>403</v>
+        <v>386</v>
       </c>
       <c r="B275" t="s">
-        <v>393</v>
-      </c>
-      <c r="C275" t="s">
-        <v>562</v>
+        <v>392</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="B276" t="s">
-        <v>394</v>
+        <v>393</v>
+      </c>
+      <c r="C276" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B277" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B278" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B279" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B280" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
+        <v>391</v>
+      </c>
+      <c r="B281" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3">
+      <c r="A282" t="s">
         <v>529</v>
       </c>
-      <c r="B281" t="s">
+      <c r="B282" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
-      <c r="A283" t="s">
+    <row r="284" spans="1:3">
+      <c r="A284" t="s">
         <v>741</v>
       </c>
-      <c r="B283" t="s">
+      <c r="B284" t="s">
         <v>760</v>
       </c>
-      <c r="C283" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="285" spans="1:3">
-      <c r="A285" t="s">
-        <v>737</v>
-      </c>
-      <c r="B285" t="s">
-        <v>738</v>
-      </c>
-      <c r="C285" t="s">
+      <c r="C284" t="s">
         <v>686</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>520</v>
+        <v>737</v>
       </c>
       <c r="B286" t="s">
-        <v>521</v>
+        <v>738</v>
+      </c>
+      <c r="C286" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>409</v>
+        <v>520</v>
       </c>
       <c r="B287" t="s">
-        <v>420</v>
+        <v>521</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B288" t="s">
-        <v>421</v>
-      </c>
-      <c r="C288" t="s">
-        <v>585</v>
+        <v>420</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>573</v>
+        <v>410</v>
       </c>
       <c r="B289" t="s">
-        <v>574</v>
+        <v>421</v>
+      </c>
+      <c r="C289" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>411</v>
+        <v>573</v>
       </c>
       <c r="B290" t="s">
-        <v>422</v>
-      </c>
-      <c r="C290" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B291" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C291" t="s">
         <v>585</v>
@@ -9523,117 +9535,120 @@
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B292" t="s">
-        <v>586</v>
+        <v>423</v>
+      </c>
+      <c r="C292" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B293" t="s">
-        <v>424</v>
+        <v>586</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B294" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B295" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B296" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B297" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B298" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>527</v>
+        <v>419</v>
       </c>
       <c r="B299" t="s">
-        <v>678</v>
+        <v>429</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>610</v>
+        <v>801</v>
       </c>
       <c r="B300" t="s">
-        <v>611</v>
+        <v>802</v>
+      </c>
+      <c r="C300" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3">
+      <c r="A301" t="s">
+        <v>527</v>
+      </c>
+      <c r="B301" t="s">
+        <v>678</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>522</v>
+        <v>610</v>
       </c>
       <c r="B302" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3">
-      <c r="A303" t="s">
-        <v>436</v>
-      </c>
-      <c r="B303" t="s">
-        <v>447</v>
+        <v>611</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>437</v>
+        <v>522</v>
       </c>
       <c r="B304" t="s">
-        <v>448</v>
-      </c>
-      <c r="C304" t="s">
-        <v>585</v>
+        <v>521</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>507</v>
+        <v>436</v>
       </c>
       <c r="B305" t="s">
-        <v>575</v>
+        <v>447</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B306" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C306" t="s">
         <v>585</v>
@@ -9641,154 +9656,173 @@
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>439</v>
+        <v>507</v>
       </c>
       <c r="B307" t="s">
-        <v>450</v>
-      </c>
-      <c r="C307" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B308" t="s">
-        <v>587</v>
+        <v>449</v>
+      </c>
+      <c r="C308" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B309" t="s">
-        <v>424</v>
+        <v>450</v>
+      </c>
+      <c r="C309" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B310" t="s">
-        <v>425</v>
+        <v>587</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B311" t="s">
-        <v>451</v>
+        <v>424</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B312" t="s">
-        <v>452</v>
+        <v>425</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B313" t="s">
-        <v>428</v>
+        <v>451</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B314" t="s">
-        <v>429</v>
+        <v>452</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>526</v>
+        <v>445</v>
       </c>
       <c r="B315" t="s">
-        <v>678</v>
+        <v>428</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>617</v>
+        <v>446</v>
       </c>
       <c r="B316" t="s">
-        <v>611</v>
+        <v>429</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3">
+      <c r="A317" t="s">
+        <v>526</v>
+      </c>
+      <c r="B317" t="s">
+        <v>678</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>735</v>
+        <v>617</v>
       </c>
       <c r="B318" t="s">
-        <v>736</v>
-      </c>
-      <c r="C318" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="319" spans="1:3">
-      <c r="A319" t="s">
-        <v>430</v>
-      </c>
-      <c r="B319" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
+        <v>735</v>
+      </c>
+      <c r="B320" t="s">
+        <v>736</v>
+      </c>
+      <c r="C320" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3">
+      <c r="A321" t="s">
+        <v>430</v>
+      </c>
+      <c r="B321" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3">
+      <c r="A322" t="s">
         <v>431</v>
       </c>
-      <c r="B320" t="s">
+      <c r="B322" t="s">
         <v>619</v>
       </c>
-      <c r="C320" t="s">
+      <c r="C322" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="321" spans="1:2">
-      <c r="A321" t="s">
+    <row r="323" spans="1:3">
+      <c r="A323" t="s">
         <v>508</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B323" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="322" spans="1:2">
-      <c r="A322" t="s">
+    <row r="324" spans="1:3">
+      <c r="A324" t="s">
         <v>432</v>
       </c>
-      <c r="B322" t="s">
+      <c r="B324" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="323" spans="1:2">
-      <c r="A323" t="s">
+    <row r="325" spans="1:3">
+      <c r="A325" t="s">
         <v>433</v>
       </c>
-      <c r="B323" t="s">
+      <c r="B325" t="s">
         <v>621</v>
       </c>
     </row>
-    <row r="324" spans="1:2">
-      <c r="A324" t="s">
+    <row r="326" spans="1:3">
+      <c r="A326" t="s">
         <v>434</v>
       </c>
-      <c r="B324" t="s">
+      <c r="B326" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="325" spans="1:2">
-      <c r="A325" t="s">
+    <row r="327" spans="1:3">
+      <c r="A327" t="s">
         <v>525</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B327" t="s">
         <v>679</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changes made to complete story: 1930
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00960130-42BC-4120-BDBF-74A2E8B5D1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5869675-6A0D-4F13-A96D-60FD11FCB6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -1992,9 +1992,6 @@
     <t>AS_HouseholdMemAbsent</t>
   </si>
   <si>
-    <t>household member is temporarily absent, need manual review.</t>
-  </si>
-  <si>
     <t>PS_PaystubsMatchEDC</t>
   </si>
   <si>
@@ -2088,9 +2085,6 @@
     <t>ICW_AssetsOver52787</t>
   </si>
   <si>
-    <t xml:space="preserve">Assets exceed the asset limit, manual review is required. </t>
-  </si>
-  <si>
     <t>TotalAssetsLimit</t>
   </si>
   <si>
@@ -2211,9 +2205,6 @@
     <t>ICW_DominiumEmployee</t>
   </si>
   <si>
-    <t>Applicant is a Dominium employee, manual review is required.</t>
-  </si>
-  <si>
     <t>SupportedIncomeTypes</t>
   </si>
   <si>
@@ -2223,9 +2214,6 @@
     <t>EDC_BothHourlyIncomeAndPSDocumented</t>
   </si>
   <si>
-    <t>Both hourly income and check stub income have been documented on the same Exact Day Calculator. Manual review is required.</t>
-  </si>
-  <si>
     <t>The {0} process has encountered a System Error.\n\nMachine Name: {1} &lt;br&gt;&lt;br&gt;LAN ID: {2} \n\nException Timestamp: {3} &lt;br&gt;&lt;br&gt;Transaction Reference: {4} &lt;br&gt;&lt;br&gt;Exception Message: {5} &lt;br&gt;&lt;br&gt;Exception Source: {6} &lt;br&gt;&lt;br&gt;Action Required: {7}</t>
   </si>
   <si>
@@ -2391,9 +2379,6 @@
     <t>PS_PayIncreaseAcrossPS</t>
   </si>
   <si>
-    <t>Regular pay rate has increase across paystubs. Manual review is required.</t>
-  </si>
-  <si>
     <t>PS_FrequencyError</t>
   </si>
   <si>
@@ -2449,6 +2434,21 @@
   </si>
   <si>
     <t>Social Security Benefits Letter is incomplete. Manual review required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assets exceed the asset limit, manual review required. </t>
+  </si>
+  <si>
+    <t>Applicant is a Dominium employee, manual review required.</t>
+  </si>
+  <si>
+    <t>household member is temporarily absent, needs manual review.</t>
+  </si>
+  <si>
+    <t>Both hourly income and check stub income have been documented on the same Exact Day Calculator. Manual review required.</t>
+  </si>
+  <si>
+    <t>Regular pay rate has increase across paystubs. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -2906,7 +2906,7 @@
         <v>207</v>
       </c>
       <c r="B7" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -2952,10 +2952,10 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B14" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -3197,7 +3197,7 @@
         <v>483</v>
       </c>
       <c r="D42" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="14.25" customHeight="1"/>
@@ -4507,7 +4507,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="B42" t="s">
         <v>480</v>
@@ -4710,10 +4710,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="B20" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -4726,10 +4726,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="B22" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -6112,42 +6112,42 @@
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="B38" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B39" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="B40" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="B41" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="B42" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7154,79 +7154,79 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="B5" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="C5" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="B6" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="C6" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="B7" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="C7" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="B8" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="C8" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="B9" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="C9" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="B10" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="C10" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="B11" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="C11" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7269,7 +7269,7 @@
         <v>205</v>
       </c>
       <c r="C17" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -7282,10 +7282,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B19" t="s">
-        <v>682</v>
+        <v>798</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7293,51 +7293,51 @@
         <v>528</v>
       </c>
       <c r="B20" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="B21" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C21" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B22" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C22" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B23" t="s">
-        <v>723</v>
+        <v>799</v>
       </c>
       <c r="C23" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="B24" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="C24" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -7385,7 +7385,7 @@
         <v>196</v>
       </c>
       <c r="B31" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -7393,7 +7393,7 @@
         <v>197</v>
       </c>
       <c r="B32" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7441,29 +7441,29 @@
         <v>649</v>
       </c>
       <c r="B38" t="s">
-        <v>650</v>
+        <v>800</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="B39" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="C39" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="B40" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="C40" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -7471,7 +7471,7 @@
         <v>543</v>
       </c>
       <c r="B41" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -7562,26 +7562,26 @@
         <v>542</v>
       </c>
       <c r="B53" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="B54" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B55" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C55" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -7671,7 +7671,7 @@
         <v>202</v>
       </c>
       <c r="B65" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -7679,7 +7679,7 @@
         <v>203</v>
       </c>
       <c r="B66" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="C66" t="s">
         <v>585</v>
@@ -7690,7 +7690,7 @@
         <v>576</v>
       </c>
       <c r="B67" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -7706,7 +7706,7 @@
         <v>552</v>
       </c>
       <c r="B69" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -7714,18 +7714,18 @@
         <v>541</v>
       </c>
       <c r="B70" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="B71" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="C71" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -7762,46 +7762,46 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="B77" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="C77" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="B78" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="C78" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="B79" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="C79" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="B80" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="C80" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -7809,7 +7809,7 @@
         <v>540</v>
       </c>
       <c r="B81" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -7822,24 +7822,24 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B84" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="C84" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="B85" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="C85" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -7898,7 +7898,7 @@
         <v>492</v>
       </c>
       <c r="C92" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -7933,46 +7933,46 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B96" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="C96" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="B97" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="C97" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="B98" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="C98" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B99" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="C99" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -7980,7 +7980,7 @@
         <v>539</v>
       </c>
       <c r="B100" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -8015,12 +8015,12 @@
         <v>577</v>
       </c>
       <c r="C105" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B106" t="s">
         <v>577</v>
@@ -8063,7 +8063,7 @@
         <v>538</v>
       </c>
       <c r="B111" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -8119,10 +8119,10 @@
         <v>624</v>
       </c>
       <c r="B119" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C119" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -8138,40 +8138,40 @@
         <v>537</v>
       </c>
       <c r="B121" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B122" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C122" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
+        <v>702</v>
+      </c>
+      <c r="B124" t="s">
+        <v>703</v>
+      </c>
+      <c r="C124" t="s">
         <v>704</v>
-      </c>
-      <c r="B124" t="s">
-        <v>705</v>
-      </c>
-      <c r="C124" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B125" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C125" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -8211,10 +8211,10 @@
         <v>554</v>
       </c>
       <c r="B131" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="C131" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -8230,7 +8230,7 @@
         <v>536</v>
       </c>
       <c r="B133" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -8270,18 +8270,18 @@
         <v>535</v>
       </c>
       <c r="B139" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="B140" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="C140" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="142" spans="1:3">
@@ -8365,7 +8365,7 @@
         <v>524</v>
       </c>
       <c r="B150" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -8381,46 +8381,46 @@
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B153" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C153" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="B154" t="s">
-        <v>727</v>
+        <v>801</v>
       </c>
       <c r="C154" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="B155" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="C155" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="B156" t="s">
-        <v>723</v>
+        <v>799</v>
       </c>
       <c r="C156" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -8433,24 +8433,24 @@
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B159" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C159" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
+        <v>655</v>
+      </c>
+      <c r="B160" t="s">
+        <v>657</v>
+      </c>
+      <c r="C160" t="s">
         <v>656</v>
-      </c>
-      <c r="B160" t="s">
-        <v>658</v>
-      </c>
-      <c r="C160" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -8485,13 +8485,13 @@
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="B164" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="C164" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -8568,40 +8568,40 @@
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
+        <v>650</v>
+      </c>
+      <c r="B174" t="s">
         <v>651</v>
-      </c>
-      <c r="B174" t="s">
-        <v>652</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B175" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B176" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="C176" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="B177" t="s">
-        <v>783</v>
+        <v>802</v>
       </c>
       <c r="C177" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -8609,18 +8609,18 @@
         <v>523</v>
       </c>
       <c r="B178" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="B180" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="C180" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -8639,7 +8639,7 @@
         <v>260</v>
       </c>
       <c r="C182" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="13.5" customHeight="1">
@@ -8650,7 +8650,7 @@
         <v>558</v>
       </c>
       <c r="C183" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -8685,7 +8685,7 @@
         <v>266</v>
       </c>
       <c r="C187" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -8736,7 +8736,7 @@
         <v>283</v>
       </c>
       <c r="C193" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -8755,7 +8755,7 @@
         <v>282</v>
       </c>
       <c r="C195" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -8792,10 +8792,10 @@
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B200" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -8803,18 +8803,18 @@
         <v>534</v>
       </c>
       <c r="B201" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B202" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C202" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -8913,10 +8913,10 @@
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B215" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="216" spans="1:3">
@@ -8924,7 +8924,7 @@
         <v>533</v>
       </c>
       <c r="B216" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -9042,10 +9042,10 @@
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="B231" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -9053,7 +9053,7 @@
         <v>532</v>
       </c>
       <c r="B232" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -9152,10 +9152,10 @@
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B245" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -9163,18 +9163,18 @@
         <v>531</v>
       </c>
       <c r="B246" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="B248" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="C248" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -9341,7 +9341,7 @@
         <v>530</v>
       </c>
       <c r="B267" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="269" spans="1:3">
@@ -9462,29 +9462,29 @@
         <v>529</v>
       </c>
       <c r="B282" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="B284" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="C284" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="B286" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="C286" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="287" spans="1:3">
@@ -9602,13 +9602,13 @@
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="B300" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="C300" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="301" spans="1:3">
@@ -9616,7 +9616,7 @@
         <v>527</v>
       </c>
       <c r="B301" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="302" spans="1:3">
@@ -9745,7 +9745,7 @@
         <v>526</v>
       </c>
       <c r="B317" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="318" spans="1:3">
@@ -9758,13 +9758,13 @@
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="B320" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="C320" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="321" spans="1:3">
@@ -9823,7 +9823,7 @@
         <v>525</v>
       </c>
       <c r="B327" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes for 1935, 1937 on Dominium Dev Board. Updated the DU for SC to replace the Part B fields even thought the third question in Part A is not answered, added the check for completion inconsistency, and added the check for 0 Annual Income listed on the ICW
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5869675-6A0D-4F13-A96D-60FD11FCB6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690924CF-651C-47AE-9DB5-A81C0F6079F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="808">
   <si>
     <t>Name</t>
   </si>
@@ -264,9 +264,6 @@
     <t>Assets need to be verified</t>
   </si>
   <si>
-    <t>Annual Income is above the Income Limit listed on the ICW.</t>
-  </si>
-  <si>
     <t>The move-in date listed is not in the future.</t>
   </si>
   <si>
@@ -2022,9 +2019,6 @@
     <t>Unable to validate findings for Self-Employment Certification. Needs manual review.</t>
   </si>
   <si>
-    <t>Unable to validate findings for ICW. Needs manual review.</t>
-  </si>
-  <si>
     <t>Unable to validate findings for Application Summary. Needs manual review.</t>
   </si>
   <si>
@@ -2121,9 +2115,6 @@
     <t>ICW_LiveInAttendant</t>
   </si>
   <si>
-    <t>Live-In Attendant documented on the ICW, manual review required.</t>
-  </si>
-  <si>
     <t>PS_MultipleIncomeDocsExists</t>
   </si>
   <si>
@@ -2449,6 +2440,30 @@
   </si>
   <si>
     <t>Regular pay rate has increase across paystubs. Manual review required.</t>
+  </si>
+  <si>
+    <t>Student Certification has inconsistent information. Please review answers in Part A to Part B for consistency.</t>
+  </si>
+  <si>
+    <t>SC_CompletionInconsistency</t>
+  </si>
+  <si>
+    <t>ICW_ZeroAnnualIncome</t>
+  </si>
+  <si>
+    <t>The Anuual Incime is listd as zero. Manual review required.</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Income Calculation Worksheet. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Annual Income is above the Income Limit listed on the Income Calculation Worksheet.</t>
+  </si>
+  <si>
+    <t>Live-In Attendant documented on the Income Calculation Worksheet. Manual review required.</t>
+  </si>
+  <si>
+    <t>Applicant is a Dominium employee. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -2903,210 +2918,210 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B12" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="B14" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B15" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B17" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B20" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B21" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B22" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B23" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B24" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B25" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B26" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B27" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C27" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B28" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
+        <v>310</v>
+      </c>
+      <c r="B29" t="s">
         <v>311</v>
-      </c>
-      <c r="B29" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>331</v>
+      </c>
+      <c r="B30" t="s">
         <v>332</v>
-      </c>
-      <c r="B30" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B31" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
@@ -3119,85 +3134,85 @@
     </row>
     <row r="33" spans="1:4" ht="14.25" customHeight="1">
       <c r="A33" t="s">
+        <v>378</v>
+      </c>
+      <c r="B33" t="s">
         <v>379</v>
-      </c>
-      <c r="B33" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B34" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B35" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="14.25" customHeight="1">
       <c r="A36" t="s">
+        <v>405</v>
+      </c>
+      <c r="B36" t="s">
         <v>406</v>
-      </c>
-      <c r="B36" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="14.25" customHeight="1">
       <c r="A37" t="s">
+        <v>453</v>
+      </c>
+      <c r="B37" t="s">
         <v>454</v>
-      </c>
-      <c r="B37" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B38" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="14.25" customHeight="1">
       <c r="A39" t="s">
+        <v>403</v>
+      </c>
+      <c r="B39" t="s">
         <v>404</v>
-      </c>
-      <c r="B39" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="14.25" customHeight="1">
       <c r="A40" t="s">
+        <v>456</v>
+      </c>
+      <c r="B40" t="s">
         <v>457</v>
-      </c>
-      <c r="B40" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B41" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B42" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D42" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="14.25" customHeight="1"/>
@@ -4179,242 +4194,242 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B1" t="s">
         <v>469</v>
-      </c>
-      <c r="B1" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B4" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B6" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B8" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B9" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B10" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
+        <v>475</v>
+      </c>
+      <c r="B11" t="s">
         <v>476</v>
-      </c>
-      <c r="B11" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B13" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B14" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B15" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
+        <v>478</v>
+      </c>
+      <c r="B16" t="s">
         <v>479</v>
-      </c>
-      <c r="B16" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B17" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B18" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B19" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B20" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B21" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
+        <v>483</v>
+      </c>
+      <c r="B22" t="s">
         <v>484</v>
-      </c>
-      <c r="B22" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B23" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B24" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B25" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B26" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B27" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B28" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B29" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B30" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4422,95 +4437,95 @@
         <v>1040</v>
       </c>
       <c r="B31" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B32" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B33" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B34" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B35" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B36" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B37" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B38" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B39" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B40" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B41" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B42" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
   </sheetData>
@@ -4710,10 +4725,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B20" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -4721,23 +4736,23 @@
         <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="B22" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B23" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5896,90 +5911,90 @@
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B13" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B14" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B16" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B17" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B18" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B19" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B20" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B21" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
@@ -5992,162 +6007,162 @@
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B23" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B24" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B27" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B28" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B29" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B30" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B32" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B33" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B35" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B36" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B37" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="B38" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B39" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="B40" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="B41" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="B42" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7128,7 +7143,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C327"/>
+  <dimension ref="A1:C329"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7146,100 +7161,100 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" t="s">
         <v>194</v>
-      </c>
-      <c r="B3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="B5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="C5" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B6" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="C6" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="B7" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="C7" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="B8" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="C8" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B9" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="C9" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="B10" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C10" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="B11" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="C11" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B13" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
         <v>71</v>
@@ -7247,847 +7262,850 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>805</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>203</v>
+      </c>
+      <c r="B17" t="s">
         <v>204</v>
       </c>
-      <c r="B17" t="s">
-        <v>205</v>
-      </c>
       <c r="C17" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>545</v>
+      </c>
+      <c r="B18" t="s">
         <v>546</v>
-      </c>
-      <c r="B18" t="s">
-        <v>547</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B19" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>528</v>
+        <v>690</v>
       </c>
       <c r="B20" t="s">
-        <v>660</v>
+        <v>806</v>
+      </c>
+      <c r="C20" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>692</v>
+        <v>704</v>
       </c>
       <c r="B21" t="s">
-        <v>693</v>
+        <v>705</v>
       </c>
       <c r="C21" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
       <c r="B22" t="s">
-        <v>708</v>
+        <v>807</v>
       </c>
       <c r="C22" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B23" t="s">
-        <v>799</v>
+        <v>723</v>
       </c>
       <c r="C23" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>722</v>
+        <v>802</v>
       </c>
       <c r="B24" t="s">
-        <v>726</v>
+        <v>803</v>
       </c>
       <c r="C24" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>181</v>
-      </c>
-      <c r="B26" t="s">
-        <v>182</v>
+        <v>682</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>527</v>
+      </c>
+      <c r="B25" t="s">
+        <v>804</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>180</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>181</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>555</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>556</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>554</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>555</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>196</v>
+        <v>81</v>
       </c>
       <c r="B31" t="s">
-        <v>788</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>84</v>
+        <v>196</v>
       </c>
       <c r="B33" t="s">
-        <v>85</v>
+        <v>786</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>625</v>
+        <v>88</v>
       </c>
       <c r="B37" t="s">
-        <v>626</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>649</v>
+        <v>624</v>
       </c>
       <c r="B38" t="s">
-        <v>800</v>
+        <v>625</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>709</v>
+        <v>648</v>
       </c>
       <c r="B39" t="s">
-        <v>710</v>
-      </c>
-      <c r="C39" t="s">
-        <v>684</v>
+        <v>797</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>794</v>
+        <v>706</v>
       </c>
       <c r="B40" t="s">
-        <v>795</v>
+        <v>707</v>
       </c>
       <c r="C40" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>543</v>
+        <v>791</v>
       </c>
       <c r="B41" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>183</v>
-      </c>
-      <c r="B43" t="s">
-        <v>185</v>
+        <v>792</v>
+      </c>
+      <c r="C41" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>542</v>
+      </c>
+      <c r="B42" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>182</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>184</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B47" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
-      </c>
-      <c r="C50" t="s">
-        <v>585</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>98</v>
+      </c>
+      <c r="C51" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>627</v>
+        <v>105</v>
       </c>
       <c r="B52" t="s">
-        <v>628</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>542</v>
+        <v>626</v>
       </c>
       <c r="B53" t="s">
-        <v>662</v>
+        <v>627</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>782</v>
+        <v>541</v>
       </c>
       <c r="B54" t="s">
-        <v>783</v>
+        <v>660</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>685</v>
+        <v>779</v>
       </c>
       <c r="B55" t="s">
-        <v>686</v>
-      </c>
-      <c r="C55" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>683</v>
+      </c>
+      <c r="B56" t="s">
         <v>684</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
-        <v>184</v>
-      </c>
-      <c r="B57" t="s">
-        <v>588</v>
+      <c r="C56" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>183</v>
       </c>
       <c r="B58" t="s">
-        <v>108</v>
-      </c>
-      <c r="C58" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B59" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="C59" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B60" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C60" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B61" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="C61" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B62" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C62" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B63" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C63" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B64" t="s">
-        <v>112</v>
+        <v>110</v>
+      </c>
+      <c r="C64" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>202</v>
+        <v>115</v>
       </c>
       <c r="B65" t="s">
-        <v>784</v>
+        <v>111</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>785</v>
-      </c>
-      <c r="C66" t="s">
-        <v>585</v>
+        <v>781</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>576</v>
+        <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>786</v>
+        <v>782</v>
+      </c>
+      <c r="C67" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>544</v>
+        <v>575</v>
       </c>
       <c r="B68" t="s">
-        <v>545</v>
+        <v>783</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="B69" t="s">
-        <v>787</v>
+        <v>544</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="B70" t="s">
-        <v>663</v>
+        <v>784</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>739</v>
+        <v>540</v>
       </c>
       <c r="B71" t="s">
-        <v>738</v>
-      </c>
-      <c r="C71" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3">
-      <c r="A73" t="s">
-        <v>158</v>
-      </c>
-      <c r="B73" t="s">
-        <v>121</v>
+        <v>661</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>736</v>
+      </c>
+      <c r="B72" t="s">
+        <v>735</v>
+      </c>
+      <c r="C72" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="B74" t="s">
-        <v>589</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B75" t="s">
-        <v>123</v>
+        <v>588</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>629</v>
+        <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>630</v>
+        <v>122</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>749</v>
+        <v>628</v>
       </c>
       <c r="B77" t="s">
-        <v>750</v>
-      </c>
-      <c r="C77" t="s">
-        <v>684</v>
+        <v>629</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>769</v>
+        <v>746</v>
       </c>
       <c r="B78" t="s">
-        <v>770</v>
+        <v>747</v>
       </c>
       <c r="C78" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B79" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="C79" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B80" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="C80" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>540</v>
+        <v>764</v>
       </c>
       <c r="B81" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3">
-      <c r="A83" t="s">
-        <v>186</v>
-      </c>
-      <c r="B83" t="s">
-        <v>187</v>
+        <v>769</v>
+      </c>
+      <c r="C81" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" t="s">
+        <v>539</v>
+      </c>
+      <c r="B82" t="s">
+        <v>662</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>748</v>
+        <v>185</v>
       </c>
       <c r="B84" t="s">
-        <v>763</v>
-      </c>
-      <c r="C84" t="s">
-        <v>684</v>
+        <v>186</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B85" t="s">
-        <v>747</v>
+        <v>760</v>
       </c>
       <c r="C85" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>125</v>
+        <v>743</v>
       </c>
       <c r="B86" t="s">
-        <v>127</v>
+        <v>744</v>
+      </c>
+      <c r="C86" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
+        <v>124</v>
+      </c>
+      <c r="B87" t="s">
         <v>126</v>
-      </c>
-      <c r="B87" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="B88" t="s">
-        <v>590</v>
+        <v>127</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B89" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B90" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B91" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B92" t="s">
-        <v>492</v>
-      </c>
-      <c r="C92" t="s">
-        <v>679</v>
+        <v>592</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B93" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C93" t="s">
-        <v>553</v>
+        <v>677</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B94" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C94" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>631</v>
+        <v>143</v>
       </c>
       <c r="B95" t="s">
-        <v>632</v>
+        <v>494</v>
+      </c>
+      <c r="C95" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>711</v>
+        <v>630</v>
       </c>
       <c r="B96" t="s">
-        <v>712</v>
-      </c>
-      <c r="C96" t="s">
-        <v>684</v>
+        <v>631</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>740</v>
+        <v>708</v>
       </c>
       <c r="B97" t="s">
-        <v>741</v>
+        <v>709</v>
       </c>
       <c r="C97" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="B98" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="C98" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="B99" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="C99" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>539</v>
+        <v>742</v>
       </c>
       <c r="B100" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3">
-      <c r="A102" t="s">
-        <v>147</v>
-      </c>
-      <c r="B102" t="s">
-        <v>150</v>
+        <v>741</v>
+      </c>
+      <c r="C100" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" t="s">
+        <v>538</v>
+      </c>
+      <c r="B101" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B103" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B104" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B105" t="s">
-        <v>577</v>
-      </c>
-      <c r="C105" t="s">
-        <v>683</v>
+        <v>151</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>682</v>
+        <v>144</v>
       </c>
       <c r="B106" t="s">
-        <v>577</v>
+        <v>576</v>
+      </c>
+      <c r="C106" t="s">
+        <v>681</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>146</v>
+        <v>680</v>
       </c>
       <c r="B107" t="s">
-        <v>129</v>
+        <v>576</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B108" t="s">
-        <v>594</v>
+        <v>128</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B109" t="s">
-        <v>130</v>
+        <v>593</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>633</v>
+        <v>131</v>
       </c>
       <c r="B110" t="s">
-        <v>634</v>
+        <v>129</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>538</v>
+        <v>632</v>
       </c>
       <c r="B111" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3">
-      <c r="A113" t="s">
-        <v>188</v>
-      </c>
-      <c r="B113" t="s">
-        <v>189</v>
+        <v>633</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" t="s">
+        <v>537</v>
+      </c>
+      <c r="B112" t="s">
+        <v>664</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>133</v>
+        <v>187</v>
       </c>
       <c r="B114" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B115" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -8095,1735 +8113,1754 @@
         <v>134</v>
       </c>
       <c r="B116" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B117" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>137</v>
+        <v>801</v>
       </c>
       <c r="B118" t="s">
-        <v>157</v>
+        <v>800</v>
+      </c>
+      <c r="C118" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>624</v>
+        <v>135</v>
       </c>
       <c r="B119" t="s">
-        <v>687</v>
-      </c>
-      <c r="C119" t="s">
-        <v>691</v>
+        <v>155</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>635</v>
+        <v>136</v>
       </c>
       <c r="B120" t="s">
-        <v>636</v>
+        <v>156</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>537</v>
+        <v>623</v>
       </c>
       <c r="B121" t="s">
-        <v>667</v>
+        <v>685</v>
+      </c>
+      <c r="C121" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>713</v>
+        <v>634</v>
       </c>
       <c r="B122" t="s">
-        <v>714</v>
-      </c>
-      <c r="C122" t="s">
-        <v>684</v>
+        <v>635</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" t="s">
+        <v>536</v>
+      </c>
+      <c r="B123" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="B124" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="C124" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3">
-      <c r="A125" t="s">
-        <v>705</v>
-      </c>
-      <c r="B125" t="s">
-        <v>706</v>
-      </c>
-      <c r="C125" t="s">
-        <v>704</v>
+        <v>682</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" t="s">
+        <v>699</v>
+      </c>
+      <c r="B126" t="s">
+        <v>700</v>
+      </c>
+      <c r="C126" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>159</v>
+        <v>702</v>
       </c>
       <c r="B127" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3">
-      <c r="A128" t="s">
-        <v>160</v>
-      </c>
-      <c r="B128" t="s">
-        <v>164</v>
+        <v>703</v>
+      </c>
+      <c r="C127" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B129" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B130" t="s">
-        <v>595</v>
+        <v>163</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>554</v>
+        <v>160</v>
       </c>
       <c r="B131" t="s">
-        <v>728</v>
-      </c>
-      <c r="C131" t="s">
-        <v>729</v>
+        <v>164</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>641</v>
+        <v>161</v>
       </c>
       <c r="B132" t="s">
-        <v>642</v>
+        <v>594</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>536</v>
+        <v>553</v>
       </c>
       <c r="B133" t="s">
-        <v>668</v>
+        <v>725</v>
+      </c>
+      <c r="C133" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
+        <v>640</v>
+      </c>
+      <c r="B134" t="s">
+        <v>641</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>192</v>
+        <v>535</v>
       </c>
       <c r="B135" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" t="s">
-        <v>166</v>
-      </c>
-      <c r="B136" t="s">
-        <v>168</v>
+        <v>666</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="B137" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>637</v>
+        <v>165</v>
       </c>
       <c r="B138" t="s">
-        <v>638</v>
+        <v>167</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>535</v>
+        <v>166</v>
       </c>
       <c r="B139" t="s">
-        <v>669</v>
+        <v>168</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>715</v>
+        <v>636</v>
       </c>
       <c r="B140" t="s">
-        <v>716</v>
-      </c>
-      <c r="C140" t="s">
-        <v>684</v>
+        <v>637</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3">
+      <c r="A141" t="s">
+        <v>534</v>
+      </c>
+      <c r="B141" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>190</v>
+        <v>712</v>
       </c>
       <c r="B142" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" t="s">
-        <v>175</v>
-      </c>
-      <c r="B143" t="s">
-        <v>172</v>
-      </c>
-      <c r="C143" t="s">
-        <v>585</v>
+        <v>713</v>
+      </c>
+      <c r="C142" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="B144" t="s">
-        <v>173</v>
-      </c>
-      <c r="C144" t="s">
-        <v>585</v>
+        <v>190</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
+        <v>174</v>
+      </c>
+      <c r="B145" t="s">
         <v>171</v>
       </c>
-      <c r="B145" t="s">
-        <v>174</v>
-      </c>
       <c r="C145" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="B146" t="s">
-        <v>200</v>
+        <v>172</v>
+      </c>
+      <c r="C146" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="B147" t="s">
-        <v>199</v>
+        <v>173</v>
+      </c>
+      <c r="C147" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="B148" t="s">
-        <v>177</v>
-      </c>
-      <c r="C148" t="s">
-        <v>585</v>
+        <v>199</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>639</v>
+        <v>197</v>
       </c>
       <c r="B149" t="s">
-        <v>640</v>
+        <v>198</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>524</v>
+        <v>175</v>
       </c>
       <c r="B150" t="s">
-        <v>670</v>
+        <v>176</v>
+      </c>
+      <c r="C150" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3">
+      <c r="A151" t="s">
+        <v>638</v>
+      </c>
+      <c r="B151" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>646</v>
+        <v>523</v>
       </c>
       <c r="B152" t="s">
-        <v>647</v>
-      </c>
-      <c r="C152" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3">
-      <c r="A153" t="s">
-        <v>718</v>
-      </c>
-      <c r="B153" t="s">
-        <v>719</v>
-      </c>
-      <c r="C153" t="s">
-        <v>684</v>
+        <v>668</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>723</v>
+        <v>645</v>
       </c>
       <c r="B154" t="s">
-        <v>801</v>
+        <v>646</v>
       </c>
       <c r="C154" t="s">
-        <v>684</v>
+        <v>647</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>781</v>
+        <v>715</v>
       </c>
       <c r="B155" t="s">
-        <v>790</v>
+        <v>716</v>
       </c>
       <c r="C155" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>730</v>
+        <v>720</v>
       </c>
       <c r="B156" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C156" t="s">
-        <v>684</v>
+        <v>682</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" t="s">
+        <v>778</v>
+      </c>
+      <c r="B157" t="s">
+        <v>787</v>
+      </c>
+      <c r="C157" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>510</v>
+        <v>727</v>
       </c>
       <c r="B158" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3">
-      <c r="A159" t="s">
-        <v>654</v>
-      </c>
-      <c r="B159" t="s">
-        <v>658</v>
-      </c>
-      <c r="C159" t="s">
-        <v>656</v>
+        <v>796</v>
+      </c>
+      <c r="C158" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>655</v>
+        <v>509</v>
       </c>
       <c r="B160" t="s">
-        <v>657</v>
-      </c>
-      <c r="C160" t="s">
-        <v>656</v>
+        <v>510</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>240</v>
+        <v>653</v>
       </c>
       <c r="B161" t="s">
-        <v>241</v>
+        <v>657</v>
       </c>
       <c r="C161" t="s">
-        <v>585</v>
+        <v>655</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>242</v>
+        <v>654</v>
       </c>
       <c r="B162" t="s">
-        <v>243</v>
+        <v>656</v>
+      </c>
+      <c r="C162" t="s">
+        <v>655</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="B163" t="s">
-        <v>557</v>
+        <v>240</v>
       </c>
       <c r="C163" t="s">
-        <v>644</v>
+        <v>584</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>779</v>
+        <v>241</v>
       </c>
       <c r="B164" t="s">
-        <v>780</v>
-      </c>
-      <c r="C164" t="s">
-        <v>684</v>
+        <v>242</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B165" t="s">
-        <v>244</v>
+        <v>556</v>
+      </c>
+      <c r="C165" t="s">
+        <v>643</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>500</v>
+        <v>776</v>
       </c>
       <c r="B166" t="s">
-        <v>509</v>
+        <v>777</v>
+      </c>
+      <c r="C166" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B167" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>248</v>
+        <v>499</v>
       </c>
       <c r="B168" t="s">
-        <v>250</v>
+        <v>508</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B169" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B170" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B171" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>300</v>
+        <v>252</v>
       </c>
       <c r="B172" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>347</v>
+        <v>254</v>
       </c>
       <c r="B173" t="s">
-        <v>348</v>
+        <v>253</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>650</v>
+        <v>299</v>
       </c>
       <c r="B174" t="s">
-        <v>651</v>
+        <v>245</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>694</v>
+        <v>346</v>
       </c>
       <c r="B175" t="s">
-        <v>695</v>
+        <v>347</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>764</v>
+        <v>649</v>
       </c>
       <c r="B176" t="s">
-        <v>765</v>
-      </c>
-      <c r="C176" t="s">
-        <v>684</v>
+        <v>650</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>778</v>
+        <v>691</v>
       </c>
       <c r="B177" t="s">
-        <v>802</v>
-      </c>
-      <c r="C177" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>523</v>
+        <v>761</v>
       </c>
       <c r="B178" t="s">
-        <v>671</v>
+        <v>762</v>
+      </c>
+      <c r="C178" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3">
+      <c r="A179" t="s">
+        <v>775</v>
+      </c>
+      <c r="B179" t="s">
+        <v>799</v>
+      </c>
+      <c r="C179" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>776</v>
+        <v>522</v>
       </c>
       <c r="B180" t="s">
-        <v>777</v>
-      </c>
-      <c r="C180" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3">
-      <c r="A181" t="s">
-        <v>512</v>
-      </c>
-      <c r="B181" t="s">
-        <v>513</v>
+        <v>669</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>257</v>
+        <v>773</v>
       </c>
       <c r="B182" t="s">
-        <v>260</v>
+        <v>774</v>
       </c>
       <c r="C182" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3" ht="13.5" customHeight="1">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>259</v>
+        <v>511</v>
       </c>
       <c r="B183" t="s">
-        <v>558</v>
-      </c>
-      <c r="C183" t="s">
-        <v>688</v>
+        <v>512</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
+        <v>256</v>
+      </c>
+      <c r="B184" t="s">
+        <v>259</v>
+      </c>
+      <c r="C184" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A185" t="s">
         <v>258</v>
       </c>
-      <c r="B184" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3">
-      <c r="A185" t="s">
-        <v>263</v>
-      </c>
       <c r="B185" t="s">
-        <v>262</v>
+        <v>557</v>
+      </c>
+      <c r="C185" t="s">
+        <v>686</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="B186" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B187" t="s">
-        <v>266</v>
-      </c>
-      <c r="C187" t="s">
-        <v>653</v>
+        <v>261</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>501</v>
+        <v>263</v>
       </c>
       <c r="B188" t="s">
-        <v>567</v>
+        <v>264</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B189" t="s">
-        <v>269</v>
+        <v>265</v>
+      </c>
+      <c r="C189" t="s">
+        <v>652</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>270</v>
+        <v>500</v>
       </c>
       <c r="B190" t="s">
-        <v>271</v>
+        <v>566</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="B191" t="s">
-        <v>285</v>
+        <v>268</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B192" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B193" t="s">
-        <v>283</v>
-      </c>
-      <c r="C193" t="s">
-        <v>653</v>
+        <v>284</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B194" t="s">
-        <v>600</v>
+        <v>283</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B195" t="s">
         <v>282</v>
       </c>
       <c r="C195" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B196" t="s">
-        <v>281</v>
+        <v>599</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="B197" t="s">
-        <v>298</v>
+        <v>281</v>
+      </c>
+      <c r="C197" t="s">
+        <v>652</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="B198" t="s">
-        <v>246</v>
+        <v>280</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="B199" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>696</v>
+        <v>298</v>
       </c>
       <c r="B200" t="s">
-        <v>695</v>
+        <v>245</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>534</v>
+        <v>301</v>
       </c>
       <c r="B201" t="s">
-        <v>672</v>
+        <v>302</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="B202" t="s">
-        <v>690</v>
-      </c>
-      <c r="C202" t="s">
-        <v>684</v>
+        <v>692</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3">
+      <c r="A203" t="s">
+        <v>533</v>
+      </c>
+      <c r="B203" t="s">
+        <v>670</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>514</v>
+        <v>687</v>
       </c>
       <c r="B204" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="205" spans="1:3">
-      <c r="A205" t="s">
-        <v>290</v>
-      </c>
-      <c r="B205" t="s">
-        <v>294</v>
-      </c>
-      <c r="C205" t="s">
-        <v>585</v>
+        <v>688</v>
+      </c>
+      <c r="C204" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
       <c r="B206" t="s">
-        <v>568</v>
+        <v>514</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B207" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C207" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>292</v>
+        <v>501</v>
       </c>
       <c r="B208" t="s">
-        <v>296</v>
+        <v>567</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B209" t="s">
-        <v>559</v>
+        <v>294</v>
+      </c>
+      <c r="C209" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="B210" t="s">
-        <v>246</v>
+        <v>295</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="B211" t="s">
-        <v>308</v>
+        <v>558</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B212" t="s">
-        <v>306</v>
+        <v>245</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B213" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B214" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>697</v>
+        <v>304</v>
       </c>
       <c r="B215" t="s">
-        <v>695</v>
+        <v>305</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>533</v>
+        <v>308</v>
       </c>
       <c r="B216" t="s">
-        <v>673</v>
+        <v>309</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3">
+      <c r="A217" t="s">
+        <v>694</v>
+      </c>
+      <c r="B217" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>516</v>
+        <v>532</v>
       </c>
       <c r="B218" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="219" spans="1:3">
-      <c r="A219" t="s">
-        <v>496</v>
-      </c>
-      <c r="B219" t="s">
-        <v>318</v>
-      </c>
-      <c r="C219" t="s">
-        <v>585</v>
+        <v>671</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
       <c r="B220" t="s">
-        <v>569</v>
+        <v>516</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>313</v>
+        <v>495</v>
       </c>
       <c r="B221" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C221" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>314</v>
+        <v>502</v>
       </c>
       <c r="B222" t="s">
-        <v>320</v>
+        <v>568</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B223" t="s">
-        <v>321</v>
+        <v>318</v>
+      </c>
+      <c r="C223" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B224" t="s">
-        <v>560</v>
+        <v>319</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B225" t="s">
-        <v>246</v>
+        <v>320</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="B226" t="s">
-        <v>323</v>
-      </c>
-      <c r="C226" t="s">
-        <v>585</v>
+        <v>559</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="B227" t="s">
-        <v>325</v>
+        <v>245</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="B228" t="s">
-        <v>326</v>
+        <v>322</v>
+      </c>
+      <c r="C228" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B229" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B230" t="s">
-        <v>254</v>
+        <v>325</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>698</v>
+        <v>327</v>
       </c>
       <c r="B231" t="s">
-        <v>695</v>
+        <v>328</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>532</v>
+        <v>329</v>
       </c>
       <c r="B232" t="s">
-        <v>674</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3">
+      <c r="A233" t="s">
+        <v>695</v>
+      </c>
+      <c r="B233" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>518</v>
+        <v>531</v>
       </c>
       <c r="B234" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
-        <v>498</v>
-      </c>
-      <c r="B235" t="s">
-        <v>336</v>
-      </c>
-      <c r="C235" t="s">
-        <v>585</v>
+        <v>672</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="B236" t="s">
-        <v>570</v>
+        <v>518</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>334</v>
+        <v>497</v>
       </c>
       <c r="B237" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C237" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>335</v>
+        <v>503</v>
       </c>
       <c r="B238" t="s">
-        <v>338</v>
+        <v>569</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>497</v>
+        <v>333</v>
       </c>
       <c r="B239" t="s">
-        <v>561</v>
+        <v>336</v>
+      </c>
+      <c r="C239" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="B240" t="s">
-        <v>246</v>
+        <v>337</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>343</v>
+        <v>496</v>
       </c>
       <c r="B241" t="s">
-        <v>339</v>
+        <v>560</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B242" t="s">
-        <v>340</v>
+        <v>245</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B243" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B244" t="s">
-        <v>254</v>
+        <v>339</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>699</v>
+        <v>344</v>
       </c>
       <c r="B245" t="s">
-        <v>695</v>
+        <v>340</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>531</v>
+        <v>345</v>
       </c>
       <c r="B246" t="s">
-        <v>675</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3">
+      <c r="A247" t="s">
+        <v>696</v>
+      </c>
+      <c r="B247" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>735</v>
+        <v>530</v>
       </c>
       <c r="B248" t="s">
-        <v>736</v>
-      </c>
-      <c r="C248" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="249" spans="1:3">
-      <c r="A249" t="s">
-        <v>548</v>
-      </c>
-      <c r="B249" t="s">
-        <v>551</v>
-      </c>
-      <c r="C249" t="s">
-        <v>583</v>
+        <v>673</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>549</v>
+        <v>732</v>
       </c>
       <c r="B250" t="s">
-        <v>550</v>
+        <v>733</v>
       </c>
       <c r="C250" t="s">
-        <v>584</v>
+        <v>682</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
+        <v>547</v>
+      </c>
+      <c r="B251" t="s">
+        <v>550</v>
+      </c>
+      <c r="C251" t="s">
         <v>582</v>
-      </c>
-      <c r="B251" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>363</v>
+        <v>548</v>
       </c>
       <c r="B252" t="s">
-        <v>349</v>
+        <v>549</v>
+      </c>
+      <c r="C252" t="s">
+        <v>583</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>364</v>
+        <v>581</v>
       </c>
       <c r="B253" t="s">
-        <v>350</v>
-      </c>
-      <c r="C253" t="s">
-        <v>585</v>
+        <v>595</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>505</v>
+        <v>362</v>
       </c>
       <c r="B254" t="s">
-        <v>571</v>
+        <v>348</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B255" t="s">
-        <v>351</v>
+        <v>349</v>
+      </c>
+      <c r="C255" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>366</v>
+        <v>504</v>
       </c>
       <c r="B256" t="s">
-        <v>352</v>
+        <v>570</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B257" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B258" t="s">
-        <v>354</v>
-      </c>
-      <c r="C258" t="s">
-        <v>585</v>
+        <v>351</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B259" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B260" t="s">
-        <v>356</v>
+        <v>353</v>
+      </c>
+      <c r="C260" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B261" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B262" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B263" t="s">
-        <v>359</v>
-      </c>
-      <c r="C263" t="s">
-        <v>585</v>
+        <v>356</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B264" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B265" t="s">
-        <v>361</v>
+        <v>358</v>
+      </c>
+      <c r="C265" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B266" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>530</v>
+        <v>374</v>
       </c>
       <c r="B267" t="s">
-        <v>659</v>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3">
+      <c r="A268" t="s">
+        <v>375</v>
+      </c>
+      <c r="B268" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>601</v>
+        <v>529</v>
       </c>
       <c r="B269" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="270" spans="1:3">
-      <c r="A270" t="s">
-        <v>383</v>
-      </c>
-      <c r="B270" t="s">
-        <v>401</v>
+        <v>658</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>384</v>
+        <v>600</v>
       </c>
       <c r="B271" t="s">
-        <v>398</v>
+        <v>601</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B272" t="s">
-        <v>399</v>
-      </c>
-      <c r="C272" t="s">
-        <v>585</v>
+        <v>400</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>506</v>
+        <v>383</v>
       </c>
       <c r="B273" t="s">
-        <v>572</v>
+        <v>397</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>402</v>
+        <v>384</v>
       </c>
       <c r="B274" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C274" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>386</v>
+        <v>505</v>
       </c>
       <c r="B275" t="s">
-        <v>392</v>
+        <v>571</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B276" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C276" t="s">
-        <v>562</v>
+        <v>584</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B277" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>389</v>
+        <v>402</v>
       </c>
       <c r="B278" t="s">
-        <v>395</v>
+        <v>392</v>
+      </c>
+      <c r="C278" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B279" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B280" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B281" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>529</v>
+        <v>389</v>
       </c>
       <c r="B282" t="s">
-        <v>676</v>
+        <v>396</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3">
+      <c r="A283" t="s">
+        <v>390</v>
+      </c>
+      <c r="B283" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>737</v>
+        <v>528</v>
       </c>
       <c r="B284" t="s">
-        <v>756</v>
-      </c>
-      <c r="C284" t="s">
-        <v>684</v>
+        <v>674</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B286" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="C286" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="287" spans="1:3">
-      <c r="A287" t="s">
-        <v>520</v>
-      </c>
-      <c r="B287" t="s">
-        <v>521</v>
+        <v>682</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>409</v>
+        <v>730</v>
       </c>
       <c r="B288" t="s">
-        <v>420</v>
+        <v>731</v>
+      </c>
+      <c r="C288" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>410</v>
+        <v>519</v>
       </c>
       <c r="B289" t="s">
-        <v>421</v>
-      </c>
-      <c r="C289" t="s">
-        <v>585</v>
+        <v>520</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>573</v>
+        <v>408</v>
       </c>
       <c r="B290" t="s">
-        <v>574</v>
+        <v>419</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B291" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C291" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>412</v>
+        <v>572</v>
       </c>
       <c r="B292" t="s">
-        <v>423</v>
-      </c>
-      <c r="C292" t="s">
-        <v>585</v>
+        <v>573</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="B293" t="s">
-        <v>586</v>
+        <v>421</v>
+      </c>
+      <c r="C293" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B294" t="s">
-        <v>424</v>
+        <v>422</v>
+      </c>
+      <c r="C294" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B295" t="s">
-        <v>425</v>
+        <v>585</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B296" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B297" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B298" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B299" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>796</v>
+        <v>417</v>
       </c>
       <c r="B300" t="s">
-        <v>797</v>
-      </c>
-      <c r="C300" t="s">
-        <v>684</v>
+        <v>427</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>527</v>
+        <v>418</v>
       </c>
       <c r="B301" t="s">
-        <v>677</v>
+        <v>428</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>610</v>
+        <v>793</v>
       </c>
       <c r="B302" t="s">
-        <v>611</v>
+        <v>794</v>
+      </c>
+      <c r="C302" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3">
+      <c r="A303" t="s">
+        <v>526</v>
+      </c>
+      <c r="B303" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>522</v>
+        <v>609</v>
       </c>
       <c r="B304" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="305" spans="1:3">
-      <c r="A305" t="s">
-        <v>436</v>
-      </c>
-      <c r="B305" t="s">
-        <v>447</v>
+        <v>610</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>437</v>
+        <v>521</v>
       </c>
       <c r="B306" t="s">
-        <v>448</v>
-      </c>
-      <c r="C306" t="s">
-        <v>585</v>
+        <v>520</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>507</v>
+        <v>435</v>
       </c>
       <c r="B307" t="s">
-        <v>575</v>
+        <v>446</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B308" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C308" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>439</v>
+        <v>506</v>
       </c>
       <c r="B309" t="s">
-        <v>450</v>
-      </c>
-      <c r="C309" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B310" t="s">
-        <v>587</v>
+        <v>448</v>
+      </c>
+      <c r="C310" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="B311" t="s">
-        <v>424</v>
+        <v>449</v>
+      </c>
+      <c r="C311" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B312" t="s">
-        <v>425</v>
+        <v>586</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B313" t="s">
-        <v>451</v>
+        <v>423</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B314" t="s">
-        <v>452</v>
+        <v>424</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B315" t="s">
-        <v>428</v>
+        <v>450</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B316" t="s">
-        <v>429</v>
+        <v>451</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>526</v>
+        <v>444</v>
       </c>
       <c r="B317" t="s">
-        <v>677</v>
+        <v>427</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>617</v>
+        <v>445</v>
       </c>
       <c r="B318" t="s">
-        <v>611</v>
+        <v>428</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3">
+      <c r="A319" t="s">
+        <v>525</v>
+      </c>
+      <c r="B319" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>731</v>
+        <v>616</v>
       </c>
       <c r="B320" t="s">
-        <v>732</v>
-      </c>
-      <c r="C320" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="321" spans="1:3">
-      <c r="A321" t="s">
-        <v>430</v>
-      </c>
-      <c r="B321" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>431</v>
+        <v>728</v>
       </c>
       <c r="B322" t="s">
-        <v>619</v>
+        <v>729</v>
       </c>
       <c r="C322" t="s">
-        <v>585</v>
+        <v>682</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>508</v>
+        <v>429</v>
       </c>
       <c r="B323" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B324" t="s">
-        <v>645</v>
+        <v>618</v>
+      </c>
+      <c r="C324" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>433</v>
+        <v>507</v>
       </c>
       <c r="B325" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="B326" t="s">
-        <v>622</v>
+        <v>644</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>525</v>
+        <v>432</v>
       </c>
       <c r="B327" t="s">
-        <v>678</v>
+        <v>620</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3">
+      <c r="A328" t="s">
+        <v>433</v>
+      </c>
+      <c r="B328" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3">
+      <c r="A329" t="s">
+        <v>524</v>
+      </c>
+      <c r="B329" t="s">
+        <v>676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update the code for 1984 - added a new asset for the lease up properties, added the login into the flow decision nodes in the process flowchart
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690924CF-651C-47AE-9DB5-A81C0F6079F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{198CEAC1-C507-4E29-B140-6053BAFD6A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="809">
   <si>
     <t>Name</t>
   </si>
@@ -2464,6 +2464,9 @@
   </si>
   <si>
     <t>Applicant is a Dominium employee. Manual review required.</t>
+  </si>
+  <si>
+    <t>LeaseUpProperties</t>
   </si>
 </sst>
 </file>
@@ -6165,7 +6168,14 @@
         <v>770</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="43" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A43" t="s">
+        <v>808</v>
+      </c>
+      <c r="B43" t="s">
+        <v>808</v>
+      </c>
+    </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="46" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
adding an asset for the max retry count for sending images to LLM
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{198CEAC1-C507-4E29-B140-6053BAFD6A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588FDAAA-F777-491B-AFF9-F756F2377036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="810">
   <si>
     <t>Name</t>
   </si>
@@ -2467,6 +2467,9 @@
   </si>
   <si>
     <t>LeaseUpProperties</t>
+  </si>
+  <si>
+    <t>LLM_Extraction_MaxRetryCount</t>
   </si>
 </sst>
 </file>
@@ -5795,7 +5798,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1012"/>
+  <dimension ref="A1:Z1013"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -6002,181 +6005,188 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>809</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>809</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A24" t="s">
         <v>205</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>205</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B24" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>237</v>
+        <v>211</v>
+      </c>
+      <c r="B25" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A27" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>272</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A27" t="s">
-        <v>273</v>
-      </c>
-      <c r="B27" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>330</v>
+        <v>273</v>
       </c>
       <c r="B28" t="s">
-        <v>330</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>489</v>
+        <v>330</v>
       </c>
       <c r="B29" t="s">
-        <v>489</v>
+        <v>330</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>489</v>
+      </c>
+      <c r="B30" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A31" t="s">
         <v>490</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A32" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A32" t="s">
+    <row r="33" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
         <v>579</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A33" s="2" t="s">
+    <row r="34" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>578</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
-        <v>580</v>
-      </c>
-      <c r="B34" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>596</v>
+        <v>580</v>
       </c>
       <c r="B35" t="s">
-        <v>596</v>
+        <v>580</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B36" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>642</v>
+        <v>597</v>
       </c>
       <c r="B37" t="s">
-        <v>642</v>
+        <v>597</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>763</v>
+        <v>642</v>
       </c>
       <c r="B38" t="s">
-        <v>763</v>
+        <v>642</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>679</v>
+        <v>763</v>
       </c>
       <c r="B39" t="s">
-        <v>679</v>
+        <v>763</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>718</v>
+        <v>679</v>
       </c>
       <c r="B40" t="s">
-        <v>718</v>
+        <v>679</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="B41" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>770</v>
+        <v>724</v>
       </c>
       <c r="B42" t="s">
-        <v>770</v>
+        <v>724</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
+        <v>770</v>
+      </c>
+      <c r="B43" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A44" t="s">
         <v>808</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>808</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7145,6 +7155,7 @@
     <row r="1010" ht="14.25" customHeight="1"/>
     <row r="1011" ht="14.25" customHeight="1"/>
     <row r="1012" ht="14.25" customHeight="1"/>
+    <row r="1013" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Parallel Processing for MID
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588FDAAA-F777-491B-AFF9-F756F2377036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAFDBE18-EECC-404B-BEBD-72D93C8F577E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2358,9 +2358,6 @@
     <t>DU_AppCredentials</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>VOE_Exists</t>
   </si>
   <si>
@@ -2470,6 +2467,9 @@
   </si>
   <si>
     <t>LLM_Extraction_MaxRetryCount</t>
+  </si>
+  <si>
+    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2927,7 +2927,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>772</v>
+        <v>809</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4528,7 +4528,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B42" t="s">
         <v>479</v>
@@ -6005,10 +6005,10 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B22" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -6181,10 +6181,10 @@
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B44" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7245,10 +7245,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>788</v>
+      </c>
+      <c r="B10" t="s">
         <v>789</v>
-      </c>
-      <c r="B10" t="s">
-        <v>790</v>
       </c>
       <c r="C10" t="s">
         <v>682</v>
@@ -7294,7 +7294,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7321,7 +7321,7 @@
         <v>678</v>
       </c>
       <c r="B19" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7329,7 +7329,7 @@
         <v>690</v>
       </c>
       <c r="B20" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="C20" t="s">
         <v>682</v>
@@ -7351,7 +7351,7 @@
         <v>717</v>
       </c>
       <c r="B22" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C22" t="s">
         <v>682</v>
@@ -7370,10 +7370,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>801</v>
+      </c>
+      <c r="B24" t="s">
         <v>802</v>
-      </c>
-      <c r="B24" t="s">
-        <v>803</v>
       </c>
       <c r="C24" t="s">
         <v>682</v>
@@ -7384,7 +7384,7 @@
         <v>527</v>
       </c>
       <c r="B25" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7432,7 +7432,7 @@
         <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7440,7 +7440,7 @@
         <v>196</v>
       </c>
       <c r="B33" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7488,7 +7488,7 @@
         <v>648</v>
       </c>
       <c r="B39" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -7504,10 +7504,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>790</v>
+      </c>
+      <c r="B41" t="s">
         <v>791</v>
-      </c>
-      <c r="B41" t="s">
-        <v>792</v>
       </c>
       <c r="C41" t="s">
         <v>682</v>
@@ -7614,10 +7614,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>778</v>
+      </c>
+      <c r="B55" t="s">
         <v>779</v>
-      </c>
-      <c r="B55" t="s">
-        <v>780</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -7718,7 +7718,7 @@
         <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -7726,7 +7726,7 @@
         <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C67" t="s">
         <v>584</v>
@@ -7737,7 +7737,7 @@
         <v>575</v>
       </c>
       <c r="B68" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -7753,7 +7753,7 @@
         <v>551</v>
       </c>
       <c r="B70" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -8147,10 +8147,10 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B118" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="C118" t="s">
         <v>682</v>
@@ -8453,7 +8453,7 @@
         <v>720</v>
       </c>
       <c r="B156" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="C156" t="s">
         <v>682</v>
@@ -8461,10 +8461,10 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B157" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C157" t="s">
         <v>682</v>
@@ -8475,7 +8475,7 @@
         <v>727</v>
       </c>
       <c r="B158" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="C158" t="s">
         <v>682</v>
@@ -8543,10 +8543,10 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
+        <v>775</v>
+      </c>
+      <c r="B166" t="s">
         <v>776</v>
-      </c>
-      <c r="B166" t="s">
-        <v>777</v>
       </c>
       <c r="C166" t="s">
         <v>682</v>
@@ -8653,10 +8653,10 @@
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B179" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C179" t="s">
         <v>682</v>
@@ -8672,10 +8672,10 @@
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
+        <v>772</v>
+      </c>
+      <c r="B182" t="s">
         <v>773</v>
-      </c>
-      <c r="B182" t="s">
-        <v>774</v>
       </c>
       <c r="C182" t="s">
         <v>682</v>
@@ -9660,10 +9660,10 @@
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
+        <v>792</v>
+      </c>
+      <c r="B302" t="s">
         <v>793</v>
-      </c>
-      <c r="B302" t="s">
-        <v>794</v>
       </c>
       <c r="C302" t="s">
         <v>682</v>

</xml_diff>

<commit_message>
I have updated DU timeout with Asset value
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37D6742-EEE1-4EC7-B040-D1D5427D26BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A2AB0C-B3D2-4211-A151-B10E8F42CA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="810">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="814">
   <si>
     <t>Name</t>
   </si>
@@ -2470,6 +2470,18 @@
   </si>
   <si>
     <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>ShortTimeDelay</t>
+  </si>
+  <si>
+    <t>MediumTimeDelay</t>
+  </si>
+  <si>
+    <t>LongTimeDelay</t>
+  </si>
+  <si>
+    <t>DU_TimeOut</t>
   </si>
 </sst>
 </file>
@@ -6187,10 +6199,38 @@
         <v>807</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
+        <v>810</v>
+      </c>
+      <c r="B45" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A46" t="s">
+        <v>811</v>
+      </c>
+      <c r="B46" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A47" t="s">
+        <v>812</v>
+      </c>
+      <c r="B47" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A48" t="s">
+        <v>813</v>
+      </c>
+      <c r="B48" t="s">
+        <v>813</v>
+      </c>
+    </row>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
     <row r="51" ht="14.25" customHeight="1"/>

</xml_diff>